<commit_message>
fix: restore corrected ETL files and standardizer improvements
</commit_message>
<xml_diff>
--- a/test_openalex.xlsx
+++ b/test_openalex.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z51"/>
+  <dimension ref="A1:Y51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,35 +526,30 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>AU_CO</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PMID</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>PMID</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>SR</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>SR</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SR_FULL</t>
         </is>
@@ -590,7 +585,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>63726</v>
+        <v>63729</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -634,33 +629,28 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>['FR', 'JP', 'DE', 'CA', 'US']</t>
+          <t>['https://openalex.org/W1496508106', 'https://openalex.org/W1571024744', 'https://openalex.org/W2024933578', 'https://openalex.org/W2035776949', 'https://openalex.org/W2040387238', 'https://openalex.org/W2047804403', 'https://openalex.org/W2063978378', 'https://openalex.org/W2097360283', 'https://openalex.org/W2097850441', 'https://openalex.org/W2118585731', 'https://openalex.org/W2146292423', 'https://openalex.org/W2152799677', 'https://openalex.org/W2153635508']</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>['Chang C, 2011, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Friedman J, 2010, PUBMED', 'Walt S, 2011, COMPUTING IN SCIENCE &amp; ENGINEERING', 'Efron B, 2004, THE ANNALS OF STATISTICS', 'Fan R, 2008, ', 'Guyon I, 2004, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Hanke M, 2009, NEUROINFORMATICS', 'Rokhlin V, 2009, SIAM JOURNAL ON MATRIX ANALYSIS AND APPLICATIONS', 'Omohundro S, 2009, ', 'Sören S, 2010, MAX PLANCK INSTITUTE FOR PLASMA PHYSICS', 'Michel V, 2011, PATTERN RECOGNITION', 'Zito T, 2008, FRONTIERS IN NEUROINFORMATICS', 'Dubois P, 2007, COMPUTING IN SCIENCE &amp; ENGINEERING']</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Fabián Pedregosa, 2012, arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Pedregosa F, 2012, ARXIV (CORNELL UNIVERSITY)</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>Pedregosa F, 2012, ARXIV (CORNELL UNIVERSITY)</t>
+          <t>Fabián Pedregosa, 2012, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -760,25 +750,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>NA, 1989, Choice Reviews Online</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>NA, 1989, CHOICE REVIEWS ONLINE</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>NA, 1989, CHOICE REVIEWS ONLINE</t>
+          <t>NA, 1989, Choice Reviews Online</t>
         </is>
       </c>
     </row>
@@ -848,7 +833,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>['AU']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -856,25 +841,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">J. R. Quinlan, 1992, </t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quinlan J, 1992, </t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quinlan J, 1992, </t>
+          <t xml:space="preserve">J. R. Quinlan, 1992, </t>
         </is>
       </c>
     </row>
@@ -956,25 +936,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Arthur Asuncion, 2007, Medical Entomology and Zoology</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Asuncion A, 2007, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Asuncion A, 2007, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
+          <t>Arthur Asuncion, 2007, Medical Entomology and Zoology</t>
         </is>
       </c>
     </row>
@@ -1052,33 +1027,28 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://openalex.org/W23418094', 'https://openalex.org/W24402856', 'https://openalex.org/W28412257', 'https://openalex.org/W43179442', 'https://openalex.org/W64096637', 'https://openalex.org/W66926763', 'https://openalex.org/W69783631', 'https://openalex.org/W122789262', 'https://openalex.org/W123339444', 'https://openalex.org/W138217685', 'https://openalex.org/W149472151', 'https://openalex.org/W173229765', 'https://openalex.org/W187357405', 'https://openalex.org/W586094522', 'https://openalex.org/W589058777', 'https://openalex.org/W1483135265', 'https://openalex.org/W1483679765', 'https://openalex.org/W1492324553', 'https://openalex.org/W1492698999', 'https://openalex.org/W1495859460', 'https://openalex.org/W1500698297', 'https://openalex.org/W1506285740', 'https://openalex.org/W1513366687', 'https://openalex.org/W1516443426', 'https://openalex.org/W1520687314', 'https://openalex.org/W1523856491', 'https://openalex.org/W1524704912', 'https://openalex.org/W1528113134', 'https://openalex.org/W1530010412', 'https://openalex.org/W1533544838', 'https://openalex.org/W1533946607', 'https://openalex.org/W1536719366', 'https://openalex.org/W1550206324', 'https://openalex.org/W1550821944', 'https://openalex.org/W1551066950', 'https://openalex.org/W1553019137', 'https://openalex.org/W1553313034', 'https://openalex.org/W1554663460', 'https://openalex.org/W1555244713', 'https://openalex.org/W1559060276', 'https://openalex.org/W1560107318', 'https://openalex.org/W1563088657', 'https://openalex.org/W1564947197', 'https://openalex.org/W1571836963', 'https://openalex.org/W1572964175', 'https://openalex.org/W1572978214', 'https://openalex.org/W1573228426', 'https://openalex.org/W1576962511', 'https://openalex.org/W1582036668', 'https://openalex.org/W1583700199', 'https://openalex.org/W1584333058', 'https://openalex.org/W1585221258', 'https://openalex.org/W1585610988', 'https://openalex.org/W1585743408', 'https://openalex.org/W1588100052', 'https://openalex.org/W1588282782', 'https://openalex.org/W1597165973', 'https://openalex.org/W1598333443', 'https://openalex.org/W1598696986', 'https://openalex.org/W1600437712', 'https://openalex.org/W1601529450', 'https://openalex.org/W1604345466', 'https://openalex.org/W1605275907', 'https://openalex.org/W1605688901', 'https://openalex.org/W1605957858', 'https://openalex.org/W1619226191', 'https://openalex.org/W1625504505', 'https://openalex.org/W1630964756', 'https://openalex.org/W1641039719', 'https://openalex.org/W1648885110', 'https://openalex.org/W1670263352', 'https://openalex.org/W1673310716', 'https://openalex.org/W1676820704', 'https://openalex.org/W1678889691', 'https://openalex.org/W1679846099', 'https://openalex.org/W1680392829', 'https://openalex.org/W1763728792', 'https://openalex.org/W1781794689', 'https://openalex.org/W1800049145', 'https://openalex.org/W1806329564', 'https://openalex.org/W1817561967', 'https://openalex.org/W1833977909', 'https://openalex.org/W1861764418', 'https://openalex.org/W1881647329', 'https://openalex.org/W1882120692', 'https://openalex.org/W1906182963', 'https://openalex.org/W1907578970', 'https://openalex.org/W1908888846', 'https://openalex.org/W1912123407', 'https://openalex.org/W1932571505', 'https://openalex.org/W1955600018', 'https://openalex.org/W1969482724', 'https://openalex.org/W1978515644', 'https://openalex.org/W1979711143', 'https://openalex.org/W1982161962', 'https://openalex.org/W1985593448', 'https://openalex.org/W1987947967', 'https://openalex.org/W1990748933', 'https://openalex.org/W1995945562', 'https://openalex.org/W2001619934', 'https://openalex.org/W2008906462', 'https://openalex.org/W2014725748', 'https://openalex.org/W2015401436', 'https://openalex.org/W2017337590', 'https://openalex.org/W2019575783', 'https://openalex.org/W2024046085', 'https://openalex.org/W2024646871', 'https://openalex.org/W2024668293', 'https://openalex.org/W2035890032', 'https://openalex.org/W2037603696', 'https://openalex.org/W2037768235', 'https://openalex.org/W2037965136', 'https://openalex.org/W2042385018', 'https://openalex.org/W2048679005', 'https://openalex.org/W2053154970', 'https://openalex.org/W2057720927', 'https://openalex.org/W2058732827', 'https://openalex.org/W2064853889', 'https://openalex.org/W2065861851', 'https://openalex.org/W2066636486', 'https://openalex.org/W2067098334', 'https://openalex.org/W2068337856', 'https://openalex.org/W2073308541', 'https://openalex.org/W2073583237', 'https://openalex.org/W2074610805', 'https://openalex.org/W2075665712', 'https://openalex.org/W2078579128', 'https://openalex.org/W2095749253', 'https://openalex.org/W2095897464', 'https://openalex.org/W2097089247', 'https://openalex.org/W2097569937', 'https://openalex.org/W2100406636', 'https://openalex.org/W2102009083', 'https://openalex.org/W2105494575', 'https://openalex.org/W2105497548', 'https://openalex.org/W2106393550', 'https://openalex.org/W2108949035', 'https://openalex.org/W2110119381', 'https://openalex.org/W2111746072', 'https://openalex.org/W2112076978', 'https://openalex.org/W2112841646', 'https://openalex.org/W2113242816', 'https://openalex.org/W2117812871', 'https://openalex.org/W2118020653', 'https://openalex.org/W2118383892', 'https://openalex.org/W2119821739', 'https://openalex.org/W2119885577', 'https://openalex.org/W2120216197', 'https://openalex.org/W2122111042', 'https://openalex.org/W2122410182', 'https://openalex.org/W2129113961', 'https://openalex.org/W2129249398', 'https://openalex.org/W2132166479', 'https://openalex.org/W2133632100', 'https://openalex.org/W2134696506', 'https://openalex.org/W2138064700', 'https://openalex.org/W2138621811', 'https://openalex.org/W2139059214', 'https://openalex.org/W2140190241', 'https://openalex.org/W2142767931', 'https://openalex.org/W2142819948', 'https://openalex.org/W2142957916', 'https://openalex.org/W2143349571', 'https://openalex.org/W2143426320', 'https://openalex.org/W2144907232', 'https://openalex.org/W2146257637', 'https://openalex.org/W2147492008', 'https://openalex.org/W2147810216', 'https://openalex.org/W2148949939', 'https://openalex.org/W2149706766', 'https://openalex.org/W2153028052', 'https://openalex.org/W2154318594', 'https://openalex.org/W2154642793', 'https://openalex.org/W2156909104', 'https://openalex.org/W2160642098', 'https://openalex.org/W2161077873', 'https://openalex.org/W2163915185', 'https://openalex.org/W2164818318', 'https://openalex.org/W2166559705', 'https://openalex.org/W2167793421', 'https://openalex.org/W2170112109', 'https://openalex.org/W2170654002', 'https://openalex.org/W2170726034', 'https://openalex.org/W2170913656', 'https://openalex.org/W2172162418', 'https://openalex.org/W2172780573', 'https://openalex.org/W2277957941', 'https://openalex.org/W2331052961', 'https://openalex.org/W2621280964', 'https://openalex.org/W2912934387', 'https://openalex.org/W2913066018', 'https://openalex.org/W2914369697', 'https://openalex.org/W2953014340', 'https://openalex.org/W2988864014', 'https://openalex.org/W3017143921', 'https://openalex.org/W3023540311', 'https://openalex.org/W3083113686', 'https://openalex.org/W3085162807', 'https://openalex.org/W3123294050', 'https://openalex.org/W3163638146', 'https://openalex.org/W3193477162', 'https://openalex.org/W3203633735', 'https://openalex.org/W3208887124']</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>['1959- B, 1994, CHOICE REVIEWS ONLINE', 'Cristianini N, 2000, CAMBRIDGE UNIVERSITY PRESS EBOOKS', ', 2014, APPLE ACADEMIC PRESS EBOOKS', 'Agrawal R, 1994, VERY LARGE DATA BASES', 'Wolpert D, 1992, NEURAL NETWORKS', 'Devroye L, 1996, STOCHASTIC MODELLING AND APPLIED PROBABILITY', 'McCallum A, 1998, ', 'Kira K, 1992, ELSEVIER EBOOKS', 'Hall M, 2000, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Egan J, 1975, ', 'Cavnar W, 1994, ', 'Pyle D, 1999, ', 'Kohavi R, 1996, ', 'Frank E, 1998, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Kimball R, 1996, ', 'Zaki M, 1997, ', 'Kushmerick N, 1997, ', 'Cypher A, 1993, ', 'Cheeseman P, 1996, ', 'Shafer J, 1996, ', 'Mehta M, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Wang Y, 1996, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Liu H, 1996, ', 'Almuallim H, 1991, NATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Drucker H, 1997, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Kerber R, 1992, NATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Schapire R, 1997, QUT EPRINTS (QUEENSLAND UNIVERSITY OF TECHNOLOGY)', 'Langley P, 1995, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Kong E, 1995, ELSEVIER EBOOKS', 'Kononenko I, 1995, ', 'Zheng Z, 2000, MACHINE LEARNING', 'Brodley C, 1996, ', 'Ting K, 1997, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Ramon J, 2000, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Almuallim H, 1992, ', 'Webb G, 1999, ', 'Kohavi R, 1996, ', 'Moore A, 1994, ELSEVIER EBOOKS', 'Bigus J, 1996, ', 'Kibler D, 1987, ELSEVIER EBOOKS', 'Omohundro S, 1987, COMPLEX SYSTEMS', 'Dhar V, 1996, ', 'Chevaleyre Y, 2001, LECTURE NOTES IN COMPUTER SCIENCE', 'Ramakrishnan R, 2000, ASSOCIATION FOR COMPUTING MACHINERY EBOOKS', 'Cherkauer K, 1996, ', 'Mann T, 1993, ', 'Holmes G, 1995, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Domingos P, 1997, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Maron O, 1998, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)', 'Giraud-Carrier C, 1996, ', 'Efron B, 1994, ', 'Ester M, 1996, ', 'Fisher R, 1936, ANNALS OF EUGENICS', 'Swets J, 1988, SCIENCE', 'Friedman N, 1997, MACHINE LEARNING', 'Cohen W, 1995, ELSEVIER EBOOKS', 'Dietterich T, 2000, MACHINE LEARNING', 'Fayyad U, 1993, INTERNATIONAL JOINT CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Dietterich T, 1995, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Srikant R, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'John G, 1994, ELSEVIER EBOOKS', 'Pelleg D, 2000, ', 'Dougherty J, 1995, ELSEVIER EBOOKS', 'Quinlan J, 1996, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Piateski G, 1991, MIT PRESS EBOOKS', 'Berry M, 1997, UNIVERSITY OF MARIBOR DIGITAL LIBRARY (UNIVERSITY OF MARIBOR)', 'Kubát M, 1998, MACHINE LEARNING', 'Kass R, 1995, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Sahami M, 1998, ', 'Langley P, 1992, ', 'Freund Y, 1998, ', 'Cleary J, 1995, ELSEVIER EBOOKS', 'Freund Y, 1999, ', 'Kohavi R, 1995, LECTURE NOTES IN COMPUTER SCIENCE', 'Langley P, 1994, ELSEVIER EBOOKS', 'Cendrowska J, 1987, INTERNATIONAL JOURNAL OF MAN-MACHINE STUDIES', 'Beck, 1986, PUBMED', 'Frank E, 1999, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'Cabena P, 1997, UNIVERSITY OF MARIBOR DIGITAL LIBRARY (UNIVERSITY OF MARIBOR)', 'Frank E, 1998, MACHINE LEARNING', 'Breiman L, 1999, MACHINE LEARNING', 'Holmes G, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Appelt D, 1999, AI COMMUNICATIONS', 'Demiröz G, 1997, LECTURE NOTES IN COMPUTER SCIENCE', 'Flach P, 2001, MACHINE LEARNING', 'Brownston L, 1985, CERN DOCUMENT SERVER (EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Moore A, 1998, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Ting K, 1997, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'Kohavi R, 1997, ', 'Oates T, 1997, ', 'Witten I, 1999, ', ', 1996, COMPUTERS &amp; MATHEMATICS WITH APPLICATIONS', 'Saitta L, 1998, MACHINE LEARNING', 'Frank E, 1999, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'RICHARDS D, 1998, INTERNATIONAL JOURNAL OF HUMAN-COMPUTER STUDIES', 'Ricci⋆ F, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Kohavi R, 1995, ', 'John G, 2013, ARXIV (CORNELL UNIVERSITY)', 'Moore A, 2021, ', 'Paynter G, 2000, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'Cohen J, 1960, EDUCATIONAL AND PSYCHOLOGICAL MEASUREMENT', 'Cortes C, 1995, MACHINE LEARNING', 'Kumar D, 1995, CHOICE REVIEWS ONLINE', 'Cover T, 1967, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Brin S, 1998, COMPUTER NETWORKS AND ISDN SYSTEMS', 'Kohavi R, 1997, ARTIFICIAL INTELLIGENCE', 'Sebastiani F, 2002, ACM COMPUTING SURVEYS', 'Freund Y, 1996, ', 'Lawson C, 1995, SOCIETY FOR INDUSTRIAL AND APPLIED MATHEMATICS EBOOKS', 'Friedman J, 2000, THE ANNALS OF STATISTICS', 'Ho T, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Ripley B, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Han J, 2000, ACM SIGMOD RECORD', 'Blum A, 1998, ', 'Stevens S, 1946, SCIENCE', 'Zhang T, 1996, ', 'Cooper G, 1992, MACHINE LEARNING', 'Dietterich T, 1997, ARTIFICIAL INTELLIGENCE', 'Friedman J, 1977, ACM TRANSACTIONS ON MATHEMATICAL SOFTWARE', 'Nigam K, 2000, MACHINE LEARNING', 'Hoerl A, 1970, TECHNOMETRICS', 'Koestler A, 1967, ', 'Schölkopf B, 1999, ', 'Brin S, 1997, ', 'Fisher D, 1987, MACHINE LEARNING', 'Vitter J, 1985, ACM TRANSACTIONS ON MATHEMATICAL SOFTWARE', 'Cessie S, 1992, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Agrawal R, 1993, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Niknian M, 1995, TECHNOMETRICS', 'Hastie T, 1998, THE ANNALS OF STATISTICS', 'Domingos P, 1999, ', 'Nigam K, 2000, ', 'Day W, 1984, JOURNAL OF CLASSIFICATION', 'Hochbaum D, 1985, MATHEMATICS OF OPERATIONS RESEARCH', 'Utgoff P, 1989, MACHINE LEARNING', 'Webb G, 2000, MACHINE LEARNING', 'Marill T, 1963, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Wang J, 2000, COGPRINTS (UNIVERSITY OF SOUTHAMPTON)', 'Langley P, 1995, COMMUNICATIONS OF THE ACM', 'Mitchell T, 1994, COMMUNICATIONS OF THE ACM', 'Aha D, 1992, INTERNATIONAL JOURNAL OF MAN-MACHINE STUDIES', 'Fürnkranz J, 1994, ELSEVIER EBOOKS', 'Liu H, 1997, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Vafaie H, 2003, ', 'Gaines B, 1995, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Wettschereck D, 1995, MACHINE LEARNING', 'Littlestone N, 1990, ', 'Bay S, 1999, INTELLIGENT DATA ANALYSIS', 'Rexine J, 1986, THE AMERICAN JOURNAL OF PHILOLOGY', 'Frank E, 2000, ', ', 1989, CHOICE REVIEWS ONLINE', 'Vapnik V, 1995, ', 'Han J, 2012, CHOICE REVIEWS ONLINE', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Breiman L, 1996, MACHINE LEARNING', 'Quinlan J, 1986, MACHINE LEARNING', 'Agrawal R, 1993, ', 'Duda R, 1973, ', 'Guyon I, 2002, MACHINE LEARNING', 'Kleinberg J, 1999, JOURNAL OF THE ACM', 'Piepel G, 1989, TECHNOMETRICS', 'Hartigan J, 1975, ', 'Ankerst M, 1999, ACM SIGMOD RECORD', 'Heckerman D, 1995, MACHINE LEARNING', 'BAYES, 1958, BIOMETRIKA', 'Chen⋆ M, 1996, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Liu B, 1998, ', 'Yan X, 2003, ', 'Holte R, 1993, MACHINE LEARNING', 'Atkinson A, 1995, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (STATISTICS IN SOCIETY)', 'Dumais S, 1998, ', 'Littlestone N, 1988, MACHINE LEARNING', 'Stone P, 2000, AUTONOMOUS ROBOTS', 'Maron O, 1997, ', 'Breiman L, 1996, MACHINE LEARNING', 'Provost F, 1997, ', 'Witten I, 1999, MORGAN KAUFMANN PUBLISHERS INC. EBOOKS', 'Friedman J, 1996, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Califf M, 1997, ', 'Buntine W, 1992, STATISTICS AND COMPUTING', 'Utgoff P, 1997, MACHINE LEARNING', 'Freitag D, 2000, MACHINE LEARNING', 'Cardie C, 1993, ELSEVIER EBOOKS', 'John G, 1995, ', 'Drummond C, 2000, ', 'Salzberg S, 1991, MACHINE LEARNING', 'Gluck M, 1985, ESCHOLARSHIP (CALIFORNIA DIGITAL LIBRARY)', 'Schölkopf B, 1998, ', 'Huffman S, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Moore A, 2000, ', 'John G, 1997, ', 'Martin B, 1995, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Li M, 1992, JOURNAL OF COMPUTER AND SYSTEM SCIENCES', 'Jabbour K, 1988, IEEE TRANSACTIONS ON POWER SYSTEMS', 'Mooney U, 2000, ', 'Komarek P, 2000, ', 'Gennari J, 1988, ', 'Bengio Y, 1999, ÉRUDIT DOCUMENTS AND DATA REPOSITORY (ÉRUDIT CONSORTIUM, UNIVERSITY OF MONTREAL)', 'Bouckaert R, 1995, DATA ARCHIVING AND NETWORKED SERVICES (DANS)', 'C.J.C. B, 1998, ', ', 2015, ', 'Johns M, 1959, ']</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Ian H. Witten, 2011, Elsevier eBooks</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Witten I, 2011, ELSEVIER EBOOKS</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>Witten I, 2011, ELSEVIER EBOOKS</t>
+          <t>Ian H. Witten, 2011, Elsevier eBooks</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1082,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>22082</v>
+        <v>22083</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1172,33 +1142,28 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>['US', 'GB']</t>
+          <t>['https://openalex.org/W1480376833', 'https://openalex.org/W1496317909', 'https://openalex.org/W2117812871', 'https://openalex.org/W3215037115', 'https://openalex.org/W4232383088', 'https://openalex.org/W4292691288']</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>['Hastie T, 2001, SPRINGER SERIES IN STATISTICS', 'Ripley B, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Robert C, 2004, SPRINGER TEXTS IN STATISTICS', 'Suykens J, 2002, WORLD SCIENTIFIC EBOOKS', 'Waserman L, 2003, ']</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Nasser M. Nasrabadi, 2007, Journal of Electronic Imaging</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Nasrabadi N, 2007, JOURNAL OF ELECTRONIC IMAGING</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>Nasrabadi N, 2007, JOURNAL OF ELECTRONIC IMAGING</t>
+          <t>Nasser M. Nasrabadi, 2007, Journal of Electronic Imaging</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1199,12 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>['David E. Goldberg']</t>
+          <t>['David E. Goldberg', 'David Robson']</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>['David E. Goldberg']</t>
+          <t>['D. Goldberg', 'David Robson']</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1249,7 +1214,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">David E. Goldberg (corresponding author), </t>
+          <t xml:space="preserve">D. Goldberg (corresponding author), </t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1276,25 +1241,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">David E. Goldberg, 1988, </t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Goldberg D, 1988, </t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Goldberg D, 1988, </t>
+          <t xml:space="preserve">David E. Goldberg, 1988, </t>
         </is>
       </c>
     </row>
@@ -1372,23 +1332,18 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">NA, 2007, </t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NA, 2007, </t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2007, </t>
         </is>
@@ -1468,33 +1423,28 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>['DE']</t>
+          <t>['https://openalex.org/W14377099', 'https://openalex.org/W44447720', 'https://openalex.org/W61071295', 'https://openalex.org/W131514509', 'https://openalex.org/W186419298', 'https://openalex.org/W336602872', 'https://openalex.org/W1213006044', 'https://openalex.org/W1484867920', 'https://openalex.org/W1486089539', 'https://openalex.org/W1486164486', 'https://openalex.org/W1496317909', 'https://openalex.org/W1497675750', 'https://openalex.org/W1505043854', 'https://openalex.org/W1506153731', 'https://openalex.org/W1510355813', 'https://openalex.org/W1512098439', 'https://openalex.org/W1512149552', 'https://openalex.org/W1515272691', 'https://openalex.org/W1543996294', 'https://openalex.org/W1549258098', 'https://openalex.org/W1550570395', 'https://openalex.org/W1551209770', 'https://openalex.org/W1554663460', 'https://openalex.org/W1564947197', 'https://openalex.org/W1567512734', 'https://openalex.org/W1571894236', 'https://openalex.org/W1574225613', 'https://openalex.org/W1598589417', 'https://openalex.org/W1601740268', 'https://openalex.org/W1604293137', 'https://openalex.org/W1607751291', 'https://openalex.org/W1618393386', 'https://openalex.org/W1618449801', 'https://openalex.org/W1628829797', 'https://openalex.org/W1633751774', 'https://openalex.org/W1642427530', 'https://openalex.org/W1648445109', 'https://openalex.org/W1654787807', 'https://openalex.org/W1755117326', 'https://openalex.org/W1859781365', 'https://openalex.org/W1963533512', 'https://openalex.org/W1965999112', 'https://openalex.org/W1967396577', 'https://openalex.org/W1975780894', 'https://openalex.org/W1976382401', 'https://openalex.org/W1976625337', 'https://openalex.org/W1978188282', 'https://openalex.org/W1978394996', 'https://openalex.org/W1981025032', 'https://openalex.org/W1982032418', 'https://openalex.org/W1982276155', 'https://openalex.org/W1986280275', 'https://openalex.org/W1995672551', 'https://openalex.org/W1998167411', 'https://openalex.org/W2000241167', 'https://openalex.org/W2003706076', 'https://openalex.org/W2003870625', 'https://openalex.org/W2006314423', 'https://openalex.org/W2008827410', 'https://openalex.org/W2014831690', 'https://openalex.org/W2015904350', 'https://openalex.org/W2018044188', 'https://openalex.org/W2019363670', 'https://openalex.org/W2020999234', 'https://openalex.org/W2023163512', 'https://openalex.org/W2033839039', 'https://openalex.org/W2041863660', 'https://openalex.org/W2047028564', 'https://openalex.org/W2049387919', 'https://openalex.org/W2056735347', 'https://openalex.org/W2062291655', 'https://openalex.org/W2063852603', 'https://openalex.org/W2065540158', 'https://openalex.org/W2069371995', 'https://openalex.org/W2069527924', 'https://openalex.org/W2072555316', 'https://openalex.org/W2078206416', 'https://openalex.org/W2081873601', 'https://openalex.org/W2085877024', 'https://openalex.org/W2087978636', 'https://openalex.org/W2088538739', 'https://openalex.org/W2090102379', 'https://openalex.org/W2090353374', 'https://openalex.org/W2093268114', 'https://openalex.org/W2094169479', 'https://openalex.org/W2094212611', 'https://openalex.org/W2096335861', 'https://openalex.org/W2098115979', 'https://openalex.org/W2098626000', 'https://openalex.org/W2098949458', 'https://openalex.org/W2100136038', 'https://openalex.org/W2101709642', 'https://openalex.org/W2103972570', 'https://openalex.org/W2104533781', 'https://openalex.org/W2106868411', 'https://openalex.org/W2107152312', 'https://openalex.org/W2107636931', 'https://openalex.org/W2107725114', 'https://openalex.org/W2108966602', 'https://openalex.org/W2111176881', 'https://openalex.org/W2111494971', 'https://openalex.org/W2112545207', 'https://openalex.org/W2114229504', 'https://openalex.org/W2114412769', 'https://openalex.org/W2115606304', 'https://openalex.org/W2116723448', 'https://openalex.org/W2117063635', 'https://openalex.org/W2117812871', 'https://openalex.org/W2118195892', 'https://openalex.org/W2123687908', 'https://openalex.org/W2124101779', 'https://openalex.org/W2124225821', 'https://openalex.org/W2126455177', 'https://openalex.org/W2127713198', 'https://openalex.org/W2129564505', 'https://openalex.org/W2129869373', 'https://openalex.org/W2130475491', 'https://openalex.org/W2130859329', 'https://openalex.org/W2137467792', 'https://openalex.org/W2137557016', 'https://openalex.org/W2137956165', 'https://openalex.org/W2139479120', 'https://openalex.org/W2140170995', 'https://openalex.org/W2140251433', 'https://openalex.org/W2141274633', 'https://openalex.org/W2141436719', 'https://openalex.org/W2142182841', 'https://openalex.org/W2142387771', 'https://openalex.org/W2142575165', 'https://openalex.org/W2143022286', 'https://openalex.org/W2143956139', 'https://openalex.org/W2144286620', 'https://openalex.org/W2145295623', 'https://openalex.org/W2146766088', 'https://openalex.org/W2148603752', 'https://openalex.org/W2149417376', 'https://openalex.org/W2149846618', 'https://openalex.org/W2151238122', 'https://openalex.org/W2152701363', 'https://openalex.org/W2152937653', 'https://openalex.org/W2153347097', 'https://openalex.org/W2153756422', 'https://openalex.org/W2156909104', 'https://openalex.org/W2158451137', 'https://openalex.org/W2158529569', 'https://openalex.org/W2160840682', 'https://openalex.org/W2161767008', 'https://openalex.org/W2162114812', 'https://openalex.org/W2163057507', 'https://openalex.org/W2167061265', 'https://openalex.org/W2167986580', 'https://openalex.org/W2168022998', 'https://openalex.org/W2169779569', 'https://openalex.org/W2170076406', 'https://openalex.org/W2170078560', 'https://openalex.org/W2170120409', 'https://openalex.org/W2170334710', 'https://openalex.org/W2171522835', 'https://openalex.org/W2172039283', 'https://openalex.org/W2296319761', 'https://openalex.org/W2408196097', 'https://openalex.org/W2464224693', 'https://openalex.org/W2548695521', 'https://openalex.org/W2554813760', 'https://openalex.org/W2782810849', 'https://openalex.org/W2797583072', 'https://openalex.org/W2798909945', 'https://openalex.org/W2904816695', 'https://openalex.org/W2916304084', 'https://openalex.org/W2989448192', 'https://openalex.org/W3014600732', 'https://openalex.org/W3017143921', 'https://openalex.org/W3023786531', 'https://openalex.org/W3048078645', 'https://openalex.org/W3119264854', 'https://openalex.org/W3127325877', 'https://openalex.org/W3134067276', 'https://openalex.org/W3140968660', 'https://openalex.org/W3148924112', 'https://openalex.org/W3165771198']</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>['1959- B, 1994, CHOICE REVIEWS ONLINE', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Platt J, 1998, THE MIT PRESS EBOOKS', 'Wiener N, 1949, THE MIT PRESS EBOOKS', 'Neal R, 1996, LECTURE NOTES IN STATISTICS', 'Cristianini N, 2000, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Suykens J, 2002, WORLD SCIENTIFIC EBOOKS', 'Devroye L, 1996, STOCHASTIC MODELLING AND APPLIED PROBABILITY', '1950- G, 2004, ELSEVIER EBOOKS', 'Wendland H, 2004, CAMBRIDGE UNIVERSITY PRESS EBOOKS', ', 2000, APPLIED PHYSICS LETTERS', 'Györfi L, 2002, SPRINGER SERIES IN STATISTICS', 'Girosi F, 1995, NEURAL COMPUTATION', 'Bartlett P, 2006, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Geisser S, 1979, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Saunders C, 1998, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Tipping M, 2003, ', 'Smola A, 2000, ', 'Winkler G, 1995, ', 'König H, 1986, OPERATOR THEORY', 'Silverman B, 1984, THE ANNALS OF STATISTICS', 'Seeger M, 2003, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Collobert R, 2000, APPLIED PHYSICS LETTERS', 'Wong E, 1979, ', 'Ritter K, 2000, LECTURE NOTES IN MATHEMATICS', 'Kammler D, 2008, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Teh Y, 2005, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'McAllester D, 2003, MACHINE LEARNING', 'Rasmussen C, 2003, ', 'Gibbs M, 1997, ', 'Seeger M, 2005, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Stitson M, 1998, THE MIT PRESS EBOOKS', 'Grenander U, 1990, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Plaskota L, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Gao F, 2000, THE ANNALS OF STATISTICS', 'Zhu H, 1997, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Silverman B, 1978, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Seeger M, 2004, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Arató M, 1982, LECTURE NOTES IN CONTROL AND INFORMATION SCIENCES', 'Pontil M, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Micchelli C, 1979, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', 'Choi T, 2018, FIGSHARE', 'Cornford D, 2002, JOURNAL OF NONPARAMETRIC STATISTICS', 'Szeliski R, 1987, NATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Grünwald P, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Hawkins D, 1989, COMMUNICATIONS IN STATISTICS - SIMULATION AND COMPUTATION', 'Minka T, 2001, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)', 'Hinton G, 1997, ', 'Neal R, 1997, ARXIV.ORG', 'Mandelbrot B, 1983, AMERICAN JOURNAL OF PHYSICS', 'Geman S, 1984, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Sacks J, 1989, STATISTICAL SCIENCE', 'Hoerl A, 2000, TECHNOMETRICS', 'Aronszajn N, 1950, TRANSACTIONS OF THE AMERICAN MATHEMATICAL SOCIETY', 'Valiant L, 1984, ', 'Arfken G, 1967, AMERICAN JOURNAL OF PHYSICS', 'Green P, 1994, ', ', 1992, CHOICE REVIEWS ONLINE', 'Bishop C, 1998, NEURAL COMPUTATION', 'Kimeldorf G, 1971, JOURNAL OF MATHEMATICAL ANALYSIS AND APPLICATIONS', 'Hand D, 2007, DRUG SAFETY', 'Mazur P, 1959, PHYSICA', 'Zhang T, 2004, THE ANNALS OF STATISTICS', 'Mackay D, 1992, NEURAL COMPUTATION', 'Schoenberg I, 1938, TRANSACTIONS OF THE AMERICAN MATHEMATICAL SOCIETY', 'Diaconis P, 1986, THE ANNALS OF STATISTICS', 'Wahba G, 1985, THE ANNALS OF STATISTICS', 'Schoenberg I, 1964, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Girard A, 2002, ', 'Rasmussen C, 2001, ', 'Solak E, 2002, ', 'O’Sullivan F, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Baxter L, 1996, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES D (THE STATISTICIAN)', 'Mackay D, 2000, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Dawid A, 1976, BIOMETRICS', 'Meir R, 2003, ', 'Cox D, 1984, SIAM JOURNAL ON NUMERICAL ANALYSIS', 'Hansen L, 1997, OPEN SYSTEMS &amp; INFORMATION DYNAMICS', 'Shepp L, 1966, THE ANNALS OF MATHEMATICAL STATISTICS', 'Eskin E, 2002, ', 'Kashyap R, 1981, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Cox D, 1990, THE ANNALS OF STATISTICS', 'Luo Z, 1997, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Williams C, 1998, NEURAL COMPUTATION', 'Freedman D, 1999, THE ANNALS OF STATISTICS', 'Poggio T, 1988, JOURNAL OF COMPLEXITY', 'Tsuda K, 2002, NEURAL COMPUTATION', 'Wahba G, 1995, MONTHLY WEATHER REVIEW', 'Rasmussen C, 2005, ', 'Schwaighofer A, 2002, ', 'Kohn R, 1987, SIAM JOURNAL ON SCIENTIFIC AND STATISTICAL COMPUTING', 'Blight B, 1975, BIOMETRIKA', 'Williams C, 2002, CAMBRIDGE UNIVERSITY ENGINEERING DEPARTMENT PUBLICATIONS DATABASE', 'Wood S, 1998, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Williams C, 2002, NEURAL INFORMATION PROCESSING SYSTEMS', 'Stein M, 1991, ANNALS OF THE INSTITUTE OF STATISTICAL MATHEMATICS', 'Girosi F, 1991, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', 'Thompson P, 1956, TELLUS A DYNAMIC METEOROLOGY AND OCEANOGRAPHY', 'Seeger M, 2003, ERA', 'Vapnik V, 1995, ', 'Wu Y, 1999, TECHNOMETRICS', 'Cressie N, 1992, TERRA NOVA', 'Bell J, 1978, MATHEMATICS OF COMPUTATION', 'Ripley B, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Müller H, 1991, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Rousseeuw P, 1984, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Dickey D, 1991, TECHNOMETRICS', 'Poggio T, 1990, PROCEEDINGS OF THE IEEE', 'Øksendal B, 2003, UNIVERSITEXT', 'Jones D, 2001, JOURNAL OF GLOBAL OPTIMIZATION', 'Williams C, 2000, ', 'Wahba G, 1975, NUMERISCHE MATHEMATIK', 'Duchon J, 1977, LECTURE NOTES IN MATHEMATICS', 'Williams C, 1995, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Cristianini N, 2006, STUDIES IN FUZZINESS AND SOFT COMPUTING', 'Collins M, 2002, THE MIT PRESS EBOOKS', 'Williams C, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Csató L, 2002, NEURAL COMPUTATION', 'Drineas P, 2005, ', ', 2000, APPLIED PHYSICS LETTERS', 'Fine S, 2002, ', 'Herbrich R, 2002, NEURAL INFORMATION PROCESSING SYSTEMS', 'Chu W, 2005, CAMBRIDGE UNIVERSITY ENGINEERING DEPARTMENT PUBLICATIONS DATABASE', 'Farlie D, 1964, OR', 'Smola A, 2000, ', 'Paciorek C, 2003, ', 'Vishwanathan S, 2004, THE MIT PRESS EBOOKS', 'Faul A, 2002, THE MIT PRESS EBOOKS', 'Mackay D, 1999, NEURAL COMPUTATION', 'Simard P, 1991, NEURAL INFORMATION PROCESSING SYSTEMS', 'Opper M, 2000, NEURAL COMPUTATION', 'Ghahramani Z, 2002, NEURAL INFORMATION PROCESSING SYSTEMS', 'Sundararajan S, 2001, NEURAL COMPUTATION', 'Rasmussen C, 2000, NEURAL INFORMATION PROCESSING SYSTEMS', 'Micchelli C, 2004, UCL DISCOVERY (UNIVERSITY COLLEGE LONDON)', 'Zhu J, 2001, ', 'Vijayakumar S, 2002, AUTONOMOUS ROBOTS', 'Murray‐Smith R, 2001, ENLIGHTEN (JURNAL BIMBINGAN DAN KONSELING ISLAM)', 'Sollich P, 2004, ', 'Seeger M, 1999, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', "Sollich P, 1998, RESEARCH PORTAL (KING'S COLLEGE LONDON)", 'Opper M, 1998, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Vivarelli F, 1998, NEURAL INFORMATION PROCESSING SYSTEMS', 'Ferrari‐Trecate G, 1998, NEURAL INFORMATION PROCESSING SYSTEMS', 'Saunders C, 2002, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Malzahn D, 2002, THE MIT PRESS EBOOKS', 'Csató L, 2002, THE MIT PRESS EBOOKS', 'Kuß M, 2005, ', 'Boyd S, 2004, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Golub G, 2012, JOHNS HOPKINS UNIVERSITY PRESS EBOOKS', 'Press W, 1994, ', 'Duda R, 1973, ', 'Kölbig K, 1995, MATHEMATICS OF COMPUTATION', 'Brown R, 1991, BIOMETRICS', ', 2004, CHOICE REVIEWS ONLINE', 'Cox D, 1966, PHYSICS TODAY', 'Ripley B, 1981, ', 'Schölkopf B, 2001, MPG.PURE (MAX PLANCK SOCIETY)', 'Platt J, 2000, THE MIT PRESS EBOOKS', 'Iaglom A, 1987, SPRINGER EBOOKS', 'Lawrence N, 2003, ', 'O’Hagan A, 1978, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Tsokos C, 1992, TECHNOMETRICS', ', 1964, ELSEVIER EBOOKS', 'Goldberg P, 1997, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Seeger M, 2003, JOURNAL OF MACHINE LEARNING RESEARCH', 'Boyle P, 2004, ', 'Berk R, 1996, TECHNOMETRICS', 'Jaakkola T, 1999, ', 'Dym H, 1989, REGIONAL CONFERENCE SERIES IN MATHEMATICS', 'Kailath T, 1971, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Yang C, 2004, ', 'Blake I, 1973, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Watkins C, 2000, THE MIT PRESS EBOOKS', 'Fowlkes C, 2005, ', 'Hájek J, 1958, CZECHOSLOVAK MATHEMATICAL JOURNAL', 'Quiñonero-Candela J, 2004, MPG.PURE (MAX PLANCK SOCIETY)']</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Rasmussen C, 2005, THE MIT PRESS EBOOKS</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>Rasmussen C, 2005, THE MIT PRESS EBOOKS</t>
+          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
         </is>
       </c>
     </row>
@@ -1572,25 +1522,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Murphy K, 2012, </t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Murphy K, 2012, </t>
+          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
         </is>
       </c>
     </row>
@@ -1624,7 +1569,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9550</v>
+        <v>9559</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1684,33 +1629,28 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W99485931', 'https://openalex.org/W1503398984', 'https://openalex.org/W1512585804', 'https://openalex.org/W1554944419', 'https://openalex.org/W1569098853', 'https://openalex.org/W1873763122', 'https://openalex.org/W1970472910', 'https://openalex.org/W1992570774', 'https://openalex.org/W1999352252', 'https://openalex.org/W2006452405', 'https://openalex.org/W2019363670', 'https://openalex.org/W2042469398', 'https://openalex.org/W2047281923', 'https://openalex.org/W2076063813', 'https://openalex.org/W2097381042', 'https://openalex.org/W2100495367', 'https://openalex.org/W2117726420', 'https://openalex.org/W2127180992', 'https://openalex.org/W2132001804', 'https://openalex.org/W2145339207', 'https://openalex.org/W2146774335', 'https://openalex.org/W2151320232', 'https://openalex.org/W2160815625', 'https://openalex.org/W2163605009', 'https://openalex.org/W2174706414', 'https://openalex.org/W2618530766', 'https://openalex.org/W3102480238', 'https://openalex.org/W4214717370', 'https://openalex.org/W4231109964', 'https://openalex.org/W4238893454', 'https://openalex.org/W4244670803', 'https://openalex.org/W4292363360']</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>['Krizhevsky A, 2017, COMMUNICATIONS OF THE ACM', 'Mnih V, 2015, NATURE', 'Sutton R, 1998, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Hinton G, 2006, SCIENCE', 'Hastie T, 2013, ', 'Schmidhuber J, 2014, NEURAL NETWORKS', 'Boyd S, 2011, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Schultz W, 1997, SCIENCE', 'Murphy K, 2012, ', 'Dwork C, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Bengio Y, 2009, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Blei D, 2012, COMMUNICATIONS OF THE ACM', 'Valiant L, 1984, ', 'Valiant L, 1984, COMMUNICATIONS OF THE ACM', 'Taylor M, 2009, JOURNAL OF MACHINE LEARNING RESEARCH', 'Thrun S, 1998, ', 'Sra S, 2011, THE MIT PRESS EBOOKS', 'Mahoney M, 2012, CHAPMAN &amp; HALL/CRC DATA MINING AND KNOWLEDGE DISCOVERY SERIES', 'Kleiner A, 2014, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Wehbe L, 2014, PLOS ONE', 'Duan R, 2014, JOURNAL OF THE ACM', 'Berthet Q, 2013, THE ANNALS OF STATISTICS', 'Blum A, 2013, JOURNAL OF THE ACM', 'Boyd M, 2011, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Chandrasekaran V, 2013, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Duchi J, 2014, JOURNAL OF THE ACM', 'Balcan M, 2012, ARXIV (CORNELL UNIVERSITY)', 'Decatur S, 2000, SIAM JOURNAL ON COMPUTING', 'Yaylalı E, 2011, WILEY ENCYCLOPEDIA OF OPERATIONS RESEARCH AND MANAGEMENT SCIENCE']</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Michael I. Jordan, 2015, Science</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Jordan M, 2015, SCIENCE</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>Jordan M, 2015, SCIENCE</t>
+          <t>Michael I. Jordan, 2015, Science</t>
         </is>
       </c>
     </row>
@@ -1784,23 +1724,18 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">NA, 2006, </t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NA, 2006, </t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2006, </t>
         </is>
@@ -1884,25 +1819,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Catherine Blake, 1998, Medical Entomology and Zoology</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Blake C, 1998, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>Blake C, 1998, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
+          <t>Catherine Blake, 1998, Medical Entomology and Zoology</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1866,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>8215</v>
+        <v>8216</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1988,25 +1918,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>PedregosaFabian, 2011, Journal of Machine Learning Research</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>PedregosaFabian, 2011, JOURNAL OF MACHINE LEARNING RESEARCH</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>PedregosaFabian, 2011, JOURNAL OF MACHINE LEARNING RESEARCH</t>
+          <t>PedregosaFabian, 2011, Journal of Machine Learning Research</t>
         </is>
       </c>
     </row>
@@ -2084,33 +2009,28 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W104184427', 'https://openalex.org/W145476170', 'https://openalex.org/W941230081', 'https://openalex.org/W1442374986', 'https://openalex.org/W1484210532', 'https://openalex.org/W1485981043', 'https://openalex.org/W1493893823', 'https://openalex.org/W1498436455', 'https://openalex.org/W1548328233', 'https://openalex.org/W1598866093', 'https://openalex.org/W1658008008', 'https://openalex.org/W1667652561', 'https://openalex.org/W1869752048', 'https://openalex.org/W1978660892', 'https://openalex.org/W1992479210', 'https://openalex.org/W2041517243', 'https://openalex.org/W2055312318', 'https://openalex.org/W2061570747', 'https://openalex.org/W2066443755', 'https://openalex.org/W2072566913', 'https://openalex.org/W2083842231', 'https://openalex.org/W2099471712', 'https://openalex.org/W2100664567', 'https://openalex.org/W2109722477', 'https://openalex.org/W2117539524', 'https://openalex.org/W2120480077', 'https://openalex.org/W2131400476', 'https://openalex.org/W2131975293', 'https://openalex.org/W2132339004', 'https://openalex.org/W2140833774', 'https://openalex.org/W2141992894', 'https://openalex.org/W2145339207', 'https://openalex.org/W2146757372', 'https://openalex.org/W2160815625', 'https://openalex.org/W2163961697', 'https://openalex.org/W2168231600', 'https://openalex.org/W2173213060', 'https://openalex.org/W2186615578', 'https://openalex.org/W2198403777', 'https://openalex.org/W2259472270', 'https://openalex.org/W2308045930', 'https://openalex.org/W2336650964', 'https://openalex.org/W2339765813', 'https://openalex.org/W2384495648', 'https://openalex.org/W2591588155', 'https://openalex.org/W2949117887', 'https://openalex.org/W2949245006', 'https://openalex.org/W2949501655', 'https://openalex.org/W2949605076', 'https://openalex.org/W2949650786', 'https://openalex.org/W2949888546', 'https://openalex.org/W2950094539', 'https://openalex.org/W2950179405', 'https://openalex.org/W2950577311', 'https://openalex.org/W2951714314', 'https://openalex.org/W2951781666']</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>['Russakovsky O, 2015, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Rumelhart D, 1986, NATURE', 'Mnih V, 2015, NATURE', '淳司 柴, 2017, JOURNAL OF JAPAN SOCIETY FOR FUZZY THEORY AND INTELLIGENT INFORMATICS', 'Dean J, 2008, COMMUNICATIONS OF THE ACM', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Zaharia M, 2012, ', 'Sutskever I, 2013, ', 'Dean J, 2012, ', ', 2000, APPLIED PHYSICS LETTERS', 'Sifis L, 2016, ARXIV (CORNELL UNIVERSITY)', 'Le Q, 2013, ', 'Hindman B, 2011, UC BERKELEY', 'Verma A, 2015, ', 'Karpathy A, 2014, ', 'Chu C, 2007, THE MIT PRESS EBOOKS', 'Jordan M, 1997, ADVANCES IN PSYCHOLOGY', 'Larochelle H, 2009, ', 'Li M, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Burrows M, 2006, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Ragan‐Kelley J, 2013, ', 'Jean S, 2015, ', 'Hinton G, 1989, ESCHOLARSHIP (CALIFORNIA DIGITAL LIBRARY)', 'Li M, 2014, ', 'Yu Y, 2008, ', 'Chilimbi T, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Collobert R, 2002, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Smola A, 2010, PROCEEDINGS OF THE VLDB ENDOWMENT', 'Byrd R, 2012, MATHEMATICAL PROGRAMMING', 'Cui H, 2016, ', 'Heigold G, 2013, ', 'Rossbach C, 2013, ', 'Chung E, 2013, ', 'Ovtcharov K, 2015, ', 'Ioffe S, 2024, ARXIV (CORNELL UNIVERSITY)', 'He K, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chen T, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chetlur S, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Józefowicz R, 2016, ARXIV (CORNELL UNIVERSITY)', 'Ba J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Xinghao P, 2017, ARXIV (CORNELL UNIVERSITY)', 'Szegedy C, 2015, ARXIV (CORNELL UNIVERSITY)', 'Nair A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Vinyals O, 2014, ARXIV (CORNELL UNIVERSITY)', 'Dai A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Crankshaw D, 2014, ARXIV (CORNELL UNIVERSITY)', 'Lavin A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Moritz P, 2015, ARXIV (CORNELL UNIVERSITY)', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Jia Y, 2014, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Szegedy C, 2014, ARXIV (CORNELL UNIVERSITY)', 'Niu F, 2011, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Martı́n Abadi, 2016, arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)</t>
+          <t>Martı́n Abadi, 2016, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2064,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>7890</v>
+        <v>7891</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2204,33 +2124,28 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>['IT']</t>
+          <t>['https://openalex.org/W12876238', 'https://openalex.org/W22906612', 'https://openalex.org/W35304842', 'https://openalex.org/W59979790', 'https://openalex.org/W74894479', 'https://openalex.org/W81384683', 'https://openalex.org/W81511778', 'https://openalex.org/W104970664', 'https://openalex.org/W107306860', 'https://openalex.org/W112196149', 'https://openalex.org/W116328816', 'https://openalex.org/W148103248', 'https://openalex.org/W166124110', 'https://openalex.org/W1482260847', 'https://openalex.org/W1487445520', 'https://openalex.org/W1490175418', 'https://openalex.org/W1493526108', 'https://openalex.org/W1505794130', 'https://openalex.org/W1507179106', 'https://openalex.org/W1508175965', 'https://openalex.org/W1513874326', 'https://openalex.org/W1514707997', 'https://openalex.org/W1520963883', 'https://openalex.org/W1522930027', 'https://openalex.org/W1523389133', 'https://openalex.org/W1523949738', 'https://openalex.org/W1533946607', 'https://openalex.org/W1544227718', 'https://openalex.org/W1547553618', 'https://openalex.org/W1550961891', 'https://openalex.org/W1553682320', 'https://openalex.org/W1556094091', 'https://openalex.org/W1561056154', 'https://openalex.org/W1574901103', 'https://openalex.org/W1576676390', 'https://openalex.org/W1577216492', 'https://openalex.org/W1578881253', 'https://openalex.org/W1591234214', 'https://openalex.org/W1592212241', 'https://openalex.org/W1594962278', 'https://openalex.org/W1597379537', 'https://openalex.org/W1601145406', 'https://openalex.org/W1619226191', 'https://openalex.org/W1620204465', 'https://openalex.org/W1813610639', 'https://openalex.org/W1857571498', 'https://openalex.org/W1907380269', 'https://openalex.org/W1924689489', 'https://openalex.org/W1966065191', 'https://openalex.org/W1969572066', 'https://openalex.org/W1970858159', 'https://openalex.org/W1970974276', 'https://openalex.org/W1971666241', 'https://openalex.org/W1973911615', 'https://openalex.org/W1975496312', 'https://openalex.org/W1977182536', 'https://openalex.org/W1978394996', 'https://openalex.org/W1979648751', 'https://openalex.org/W1980776671', 'https://openalex.org/W1983078185', 'https://openalex.org/W1986913017', 'https://openalex.org/W1988711048', 'https://openalex.org/W1989568037', 'https://openalex.org/W1989738209', 'https://openalex.org/W1993657037', 'https://openalex.org/W1993934121', 'https://openalex.org/W1995014490', 'https://openalex.org/W2001664274', 'https://openalex.org/W2002675557', 'https://openalex.org/W2002857471', 'https://openalex.org/W2003436527', 'https://openalex.org/W2004180556', 'https://openalex.org/W2004871537', 'https://openalex.org/W2005422315', 'https://openalex.org/W2005758492', 'https://openalex.org/W2006119904', 'https://openalex.org/W2006187024', 'https://openalex.org/W2007395264', 'https://openalex.org/W2007512902', 'https://openalex.org/W2008931716', 'https://openalex.org/W2009190245', 'https://openalex.org/W2010652031', 'https://openalex.org/W2013657661', 'https://openalex.org/W2015267443', 'https://openalex.org/W2015518873', 'https://openalex.org/W2017867386', 'https://openalex.org/W2019778169', 'https://openalex.org/W2020316999', 'https://openalex.org/W2025451713', 'https://openalex.org/W2029609769', 'https://openalex.org/W2033751006', 'https://openalex.org/W2035754578', 'https://openalex.org/W2040424159', 'https://openalex.org/W2041726831', 'https://openalex.org/W2043909051', 'https://openalex.org/W2045812729', 'https://openalex.org/W2047031127', 'https://openalex.org/W2049384587', 'https://openalex.org/W2053463056', 'https://openalex.org/W2058982198', 'https://openalex.org/W2059019405', 'https://openalex.org/W2060216474', 'https://openalex.org/W2060476676', 'https://openalex.org/W2060704583', 'https://openalex.org/W2062847911', 'https://openalex.org/W2062914707', 'https://openalex.org/W2063198646', 'https://openalex.org/W2063862666', 'https://openalex.org/W2064580901', 'https://openalex.org/W2065010255', 'https://openalex.org/W2065747622', 'https://openalex.org/W2066462377', 'https://openalex.org/W2071415686', 'https://openalex.org/W2071664212', 'https://openalex.org/W2076008912', 'https://openalex.org/W2077777431', 'https://openalex.org/W2080251601', 'https://openalex.org/W2084044465', 'https://openalex.org/W2085302848', 'https://openalex.org/W2085989833', 'https://openalex.org/W2087609354', 'https://openalex.org/W2088658068', 'https://openalex.org/W2092134162', 'https://openalex.org/W2092488901', 'https://openalex.org/W2092689128', 'https://openalex.org/W2093098531', 'https://openalex.org/W2094934653', 'https://openalex.org/W2096152098', 'https://openalex.org/W2096411881', 'https://openalex.org/W2097089247', 'https://openalex.org/W2097847889', 'https://openalex.org/W2101154521', 'https://openalex.org/W2104808840', 'https://openalex.org/W2106365165', 'https://openalex.org/W2107008379', 'https://openalex.org/W2107827038', 'https://openalex.org/W2110224739', 'https://openalex.org/W2114535528', 'https://openalex.org/W2125776553', 'https://openalex.org/W2126502509', 'https://openalex.org/W2126631147', 'https://openalex.org/W2126850915', 'https://openalex.org/W2127994451', 'https://openalex.org/W2130337399', 'https://openalex.org/W2132315067', 'https://openalex.org/W2133890944', 'https://openalex.org/W2135276756', 'https://openalex.org/W2139578439', 'https://openalex.org/W2140785063', 'https://openalex.org/W2140956226', 'https://openalex.org/W2142515059', 'https://openalex.org/W2145036943', 'https://openalex.org/W2145296344', 'https://openalex.org/W2146888100', 'https://openalex.org/W2147152072', 'https://openalex.org/W2149684865', 'https://openalex.org/W2151801809', 'https://openalex.org/W2153211312', 'https://openalex.org/W2153962014', 'https://openalex.org/W2158738673', 'https://openalex.org/W2165612380', 'https://openalex.org/W2169384781', 'https://openalex.org/W2170654002', 'https://openalex.org/W2172142456', 'https://openalex.org/W2174678383', 'https://openalex.org/W2435251607', 'https://openalex.org/W2561675875', 'https://openalex.org/W2798573942', 'https://openalex.org/W2915186198', 'https://openalex.org/W2949696181', 'https://openalex.org/W2952299822', 'https://openalex.org/W2953123431', 'https://openalex.org/W3042893949', 'https://openalex.org/W3157411736', 'https://openalex.org/W4205241946', 'https://openalex.org/W4240008182', 'https://openalex.org/W4249379282', 'https://openalex.org/W4285719527', 'https://openalex.org/W6604296810', 'https://openalex.org/W6614676750', 'https://openalex.org/W6629232668', 'https://openalex.org/W6630268012', 'https://openalex.org/W6631307659', 'https://openalex.org/W6632118081', 'https://openalex.org/W6633640926', 'https://openalex.org/W6635379667', 'https://openalex.org/W6635548358', 'https://openalex.org/W6636628491', 'https://openalex.org/W6638423001', 'https://openalex.org/W6641777427', 'https://openalex.org/W6643036076', 'https://openalex.org/W6644484350', 'https://openalex.org/W6666817399', 'https://openalex.org/W6673691841', 'https://openalex.org/W6673781366', 'https://openalex.org/W6679004887', 'https://openalex.org/W6679453733', 'https://openalex.org/W6681835404', 'https://openalex.org/W6682342947', 'https://openalex.org/W6738852829', 'https://openalex.org/W6792154874', 'https://openalex.org/W6794861161', 'https://openalex.org/W7046466245', 'https://openalex.org/W7064660697']</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>['John G, 1994, ELSEVIER EBOOKS', 'Lewis D, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Lang K, 1995, ELSEVIER EBOOKS', 'Cavnar W, 1994, ', 'Lewis D, 1994, ELSEVIER EBOOKS', 'Jones K, 1997, MORGAN KAUFMANN PUBLISHERS INC. EBOOKS', 'Koller D, 1997, ', 'McCallum A, 1998, ', 'Klinkenberg R, 2000, ', 'Cohen W, 1996, ', 'Lewis D, 1991, SCHOLARWORKS@UMASSAMHERST (UNIVERSITY OF MASSACHUSETTS AMHERST)', 'Cohen W, 1999, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Yang Y, 2002, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Scott S, 1999, ', 'Galavotti L, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Liere R, 1997, ', 'Caropreso M, 2001, ', 'Mladenić D, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Weigend A, 1999, INFORMATION RETRIEVAL', 'Wermter S, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Taira H, 1999, ', 'Willett P, 1988, ', 'Roussinov D, 1998, UA CAMPUS REPOSITORY (THE UNIVERSITY OF ARIZONA)', 'Fuhr N, 1991, ', 'Diao Y, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Escudero G, 2000, EUROPEAN CONFERENCE ON MACHINE LEARNING', 'Frasconi P, 2002, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Myers K, 2000, ', 'Joachims T, 2002, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Forsyth R, 1999, ', 'Cohen W, 1995, ELSEVIER EBOOKS', ', 2002, PROGRAM ELECTRONIC LIBRARY AND INFORMATION SYSTEMS', 'Lam W, 1997, INTERNATIONAL JOINT CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Fuhr N, 1985, ', 'Fuhr N, 1984, INTERNATIONAL ACM SIGIR CONFERENCE ON RESEARCH AND DEVELOPMENT IN INFORMATION RETRIEVAL', 'Attardi G, 1998, ZENODO (CERN EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Hull D, 1997, ', 'Sable C, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Lim J, 1999, ', 'Manning C, 1999, ', 'McCallum A, 2022, ', 'Roth D, 1998, ARXIV.ORG', 'Dagan I, 1997, ARXIV.ORG', 'Rodríguez M, 1997, ARXIV.ORG', 'Lewis D, 1994, ACM TRANSACTIONS ON OFFICE INFORMATION SYSTEMS', 'Knorz G, 1982, INTERNATIONAL ACM SIGIR CONFERENCE ON RESEARCH AND DEVELOPMENT IN INFORMATION RETRIEVAL', 'Fangmeyer H, 1968, IFIP CONGRESS', 'Díaz A, 1998, ', 'Lewis D, 1999, INTERNATIONAL ACM SIGIR CONFERENCE ON RESEARCH AND DEVELOPMENT IN INFORMATION RETRIEVAL', 'Tong R, 1992, TEXT RETRIEVAL CONFERENCE', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Yang Y, 1999, ', 'Schapire R, 2000, MACHINE LEARNING', 'Robertson S, 1976, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Chakrabarti S, 1998, COMPUTER NETWORKS AND ISDN SYSTEMS', 'Weikum G, 2002, ACM SIGMOD RECORD', 'Tumer K, 1996, CONNECTION SCIENCE', 'Maron M, 1961, JOURNAL OF THE ACM', 'Gale W, 1992, COMPUTERS AND THE HUMANITIES', 'Schütze H, 1995, ', 'Ng H, 1997, ', 'Larkey L, 1996, ', 'Yang Y, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Crestani F, 1998, ACM COMPUTING SURVEYS', 'Schapire R, 1998, ', 'Masand B, 1992, ', 'Weiss S, 1999, IEEE INTELLIGENT SYSTEMS AND THEIR APPLICATIONS', 'Fuhr N, 1991, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Singhal A, 1996, INFORMATION PROCESSING &amp; MANAGEMENT', 'Yang Y, 1995, ', 'Lam W, 1998, ', 'Wong S, 1995, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Hull D, 1994, ', 'Dörre J, 1999, ', 'Tzeras K, 1993, ', 'Fürnkranz J, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Iwayama M, 1995, ', 'Merkl D, 1998, NEUROCOMPUTING', 'Cooper W, 1995, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Fuhr N, 1989, INFORMATION PROCESSING &amp; MANAGEMENT', 'Singhal A, 1997, ', 'Kim Y, 2000, ', 'Frasconi P, 2001, ', 'Biebricher P, 1988, ', 'Iyer R, 2000, ', 'Knight K, 1999, COMMUNICATIONS OF THE ACM', 'Li P, 1996, CONNECTION SCIENCE', 'Papka R, 1998, ', 'Yu K, 1998, ', 'Cooper W, 1991, ', 'Klingbiel P, 1973, INFORMATION STORAGE AND RETRIEVAL', 'Field B, 1975, JOURNAL OF DOCUMENTATION', 'Guthrie L, 1994, ', 'Sable C, 2000, INTERNATIONAL JOURNAL ON DIGITAL LIBRARIES', 'Liddy E, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Klingbiel P, 1973, INFORMATION STORAGE AND RETRIEVAL', 'Robertson S, 1984, JOURNAL OF DOCUMENTATION', 'Hoyle W, 1973, INFORMATION STORAGE AND RETRIEVAL', 'Wong J, 1996, ACM SIGIR FORUM', 'Cleverdon C, 1984, INFORMATION SERVICES &amp; USE', 'Domingos P, 1997, MACHINE LEARNING', 'Nigam K, 2000, MACHINE LEARNING', 'Joachims T, 1999, ', 'Yang Y, 1999, INFORMATION RETRIEVAL', 'Lewis D, 1994, ARXIV (CORNELL UNIVERSITY)', 'Belkin N, 1992, COMMUNICATIONS OF THE ACM', 'Schütze H, 1998, ', 'Joachims T, 1997, ', 'Apté C, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Saračević T, 1975, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Dumais S, 2000, ', 'Chakrabarti S, 1998, ', 'Baker L, 1998, ', 'Lewis D, 1992, ', 'Lewis D, 1996, ', 'Rijsbergen C, 1977, JOURNAL OF DOCUMENTATION', 'Androutsopoulos I, 2000, ', 'Lewis D, 1995, ACM SIGIR FORUM', 'Li Y, 1998, THE COMPUTER JOURNAL', 'Nigam K, 1998, ', 'Larkey L, 1998, ', 'Chakrabarti S, 1998, THE VLDB JOURNAL', 'Larkey L, 1999, ', 'Lam S, 2003, ', 'Borko H, 1963, JOURNAL OF THE ACM', 'Creecy R, 1992, COMMUNICATIONS OF THE ACM', 'Oh H, 2000, ', 'Attardi G, 1999, CINECA IRIS INSTITUTIAL RESEARCH INFORMATION SYSTEM (UNIVERSITY OF PISA)', 'Hayes P, 2002, ', 'Amati G, 1999, INFORMATION PROCESSING &amp; MANAGEMENT', 'Heaps H, 1973, INFORMATION AND CONTROL', 'Riloff E, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Cohen W, 1998, ', 'Hull D, 1996, ', 'Ruiz M, 1999, ', 'Gövert N, 1999, ', 'Ragas H, 1998, ', 'Li H, 1999, ', 'Clack C, 1997, ', 'Hamill K, 1980, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Fuhr N, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Moulinier I, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Rau L, 1991, ', 'Goodman M, 1990, INNOVATIVE APPLICATIONS OF ARTIFICIAL INTELLIGENCE', 'Junker M, 1998, INTERNATIONAL JOURNAL ON DOCUMENT ANALYSIS AND RECOGNITION (IJDAR)', 'Gray W, 1971, INFORMATION STORAGE AND RETRIEVAL', 'Brückner T, 1997, TEXT RETRIEVAL CONFERENCE', ', 1999, INDUSTRIAL ROBOT THE INTERNATIONAL JOURNAL OF ROBOTICS RESEARCH AND APPLICATION', 'Deerwester S, 1990, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Salton G, 1975, COMMUNICATIONS OF THE ACM', 'Yang Y, 1997, ', 'Drucker H, 1999, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Dumais S, 1998, ', 'Subashini D, 1993, JOURNAL OF COMPUTATIONAL AND APPLIED MATHEMATICS', 'Willett P, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Kessler B, 1997, ', 'Lewis D, 1995, ', 'Lam W, 1999, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Escudero G, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Raghavan V, 2004, CHAPMAN &amp; HALL/CRC COMPUTER AND INFORMATION SCIENCE SERIES', 'Robertson S, 1988, TAYLOR GRAHAM PUBLISHING EBOOKS', 'Riloff E, 1995, ', 'Ruiz M, 1999, ACM SIGIR FORUM', 'Moulinier I, 1996, ', 'Sebastiani F, 2000, ', 'Denoyer L, 2001, ', 'Tauritz D, 2000, INFORMATION SCIENCES', 'Ignatow G, 2017, ', 'Kessler B, 1997, ARXIV.ORG', 'Dagan I, 1997, ARXIV (CORNELL UNIVERSITY)', 'Institute N, 2020, DEFINITIONS', 'Escudero G, 2000, ARXIV.ORG']</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Fabrizio Sebastiani, 2002, ACM Computing Surveys</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Sebastiani F, 2002, ACM COMPUTING SURVEYS</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>Sebastiani F, 2002, ACM COMPUTING SURVEYS</t>
+          <t>Fabrizio Sebastiani, 2002, ACM Computing Surveys</t>
         </is>
       </c>
     </row>
@@ -2296,33 +2211,28 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W1534707631', 'https://openalex.org/W1573640198', 'https://openalex.org/W1594031697', 'https://openalex.org/W1604329830', 'https://openalex.org/W2149706766', 'https://openalex.org/W3085162807']</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>['Gordon A, 1984, BIOMETRICS', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Quinlan J, 1986, MACHINE LEARNING', 'Mingers J, 1989, MACHINE LEARNING', 'Quinlan J, 1989, ELSEVIER EBOOKS', 'Schaffer C, 1992, ELSEVIER EBOOKS']</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salzberg S, 1994, </t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Salzberg S, 1994, </t>
+          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
         </is>
       </c>
     </row>
@@ -2416,25 +2326,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>NA, 2007, Kybernetes</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>NA, 2007, KYBERNETES</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>NA, 2007, KYBERNETES</t>
+          <t>NA, 2007, Kybernetes</t>
         </is>
       </c>
     </row>
@@ -2512,33 +2417,28 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://openalex.org/W1442374986', 'https://openalex.org/W1484210532', 'https://openalex.org/W1487337216', 'https://openalex.org/W1498436455', 'https://openalex.org/W1526734559', 'https://openalex.org/W1548328233', 'https://openalex.org/W1598866093', 'https://openalex.org/W1614298861', 'https://openalex.org/W1658008008', 'https://openalex.org/W1667652561', 'https://openalex.org/W1738019091', 'https://openalex.org/W1827297289', 'https://openalex.org/W1869752048', 'https://openalex.org/W1947291763', 'https://openalex.org/W1978660892', 'https://openalex.org/W1978924650', 'https://openalex.org/W2002257715', 'https://openalex.org/W2016053056', 'https://openalex.org/W2017351599', 'https://openalex.org/W2032036568', 'https://openalex.org/W2035424729', 'https://openalex.org/W2055312318', 'https://openalex.org/W2064675550', 'https://openalex.org/W2082171780', 'https://openalex.org/W2097117768', 'https://openalex.org/W2100830825', 'https://openalex.org/W2123024445', 'https://openalex.org/W2130942839', 'https://openalex.org/W2131975293', 'https://openalex.org/W2138243089', 'https://openalex.org/W2141992894', 'https://openalex.org/W2146757372', 'https://openalex.org/W2155893237', 'https://openalex.org/W2160815625', 'https://openalex.org/W2168231600', 'https://openalex.org/W2171532807', 'https://openalex.org/W2181607856', 'https://openalex.org/W2253807446', 'https://openalex.org/W2507756961', 'https://openalex.org/W2949117887', 'https://openalex.org/W2950789693', 'https://openalex.org/W2951781666']</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>['Hochreiter S, 1997, NEURAL COMPUTATION', 'Szegedy C, 2015, ', 'Rumelhart D, 1986, NATURE', 'Jia Y, 2014, ', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Karpathy A, 2014, ', 'Zaharia M, 2012, ', 'Dean J, 2012, ', 'Isard M, 2007, ', 'Frome A, 2013, ', 'Dongarra J, 1990, ACM TRANSACTIONS ON MATHEMATICAL SOFTWARE', 'Verma A, 2015, ', 'Vinyals O, 2015, NEURAL INFORMATION PROCESSING SYSTEMS', 'Recht B, 2011, NEURAL INFORMATION PROCESSING SYSTEMS', 'Ragan‐Kelley J, 2013, ', 'Ranzato M, 2012, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Murray D, 2013, ', 'Chilimbi T, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Collobert R, 2002, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Zeiler M, 2013, ', 'Arvind A, 1990, IEEE TRANSACTIONS ON COMPUTERS', 'Yu D, 2014, ', 'Chambers C, 2010, ', 'Heigold G, 2013, ', 'Murray D, 2011, ', 'Rossbach C, 2013, ', 'Angelova A, 2015, ', 'Click C, 1995, ', 'Gónzalez-Domínguez J, 2014, NEURAL NETWORKS', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Ioffe S, 2024, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Niu F, 2011, ARXIV (CORNELL UNIVERSITY)', 'Chetlur S, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ba J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Goodfellow I, 2013, ARXIV (CORNELL UNIVERSITY)', 'Nair A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Vinyals O, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ramsundar B, 2015, ARXIV (CORNELL UNIVERSITY)', 'Le Q, 2011, ARXIV (CORNELL UNIVERSITY)', 'Maddison C, 2014, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Martı́n Abadi, 2016, arXiv (Cornell University)-a</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)-a</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)</t>
+          <t>Martı́n Abadi, 2016, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2472,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>6503</v>
+        <v>6533</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2624,33 +2524,28 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W196871588', 'https://openalex.org/W1538131130', 'https://openalex.org/W1543241987', 'https://openalex.org/W1731081199', 'https://openalex.org/W1856502440', 'https://openalex.org/W1899249567', 'https://openalex.org/W1972005403', 'https://openalex.org/W1972576201', 'https://openalex.org/W1976068300', 'https://openalex.org/W1979769287', 'https://openalex.org/W2000359198', 'https://openalex.org/W2002355073', 'https://openalex.org/W2017880874', 'https://openalex.org/W2018159038', 'https://openalex.org/W2019465613', 'https://openalex.org/W2020561998', 'https://openalex.org/W2025444507', 'https://openalex.org/W2060229389', 'https://openalex.org/W2072072671', 'https://openalex.org/W2099471712', 'https://openalex.org/W2101371964', 'https://openalex.org/W2125645174', 'https://openalex.org/W2134164499', 'https://openalex.org/W2142894919', 'https://openalex.org/W2143225719', 'https://openalex.org/W2149498546', 'https://openalex.org/W2158985775', 'https://openalex.org/W2194775991', 'https://openalex.org/W2212370034', 'https://openalex.org/W2234882433', 'https://openalex.org/W2239232218', 'https://openalex.org/W2261689926', 'https://openalex.org/W2277172374', 'https://openalex.org/W2323851192', 'https://openalex.org/W2402144811', 'https://openalex.org/W2474090883', 'https://openalex.org/W2486824498', 'https://openalex.org/W2507348356', 'https://openalex.org/W2534240011', 'https://openalex.org/W2550848904', 'https://openalex.org/W2551156993', 'https://openalex.org/W2558748708', 'https://openalex.org/W2573864470', 'https://openalex.org/W2600297185', 'https://openalex.org/W2605147767', 'https://openalex.org/W2619381903', 'https://openalex.org/W2742127985', 'https://openalex.org/W2749028154', 'https://openalex.org/W2777417212', 'https://openalex.org/W2783378529', 'https://openalex.org/W2786232134', 'https://openalex.org/W2787931125', 'https://openalex.org/W2803629276', 'https://openalex.org/W2809090039', 'https://openalex.org/W2810026216', 'https://openalex.org/W2811199191', 'https://openalex.org/W2856628251', 'https://openalex.org/W2884775584', 'https://openalex.org/W2886802770', 'https://openalex.org/W2887569307', 'https://openalex.org/W2890889625', 'https://openalex.org/W2890968382', 'https://openalex.org/W2893749619', 'https://openalex.org/W2893813411', 'https://openalex.org/W2896549049', 'https://openalex.org/W2897097528', 'https://openalex.org/W2899283552', 'https://openalex.org/W2899971035', 'https://openalex.org/W2900369848', 'https://openalex.org/W2901203181', 'https://openalex.org/W2907047316', 'https://openalex.org/W2908541468', 'https://openalex.org/W2909320927', 'https://openalex.org/W2912389156', 'https://openalex.org/W2912465314', 'https://openalex.org/W2912649832', 'https://openalex.org/W2913323966', 'https://openalex.org/W2914483840', 'https://openalex.org/W2914520121', 'https://openalex.org/W2919958648', 'https://openalex.org/W2936357167', 'https://openalex.org/W2945102878', 'https://openalex.org/W2946794331', 'https://openalex.org/W2946866513', 'https://openalex.org/W2947072793', 'https://openalex.org/W2951392159', 'https://openalex.org/W2952046647', 'https://openalex.org/W2959995783', 'https://openalex.org/W2962793481', 'https://openalex.org/W2963021886', 'https://openalex.org/W2963063862', 'https://openalex.org/W2963095610', 'https://openalex.org/W2963190151', 'https://openalex.org/W2963518130', 'https://openalex.org/W2963634130', 'https://openalex.org/W2963716063', 'https://openalex.org/W2963755523', 'https://openalex.org/W2963901342', 'https://openalex.org/W2964059111', 'https://openalex.org/W2964088238', 'https://openalex.org/W2964121744', 'https://openalex.org/W2964135722', 'https://openalex.org/W2964212578', 'https://openalex.org/W2964268978', 'https://openalex.org/W2966284335', 'https://openalex.org/W2969381807', 'https://openalex.org/W2970100546', 'https://openalex.org/W2970971581', 'https://openalex.org/W2971095480', 'https://openalex.org/W2971343405', 'https://openalex.org/W2972153210', 'https://openalex.org/W2973886134', 'https://openalex.org/W2975003945', 'https://openalex.org/W2977109506', 'https://openalex.org/W2978281981', 'https://openalex.org/W2979712029', 'https://openalex.org/W2979786244', 'https://openalex.org/W2980147119', 'https://openalex.org/W2980592884', 'https://openalex.org/W2980973551', 'https://openalex.org/W2983902802', 'https://openalex.org/W2991298115', 'https://openalex.org/W2991550674', 'https://openalex.org/W2994626356', 'https://openalex.org/W2994747787', 'https://openalex.org/W2997814214', 'https://openalex.org/W2999026783', 'https://openalex.org/W2999467285', 'https://openalex.org/W3003747211', 'https://openalex.org/W3003922491', 'https://openalex.org/W3004450693', 'https://openalex.org/W3005610174', 'https://openalex.org/W3007470329', 'https://openalex.org/W3007740214', 'https://openalex.org/W3008453832', 'https://openalex.org/W3009784374', 'https://openalex.org/W3010849941', 'https://openalex.org/W3011147100', 'https://openalex.org/W3011806874', 'https://openalex.org/W3012417314', 'https://openalex.org/W3012621877', 'https://openalex.org/W3014009018', 'https://openalex.org/W3014468003', 'https://openalex.org/W3015176898', 'https://openalex.org/W3015606043', 'https://openalex.org/W3015865829', 'https://openalex.org/W3016703299', 'https://openalex.org/W3022657828', 'https://openalex.org/W3023982288', 'https://openalex.org/W3025645353', 'https://openalex.org/W3026222427', 'https://openalex.org/W3028316595', 'https://openalex.org/W3028529071', 'https://openalex.org/W3035493266', 'https://openalex.org/W3036843665', 'https://openalex.org/W3037090957', 'https://openalex.org/W3039304986', 'https://openalex.org/W3040277050', 'https://openalex.org/W3041984619', 'https://openalex.org/W3043174105', 'https://openalex.org/W3043516796', 'https://openalex.org/W3045146186', 'https://openalex.org/W3046173836', 'https://openalex.org/W3047001618', 'https://openalex.org/W3048241795', 'https://openalex.org/W3049075514', 'https://openalex.org/W3080393992', 'https://openalex.org/W3081814969', 'https://openalex.org/W3082908155', 'https://openalex.org/W3082977546', 'https://openalex.org/W3084017095', 'https://openalex.org/W3088681382', 'https://openalex.org/W3088691598', 'https://openalex.org/W3088877001', 'https://openalex.org/W3093018961', 'https://openalex.org/W3093190107', 'https://openalex.org/W3093786597', 'https://openalex.org/W3093990252', 'https://openalex.org/W3096173239', 'https://openalex.org/W3096732413', 'https://openalex.org/W3098172061', 'https://openalex.org/W3098195931', 'https://openalex.org/W3098370560', 'https://openalex.org/W3098546160', 'https://openalex.org/W3098951945', 'https://openalex.org/W3099849883', 'https://openalex.org/W3100156752', 'https://openalex.org/W3101260193', 'https://openalex.org/W3101396145', 'https://openalex.org/W3102139197', 'https://openalex.org/W3102569296', 'https://openalex.org/W3102697518', 'https://openalex.org/W3102845444', 'https://openalex.org/W3102921872', 'https://openalex.org/W3103242287', 'https://openalex.org/W3104150464', 'https://openalex.org/W3104873019', 'https://openalex.org/W3105982350', 'https://openalex.org/W3106050203', 'https://openalex.org/W3107691001', 'https://openalex.org/W3107973042', 'https://openalex.org/W3112233611', 'https://openalex.org/W3112264320', 'https://openalex.org/W3116268267', 'https://openalex.org/W3118310857', 'https://openalex.org/W3125167458', 'https://openalex.org/W3128400532', 'https://openalex.org/W3129530645', 'https://openalex.org/W3129610195', 'https://openalex.org/W3132277775', 'https://openalex.org/W3133338006', 'https://openalex.org/W3133608513', 'https://openalex.org/W3137240924', 'https://openalex.org/W3137474564', 'https://openalex.org/W3138463430', 'https://openalex.org/W3145000844', 'https://openalex.org/W3148629269', 'https://openalex.org/W3168386838', 'https://openalex.org/W3181271387', 'https://openalex.org/W3201460085', 'https://openalex.org/W3207890637', 'https://openalex.org/W4230953281', 'https://openalex.org/W4234008654', 'https://openalex.org/W6694756022', 'https://openalex.org/W6713134421', 'https://openalex.org/W6755308174', 'https://openalex.org/W6763197053', 'https://openalex.org/W6787451610']</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>['He K, 2016, ', 'Plimpton S, 1995, JOURNAL OF COMPUTATIONAL PHYSICS', '淳司 柴, 2017, JOURNAL OF JAPAN SOCIETY FOR FUZZY THEORY AND INTELLIGENT INFORMATICS', 'Ganin Y, 2017, ADVANCES IN COMPUTER VISION AND PATTERN RECOGNITION', 'Abadi M, 2016, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Byrd R, 1995, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Behler J, 2007, PHYSICAL REVIEW LETTERS', 'Xiu D, 2002, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Brunton S, 2016, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'LeCun Y, 1998, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Bronstein M, 2017, IEEE SIGNAL PROCESSING MAGAZINE', 'Schmidt M, 2009, SCIENCE', 'Lagaris I, 1998, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Zhang L, 2018, PHYSICAL REVIEW LETTERS', 'Sirignano J, 2018, JOURNAL OF COMPUTATIONAL PHYSICS', 'Alnæs M, 2015, DEPARTMENT OF EARTH SCIENCES EPRINTS REPOSITORY', 'Stuart A, 2010, ACTA NUMERICA', 'Rackauckas C, 2017, JOURNAL OF OPEN RESEARCH SOFTWARE', 'Bruna J, 2013, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Ling J, 2016, JOURNAL OF FLUID MECHANICS', 'Lusch B, 2018, NATURE COMMUNICATIONS', 'Kimeldorf G, 1970, THE ANNALS OF MATHEMATICAL STATISTICS', 'Hart J, 2006, EARTH-SCIENCE REVIEWS', 'Jasak H, 2007, ', 'Hachmann J, 2011, THE JOURNAL OF PHYSICAL CHEMISTRY LETTERS', 'Mallat S, 2016, PHILOSOPHICAL TRANSACTIONS OF THE ROYAL SOCIETY A MATHEMATICAL PHYSICAL AND ENGINEERING SCIENCES', 'Weinan E, 2017, COMMUNICATIONS IN MATHEMATICS AND STATISTICS', 'Raissi M, 2017, JOURNAL OF COMPUTATIONAL PHYSICS', 'Poggio T, 2017, INTERNATIONAL JOURNAL OF AUTOMATION AND COMPUTING', 'Blum A, 1992, NEURAL NETWORKS', 'Marzouk Y, 2006, JOURNAL OF COMPUTATIONAL PHYSICS', 'Lee J, 2016, CONFERENCE ON LEARNING THEORY', 'Micchelli C, 1977, ', 'Raissi M, 2017, JOURNAL OF COMPUTATIONAL PHYSICS', 'Raissi M, 2018, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'González‐García R, 1998, COMPUTERS &amp; CHEMICAL ENGINEERING', 'Diaconis P, 1988, ', 'Owhadi H, 2015, MULTISCALE MODELING AND SIMULATION', 'Stoudenmire E, 2016, NEURAL INFORMATION PROCESSING SYSTEMS', 'Owhadi H, 2006, COMMUNICATIONS ON PURE AND APPLIED MATHEMATICS', 'McFall K, 2009, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Rico-Martı́nez R, 1992, CHEMICAL ENGINEERING COMMUNICATIONS', 'Larkin F, 1972, ROCKY MOUNTAIN JOURNAL OF MATHEMATICS', 'Beidokhti R, 2009, JOURNAL OF THE FRANKLIN INSTITUTE', 'Rovelli C, 2011, FOUNDATIONS OF PHYSICS', 'Rico-Martı́nez R, 2002, ', 'Reisert M, 2007, ', 'Choromanska A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Kondor R, 2018, ARXIV (CORNELL UNIVERSITY)', 'Kadri H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Zhu J, 2017, ', 'Raissi M, 2018, JOURNAL OF COMPUTATIONAL PHYSICS', 'Reichstein M, 2019, NATURE', 'Han J, 2018, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Belkin M, 2019, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Zhu Y, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Bianco S, 2018, IEEE ACCESS', 'Meng X, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Mei S, 2018, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Zhang D, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Xu Z, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Iten R, 2020, PHYSICAL REVIEW LETTERS', 'Tripathy R, 2018, JOURNAL OF COMPUTATIONAL PHYSICS', 'Yang Y, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Geneva N, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Pun G, 2019, NATURE COMMUNICATIONS', 'Kurth T, 2018, ', 'Gardner J, 2018, NEURAL INFORMATION PROCESSING SYSTEMS', 'Poole B, 2016, ARXIV (CORNELL UNIVERSITY)', 'Frostig R, 2018, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Reddy D, 2018, MODELING EARTH SYSTEMS AND ENVIRONMENT', 'Geiger M, 2020, JOURNAL OF STATISTICAL MECHANICS THEORY AND EXPERIMENT', 'Wu J, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Karumuri S, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Grohs P, 2023, MEMOIRS OF THE AMERICAN MATHEMATICAL SOCIETY', 'He J, 2020, JOURNAL OF COMPUTATIONAL MATHEMATICS', 'Geiger M, 2019, PHYSICAL REVIEW. E', 'He J, 2019, SCIENCE CHINA MATHEMATICS', 'Winovich N, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Owhadi H, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Pang G, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Hy T, 2018, THE JOURNAL OF CHEMICAL PHYSICS', 'Spigler S, 2019, JOURNAL OF PHYSICS A MATHEMATICAL AND THEORETICAL', 'Yang Y, 2019, COMPUTATIONAL MECHANICS', 'Yang G, 2017, NEURAL INFORMATION PROCESSING SYSTEMS', 'Kemeth F, 2018, IEEE ACCESS', 'Tai K, 2019, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Winkens J, 2018, ', 'Huang D, 2019, ARXIV (CORNELL UNIVERSITY)', 'Gal Y, 2015, ARXIV (CORNELL UNIVERSITY)', 'Brock A, 2018, ARXIV (CORNELL UNIVERSITY)', 'Jacot A, 2018, ARXIV (CORNELL UNIVERSITY)', 'Cohen T, 2019, ARXIV (CORNELL UNIVERSITY)', 'Rahaman N, 2018, ARXIV (CORNELL UNIVERSITY)', 'Erichson N, 2019, ARXIV (CORNELL UNIVERSITY)', 'Mattheakis M, 2019, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2019, ARXIV (CORNELL UNIVERSITY)', 'Kuan-Lin C, 2021, DROPS (SCHLOSS DAGSTUHL – LEIBNIZ CENTER FOR INFORMATICS)', 'Lu L, 2021, NATURE MACHINE INTELLIGENCE', 'Yu L, 2017, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Raissi M, 2020, SCIENCE', 'He X, 2020, KNOWLEDGE-BASED SYSTEMS', 'Jagtap A, 2020, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Yang L, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Newman D, 1998, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Elsken T, 2019, ARXIV (CORNELL UNIVERSITY)', 'Kharazmi E, 2020, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Kissas G, 2019, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Alber M, 2019, NPJ DIGITAL MEDICINE', 'Tartakovsky A, 2020, WATER RESOURCES RESEARCH', 'Pfau D, 2020, PHYSICAL REVIEW RESEARCH', 'Yang L, 2020, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Haghighat E, 2020, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Lu L, 2020, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Zhang D, 2020, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Hospedales T, 2021, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Jagtap A, 2020, PROCEEDINGS OF THE ROYAL SOCIETY A MATHEMATICAL PHYSICAL AND ENGINEERING SCIENCES', 'Wang W, 2019, NPJ COMPUTATIONAL MATERIALS', 'Xu K, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Sheng H, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Nakata A, 2020, THE JOURNAL OF CHEMICAL PHYSICS', 'Chen F, 2020, THE JOURNAL OF OPEN SOURCE SOFTWARE', 'Owhadi H, 2019, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Fan D, 2019, SCIENCE ROBOTICS', 'Darbon J, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Basri R, 2019, ARXIV (CORNELL UNIVERSITY)', 'Novak R, 2020, INTERNATIONAL CONFERENCE ON LEARNING REPRESENTATIONS', 'Jia J, 2019, ARXIV (CORNELL UNIVERSITY)', 'Jo H, 2020, NETWORKS AND HETEROGENEOUS MEDIA', 'Tsai Y, 2019, ', 'Owhadi H, 2019, NOTICES OF THE AMERICAN MATHEMATICAL SOCIETY', 'Bettencourt J, 2019, ', 'Paszke A, 2019, ARXIV (CORNELL UNIVERSITY)', 'Rackauckas C, 2020, RESEARCH SQUARE', 'Kharazmi E, 2019, ARXIV (CORNELL UNIVERSITY)', 'Wang S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Jia X, 2020, ARXIV (CORNELL UNIVERSITY)', 'Koryagin A, 2019, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2019, ARXIV (CORNELL UNIVERSITY)', 'Kunitski M, 2019, GSI REPOSITORY (GERMAN FEDERAL GOVERNMENT)', 'Lagaris I, 1998, ', 'Jagtap A, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'N. K, 2019, REPEC: RESEARCH PAPERS IN ECONOMICS', 'Kashefi A, 2021, PHYSICS OF FLUIDS', 'Shin Y, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Jin P, 2020, NEURAL NETWORKS', 'Liu Z, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Dong S, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Sirignano J, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Tancik M, 2020, NEURAL INFORMATION PROCESSING SYSTEMS', 'Mu S, 2019, UNIVERSITY OF REGENSBURG PUBLICATION SERVER (UNIVERSITY OF REGENSBURG)', 'Wang S, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Mathews A, 2021, PHYSICAL REVIEW. E', 'Cai W, 2020, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Li D, 2020, WATER RESOURCES RESEARCH', 'Reyes B, 2021, PHYSICAL REVIEW FLUIDS', 'Lagari P, 2020, INTERNATIONAL JOURNAL OF ARTIFICIAL INTELLIGENCE TOOLS', 'Wang B, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Li Z, 2020, CALTECHAUTHORS (CALIFORNIA INSTITUTE OF TECHNOLOGY)', 'Arbabi H, 2020, JOM', 'Guo M, 2022, JOURNAL OF ENGINEERING MECHANICS', 'Nelsen N, 2021, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Mishra S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Tancik M, 2020, ARXIV (CORNELL UNIVERSITY)', 'Pun G, , REPEC: RESEARCH PAPERS IN ECONOMICS', 'Wujie W, 2019, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)', 'Wang S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Wight C, 2020, ARXIV (CORNELL UNIVERSITY)', 'Mishra S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Mao Z, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Owhadi H, 2020, CALTECHAUTHORS (CALIFORNIA INSTITUTE OF TECHNOLOGY)', 'Pfrommer S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Rotskoff G, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Lee J, 2020, ARXIV (CORNELL UNIVERSITY)', 'Wang S, 2021, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Cai S, 2021, JOURNAL OF FLUID MECHANICS', 'Sard A, 1963, MATHEMATICAL SURVEYS AND MONOGRAPHS', 'Jia W, 2020, ', 'Li Z, 2021, CALTECHAUTHORS (CALIFORNIA INSTITUTE OF TECHNOLOGY)', 'Cai S, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', ', 2017, AUERBACH PUBLICATIONS EBOOKS', 'Lanthaler S, 2022, TRANSACTIONS OF MATHEMATICS AND ITS APPLICATIONS', 'Hennigh O, 2021, LECTURE NOTES IN COMPUTER SCIENCE', 'Patel R, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Mao Z, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Hamzi B, 2021, PHYSICA D NONLINEAR PHENOMENA', 'Yang Y, 2020, PROCEEDINGS OF THE ROYAL SOCIETY A MATHEMATICAL PHYSICAL AND ENGINEERING SCIENCES', 'Yang L, 2022, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Manickam I, 2021, ', 'Zhu W, 2020, AGU FALL MEETING ABSTRACTS', 'Hennigh O, 2020, ARXIV (CORNELL UNIVERSITY)', 'Deng B, 2021, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Karniadakis G, 2021, NATURE REVIEWS PHYSICS</t>
-        </is>
-      </c>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>Karniadakis G, 2021, NATURE REVIEWS PHYSICS</t>
+          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2579,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>7839</v>
+        <v>7843</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2736,33 +2631,28 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W195465510', 'https://openalex.org/W1482451543', 'https://openalex.org/W1553313034', 'https://openalex.org/W1578772208', 'https://openalex.org/W1605688901', 'https://openalex.org/W1676820704', 'https://openalex.org/W1970074386', 'https://openalex.org/W1988790447', 'https://openalex.org/W1991418450', 'https://openalex.org/W2019778169', 'https://openalex.org/W2027197837', 'https://openalex.org/W2032210760', 'https://openalex.org/W2037699108', 'https://openalex.org/W2042614373', 'https://openalex.org/W2098191394', 'https://openalex.org/W2112076978', 'https://openalex.org/W2135293965', 'https://openalex.org/W2148520070', 'https://openalex.org/W2152761983', 'https://openalex.org/W2912934387', 'https://openalex.org/W2914859268', 'https://openalex.org/W4212774754', 'https://openalex.org/W4242746271', 'https://openalex.org/W6676769703', 'https://openalex.org/W6808111085']</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>['Freund Y, 1997, JOURNAL OF COMPUTER AND SYSTEM SCIENCES', 'Breiman L, 1996, MACHINE LEARNING', ', 1996, COMPUTERS &amp; MATHEMATICS WITH APPLICATIONS', 'Freund Y, 1996, ', 'Hansen L, 1990, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Dietterich T, 2000, MACHINE LEARNING', 'Dietterich T, 1995, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Bauer E, 1999, MACHINE LEARNING', 'Schapire R, 1998, ', 'Hornik K, 1990, NEURAL NETWORKS', 'Neal R, 2011, ', 'Hyafil L, 1976, INFORMATION PROCESSING LETTERS', 'Tumer K, 1996, CONNECTION SCIENCE', 'Schapire R, 1997, QUT EPRINTS (QUEENSLAND UNIVERSITY OF TECHNOLOGY)', 'Fisher D, 1997, ', 'Kolen J, 1990, ', 'Schapire R, 1997, ', 'Ali K, 1994, MACHINE LEARNING', 'Raviv Y, 1996, CONNECTION SCIENCE', 'Ali K, 1996, MACHINE LEARNING', 'Kwok S, 1990, MACHINE INTELLIGENCE AND PATTERN RECOGNITION', 'Parmanto B, 1995, ']</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Thomas G. Dietterich, 2000, Lecture notes in computer science</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Dietterich T, 2000, LECTURE NOTES IN COMPUTER SCIENCE</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>Dietterich T, 2000, LECTURE NOTES IN COMPUTER SCIENCE</t>
+          <t>Thomas G. Dietterich, 2000, Lecture notes in computer science</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2686,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>4429</v>
+        <v>4433</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -2852,33 +2742,28 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>['RU', 'ES', 'DE', 'US']</t>
+          <t>['https://openalex.org/W51943945', 'https://openalex.org/W118877790', 'https://openalex.org/W199424061', 'https://openalex.org/W882068046', 'https://openalex.org/W999198455', 'https://openalex.org/W1479793620', 'https://openalex.org/W1492999010', 'https://openalex.org/W1503870031', 'https://openalex.org/W1529944915', 'https://openalex.org/W1534582174', 'https://openalex.org/W1559984405', 'https://openalex.org/W1568345435', 'https://openalex.org/W1631356911', 'https://openalex.org/W1684389741', 'https://openalex.org/W1703581136', 'https://openalex.org/W1743210689', 'https://openalex.org/W1872619987', 'https://openalex.org/W1965702053', 'https://openalex.org/W1968390152', 'https://openalex.org/W1968561119', 'https://openalex.org/W1979692035', 'https://openalex.org/W1980314119', 'https://openalex.org/W1981783889', 'https://openalex.org/W1983561139', 'https://openalex.org/W1988369744', 'https://openalex.org/W1994630055', 'https://openalex.org/W2001157051', 'https://openalex.org/W2010505240', 'https://openalex.org/W2015811642', 'https://openalex.org/W2019658260', 'https://openalex.org/W2021276590', 'https://openalex.org/W2022786335', 'https://openalex.org/W2028918948', 'https://openalex.org/W2030545386', 'https://openalex.org/W2035551859', 'https://openalex.org/W2040792108', 'https://openalex.org/W2040870580', 'https://openalex.org/W2041506125', 'https://openalex.org/W2042127289', 'https://openalex.org/W2046481556', 'https://openalex.org/W2051446825', 'https://openalex.org/W2055784634', 'https://openalex.org/W2064517571', 'https://openalex.org/W2069563009', 'https://openalex.org/W2075236172', 'https://openalex.org/W2086236885', 'https://openalex.org/W2097981279', 'https://openalex.org/W2101403221', 'https://openalex.org/W2103956991', 'https://openalex.org/W2104944940', 'https://openalex.org/W2106090814', 'https://openalex.org/W2110322033', 'https://openalex.org/W2120480077', 'https://openalex.org/W2120802379', 'https://openalex.org/W2124269824', 'https://openalex.org/W2153346333', 'https://openalex.org/W2153887174', 'https://openalex.org/W2155728415', 'https://openalex.org/W2156909104', 'https://openalex.org/W2170504083', 'https://openalex.org/W2188879252', 'https://openalex.org/W2195198640', 'https://openalex.org/W2207520826', 'https://openalex.org/W2207698480', 'https://openalex.org/W2221147613', 'https://openalex.org/W2262683142', 'https://openalex.org/W2266138411', 'https://openalex.org/W2272691542', 'https://openalex.org/W2306477081', 'https://openalex.org/W2327049932', 'https://openalex.org/W2334150129', 'https://openalex.org/W2337082154', 'https://openalex.org/W2341702711', 'https://openalex.org/W2397157153', 'https://openalex.org/W2409645286', 'https://openalex.org/W2419175238', 'https://openalex.org/W2468412683', 'https://openalex.org/W2478948476', 'https://openalex.org/W2489886790', 'https://openalex.org/W2490964415', 'https://openalex.org/W2495424399', 'https://openalex.org/W2516533688', 'https://openalex.org/W2517233404', 'https://openalex.org/W2521267242', 'https://openalex.org/W2528744766', 'https://openalex.org/W2557392572', 'https://openalex.org/W2560386163', 'https://openalex.org/W2571629069', 'https://openalex.org/W2579928628', 'https://openalex.org/W2580674237', 'https://openalex.org/W2582909346', 'https://openalex.org/W2595654587', 'https://openalex.org/W2604642811', 'https://openalex.org/W2607911764', 'https://openalex.org/W2612799626', 'https://openalex.org/W2751668559', 'https://openalex.org/W2764347725', 'https://openalex.org/W2766518897', 'https://openalex.org/W2768556639', 'https://openalex.org/W2919115771', 'https://openalex.org/W2949537205', 'https://openalex.org/W2951663210', 'https://openalex.org/W2952050628', 'https://openalex.org/W2962688653', 'https://openalex.org/W2962821153', 'https://openalex.org/W2962954040', 'https://openalex.org/W2963060324', 'https://openalex.org/W2963331258', 'https://openalex.org/W2963614945', 'https://openalex.org/W2963762919', 'https://openalex.org/W2964039664', 'https://openalex.org/W3022610800', 'https://openalex.org/W3023478445', 'https://openalex.org/W3098126014', 'https://openalex.org/W3098768946', 'https://openalex.org/W3098965398', 'https://openalex.org/W3099695580', 'https://openalex.org/W3100863707', 'https://openalex.org/W3101664568', 'https://openalex.org/W3102047485', 'https://openalex.org/W3103372543', 'https://openalex.org/W3104450852', 'https://openalex.org/W3104599990', 'https://openalex.org/W3105377867', 'https://openalex.org/W3106418633', 'https://openalex.org/W3111297213', 'https://openalex.org/W4230674625', 'https://openalex.org/W4297801632', 'https://openalex.org/W4301805094', 'https://openalex.org/W6687462962']</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>['Nielsen M, 2002, AMERICAN JOURNAL OF PHYSICS', 'Rosenblatt F, 1958, PSYCHOLOGICAL REVIEW', 'Harrow A, 2009, PHYSICAL REVIEW LETTERS', 'Lloyd S, 1996, SCIENCE', 'Rebentrost P, 2014, PHYSICAL REVIEW LETTERS', 'Lloyd S, 2014, NATURE PHYSICS', 'Schuld M, 2014, CONTEMPORARY PHYSICS', 'Giovannetti V, 2008, PHYSICAL REVIEW LETTERS', 'Brunner D, 2013, NATURE COMMUNICATIONS', 'Rønnow T, 2014, SCIENCE', 'Wiebe N, 2012, PHYSICAL REVIEW LETTERS', 'Aaronson S, 2015, NATURE PHYSICS', 'Wittek P, 2014, ', 'Temme K, 2011, NATURE', 'Dolde F, 2014, NATURE COMMUNICATIONS', 'Clader B, 2013, PHYSICAL REVIEW LETTERS', 'Ventura D, 2000, INFORMATION SCIENCES', 'Li Z, 2015, PHYSICAL REVIEW LETTERS', 'Wiebe N, 2014, PHYSICAL REVIEW LETTERS', 'Zeidler D, 2001, PHYSICAL REVIEW A', 'Cai X, 2015, PHYSICAL REVIEW LETTERS', 'Paparo G, 2014, PHYSICAL REVIEW X', 'Hentschel A, 2010, PHYSICAL REVIEW LETTERS', 'Biamonte J, 2008, PHYSICAL REVIEW A', 'Bisio A, 2010, PHYSICAL REVIEW A', 'Zahedinejad E, 2015, PHYSICAL REVIEW LETTERS', 'Low G, 2014, PHYSICAL REVIEW A', 'Anguita D, 2003, NEURAL NETWORKS', 'Lovett N, 2013, PHYSICAL REVIEW LETTERS', 'Sasaki M, 2001, PHYSICAL REVIEW A', 'Sentís G, 2012, SCIENTIFIC REPORTS', 'Whitfield J, 2012, EUROPHYSICS LETTERS (EPL)', 'Neigovzen R, 2009, PHYSICAL REVIEW A', 'Wiebe N, 2015, NEW JOURNAL OF PHYSICS', 'Karimi K, 2011, QUANTUM INFORMATION PROCESSING', 'Dunjko V, 2015, NEW JOURNAL OF PHYSICS', 'Sentís G, 2015, EPJ QUANTUM TECHNOLOGY', 'Tezak N, 2015, EPJ QUANTUM TECHNOLOGY', 'Pons M, 2007, PHYSICAL REVIEW LETTERS', 'Freitas N, 2011, ', 'Lloyd S, 2016, NEW JOURNAL OF PHYSICS', 'Amstrup B, 1995, THE JOURNAL OF PHYSICAL CHEMISTRY', 'Farhi E, 2014, ARXIV (CORNELL UNIVERSITY)', 'Lloyd S, 2013, ARXIV (CORNELL UNIVERSITY)', 'Hermans M, 2015, ARXIV (CORNELL UNIVERSITY)', 'Denchev V, 2012, ARXIV (CORNELL UNIVERSITY)', 'Denchev V, 2015, ARXIV (CORNELL UNIVERSITY)', 'Scherer A, 2015, ARXIV (CORNELL UNIVERSITY)', 'LeCun Y, 2015, NATURE', 'Vapnik V, 1995, ', 'Law J, 2001, ACM SIGSOFT SOFTWARE ENGINEERING NOTES', 'Carleo G, 2017, SCIENCE', 'Le Q, 2013, ', 'Carrasquilla J, 2017, NATURE PHYSICS', 'Dunjko V, 2016, PHYSICAL REVIEW LETTERS', 'Christoph D, 1996, ARXIV.ORG', 'Broecker P, 2017, SCIENTIFIC REPORTS', 'Schuld M, 2016, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Wan K, 2017, NPJ QUANTUM INFORMATION', 'Lloyd S, 2016, NATURE COMMUNICATIONS', 'Schuld M, 2017, EUROPHYSICS LETTERS (EPL)', 'Wossnig L, 2018, PHYSICAL REVIEW LETTERS', 'Benedetti M, 2016, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Granade C, 2012, NEW JOURNAL OF PHYSICS', 'Kieferová M, 2017, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Aı̈meur E, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Yung M, 2012, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Rebentrost P, 2018, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Arunachalam S, 2015, NEW JOURNAL OF PHYSICS', 'Zhao Z, 2019, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Lau H, 2017, PHYSICAL REVIEW LETTERS', 'Palittapongarnpim P, 2017, NEUROCOMPUTING', 'Lamata L, 2017, SCIENTIFIC REPORTS', 'and A, 2017, QUANTUM INFORMATION AND COMPUTATION', 'Kimmel S, 2017, NPJ QUANTUM INFORMATION', 'Zahedinejad E, 2016, PHYSICAL REVIEW APPLIED', 'August M, 2017, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'O’Gorman B, 2015, THE EUROPEAN PHYSICAL JOURNAL SPECIAL TOPICS', 'Mavadia S, 2017, NATURE COMMUNICATIONS', 'Scherer A, 2017, QUANTUM INFORMATION PROCESSING', 'Banchi L, 2016, NPJ QUANTUM INFORMATION', 'Heras U, 2016, PHYSICAL REVIEW LETTERS', 'Alvarez-Rodriguez U, 2017, SCIENTIFIC REPORTS', 'Sentís G, 2017, ARXIV (CORNELL UNIVERSITY)', 'Monràs A, 2017, PHYSICAL REVIEW LETTERS', 'Dumoulin V, 2014, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Wittek P, 2017, SCIENTIFIC REPORTS', 'Bisio A, 2011, PHYSICS LETTERS A', 'Somma R, 2016, BULLETIN OF THE AMERICAN PHYSICAL SOCIETY', 'Palittapongarnpim P, 2016, KTH PUBLICATION DATABASE DIVA (KTH ROYAL INSTITUTE OF TECHNOLOGY)', 'Alvarez-Rodriguez U, 2016, ARXIV (CORNELL UNIVERSITY)', 'Lu D, 2017, ARXIV (CORNELL UNIVERSITY)', 'Adachi S, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kerenidis I, 2016, ARXIV (CORNELL UNIVERSITY)', 'Adcock J, 2015, ARXIV (CORNELL UNIVERSITY)', 'Marvian I, 2016, ARXIV (CORNELL UNIVERSITY)', 'Dridi R, 2015, ARXIV (CORNELL UNIVERSITY)', 'Schuld M, 2017, ARXIV (CORNELL UNIVERSITY)', 'Vapnik V, 2000, ', 'Shor P, 1997, SIAM JOURNAL ON COMPUTING', 'Schuld M, 2014, ', 'Kerenidis I, 2017, DR-NTU (NANYANG TECHNOLOGICAL UNIVERSITY)', 'Wiebe N, 2015, QUANTUM INFORMATION AND COMPUTATION', 'Wittek P, 2014, ELSEVIER EBOOKS', 'Wiebe N, 2016, NEURAL INFORMATION PROCESSING SYSTEMS', 'Banchi L, 2016, MPG.PURE (MAX PLANCK SOCIETY)', 'Tiersch M, 2015, SCIENTIFIC REPORTS', 'Unai Á, 2018, LA REFERENCIA (RED FEDERADA DE REPOSITORIOS INSTITUCIONALES DE PUBLICACIONES CIENTÍFICAS)', 'M F, 2013, OXFORD UNIVERSITY RESEARCH ARCHIVE (ORA) (UNIVERSITY OF OXFORD)', 'Chatterjee R, 2017, QUANTUM INFORMATION AND COMPUTATION', 'Seth L, 2016, RWTH PUBLICATIONS (RWTH AACHEN)', 'Kulchytskyy B, 2016, BULLETIN OF THE AMERICAN PHYSICAL SOCIETY', 'Adcock J, , BRISTOL RESEARCH (UNIVERSITY OF BRISTOL)', 'Arunachalam S, 2017, ARXIV (CORNELL UNIVERSITY)', 'Low G, 2014, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)']</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Jacob Biamonte, 2017, Nature</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Biamonte J, 2017, NATURE</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>Biamonte J, 2017, NATURE</t>
+          <t>Jacob Biamonte, 2017, Nature</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2797,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>5851</v>
+        <v>5862</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2968,33 +2853,28 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>['HK', 'CN']</t>
+          <t>['https://openalex.org/W150223756', 'https://openalex.org/W162878246', 'https://openalex.org/W199752024', 'https://openalex.org/W1484769234', 'https://openalex.org/W1485800369', 'https://openalex.org/W1488526968', 'https://openalex.org/W1510952750', 'https://openalex.org/W1559506103', 'https://openalex.org/W1574534563', 'https://openalex.org/W1964366273', 'https://openalex.org/W1968265138', 'https://openalex.org/W1971991172', 'https://openalex.org/W1985511977', 'https://openalex.org/W2016758618', 'https://openalex.org/W2024652123', 'https://openalex.org/W2027471022', 'https://openalex.org/W2041416246', 'https://openalex.org/W2053637704', 'https://openalex.org/W2082624086', 'https://openalex.org/W2092422002', 'https://openalex.org/W2093367651', 'https://openalex.org/W2109426455', 'https://openalex.org/W2112022568', 'https://openalex.org/W2112340198', 'https://openalex.org/W2128906841', 'https://openalex.org/W2132737349', 'https://openalex.org/W2137351756', 'https://openalex.org/W2139336600', 'https://openalex.org/W2159024459', 'https://openalex.org/W2165698076', 'https://openalex.org/W2257979135', 'https://openalex.org/W2283463896', 'https://openalex.org/W2295292576', 'https://openalex.org/W2317339301', 'https://openalex.org/W2435473771', 'https://openalex.org/W2473418344', 'https://openalex.org/W2530417694', 'https://openalex.org/W2536058570', 'https://openalex.org/W2577421826', 'https://openalex.org/W2585580772', 'https://openalex.org/W2591882872', 'https://openalex.org/W2606882085', 'https://openalex.org/W2618494520', 'https://openalex.org/W2679684481', 'https://openalex.org/W2701059868', 'https://openalex.org/W2757853533', 'https://openalex.org/W2765200655', 'https://openalex.org/W2766255512', 'https://openalex.org/W2767079719', 'https://openalex.org/W2768347741', 'https://openalex.org/W2773194476', 'https://openalex.org/W2774000609', 'https://openalex.org/W2777914285', 'https://openalex.org/W2781091734', 'https://openalex.org/W2788629937', 'https://openalex.org/W2793216106', 'https://openalex.org/W2793925626', 'https://openalex.org/W2794888826', 'https://openalex.org/W2798551148', 'https://openalex.org/W2799803467', 'https://openalex.org/W2801958627', 'https://openalex.org/W2807006176', 'https://openalex.org/W2810065831', 'https://openalex.org/W2886722183', 'https://openalex.org/W2895865029', 'https://openalex.org/W2914304175', 'https://openalex.org/W2949140995', 'https://openalex.org/W2950460048', 'https://openalex.org/W2951152347', 'https://openalex.org/W2951368041', 'https://openalex.org/W2951798842', 'https://openalex.org/W2962877476', 'https://openalex.org/W2963106566', 'https://openalex.org/W2990138404', 'https://openalex.org/W3029558105', 'https://openalex.org/W3209546151', 'https://openalex.org/W4248358572', 'https://openalex.org/W4249529812', 'https://openalex.org/W4300427714', 'https://openalex.org/W4301418013', 'https://openalex.org/W4301483968', 'https://openalex.org/W6606067566', 'https://openalex.org/W6732586565', 'https://openalex.org/W6738383168', 'https://openalex.org/W6807767519']</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>['Pan S, 2009, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Silver D, 2016, NATURE', 'Sweeney L, 2002, INTERNATIONAL JOURNAL OF UNCERTAINTY FUZZINESS AND KNOWLEDGE-BASED SYSTEMS', 'Abadi M, 2016, ', 'Goldreich O, 1987, ', 'Bonawitz K, 2017, ', 'Dwork C, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Agrawal R, 2000, ACM SIGMOD RECORD', 'Yao A, 1982, FOUNDATIONS OF COMPUTER SCIENCE', 'Shokri R, 2015, ', 'Mohassel P, 2017, ', 'Rivest R, 1978, ', 'Dowlin N, 2016, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Hitaj B, 2017, ', 'Acar A, 2018, ACM COMPUTING SURVEYS', 'Vaidya J, 2002, ', 'Clifton C, 2010, ', 'Liu J, 2017, ', 'Bogdanov D, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Vaidya J, 2003, ', 'Ho Q, 2013, PUBMED', 'Song S, 2013, ', 'Nikolaenko V, 2013, ', 'Araki T, 2016, ', 'Du W, 2004, ', 'Du W, 2002, SYRACUSE UNIVERSITY LIBRARIES (SYRACUSE UNIVERSITY)', 'Du W, 2005, ', 'Zhang Q, 2015, IEEE TRANSACTIONS ON COMPUTERS', 'Vaidya J, 2004, ', 'Yuan J, 2013, IEEE TRANSACTIONS ON PARALLEL AND DISTRIBUTED SYSTEMS', 'Yu H, 2006, ', 'Yu H, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Scannapieco M, 2007, ', 'Aono Y, 2016, ', 'Sanil A, 2004, ', 'Karr A, 2009, ', 'Hall R, 2011, ', 'Mohassel P, 2015, ', 'Bahmani R, 2017, LECTURE NOTES IN COMPUTER SCIENCE', 'McMahan H, 2017, ', 'Vaidya J, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Wan L, 2007, ', 'Liang G, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Faltings B, 2017, SYNTHESIS LECTURES ON ARTIFICIAL INTELLIGENCE AND MACHINE LEARNING', 'Konečný J, 2016, ARXIV (CORNELL UNIVERSITY)', 'McMahan H, 2016, ARXIV (CORNELL UNIVERSITY)', 'Hesamifard E, 2017, ARXIV (CORNELL UNIVERSITY)', 'Chabanne H, 2017, IACR CRYPTOLOGY EPRINT ARCHIVE', 'Smith V, 2017, ARXIV (CORNELL UNIVERSITY)', ', 2007, THE MIT PRESS EBOOKS', 'Leen T, 2000, ', 'Agrawal R, 2000, ', 'Phong L, 2017, IEEE TRANSACTIONS ON INFORMATION FORENSICS AND SECURITY', 'Mohassel P, 2018, ', 'Riazi M, 2018, ', 'Bourse F, 2018, LECTURE NOTES IN COMPUTER SCIENCE', 'Kim M, 2018, JMIR MEDICAL INFORMATICS', 'Wang S, 2018, ', 'Rouhani B, 2018, 2018 55TH ACM/ESDA/IEEE DESIGN AUTOMATION CONFERENCE (DAC)', 'Kim H, 2018, ', 'Melis L, 2018, ARXIV (CORNELL UNIVERSITY)', 'Chen F, 2018, ', 'Cheng Y, 2019, ', 'Bourse F, 2018, IACR CRYPTOLOGY EPRINT ARCHIVE', 'Faltings B, 2017, SYNTHESIS LECTURES ON ARTIFICIAL INTELLIGENCE AND MACHINE LEARNING', 'Zhao Y, 2018, ARXIV (CORNELL UNIVERSITY)', 'Dariusz W, 2019, SGEM INTERNATIONAL MULTIDISCIPLINARY SCIENTIFIC CONFERENCES ON SOCIAL SCIENCES AND ARTS', 'Bagdasaryan E, 2018, ARXIV (CORNELL UNIVERSITY)', 'Lin Y, 2017, ARXIV (CORNELL UNIVERSITY)', 'Geyer R, 2017, ARXIV (CORNELL UNIVERSITY)', 'Hardy S, 2017, ARXIV (CORNELL UNIVERSITY)', 'Hitaj B, 2017, ARXIV (CORNELL UNIVERSITY)', 'Gascón A, 2016, IACR CRYPTOLOGY EPRINT ARCHIVE', ', 1999, ', 'Nock R, 2018, ARXIV (CORNELL UNIVERSITY)', 'Kilbertus N, 2025, WARWICK RESEARCH ARCHIVE PORTAL (UNIVERSITY OF WARWICK)', 'Su L, 2018, ARXIV (CORNELL UNIVERSITY)', 'Giacomelli I, 2017, IACR CRYPTOLOGY EPRINT ARCHIVE']</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Qiang Yang, 2019, ACM Transactions on Intelligent Systems and Technology</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Yang Q, 2019, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY</t>
-        </is>
-      </c>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>Yang Q, 2019, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY</t>
+          <t>Qiang Yang, 2019, ACM Transactions on Intelligent Systems and Technology</t>
         </is>
       </c>
     </row>
@@ -3080,33 +2960,28 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W104184427', 'https://openalex.org/W145476170', 'https://openalex.org/W1425731158', 'https://openalex.org/W1442374986', 'https://openalex.org/W1485981043', 'https://openalex.org/W1493893823', 'https://openalex.org/W1498436455', 'https://openalex.org/W1526734559', 'https://openalex.org/W1539309091', 'https://openalex.org/W1548328233', 'https://openalex.org/W1598866093', 'https://openalex.org/W1658008008', 'https://openalex.org/W1667652561', 'https://openalex.org/W1815076433', 'https://openalex.org/W1947291763', 'https://openalex.org/W1978660892', 'https://openalex.org/W2016053056', 'https://openalex.org/W2032036568', 'https://openalex.org/W2035424729', 'https://openalex.org/W2041517243', 'https://openalex.org/W2061570747', 'https://openalex.org/W2064675550', 'https://openalex.org/W2066443755', 'https://openalex.org/W2083842231', 'https://openalex.org/W2097117768', 'https://openalex.org/W2100664567', 'https://openalex.org/W2100830825', 'https://openalex.org/W2117539524', 'https://openalex.org/W2122465391', 'https://openalex.org/W2131975293', 'https://openalex.org/W2132339004', 'https://openalex.org/W2140833774', 'https://openalex.org/W2141992894', 'https://openalex.org/W2145339207', 'https://openalex.org/W2146502635', 'https://openalex.org/W2146757372', 'https://openalex.org/W2147527908', 'https://openalex.org/W2160815625', 'https://openalex.org/W2168231600', 'https://openalex.org/W2172654076', 'https://openalex.org/W2186615578', 'https://openalex.org/W2194775991', 'https://openalex.org/W2253807446', 'https://openalex.org/W2259472270', 'https://openalex.org/W2336650964', 'https://openalex.org/W2339765813', 'https://openalex.org/W2384495648', 'https://openalex.org/W2521218765', 'https://openalex.org/W2525778437', 'https://openalex.org/W2618530766', 'https://openalex.org/W2949117887', 'https://openalex.org/W2949888546', 'https://openalex.org/W2950577311', 'https://openalex.org/W2951781666', 'https://openalex.org/W2962844195']</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>['He K, 2016, ', 'Hochreiter S, 1997, NEURAL COMPUTATION', 'Szegedy C, 2015, ', 'Russakovsky O, 2015, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Rumelhart D, 1986, NATURE', 'Mnih V, 2015, NATURE', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Duchi J, 2010, ', 'Karpathy A, 2014, ', 'Zaharia M, 2012, ', 'Sutskever I, 2013, ', 'Dayalan M, 2018, INTERNATIONAL JOURNAL OF RESEARCH AND ENGINEERING', 'Dean J, 2012, ', 'Isard M, 2007, ', ', 2000, APPLIED PHYSICS LETTERS', 'Sifis L, 2016, ARXIV (CORNELL UNIVERSITY)', 'Verma A, 2015, ', 'Jordan M, 1997, ADVANCES IN PSYCHOLOGY', 'Larochelle H, 2009, ', 'Li M, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Lavin A, 2016, ', 'Jean S, 2015, ', 'Hinton G, 1989, ESCHOLARSHIP (CALIFORNIA DIGITAL LIBRARY)', 'Yu Y, 2008, ', 'Ranzato M, 2012, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Chilimbi T, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Collobert R, 2002, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Smola A, 2010, PROCEEDINGS OF THE VLDB ENDOWMENT', 'Zeiler M, 2013, ', 'Byrd R, 2012, MATHEMATICAL PROGRAMMING', 'Cui H, 2016, ', 'Heigold G, 2013, ', 'McSherry F, 2015, ', 'Rossbach C, 2013, ', 'Chung E, 2013, ', 'Chelba C, 2014, ', 'Angelova A, 2015, ', 'Gónzalez-Domínguez J, 2014, NEURAL NETWORKS', 'Murray D, 2016, COMMUNICATIONS OF THE ACM', 'Wu Y, 2016, ARXIV (CORNELL UNIVERSITY)', 'Pascanu R, 2012, ARXIV (CORNELL UNIVERSITY)', 'Chen T, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chetlur S, 2014, ARXIV (CORNELL UNIVERSITY)', 'Mnih V, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Józefowicz R, 2016, ARXIV (CORNELL UNIVERSITY)', 'Xinghao P, 2017, ARXIV (CORNELL UNIVERSITY)', 'Nair A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Maddison C, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ioffe S, 2024, ARXIV (CORNELL UNIVERSITY)', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Niu F, 2011, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Martı́n Abadi, 2016, Operating Systems Design and Implementation</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Abadi M, 2016, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION</t>
-        </is>
-      </c>
-      <c r="Z25" t="inlineStr">
-        <is>
-          <t>Abadi M, 2016, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION</t>
+          <t>Martı́n Abadi, 2016, Operating Systems Design and Implementation</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3015,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>7219</v>
+        <v>7225</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -3196,33 +3071,28 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>['AU']</t>
+          <t>['https://openalex.org/W102612133', 'https://openalex.org/W1479940792', 'https://openalex.org/W1488460165', 'https://openalex.org/W1489095897', 'https://openalex.org/W1515026043', 'https://openalex.org/W1533986854', 'https://openalex.org/W1541145887', 'https://openalex.org/W1587362683', 'https://openalex.org/W1588861010', 'https://openalex.org/W1594031697', 'https://openalex.org/W1623080549', 'https://openalex.org/W1704669313', 'https://openalex.org/W1770825568', 'https://openalex.org/W1784695092', 'https://openalex.org/W1967760155', 'https://openalex.org/W1969341260', 'https://openalex.org/W1969557815', 'https://openalex.org/W1983523174', 'https://openalex.org/W1989164753', 'https://openalex.org/W1995023359', 'https://openalex.org/W2002096058', 'https://openalex.org/W2026980413', 'https://openalex.org/W2049172236', 'https://openalex.org/W2050206309', 'https://openalex.org/W2060136512', 'https://openalex.org/W2102150307', 'https://openalex.org/W2110323455', 'https://openalex.org/W2116939452', 'https://openalex.org/W2117897510', 'https://openalex.org/W2125055259', 'https://openalex.org/W2135346934', 'https://openalex.org/W2145224695', 'https://openalex.org/W2157825442', 'https://openalex.org/W2322002063', 'https://openalex.org/W2766736793', 'https://openalex.org/W2921629193', 'https://openalex.org/W2988864014', 'https://openalex.org/W3015981925', 'https://openalex.org/W3085162807', 'https://openalex.org/W3137161744', 'https://openalex.org/W4233107852', 'https://openalex.org/W4254952533', 'https://openalex.org/W4300993416', 'https://openalex.org/W4400445037', 'https://openalex.org/W6629338572', 'https://openalex.org/W6632481002', 'https://openalex.org/W6635398855', 'https://openalex.org/W6642591540', 'https://openalex.org/W6650814897', 'https://openalex.org/W6676534550', 'https://openalex.org/W6682610290', 'https://openalex.org/W7020983598']</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>['Gordon A, 1984, BIOMETRICS', 'Quinlan J, 1992, ', 'Hanley J, 1982, RADIOLOGY', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Efron B, 1979, THE ANNALS OF STATISTICS', 'Fukunaga K, 1990, ELSEVIER EBOOKS', 'Green D, 1966, ', 'Ingleby J, 1967, JOURNAL OF SOUND AND VIBRATION', 'Hanley J, 1983, RADIOLOGY', 'Fukunaga K, 1990, ACADEMIC PRESS PROFESSIONAL, INC. EBOOKS', ', 2009, ', 'Devijver P, 1982, PRENTICE-HALL INTERNATIONAL EBOOKS', 'Beckman R, 1973, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Mullin A, 1963, AMERICAN MATHEMATICAL MONTHLY', 'Nguyen D, 1990, ', 'Swets J, 1982, ', 'Ziegel E, 2000, TECHNOMETRICS', 'Kavzoğlu T, 2024, ', 'Wolberg W, 1990, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Loader C, 1999, STATISCTICS AND COMPUTING/STATISTICS AND COMPUTING', 'Weiss S, 1991, ', 'Dorfman D, 1969, JOURNAL OF MATHEMATICAL PSYCHOLOGY', 'Smith J, 1988, PUBMED CENTRAL', 'Moore B, 1982, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (GENERAL)', 'Swets J, 1979, INVESTIGATIVE RADIOLOGY', 'Detrano R, 1989, THE AMERICAN JOURNAL OF CARDIOLOGY', 'Gennari J, 1989, ARTIFICIAL INTELLIGENCE', 'Robinson J, 1990, TECHNOMETRICS', 'Schaffer C, 1993, MACHINE LEARNING', 'Picinbono B, 1995, IEEE TRANSACTIONS ON AEROSPACE AND ELECTRONIC SYSTEMS', 'Ivakhnenko A, 1976, CYBERNETICS AND SYSTEMS ANALYSIS', ', 1989, CHOICE REVIEWS ONLINE', 'Schaffer C, 1993, MACHINE LEARNING', 'Friedman J, 1994, ', 'Cherkassky V, 1996, CERN DOCUMENT SERVER (EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Nelson L, 1994, JOURNAL OF QUALITY TECHNOLOGY', 'Walker R, 2002, ', 'Ray M, 1994, THE ANNALS OF THORACIC SURGERY', 'Lovell B, 1996, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Raubertas R, 1994, MEDICAL DECISION MAKING', 'Bradley A, 2002, ', 'Rumelhart D, 1985, ', 'Gennari J, 1988, ', 'Twomey J, 2002, IEEE INTERNATIONAL CONFERENCE ON NEURAL NETWORKS']</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Bradley A, 1997, PATTERN RECOGNITION</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>Bradley A, 1997, PATTERN RECOGNITION</t>
+          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
         </is>
       </c>
     </row>
@@ -3304,25 +3174,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Chris Bishop, 2006, Springer eBooks</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Bishop C, 2006, SPRINGER EBOOKS</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>Bishop C, 2006, SPRINGER EBOOKS</t>
+          <t>Chris Bishop, 2006, Springer eBooks</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3281,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>['CA']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3424,25 +3289,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Radford M. Neal, 2007, Technometrics</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Neal R, 2007, TECHNOMETRICS</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
-        <is>
-          <t>Neal R, 2007, TECHNOMETRICS</t>
+          <t>Radford M. Neal, 2007, Technometrics</t>
         </is>
       </c>
     </row>
@@ -3520,33 +3380,28 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>['CA', 'US']</t>
+          <t>['https://openalex.org/W60686164', 'https://openalex.org/W78356000', 'https://openalex.org/W84569508', 'https://openalex.org/W1497675750', 'https://openalex.org/W1746819321', 'https://openalex.org/W1973333099', 'https://openalex.org/W2061144551', 'https://openalex.org/W2097998348', 'https://openalex.org/W2099201756', 'https://openalex.org/W2106411961', 'https://openalex.org/W2106869737', 'https://openalex.org/W2119595900', 'https://openalex.org/W2129458072', 'https://openalex.org/W2132984949', 'https://openalex.org/W2141125852', 'https://openalex.org/W2147196093', 'https://openalex.org/W2151238122', 'https://openalex.org/W2165599843', 'https://openalex.org/W2189424119', 'https://openalex.org/W2197776371', 'https://openalex.org/W2951665052', 'https://openalex.org/W2964172739', 'https://openalex.org/W3118608800']</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>['Rasmussen C, 2005, THE MIT PRESS EBOOKS', 'Bergstra J, 2012, ', 'Kennedy M, 2001, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Cireşan D, 2012, ', 'Bergstra J, 2011, ', 'Hutter F, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Jones D, 2001, JOURNAL OF GLOBAL OPTIMIZATION', 'Hoffman M, 2010, ', 'Kushner H, 1964, JOURNAL OF BASIC ENGINEERING', 'Kumar M, 2010, NEURAL INFORMATION PROCESSING SYSTEMS', 'Bonilla E, 2007, EDINBURGH RESEARCH EXPLORER', 'Yu C, 2009, ', 'Saxe A, 2011, ', 'Bull A, 2011, JOURNAL OF MACHINE LEARNING RESEARCH', 'Teh Y, 2005, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Mahendran N, 2012, ', 'Miller K, 2012, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Krizhevsky A, 2024, ', 'Brochu E, 2010, ARXIV (CORNELL UNIVERSITY)', 'Srinivas N, 2009, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Coates A, 2024, ', 'Murray I, 2010, ARXIV (CORNELL UNIVERSITY)', 'Ginsbourger D, 2011, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)']</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W29" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Snoek J, 2012, ARXIV (CORNELL UNIVERSITY)</t>
-        </is>
-      </c>
-      <c r="Z29" t="inlineStr">
-        <is>
-          <t>Snoek J, 2012, ARXIV (CORNELL UNIVERSITY)</t>
+          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3435,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>4501</v>
+        <v>4515</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -3636,33 +3491,28 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>['GB', 'US', 'KR']</t>
+          <t>['https://openalex.org/W617139115', 'https://openalex.org/W639205477', 'https://openalex.org/W1491105865', 'https://openalex.org/W1492999010', 'https://openalex.org/W1510073064', 'https://openalex.org/W1565640256', 'https://openalex.org/W1625305535', 'https://openalex.org/W1710476689', 'https://openalex.org/W1757990252', 'https://openalex.org/W1865667476', 'https://openalex.org/W1968761064', 'https://openalex.org/W1976492731', 'https://openalex.org/W1979769287', 'https://openalex.org/W1982589276', 'https://openalex.org/W1982598895', 'https://openalex.org/W1992985800', 'https://openalex.org/W1997974358', 'https://openalex.org/W2007400012', 'https://openalex.org/W2020786104', 'https://openalex.org/W2025679679', 'https://openalex.org/W2030843415', 'https://openalex.org/W2030976617', 'https://openalex.org/W2032026767', 'https://openalex.org/W2034097448', 'https://openalex.org/W2036524141', 'https://openalex.org/W2052226480', 'https://openalex.org/W2052891002', 'https://openalex.org/W2057069496', 'https://openalex.org/W2058452634', 'https://openalex.org/W2063007245', 'https://openalex.org/W2067250248', 'https://openalex.org/W2074616700', 'https://openalex.org/W2076063813', 'https://openalex.org/W2081413236', 'https://openalex.org/W2083415705', 'https://openalex.org/W2104489082', 'https://openalex.org/W2123306226', 'https://openalex.org/W2124234891', 'https://openalex.org/W2127168465', 'https://openalex.org/W2128245586', 'https://openalex.org/W2134164499', 'https://openalex.org/W2138178257', 'https://openalex.org/W2157886206', 'https://openalex.org/W2164524421', 'https://openalex.org/W2173027866', 'https://openalex.org/W2194321275', 'https://openalex.org/W2217912240', 'https://openalex.org/W2230728100', 'https://openalex.org/W2279490987', 'https://openalex.org/W2310703973', 'https://openalex.org/W2324964582', 'https://openalex.org/W2325264655', 'https://openalex.org/W2328928309', 'https://openalex.org/W2337082154', 'https://openalex.org/W2338402873', 'https://openalex.org/W2346180883', 'https://openalex.org/W2346400664', 'https://openalex.org/W2347129741', 'https://openalex.org/W2349487082', 'https://openalex.org/W2418973097', 'https://openalex.org/W2468638527', 'https://openalex.org/W2477622860', 'https://openalex.org/W2478294658', 'https://openalex.org/W2503662290', 'https://openalex.org/W2509907061', 'https://openalex.org/W2520022941', 'https://openalex.org/W2520500207', 'https://openalex.org/W2521267242', 'https://openalex.org/W2525748878', 'https://openalex.org/W2531602199', 'https://openalex.org/W2537064446', 'https://openalex.org/W2540627216', 'https://openalex.org/W2541404351', 'https://openalex.org/W2559394418', 'https://openalex.org/W2565684601', 'https://openalex.org/W2571050567', 'https://openalex.org/W2580919858', 'https://openalex.org/W2591366729', 'https://openalex.org/W2599053724', 'https://openalex.org/W2606044016', 'https://openalex.org/W2611413954', 'https://openalex.org/W2618625858', 'https://openalex.org/W2619580215', 'https://openalex.org/W2620846205', 'https://openalex.org/W2621738901', 'https://openalex.org/W2621742623', 'https://openalex.org/W2734520197', 'https://openalex.org/W2740407088', 'https://openalex.org/W2746244909', 'https://openalex.org/W2747592475', 'https://openalex.org/W2752180799', 'https://openalex.org/W2753962198', 'https://openalex.org/W2766362701', 'https://openalex.org/W2789615344', 'https://openalex.org/W2951016506', 'https://openalex.org/W2963094133', 'https://openalex.org/W2964113829', 'https://openalex.org/W2964116922', 'https://openalex.org/W2964217201', 'https://openalex.org/W3037315640', 'https://openalex.org/W3099950071', 'https://openalex.org/W4240502307', 'https://openalex.org/W4252359241', 'https://openalex.org/W6637568146', 'https://openalex.org/W6730103093', 'https://openalex.org/W6735944222', 'https://openalex.org/W6910696677']</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>['Kohn W, 1965, PHYSICAL REVIEW', 'Schmidhuber J, 2014, NEURAL NETWORKS', 'Jain A, 2013, APL MATERIALS', 'Shawe‐Taylor J, 2004, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Sterling T, 2015, JOURNAL OF CHEMICAL INFORMATION AND MODELING', 'Harrow A, 2009, PHYSICAL REVIEW LETTERS', 'Bartók A, 2010, PHYSICAL REVIEW LETTERS', 'Lake B, 2015, SCIENCE', 'Schmidt M, 2009, SCIENCE', 'Drori I, 2022, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Saal J, 2013, JOM', 'Rupp M, 2012, PHYSICAL REVIEW LETTERS', 'Hansch C, 1964, JOURNAL OF THE AMERICAN CHEMICAL SOCIETY', 'Curtarolo S, 2013, NATURE MATERIALS', 'Tropsha A, 2010, MOLECULAR INFORMATICS', 'Dirac P, 1929, PROCEEDINGS OF THE ROYAL SOCIETY OF LONDON SERIES A CONTAINING PAPERS OF A MATHEMATICAL AND PHYSICAL CHARACTER', 'Lejaeghere K, 2016, SCIENCE', 'Aspuru‐Guzik A, 2005, SCIENCE', 'Ghiringhelli L, 2015, PHYSICAL REVIEW LETTERS', 'Hand D, 2001, INTERNATIONAL STATISTICAL REVIEW', 'Pilania G, 2013, SCIENTIFIC REPORTS', 'Fourches D, 2010, JOURNAL OF CHEMICAL INFORMATION AND MODELING', 'Billinge S, 2007, SCIENCE', 'Corey E, 1969, SCIENCE', 'Hachmann J, 2011, THE JOURNAL OF PHYSICAL CHEMISTRY LETTERS', 'Snyder J, 2012, PHYSICAL REVIEW LETTERS', 'Havu V, 2009, JOURNAL OF COMPUTATIONAL PHYSICS', 'Hautier G, 2010, CHEMISTRY OF MATERIALS', 'Schütt K, 2014, PHYSICAL REVIEW B', 'Calderón C, 2015, COMPUTATIONAL MATERIALS SCIENCE', 'Faber F, 2016, PHYSICAL REVIEW LETTERS', 'Shakhnarovich G, 2005, ', 'Kalinin S, 2015, NATURE MATERIALS', 'Handley C, 2010, THE JOURNAL OF PHYSICAL CHEMISTRY A', 'Franceschetti A, 1999, NATURE', 'Christensen R, 2015, CATALYSIS SCIENCE &amp; TECHNOLOGY', 'Fleuren W, 2015, METHODS', 'Kireeva N, 2012, MOLECULAR INFORMATICS', 'Pople J, 1999, ANGEWANDTE CHEMIE INTERNATIONAL EDITION', 'Bonchev D, 1994, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Albuquerque V, 2008, NONDESTRUCTIVE TESTING AND EVALUATION', 'Wicker J, 2014, CRYSTENGCOMM', 'Kühn C, 1996, THE JOURNAL OF PHYSICAL CHEMISTRY', 'Walsh A, 2015, NATURE CHEMISTRY', ', 2013, ', 'Oprea T, 2006, DRUG DISCOVERY TODAY TECHNOLOGIES', 'Kiselyova N, 1998, JOURNAL OF ALLOYS AND COMPOUNDS', 'Duvenaud D, 2015, ARXIV (CORNELL UNIVERSITY)', 'Jastrzȩbski S, 2016, ARXIV (CORNELL UNIVERSITY)', 'Biamonte J, 2017, NATURE', 'Smith J, 2017, CHEMICAL SCIENCE', 'Segler M, 2018, NATURE', 'Raccuglia P, 2016, NATURE', ', 2021, ENCYCLOPEDIA OF THE UN SUSTAINABLE DEVELOPMENT GOALS', 'Rudy S, 2017, SCIENCE ADVANCES', 'Wellendorff J, 2012, PHYSICAL REVIEW B', 'Carrasquilla J, 2017, NATURE PHYSICS', 'Steane A, 1998, REPORTS ON PROGRESS IN PHYSICS', 'Agrawal A, 2016, APL MATERIALS', 'Mardirossian N, 2016, THE JOURNAL OF CHEMICAL PHYSICS', 'Gómez‐Bombarelli R, 2016, NATURE MATERIALS', 'Altae-Tran H, 2017, ACS CENTRAL SCIENCE', 'Reiher M, 2017, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Behler J, 2017, ANGEWANDTE CHEMIE INTERNATIONAL EDITION', 'Faber F, 2017, JOURNAL OF CHEMICAL THEORY AND COMPUTATION', 'Isayev O, 2017, NATURE COMMUNICATIONS', 'Szymkuć S, 2016, ANGEWANDTE CHEMIE INTERNATIONAL EDITION', 'Segler M, 2017, CHEMISTRY - A EUROPEAN JOURNAL', 'Brockherde F, 2017, NATURE COMMUNICATIONS', 'Liu B, 2017, ACS CENTRAL SCIENCE', 'Pulido A, 2017, NATURE', 'Kim E, 2017, CHEMISTRY OF MATERIALS', 'Dunjko V, 2016, PHYSICAL REVIEW LETTERS', 'Ward L, 2017, PHYSICAL REVIEW. B./PHYSICAL REVIEW. B', 'Oliynyk A, 2016, CHEMISTRY OF MATERIALS', 'Klucznik T, 2018, CHEM', 'Duan Y, 2017, NEURAL INFORMATION PROCESSING SYSTEMS', 'Hill J, 2016, MRS BULLETIN', 'Davies D, 2016, CHEM', 'Pensak D, 1977, ACS SYMPOSIUM SERIES', 'Legrain F, 2017, THE JOURNAL OF PHYSICAL CHEMISTRY B', 'Ziatdinov M, 2017, NPJ COMPUTATIONAL MATERIALS', 'Dragone V, 2017, NATURE COMMUNICATIONS', 'Wilkinson K, 2014, JOURNAL OF CHEMICAL THEORY AND COMPUTATION', 'Norbert J, 2011, STUDIES IN COMPUTATIONAL INTELLIGENCE', 'Seko A, 2018, ', 'Arita M, 2014, JOURNAL OF CHEMICAL THEORY AND COMPUTATION', 'Coudert F, 2017, CHEMISTRY OF MATERIALS', 'Tetko I, 2016, MOLECULAR INFORMATICS', 'Cole J, 2016, ACTA CRYSTALLOGRAPHICA SECTION B STRUCTURAL SCIENCE CRYSTAL ENGINEERING AND MATERIALS', 'Boyd D, 2013, ACS SYMPOSIUM SERIES', 'Moot T, 2016, MATERIALS DISCOVERY', 'Pillong M, 2017, CRYSTENGCOMM', 'Trabesinger A, 2017, NATURE', 'Hui Y, 2019, ADVANCES IN INTELLIGENT SYSTEMS AND COMPUTING', 'Guimaraes G, 2017, ARXIV (CORNELL UNIVERSITY)', 'Nam J, 2016, ARXIV (CORNELL UNIVERSITY)', 'Calderón C, 2015, ARXIV (CORNELL UNIVERSITY)', 'F. B, 2017, MPG.PURE (MAX PLANCK SOCIETY)', 'R.B. M, 1993, JOURNAL OF MOLECULAR STRUCTURE THEOCHEM', 'Rokach L, 2009, ']</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Keith T. Butler, 2018, Nature</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Butler K, 2018, NATURE</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
-        <is>
-          <t>Butler K, 2018, NATURE</t>
+          <t>Keith T. Butler, 2018, Nature</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3581,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>['US', 'CA']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3739,25 +3589,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">William W. Cohen, 2008, </t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cohen W, 2008, </t>
-        </is>
-      </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cohen W, 2008, </t>
+          <t xml:space="preserve">William W. Cohen, 2008, </t>
         </is>
       </c>
     </row>
@@ -3791,7 +3636,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>3936</v>
+        <v>3948</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -3847,33 +3692,28 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W1524493166', 'https://openalex.org/W1529983430', 'https://openalex.org/W2005440935', 'https://openalex.org/W2009184733', 'https://openalex.org/W2009954208', 'https://openalex.org/W2027540165', 'https://openalex.org/W2033163059', 'https://openalex.org/W2033609349', 'https://openalex.org/W2043092953', 'https://openalex.org/W2054076956', 'https://openalex.org/W2083721602', 'https://openalex.org/W2096849439', 'https://openalex.org/W2103018059', 'https://openalex.org/W2103889389', 'https://openalex.org/W2119472226', 'https://openalex.org/W2137767404', 'https://openalex.org/W2147246123', 'https://openalex.org/W2166187912', 'https://openalex.org/W2167414941', 'https://openalex.org/W2174931596', 'https://openalex.org/W2267932926', 'https://openalex.org/W2276530525', 'https://openalex.org/W2337116044', 'https://openalex.org/W2415841860', 'https://openalex.org/W2468431774', 'https://openalex.org/W2512902140', 'https://openalex.org/W2515682654', 'https://openalex.org/W2528491735', 'https://openalex.org/W2530247697', 'https://openalex.org/W2548723212', 'https://openalex.org/W2557738935', 'https://openalex.org/W2581082771', 'https://openalex.org/W2598272139', 'https://openalex.org/W2732701910', 'https://openalex.org/W2734356183', 'https://openalex.org/W2738975713', 'https://openalex.org/W2740060821', 'https://openalex.org/W2752747624', 'https://openalex.org/W2753059860', 'https://openalex.org/W2754518417', 'https://openalex.org/W2758348074', 'https://openalex.org/W2762741128', 'https://openalex.org/W2772246530', 'https://openalex.org/W2772723798', 'https://openalex.org/W2782945064', 'https://openalex.org/W2784499877', 'https://openalex.org/W2785268987', 'https://openalex.org/W2785526886', 'https://openalex.org/W2788633781', 'https://openalex.org/W2789894922', 'https://openalex.org/W2790444357', 'https://openalex.org/W2791819448', 'https://openalex.org/W2792902933', 'https://openalex.org/W2793267369', 'https://openalex.org/W2794457162', 'https://openalex.org/W2799837895', 'https://openalex.org/W2804685074', 'https://openalex.org/W2809453031', 'https://openalex.org/W2886281300', 'https://openalex.org/W2887623535', 'https://openalex.org/W2887719255', 'https://openalex.org/W2888109941', 'https://openalex.org/W2889242407', 'https://openalex.org/W2889494558', 'https://openalex.org/W2894917609', 'https://openalex.org/W2896385413', 'https://openalex.org/W2896817483', 'https://openalex.org/W2897434820', 'https://openalex.org/W2899560923', 'https://openalex.org/W2902802452', 'https://openalex.org/W2908201961', 'https://openalex.org/W2914579361', 'https://openalex.org/W2916105049', 'https://openalex.org/W2919115771', 'https://openalex.org/W3098949126', 'https://openalex.org/W4205374244', 'https://openalex.org/W4212774754', 'https://openalex.org/W4296220420']</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>['Esteva A, 2017, NATURE', 'Gulshan V, 2016, JAMA', 'Haynes A, 2009, NEW ENGLAND JOURNAL OF MEDICINE', 'Kermany D, 2018, CELL', 'Bejnordi B, 2017, JAMA', 'Rajkomar A, 2018, NPJ DIGITAL MEDICINE', 'Ting D, 2017, JAMA', 'Beam A, 2018, JAMA', 'Poplin R, 2018, NATURE BIOMEDICAL ENGINEERING', 'Halevy A, 2009, IEEE INTELLIGENT SYSTEMS', 'Castelvecchi D, 2016, NATURE', 'Sinsky C, 2016, ANNALS OF INTERNAL MEDICINE', 'Bates D, 2014, HEALTH AFFAIRS', 'Cabitza F, 2017, JAMA', 'Arndt B, 2017, THE ANNALS OF FAMILY MEDICINE', 'Mandel J, 2016, JOURNAL OF THE AMERICAN MEDICAL INFORMATICS ASSOCIATION', 'Frieden T, 2017, NEW ENGLAND JOURNAL OF MEDICINE', 'Muntner P, 2014, JAMA', 'Krumholz H, 2014, HEALTH AFFAIRS', 'Hersh W, 2013, MEDICAL CARE', 'Krause J, 2018, OPHTHALMOLOGY', 'Elmore J, 2017, BMJ', 'Jong M, 2017, THE LANCET', 'Lyell D, 2016, JOURNAL OF THE AMERICAN MEDICAL INFORMATICS ASSOCIATION', 'Schneeweiß S, 2014, NEW ENGLAND JOURNAL OF MEDICINE', 'Mandl K, 2001, BMJ', 'Cohen I, 2014, HEALTH AFFAIRS', 'Lindenauer P, 2012, JAMA', 'Kesselheim A, 2011, HEALTH AFFAIRS', 'Obermeyer Z, 2017, NEW ENGLAND JOURNAL OF MEDICINE', 'Erickson S, 2017, ANNALS OF INTERNAL MEDICINE', 'Schwartz W, 1970, NEW ENGLAND JOURNAL OF MEDICINE', 'Hill R, 2013, THE AMERICAN JOURNAL OF EMERGENCY MEDICINE', 'Amarasingham R, 2014, HEALTH AFFAIRS', 'Mamykina L, 2016, ACADEMIC MEDICINE', 'Shuren J, 2016, JAMA', 'Fiore L, 2016, NEW ENGLAND JOURNAL OF MEDICINE', 'Bakris G, 2018, NEW ENGLAND JOURNAL OF MEDICINE', 'Escobar G, 2016, JOURNAL OF HOSPITAL MEDICINE', 'McGlynn E, 2015, JAMA', 'Mandl K, 2016, NEW ENGLAND JOURNAL OF MEDICINE', 'Sniderman A, 2015, JAMA', 'Steinhubl S, 2018, THE LANCET', 'Schuster M, 2017, JAMA', 'Slack W, 1966, NEW ENGLAND JOURNAL OF MEDICINE', 'Oxentenko A, 2010, ARCHIVES OF INTERNAL MEDICINE', 'Reis B, 2009, BMJ', 'Gabriels K, 2018, JOURNAL OF MEDICAL INTERNET RESEARCH', 'Sittig D, 2015, JOURNAL OF THE AMERICAN MEDICAL INFORMATICS ASSOCIATION', 'Rajkomar A, 2016, JMIR MEDICAL INFORMATICS', 'LeCun Y, 2015, NATURE', ', 1996, COMPUTERS &amp; MATHEMATICS WITH APPLICATIONS', 'Topol E, 2018, NATURE MEDICINE', 'Fauw J, 2018, NATURE MEDICINE', 'Alvin R, 2018, ', 'Ford I, 2016, NEW ENGLAND JOURNAL OF MEDICINE', 'Gianfrancesco M, 2018, JAMA INTERNAL MEDICINE', 'Rajkomar A, 2018, ANNALS OF INTERNAL MEDICINE', 'Chilamkurthy S, 2018, THE LANCET', 'Wang P, 2019, GUT', 'Hinton G, 2018, JAMA', 'Grinfeld J, 2018, NEW ENGLAND JOURNAL OF MEDICINE', 'Denis F, 2019, JAMA', 'Tison G, 2018, JAMA CARDIOLOGY', 'Mori Y, 2018, ANNALS OF INTERNAL MEDICINE', 'Steiner D, 2018, THE AMERICAN JOURNAL OF SURGICAL PATHOLOGY', 'Liu Y, 2018, ARCHIVES OF PATHOLOGY &amp; LABORATORY MEDICINE', 'Morawski K, 2018, JAMA INTERNAL MEDICINE', 'Howe J, 2018, JAMA', 'Fraser H, 2018, THE LANCET', 'Kale M, 2018, BMJ', 'Das J, 2018, BMJ', 'Schwartz W, 1987, NEW ENGLAND JOURNAL OF MEDICINE', 'Galloway C, 2018, JOURNAL OF THE AMERICAN COLLEGE OF CARDIOLOGY', 'Berwick D, 2018, JAMA', 'Auerbach A, 2018, ANNALS OF INTERNAL MEDICINE', 'Kannan A, 2018, ', 'Lee V, 2018, JAMA']</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Rajkomar A, 2019, NEW ENGLAND JOURNAL OF MEDICINE</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
-        <is>
-          <t>Rajkomar A, 2019, NEW ENGLAND JOURNAL OF MEDICINE</t>
+          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
         </is>
       </c>
     </row>
@@ -3959,33 +3799,28 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>['DE']</t>
+          <t>['https://openalex.org/W740415', 'https://openalex.org/W1504694836', 'https://openalex.org/W1978394996', 'https://openalex.org/W2023677852', 'https://openalex.org/W2087614174', 'https://openalex.org/W2096152098', 'https://openalex.org/W2114535528', 'https://openalex.org/W2119821739', 'https://openalex.org/W2125055259', 'https://openalex.org/W2149684865', 'https://openalex.org/W2156909104', 'https://openalex.org/W2164547069', 'https://openalex.org/W2435251607', 'https://openalex.org/W6821113053']</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>['Vapnik V, 1995, ', 'Cortes C, 1995, MACHINE LEARNING', 'Quinlan J, 1992, ', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Salzberg S, 1994, ', 'Yang Y, 1997, ', 'Rocchio J, 1971, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Vapnik V, 1995, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Yang Y, 1999, INFORMATION RETRIEVAL', 'Joachims T, 1997, ', 'Kivinen J, 1997, ARTIFICIAL INTELLIGENCE', 'Kivinen J, 1995, ']</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Thorsten Joachims, 1998, Lecture notes in computer science</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
-        <is>
-          <t>Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE</t>
+          <t>Thorsten Joachims, 1998, Lecture notes in computer science</t>
         </is>
       </c>
     </row>
@@ -4019,7 +3854,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>6646</v>
+        <v>6648</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -4063,33 +3898,28 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>['HK', 'CN']</t>
+          <t>['https://openalex.org/W588441650', 'https://openalex.org/W962117656', 'https://openalex.org/W1514535095', 'https://openalex.org/W1568514080', 'https://openalex.org/W1606347560', 'https://openalex.org/W1810943226', 'https://openalex.org/W1815076433', 'https://openalex.org/W1867429401', 'https://openalex.org/W1903029394', 'https://openalex.org/W1905882502', 'https://openalex.org/W1947481528', 'https://openalex.org/W1982479097', 'https://openalex.org/W2024414272', 'https://openalex.org/W2030459037', 'https://openalex.org/W2064675550', 'https://openalex.org/W2079565659', 'https://openalex.org/W2116435618', 'https://openalex.org/W2130942839', 'https://openalex.org/W2157331557', 'https://openalex.org/W2557283755', 'https://openalex.org/W2787727108', 'https://openalex.org/W2950635152', 'https://openalex.org/W2951183276', 'https://openalex.org/W2952453038', 'https://openalex.org/W4233546237', 'https://openalex.org/W4294306266', 'https://openalex.org/W4308909683']</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>['Hochreiter S, 1997, NEURAL COMPUTATION', 'Long J, 2015, ', 'Cho K, 2014, ', 'Goodfellow I, 2016, MIT PRESS EBOOKS', 'Donahue J, 2015, ', 'Karpathy A, 2015, ', 'Davide B, 2013, DROPS (SCHLOSS DAGSTUHL – LEIBNIZ CENTER FOR INFORMATICS)', 'Brox T, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Sun J, 2013, BULLETIN OF THE AMERICAN METEOROLOGICAL SOCIETY', 'Germann U, 2002, MONTHLY WEATHER REVIEW', 'Bridson R, 2011, ', 'Bridson R, 2015, ', 'Klein B, 2015, ', 'Sakaino H, 2012, IEEE TRANSACTIONS ON GEOSCIENCE AND REMOTE SENSING', 'Woo W, 2014, 27TH CONFERENCE ON SEVERE LOCAL STORMS', 'Douglas R, 1990, AMERICAN METEOROLOGICAL SOCIETY EBOOKS', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2015, ARXIV (CORNELL UNIVERSITY)', 'Pascanu R, 2012, ARXIV (CORNELL UNIVERSITY)', 'Cho K, 2014, ARXIV (CORNELL UNIVERSITY)', 'Long J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Srivastava N, 2015, ARXIV (CORNELL UNIVERSITY)', 'Donahue J, 2014, ', 'Bastien F, 2012, ARXIV (CORNELL UNIVERSITY)', 'Ranzato M, 2014, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Xingjian Shi, 2015, arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Shi X, 2015, ARXIV (CORNELL UNIVERSITY)</t>
-        </is>
-      </c>
-      <c r="Z34" t="inlineStr">
-        <is>
-          <t>Shi X, 2015, ARXIV (CORNELL UNIVERSITY)</t>
+          <t>Xingjian Shi, 2015, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -4175,33 +4005,28 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>['DE']</t>
+          <t>['https://openalex.org/W1657213141', 'https://openalex.org/W1746680969', 'https://openalex.org/W2117063635', 'https://openalex.org/W2129564505']</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>['Jordan M, 1998, ', 'Williams C, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Csató L, 2002, NEURAL COMPUTATION', 'Williams C, 1998, ']</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W35" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Carl Edward Rasmussen, 2004, Lecture notes in computer science</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Rasmussen C, 2004, LECTURE NOTES IN COMPUTER SCIENCE</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>Rasmussen C, 2004, LECTURE NOTES IN COMPUTER SCIENCE</t>
+          <t>Carl Edward Rasmussen, 2004, Lecture notes in computer science</t>
         </is>
       </c>
     </row>
@@ -4283,33 +4108,28 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W1505356468', 'https://openalex.org/W1535810436', 'https://openalex.org/W1629097610', 'https://openalex.org/W2029538739', 'https://openalex.org/W2030811966', 'https://openalex.org/W2035720976', 'https://openalex.org/W2043919728', 'https://openalex.org/W2068484625', 'https://openalex.org/W2086161653', 'https://openalex.org/W2098921539', 'https://openalex.org/W2101159990', 'https://openalex.org/W2113651538', 'https://openalex.org/W2119821739', 'https://openalex.org/W2127218421', 'https://openalex.org/W2129191766', 'https://openalex.org/W2135046866', 'https://openalex.org/W2137515395', 'https://openalex.org/W2147880316', 'https://openalex.org/W2150102617', 'https://openalex.org/W2154451187', 'https://openalex.org/W2322150470', 'https://openalex.org/W2416173357', 'https://openalex.org/W2766736793', 'https://openalex.org/W2990138404', 'https://openalex.org/W3207342693', 'https://openalex.org/W4238284510']</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>['Tibshirani R, 1996, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Cortes C, 1995, MACHINE LEARNING', 'MacQueen J, 1967, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', ', 2007, THE MIT PRESS EBOOKS', 'Lafferty J, 2001, SCHOLARLY COMMONS (UNIVERSITY OF PENNSYLVANIA)', 'Dennis J, 1996, SOCIETY FOR INDUSTRIAL AND APPLIED MATHEMATICS EBOOKS', 'Vapnik V, 2015, ', 'Lewis D, 2004, GOLDSMITHS (UNIVERSITY OF LONDON)', 'Vapnik V, 1971, THEORY OF PROBABILITY AND ITS APPLICATIONS', 'Joachims T, 2006, ', 'Polyak B, 1992, SIAM JOURNAL ON CONTROL AND OPTIMIZATION', 'Bottou L, 2011, THE MIT PRESS EBOOKS', 'Tsybakov A, 2004, THE ANNALS OF STATISTICS', 'Bordes A, 2009, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Lin C, 2007, ', 'Shalev‐Shwartz S, 2008, ', 'Massart P, 2000, ANNALES DE LA FACULTÉ DES SCIENCES DE TOULOUSE MATHÉMATIQUES', 'Bottou L, 2005, APPLIED STOCHASTIC MODELS IN BUSINESS AND INDUSTRY', 'Lee W, 1998, IEEE TRANSACTIONS ON INFORMATION THEORY', "Bousquet O, 2002, OPENGREY (INSTITUT DE L'INFORMATION SCIENTIFIQUE ET TECHNIQUE)", 'Murata N, 1999, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Rumelhart D, 1985, ', 'Widrow B, 1960, ', 'Xu W, 2011, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">Léon Bottou, 2010, </t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottou L, 2010, </t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bottou L, 2010, </t>
+          <t xml:space="preserve">Léon Bottou, 2010, </t>
         </is>
       </c>
     </row>
@@ -4354,7 +4174,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>['Nijssen, Siegfried']</t>
+          <t>['Sammut, Claude 1956-']</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -4364,7 +4184,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Nijssen, Siegfried (corresponding author), University Of New south Wales</t>
+          <t>Sammut, Claude 1956- (corresponding author), University Of New south Wales</t>
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -4379,7 +4199,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>['AU']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4387,25 +4207,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">Claude Sammut, 2010, </t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sammut C, 2010, </t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sammut C, 2010, </t>
+          <t xml:space="preserve">Claude Sammut, 2010, </t>
         </is>
       </c>
     </row>
@@ -4439,7 +4254,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>8893</v>
+        <v>8918</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -4495,33 +4310,28 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W1492170170', 'https://openalex.org/W1537462412', 'https://openalex.org/W1731081199', 'https://openalex.org/W1746506709', 'https://openalex.org/W1905782493', 'https://openalex.org/W1973682096', 'https://openalex.org/W1984314602', 'https://openalex.org/W1994407253', 'https://openalex.org/W2013587512', 'https://openalex.org/W2026905436', 'https://openalex.org/W2046945713', 'https://openalex.org/W2072136246', 'https://openalex.org/W2082262280', 'https://openalex.org/W2132166479', 'https://openalex.org/W2134598164', 'https://openalex.org/W2141097525', 'https://openalex.org/W2149033360', 'https://openalex.org/W2163598528', 'https://openalex.org/W2239135493', 'https://openalex.org/W2248060815', 'https://openalex.org/W2467510144', 'https://openalex.org/W2493343568', 'https://openalex.org/W2579555219', 'https://openalex.org/W2604231045', 'https://openalex.org/W2613140028', 'https://openalex.org/W2621305858', 'https://openalex.org/W2743731382', 'https://openalex.org/W2752988282', 'https://openalex.org/W2765813195', 'https://openalex.org/W2767442356', 'https://openalex.org/W2778670458', 'https://openalex.org/W2798857668', 'https://openalex.org/W2811104224', 'https://openalex.org/W2811374795', 'https://openalex.org/W2894881080', 'https://openalex.org/W2895051075', 'https://openalex.org/W2896176822', 'https://openalex.org/W2898694742', 'https://openalex.org/W2899360465', 'https://openalex.org/W2901939789', 'https://openalex.org/W2902991393', 'https://openalex.org/W2910705748', 'https://openalex.org/W2962689739', 'https://openalex.org/W2963125461', 'https://openalex.org/W2963533879', 'https://openalex.org/W2963816926', 'https://openalex.org/W2964134873', 'https://openalex.org/W2964180856', 'https://openalex.org/W3085162807', 'https://openalex.org/W3098636317', 'https://openalex.org/W3102221121', 'https://openalex.org/W3102834905', 'https://openalex.org/W3122175177', 'https://openalex.org/W4234008654', 'https://openalex.org/W6743543778']</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>['Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Miller G, 1956, PSYCHOLOGICAL REVIEW', 'Miller G, 1994, PSYCHOLOGICAL REVIEW', 'Ganin Y, 2017, ADVANCES IN COMPUTER VISION AND PATTERN RECOGNITION', 'Fayyad U, 1996, ', 'Goodman B, 2017, AI MAGAZINE', 'Murdoch W, 2019, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Holte R, 1993, MACHINE LEARNING', 'Zech J, 2018, PLOS MEDICINE', 'Cowan N, 2010, CURRENT DIRECTIONS IN PSYCHOLOGICAL SCIENCE', 'Mittelstadt B, 2019, ', 'Hand D, 2006, STATISTICAL SCIENCE', 'Freitas A, 2014, ACM SIGKDD EXPLORATIONS NEWSLETTER', 'Lou Y, 2013, ', 'Lou Y, 2012, ', 'Huysmans J, 2010, DECISION SUPPORT SYSTEMS', 'Li O, 2018, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Ustun B, 2017, JAMA PSYCHIATRY', 'Brennan T, 2008, CRIMINAL JUSTICE AND BEHAVIOR', 'Flores A, 2016, FEDERAL PROBATION', 'Razavian N, 2015, BIG DATA', 'Zeng J, 2016, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (STATISTICS IN SOCIETY)', 'Wang F, 2015, INTERNATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE AND STATISTICS', 'Rudin C, 2018, ARXIV (CORNELL UNIVERSITY)', 'Goodman B, 2016, ARXIV (CORNELL UNIVERSITY)', 'Tollenaar N, 2012, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (STATISTICS IN SOCIETY)', 'Rudin C, 2018, INFORMS JOURNAL ON APPLIED ANALYTICS', 'Gupta M, 2016, JOURNAL OF MACHINE LEARNING RESEARCH', 'Rudin C, 2020, HARVARD DATA SCIENCE REVIEW', 'Rüping S, 2006, ', 'Rudin C, 2010, MACHINE LEARNING', 'Ustun B, 2017, ', 'Auer P, 1995, ELSEVIER EBOOKS', 'Carrizosa E, 2009, INFORMS JOURNAL ON COMPUTING', 'Wang J, 2018, ', 'Gallagher N, 2017, NEURAL INFORMATION PROCESSING SYSTEMS', 'Chang A, 2012, MACHINE LEARNING', 'Goel A, 2017, AI MAGAZINE', 'Wang F, 2018, BIOSTATISTICS', 'Mannshardt E, 2018, SIGNIFICANCE', 'Neri P, 2018, INFORMS JOURNAL ON APPLIED ANALYTICS', ', , VIEW', 'Chen C, 2018, ARXIV (CORNELL UNIVERSITY)', 'Li O, 2017, ARXIV (CORNELL UNIVERSITY)', 'Chen C, 2018, ARXIV (CORNELL UNIVERSITY)', 'Carrière M, 2017, ARXIV (CORNELL UNIVERSITY)', "Sokolovska N, 2018, BASE INSTITUTIONNELLE DE RECHERCHE DE L'UNIVERSITÉ PARIS-DAUPHINE (BIRD) (UNIVERSITY PARIS-DAUPHINE)", ', 2017, AUERBACH PUBLICATIONS EBOOKS']</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Rudin C, 2019, NATURE MACHINE INTELLIGENCE</t>
-        </is>
-      </c>
-      <c r="Z38" t="inlineStr">
-        <is>
-          <t>Rudin C, 2019, NATURE MACHINE INTELLIGENCE</t>
+          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4365,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>3407</v>
+        <v>3409</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -4615,33 +4425,28 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>['US']</t>
+          <t>['https://openalex.org/W40442397', 'https://openalex.org/W1480376833', 'https://openalex.org/W1678356000', 'https://openalex.org/W1808991731', 'https://openalex.org/W1902027874', 'https://openalex.org/W1976196376', 'https://openalex.org/W2011999110', 'https://openalex.org/W2021701428', 'https://openalex.org/W2029243817', 'https://openalex.org/W2052825782', 'https://openalex.org/W2072128103', 'https://openalex.org/W2073751243', 'https://openalex.org/W2105464873', 'https://openalex.org/W2106665921', 'https://openalex.org/W2110243528', 'https://openalex.org/W2112289645', 'https://openalex.org/W2112592817', 'https://openalex.org/W2113606819', 'https://openalex.org/W2116802246', 'https://openalex.org/W2119361626', 'https://openalex.org/W2120480077', 'https://openalex.org/W2121495423', 'https://openalex.org/W2122111042', 'https://openalex.org/W2127482775', 'https://openalex.org/W2135046866', 'https://openalex.org/W2139212933', 'https://openalex.org/W2147461734', 'https://openalex.org/W2149298154', 'https://openalex.org/W2152072062', 'https://openalex.org/W2158927033', 'https://openalex.org/W2162586165', 'https://openalex.org/W2163697531', 'https://openalex.org/W2164434252', 'https://openalex.org/W2345255551', 'https://openalex.org/W2787894218', 'https://openalex.org/W2911964244', 'https://openalex.org/W2912934387', 'https://openalex.org/W2963481018', 'https://openalex.org/W2998216295', 'https://openalex.org/W3099478002', 'https://openalex.org/W4212883601', 'https://openalex.org/W4231109964', 'https://openalex.org/W4243607236', 'https://openalex.org/W4285719527', 'https://openalex.org/W6601599523', 'https://openalex.org/W6676903177', 'https://openalex.org/W7066667914']</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>['Breiman L, 2001, MACHINE LEARNING', 'Tibshirani R, 1996, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Friedman J, 2001, THE ANNALS OF STATISTICS', 'Hastie T, 2001, SPRINGER SERIES IN STATISTICS', 'Hastie T, 2009, SPRINGER SERIES IN STATISTICS', 'Breiman L, 1996, MACHINE LEARNING', 'Burges C, 1998, DATA MINING AND KNOWLEDGE DISCOVERY', 'Breiman L, 1996, MACHINE LEARNING', 'Cover T, 1967, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Lee D, 1999, NATURE', 'GuyonIsabelle, 2003, JOURNAL OF MACHINE LEARNING RESEARCH', 'Bengio Y, 2009, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Lip G, 2009, CHEST JOURNAL', 'Vapnik V, 1999, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Bengio Y, 2009, NOW PUBLISHERS, INC. EBOOKS', 'Olshausen B, 1997, VISION RESEARCH', 'Pitt B, 2014, NEW ENGLAND JOURNAL OF MEDICINE', 'Ishwaran H, 2008, THE ANNALS OF APPLIED STATISTICS', 'Lee H, 2007, THE MIT PRESS EBOOKS', 'D’Agostino R, 2001, JAMA', 'Woodruff P, 2009, AMERICAN JOURNAL OF RESPIRATORY AND CRITICAL CARE MEDICINE', 'Le Q, 2013, ', 'Corren J, 2011, NEW ENGLAND JOURNAL OF MEDICINE', 'Ishwaran H, 2008, ', 'O’Mahony C, 2013, EUROPEAN HEART JOURNAL', 'James M, 2012, PHYSIOLOGICAL REVIEWS', 'Shah S, 2014, CIRCULATION', 'Beck A, 2011, SCIENCE TRANSLATIONAL MEDICINE', 'Koren Y, 2009, ', 'Peña‐Castillo L, 2008, GENOME BIOLOGY', 'Abu‐Mostafa Y, 2012, ', 'Hsich E, 2010, CIRCULATION CARDIOVASCULAR QUALITY AND OUTCOMES', 'Cheng W, 2013, SCIENCE TRANSLATIONAL MEDICINE', 'Margolin A, 2013, SCIENCE TRANSLATIONAL MEDICINE', 'Udelson J, 2011, CIRCULATION', 'Kannel W, 1975, CIRCULATION', 'Cheng W, 2013, PLOS COMPUTATIONAL BIOLOGY', 'Gorodeski E, 2011, CIRCULATION CARDIOVASCULAR QUALITY AND OUTCOMES', 'Deo R, 2014, GENOME BIOLOGY', 'Yogatama D, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ausiello D, 2014, EUROPE PMC (PUBMED CENTRAL)']</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Rahul C. Deo, 2015, Circulation</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>Deo R, 2015, CIRCULATION</t>
-        </is>
-      </c>
-      <c r="Z39" t="inlineStr">
-        <is>
-          <t>Deo R, 2015, CIRCULATION</t>
+          <t>Rahul C. Deo, 2015, Circulation</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4480,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>4194</v>
+        <v>4207</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -4731,33 +4536,28 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>['GB', 'US']</t>
+          <t>['https://openalex.org/W8316075', 'https://openalex.org/W21006490', 'https://openalex.org/W22229905', 'https://openalex.org/W59175527', 'https://openalex.org/W68733909', 'https://openalex.org/W129606432', 'https://openalex.org/W155596317', 'https://openalex.org/W189596042', 'https://openalex.org/W199018803', 'https://openalex.org/W262578090', 'https://openalex.org/W854541894', 'https://openalex.org/W877909479', 'https://openalex.org/W956551720', 'https://openalex.org/W1123427201', 'https://openalex.org/W1480583224', 'https://openalex.org/W1481820510', 'https://openalex.org/W1488163396', 'https://openalex.org/W1503933356', 'https://openalex.org/W1514535095', 'https://openalex.org/W1522301498', 'https://openalex.org/W1523385540', 'https://openalex.org/W1527575280', 'https://openalex.org/W1528056001', 'https://openalex.org/W1533861849', 'https://openalex.org/W1540429825', 'https://openalex.org/W1555767263', 'https://openalex.org/W1566289585', 'https://openalex.org/W1572567476', 'https://openalex.org/W1573040851', 'https://openalex.org/W1586939924', 'https://openalex.org/W1601567445', 'https://openalex.org/W1628307106', 'https://openalex.org/W1651753422', 'https://openalex.org/W1664311846', 'https://openalex.org/W1686810756', 'https://openalex.org/W1687846465', 'https://openalex.org/W1753482797', 'https://openalex.org/W1762503104', 'https://openalex.org/W1766290689', 'https://openalex.org/W1773149199', 'https://openalex.org/W1811254738', 'https://openalex.org/W1822526425', 'https://openalex.org/W1828348983', 'https://openalex.org/W1836465849', 'https://openalex.org/W1858383477', 'https://openalex.org/W1870428314', 'https://openalex.org/W1872883209', 'https://openalex.org/W1883346539', 'https://openalex.org/W1889038981', 'https://openalex.org/W1889081078', 'https://openalex.org/W1893116441', 'https://openalex.org/W1895577753', 'https://openalex.org/W1897761818', 'https://openalex.org/W1905882502', 'https://openalex.org/W1906515132', 'https://openalex.org/W1922557984', 'https://openalex.org/W1931795219', 'https://openalex.org/W1933065844', 'https://openalex.org/W1933349210', 'https://openalex.org/W1956340063', 'https://openalex.org/W1963540633', 'https://openalex.org/W1964073652', 'https://openalex.org/W1966811077', 'https://openalex.org/W1969616664', 'https://openalex.org/W1970055505', 'https://openalex.org/W1971791733', 'https://openalex.org/W1976066595', 'https://openalex.org/W1977547683', 'https://openalex.org/W1985867508', 'https://openalex.org/W1986451414', 'https://openalex.org/W1987835821', 'https://openalex.org/W1996418862', 'https://openalex.org/W1996478295', 'https://openalex.org/W2000911139', 'https://openalex.org/W2003333103', 'https://openalex.org/W2006969979', 'https://openalex.org/W2009059481', 'https://openalex.org/W2012237712', 'https://openalex.org/W2015394094', 'https://openalex.org/W2015412875', 'https://openalex.org/W2019024625', 'https://openalex.org/W2022799064', 'https://openalex.org/W2025341678', 'https://openalex.org/W2025638820', 'https://openalex.org/W2026012689', 'https://openalex.org/W2026243162', 'https://openalex.org/W2038698865', 'https://openalex.org/W2041288440', 'https://openalex.org/W2042608483', 'https://openalex.org/W2048343491', 'https://openalex.org/W2048679005', 'https://openalex.org/W2051721233', 'https://openalex.org/W2053101950', 'https://openalex.org/W2057568625', 'https://openalex.org/W2058616948', 'https://openalex.org/W2061781940', 'https://openalex.org/W2062632672', 'https://openalex.org/W2062955551', 'https://openalex.org/W2063036810', 'https://openalex.org/W2063330527', 'https://openalex.org/W2064675550', 'https://openalex.org/W2066667210', 'https://openalex.org/W2068676460', 'https://openalex.org/W2069682406', 'https://openalex.org/W2077395415', 'https://openalex.org/W2080576537', 'https://openalex.org/W2083885588', 'https://openalex.org/W2090048052', 'https://openalex.org/W2095705004', 'https://openalex.org/W2096391593', 'https://openalex.org/W2098411764', 'https://openalex.org/W2098562545', 'https://openalex.org/W2099471712', 'https://openalex.org/W2100235303', 'https://openalex.org/W2100561338', 'https://openalex.org/W2101105183', 'https://openalex.org/W2101534792', 'https://openalex.org/W2102765684', 'https://openalex.org/W2105103432', 'https://openalex.org/W2106277773', 'https://openalex.org/W2108710284', 'https://openalex.org/W2109586012', 'https://openalex.org/W2109743529', 'https://openalex.org/W2111078031', 'https://openalex.org/W2111645492', 'https://openalex.org/W2112019442', 'https://openalex.org/W2112184938', 'https://openalex.org/W2112912048', 'https://openalex.org/W2113507809', 'https://openalex.org/W2118714046', 'https://openalex.org/W2119288237', 'https://openalex.org/W2120776756', 'https://openalex.org/W2123024445', 'https://openalex.org/W2124033848', 'https://openalex.org/W2124372976', 'https://openalex.org/W2125336414', 'https://openalex.org/W2125366733', 'https://openalex.org/W2126598020', 'https://openalex.org/W2128856065', 'https://openalex.org/W2129142580', 'https://openalex.org/W2129360799', 'https://openalex.org/W2129382193', 'https://openalex.org/W2130055251', 'https://openalex.org/W2130162821', 'https://openalex.org/W2130942839', 'https://openalex.org/W2131179926', 'https://openalex.org/W2133459682', 'https://openalex.org/W2133564696', 'https://openalex.org/W2135776491', 'https://openalex.org/W2136922672', 'https://openalex.org/W2136985729', 'https://openalex.org/W2137735870', 'https://openalex.org/W2137806537', 'https://openalex.org/W2141477623', 'https://openalex.org/W2142192571', 'https://openalex.org/W2142900973', 'https://openalex.org/W2143449221', 'https://openalex.org/W2143492886', 'https://openalex.org/W2143612262', 'https://openalex.org/W2143926884', 'https://openalex.org/W2145056192', 'https://openalex.org/W2147880316', 'https://openalex.org/W2147885303', 'https://openalex.org/W2148298736', 'https://openalex.org/W2149172860', 'https://openalex.org/W2149557440', 'https://openalex.org/W2149940198', 'https://openalex.org/W2150295085', 'https://openalex.org/W2150658333', 'https://openalex.org/W2150696241', 'https://openalex.org/W2150824314', 'https://openalex.org/W2151096985', 'https://openalex.org/W2151103935', 'https://openalex.org/W2152239535', 'https://openalex.org/W2153579005', 'https://openalex.org/W2153927146', 'https://openalex.org/W2156303437', 'https://openalex.org/W2156503193', 'https://openalex.org/W2159973364', 'https://openalex.org/W2160815625', 'https://openalex.org/W2163108352', 'https://openalex.org/W2163605009', 'https://openalex.org/W2163922914', 'https://openalex.org/W2164186291', 'https://openalex.org/W2164450870', 'https://openalex.org/W2164587673', 'https://openalex.org/W2164699598', 'https://openalex.org/W2167103782', 'https://openalex.org/W2173180041', 'https://openalex.org/W2180844455', 'https://openalex.org/W2181691731', 'https://openalex.org/W2184045248', 'https://openalex.org/W2184188583', 'https://openalex.org/W2185175083', 'https://openalex.org/W2201007611', 'https://openalex.org/W2203543769', 'https://openalex.org/W2220981600', 'https://openalex.org/W2250742840', 'https://openalex.org/W2250842428', 'https://openalex.org/W2251353663', 'https://openalex.org/W2251394420', 'https://openalex.org/W2251885125', 'https://openalex.org/W2251970440', 'https://openalex.org/W2252122141', 'https://openalex.org/W2252238675', 'https://openalex.org/W2266728343', 'https://openalex.org/W2267126114', 'https://openalex.org/W2282219577', 'https://openalex.org/W2291822808', 'https://openalex.org/W2293453011', 'https://openalex.org/W2294797155', 'https://openalex.org/W2296613712', 'https://openalex.org/W2316138215', 'https://openalex.org/W2327501763', 'https://openalex.org/W2342662179', 'https://openalex.org/W2388114291', 'https://openalex.org/W2397159106', 'https://openalex.org/W2399507222', 'https://openalex.org/W2399733683', 'https://openalex.org/W2402955625', 'https://openalex.org/W2405756170', 'https://openalex.org/W2411037331', 'https://openalex.org/W2418349398', 'https://openalex.org/W2434537049', 'https://openalex.org/W2462496837', 'https://openalex.org/W2470413457', 'https://openalex.org/W2489434015', 'https://openalex.org/W2494980014', 'https://openalex.org/W2519091744', 'https://openalex.org/W2519656895', 'https://openalex.org/W2520160253', 'https://openalex.org/W2546919788', 'https://openalex.org/W2557865186', 'https://openalex.org/W2579317665', 'https://openalex.org/W2914699769', 'https://openalex.org/W2949465329', 'https://openalex.org/W2953318193', 'https://openalex.org/W2962706528', 'https://openalex.org/W2962756039', 'https://openalex.org/W2962835968', 'https://openalex.org/W2963082528', 'https://openalex.org/W2963109634', 'https://openalex.org/W2963143316', 'https://openalex.org/W2963192057', 'https://openalex.org/W2963260436', 'https://openalex.org/W2963324994', 'https://openalex.org/W2963383024', 'https://openalex.org/W2963389687', 'https://openalex.org/W2963410018', 'https://openalex.org/W2963576560', 'https://openalex.org/W2963579811', 'https://openalex.org/W2963605190', 'https://openalex.org/W2963656855', 'https://openalex.org/W2963735856', 'https://openalex.org/W2963811219', 'https://openalex.org/W2963899908', 'https://openalex.org/W2963954913', 'https://openalex.org/W2964040984', 'https://openalex.org/W2964118342', 'https://openalex.org/W2964121744', 'https://openalex.org/W2964217371', 'https://openalex.org/W2964241990', 'https://openalex.org/W2964308564', 'https://openalex.org/W2964345931', 'https://openalex.org/W3000384245', 'https://openalex.org/W3023993913', 'https://openalex.org/W3087871082', 'https://openalex.org/W3125032682', 'https://openalex.org/W4211232216', 'https://openalex.org/W4212844288', 'https://openalex.org/W4240592325', 'https://openalex.org/W4244018879', 'https://openalex.org/W4245655784', 'https://openalex.org/W4252331534', 'https://openalex.org/W4285719527', 'https://openalex.org/W4293665662', 'https://openalex.org/W4294170691', 'https://openalex.org/W4297813007', 'https://openalex.org/W4299801216', 'https://openalex.org/W4302613066', 'https://openalex.org/W4320013936', 'https://openalex.org/W6600334730', 'https://openalex.org/W6600827882', 'https://openalex.org/W6605295763', 'https://openalex.org/W6606244218', 'https://openalex.org/W6606327593', 'https://openalex.org/W6607775107', 'https://openalex.org/W6608183366', 'https://openalex.org/W6623517193', 'https://openalex.org/W6623995992', 'https://openalex.org/W6625044600', 'https://openalex.org/W6628794645', 'https://openalex.org/W6629203210', 'https://openalex.org/W6630875275', 'https://openalex.org/W6631190155', 'https://openalex.org/W6631216910', 'https://openalex.org/W6631516269', 'https://openalex.org/W6631943919', 'https://openalex.org/W6634126550', 'https://openalex.org/W6636447180', 'https://openalex.org/W6636942303', 'https://openalex.org/W6637306801', 'https://openalex.org/W6637373629', 'https://openalex.org/W6637698695', 'https://openalex.org/W6637971603', 'https://openalex.org/W6637989529', 'https://openalex.org/W6638549007', 'https://openalex.org/W6638667902', 'https://openalex.org/W6638742206', 'https://openalex.org/W6639103823', 'https://openalex.org/W6639118148', 'https://openalex.org/W6639283537', 'https://openalex.org/W6639358663', 'https://openalex.org/W6639432524', 'https://openalex.org/W6639434097', 'https://openalex.org/W6640257717', 'https://openalex.org/W6640296258', 'https://openalex.org/W6640764460', 'https://openalex.org/W6650605322', 'https://openalex.org/W6652311901', 'https://openalex.org/W6674330103', 'https://openalex.org/W6675048546', 'https://openalex.org/W6676380891', 'https://openalex.org/W6676497082', 'https://openalex.org/W6676647902', 'https://openalex.org/W6676709516', 'https://openalex.org/W6678360021', 'https://openalex.org/W6678470764', 'https://openalex.org/W6678809451', 'https://openalex.org/W6679434410', 'https://openalex.org/W6679436768', 'https://openalex.org/W6680094886', 'https://openalex.org/W6680336390', 'https://openalex.org/W6681184217', 'https://openalex.org/W6682082992', 'https://openalex.org/W6682086108', 'https://openalex.org/W6682222085', 'https://openalex.org/W6682511423', 'https://openalex.org/W6682691769', 'https://openalex.org/W6682864246', 'https://openalex.org/W6683074461', 'https://openalex.org/W6683167905', 'https://openalex.org/W6683277684', 'https://openalex.org/W6684191040', 'https://openalex.org/W6684209796', 'https://openalex.org/W6685183736', 'https://openalex.org/W6685527872', 'https://openalex.org/W6686207219', 'https://openalex.org/W6687543112', 'https://openalex.org/W6687672932', 'https://openalex.org/W6688143368', 'https://openalex.org/W6691419566', 'https://openalex.org/W6691647468', 'https://openalex.org/W6692004142', 'https://openalex.org/W6696843773', 'https://openalex.org/W6697449767', 'https://openalex.org/W6712426025', 'https://openalex.org/W6712802073', 'https://openalex.org/W6713645886', 'https://openalex.org/W6717487601', 'https://openalex.org/W6726977916', 'https://openalex.org/W6727336983', 'https://openalex.org/W6729831399', 'https://openalex.org/W6730042849', 'https://openalex.org/W6730666313', 'https://openalex.org/W6732843983', 'https://openalex.org/W6845679800', 'https://openalex.org/W6898505805', 'https://openalex.org/W7011438494']</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>['Glorot X, 2010, ', 'Zhu Y, 2015, ', 'Salakhutdinov R, 2009, ', 'Plummer B, 2015, ', 'Kalchbrenner N, 2013, ', 'Hodosh M, 2013, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Andrew G, 2013, ', 'Ghahramani Z, 1997, MACHINE LEARNING', 'Yao L, 2015, ', 'Sutton C, 2007, THE MIT PRESS EBOOKS', 'Weston J, 2011, ', 'Pan Y, 2016, ', 'Wang W, 2015, ', 'Kumar S, 2012, ', 'Mitchell M, 2012, CONFERENCE OF THE EUROPEAN CHAPTER OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Louwerse M, 2010, TOPICS IN COGNITIVE SCIENCE', 'Kahou S, 2015, JOURNAL ON MULTIMODAL USER INTERFACES', 'Gregory K, 2014, IT UNIVERSITY OF COPENHAGEN (IT UNIVERSITY OF COPENHAGEN)', 'Li S, 2011, ', 'Kojima A, 2002, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Yang Y, 2011, ', 'Xu R, 2015, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Castellano G, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Mroueh Y, 2015, ', 'Glodek M, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Cour T, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Gupta A, 2021, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Morvant E, 2014, LECTURE NOTES IN COMPUTER SCIENCE', 'Bojanowski P, 2015, ', 'Feng Y, 2010, EDINBURGH RESEARCH EXPLORER (UNIVERSITY OF EDINBURGH)', 'Wei Y, 2016, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Chen Y, 2004, ', 'Sjölander K, 2003, ', 'Wu Z, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Naim I, 2014, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Khapra M, 2010, ', 'Deena S, 2009, LECTURE NOTES IN COMPUTER SCIENCE', 'Kingma D, 2014, UVA-DARE (UNIVERSITY OF AMSTERDAM)', 'Simonyan K, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ioffe S, 2015, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chorowski J, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chen X, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kiros R, 2014, ARXIV (CORNELL UNIVERSITY)', 'Mao J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Gao H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Torabi A, 2015, ARXIV (CORNELL UNIVERSITY)', 'McFee B, 2010, ARXIV (CORNELL UNIVERSITY)', 'Christoudias C, 2012, ARXIV (CORNELL UNIVERSITY)', 'Lebret R, 2015, ARXIV (CORNELL UNIVERSITY)', 'Vinyals O, 2015, ', 'McGurk H, 1976, NATURE', 'Blum A, 1998, ', 'Hotelling H, 1936, BIOMETRIKA', 'Karpathy A, 2015, ', 'Vedantam R, 2015, ', 'Antol S, 2015, ', 'Brown P, 1993, ', 'Farhadi A, 2010, LECTURE NOTES IN COMPUTER SCIENCE', 'Atrey P, 2010, MULTIMEDIA SYSTEMS', 'Kulkarni G, 2013, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Vogel S, 1996, ', 'Juang B, 1991, TECHNOMETRICS', 'D’Mello S, 2015, ACM COMPUTING SURVEYS', 'Feng F, 2014, ', 'Valstar M, 2013, ', 'Bronstein M, 2010, ', 'Kim Y, 2013, ', 'Lienhart R, 1998, PROCEEDINGS OF SPIE, THE INTERNATIONAL SOCIETY FOR OPTICAL ENGINEERING/PROCEEDINGS OF SPIE', 'Kruskal J, 1983, SIAM REVIEW', 'Yao B, 2010, PROCEEDINGS OF THE IEEE', 'Wöllmer M, 2012, IMAGE AND VISION COMPUTING', 'Ouyang W, 2014, ', 'Evangelopoulos G, 2013, IEEE TRANSACTIONS ON MULTIMEDIA', 'Socher R, 2010, ', 'Li Y, 2014, NEUROCOMPUTING', 'Zitnick C, 2013, ', 'Kong C, 2014, ', 'Huang J, 2013, ', 'Sargin M, 2007, IEEE TRANSACTIONS ON MULTIMEDIA', 'Zhou F, 2012, ', 'Mei H, 2016, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Liu F, 2013, IEEE JOURNAL OF BIOMEDICAL AND HEALTH INFORMATICS', 'Rohrbach A, 2015, LECTURE NOTES IN COMPUTER SCIENCE', 'Chen S, 2015, ', 'Sarah T, 2012, ', 'Baltrušaitis T, 2013, ', 'Chen J, 2014, ', 'Zen H, 2012, IEEE TRANSACTIONS ON AUDIO SPEECH AND LANGUAGE PROCESSING', 'Tapaswi M, 2015, ', 'Arora R, 2013, ', 'Feng F, 2014, NEUROCOMPUTING', 'Bourlard H, 2002, ', 'Yeh Y, 2012, IEEE TRANSACTIONS ON MULTIMEDIA', 'Noulas A, 2011, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Jiang X, 2014, PATTERN RECOGNITION LETTERS', 'Haubold A, 2007, ', 'Tapaswi M, 2014, INTERNATIONAL JOURNAL OF MULTIMEDIA INFORMATION RETRIEVAL', 'Wu D, 2014, ', 'Klein B, 2014, ARXIV (CORNELL UNIVERSITY)', 'Hochreiter S, 1997, NEURAL COMPUTATION', 'Srivastava N, 2014, ', '淳司 柴, 2017, JOURNAL OF JAPAN SOCIETY FOR FUZZY THEORY AND INTELLIGENT INFORMATICS', 'Papineni K, 2001, ', 'Hinton G, 2006, NEURAL COMPUTATION', 'Hardoon D, 2004, NEURAL COMPUTATION', 'Denkowski M, 2014, ', 'Frome A, 2013, ', 'Farhadi A, 2009, 2009 IEEE CONFERENCE ON COMPUTER VISION AND PATTERN RECOGNITION', 'Gönen M, 2011, ', 'Rasiwasia N, 2010, ', 'Zen H, 2009, SPEECH COMMUNICATION', 'Suk H, 2014, NEUROIMAGE', 'Ordóñez V, 2011, ', 'James A, 2014, INFORMATION FUSION', 'Bruni E, 2014, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Carletta J, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Gehler P, 2009, ', 'Pomianos G, 2003, PROCEEDINGS OF THE IEEE', 'Bigham J, 2010, ', 'Lai P, 2000, INTERNATIONAL JOURNAL OF NEURAL SYSTEMS', 'Quattoni A, 2007, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Regneri M, 2013, TRANSACTIONS OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Snoek C, 2004, MULTIMEDIA TOOLS AND APPLICATIONS', 'Anagnostopoulos C, 2012, ARTIFICIAL INTELLIGENCE REVIEW', 'Weston J, 2010, MACHINE LEARNING', 'Coyne B, 2001, ', 'Bucak S, 2014, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'McKeown G, 2010, ', 'Schuller B, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Devlin J, 2015, ', 'Bojanowski P, 2014, LECTURE NOTES IN COMPUTER SCIENCE', 'Wu Z, 2014, ', 'Elliott D, 2014, ', 'Mason R, 2014, ', 'Ramírez G, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Anderson R, 2013, ', 'Song Y, 2012, ', 'Slaney M, 2000, NEURAL INFORMATION PROCESSING SYSTEMS', 'Lan Z, 2013, MULTIMEDIA TOOLS AND APPLICATIONS', 'Chang A, 2015, ', 'Gurban M, 2008, ', 'Krogel M, 2004, MACHINE LEARNING', 'Garg A, 2003, PROCEEDINGS OF THE IEEE', 'Christoudias C, 2006, ', 'Cosi P, 2002, ', 'Bahdanau D, 2014, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Socher R, 2013, ARXIV (CORNELL UNIVERSITY)', 'Karpathy A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2017, COMMUNICATIONS OF THE ACM', 'Lowe D, 2004, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Lafferty J, 2001, SCHOLARLY COMMONS (UNIVERSITY OF PENNSYLVANIA)', 'Bengio Y, 2013, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Graves A, 2013, ', 'Zeng Z, 2008, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Young P, 2014, TRANSACTIONS OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Ngiam J, 2011, ', 'Hinton G, 2012, ', 'Lin C, 2003, ', 'Hunt A, 2002, ', 'Brand M, 2002, ', 'Socher R, 2014, TRANSACTIONS OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Palatucci M, 2018, FIGSHARE', 'Soleymani M, 2011, IEEE TRANSACTIONS ON AFFECTIVE COMPUTING', 'Bregler C, 1997, ', 'Zhang D, 2014, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Malinowski M, 2015, ', 'Guadarrama S, 2013, ', 'Nicolaou M, 2011, IEEE TRANSACTIONS ON AFFECTIVE COMPUTING', 'Jia X, 2015, ', 'Harvey D, 2009, ', 'Bruni E, 2012, INSTITUTIONAL RESEARCH INFORMATION SYSTEM (UNIVERSITÀ DEGLI STUDI DI TRENTO)', 'Кузнецова П, 2012, ', 'Hendricks L, 2016, ', 'Elliott D, 2013, ', 'Kiela D, 2014, ', 'Левин, 2003, ', 'Silberer C, 2014, ', 'Nefian A, 2002, IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS SPEECH AND SIGNAL PROCESSING', 'Yuhas B, 1989, IEEE COMMUNICATIONS MAGAZINE', 'Wöllmer M, 2010, ', 'Zhou F, 2009, ', 'Thomason J, 2014, ', 'Sikka K, 2013, ', 'Qin T, 2008, ', 'Yu H, 2013, ', 'Wang D, 2015, INTERNATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Sarkar A, 2001, ', 'Song Y, 2012, ', 'Nakov P, 2012, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Yagcioglu S, 2015, ', 'Shariat S, 2011, ', 'Masuko T, 2002, ', 'Reiter S, 2007, ', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Simonyan K, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ratnaparkhi A, 2000, ARXIV.ORG', 'Feichtenhofer C, 2016, ', 'Chan W, 2016, ', 'Fukui A, 2016, ', 'Mao J, 2016, ', 'Yu L, 2016, LECTURE NOTES IN COMPUTER SCIENCE', 'Jiang Q, 2017, ', 'Trigeorgis G, 2016, ', 'Wang L, 2016, ', 'Yu H, 2016, ', 'Poria S, 2015, ', 'Müller M, 2008, ', 'Fan Y, 2014, ', 'Bernardi R, 2016, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Rohrbach A, 2017, INTERNATIONAL JOURNAL OF COMPUTER VISION', ', 2009, ENCYCLOPEDIA OF BIOMETRICS', 'Cao Y, 2016, ', 'Nojavanasghari B, 2016, ', 'Shutova E, 2016, ', 'Srivastava N, 2012, ', 'Mahasseni B, 2016, ', 'Rajagopalan S, 2016, LECTURE NOTES IN COMPUTER SCIENCE', 'Gebru I, 2017, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Baroni M, 2015, LANGUAGE AND LINGUISTICS COMPASS', 'Lazaridou A, 2014, ', 'Kiela D, 2015, ', 'Silberer C, 2012, EDINBURGH RESEARCH EXPLORER (UNIVERSITY OF EDINBURGH)', 'Gao H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kiela D, 2015, ', 'Trigeorgis G, 2016, ', 'Jin Q, 2016, ', 'Song Y, 2016, INTERNATIONAL JOINT CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Naim I, 2015, ', 'Anguera X, 2014, ', 'Moon S, 2014, ', 'Oord A, 2016, ARXIV (CORNELL UNIVERSITY)', 'Reed S, 2016, ARXIV (CORNELL UNIVERSITY)', 'Oord A, 2016, ARXIV (CORNELL UNIVERSITY)', 'Xiong C, 2016, ARXIV (CORNELL UNIVERSITY)', 'Oord A, 2016, ARXIV (CORNELL UNIVERSITY)', 'Collobert R, 2016, ARXIV (CORNELL UNIVERSITY)', 'Lu J, 2016, ARXIV (CORNELL UNIVERSITY)', 'Kuan-Lin C, 2021, DROPS (SCHLOSS DAGSTUHL – LEIBNIZ CENTER FOR INFORMATICS)', 'Labaca-Castro R, 2023, ', 'Barsalou L, 2007, ANNUAL REVIEW OF PSYCHOLOGY', 'Yang Z, 2016, ', ', 2007, ', 'Xu H, 2016, LECTURE NOTES IN COMPUTER SCIENCE', 'Juang B, 1991, TECHNOMETRICS', 'Hu R, 2016, ', 'Xiong C, 2016, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Huang T, 2016, ', 'Zeng K, 2017, ', 'Torre F, 2011, ', 'Nefian, 2002, IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS SPEECH AND SIGNAL PROCESSING', 'McFeeBrian, 2011, JOURNAL OF MACHINE LEARNING RESEARCH', 'Bourlard H, 1996, 4TH INTERNATIONAL CONFERENCE ON SPOKEN LANGUAGE PROCESSING (ICSLP 1996)', 'Zhang H, 2016, ', 'Ghahramani Z, 1996, ', 'Mei H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Klein B, 2014, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W40" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Tadas Baltrušaitis, 2018, IEEE Transactions on Pattern Analysis and Machine Intelligence</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>Baltrušaitis T, 2018, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE</t>
-        </is>
-      </c>
-      <c r="Z40" t="inlineStr">
-        <is>
-          <t>Baltrušaitis T, 2018, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE</t>
+          <t>Tadas Baltrušaitis, 2018, IEEE Transactions on Pattern Analysis and Machine Intelligence</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4591,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>5100</v>
+        <v>5107</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -4847,33 +4647,28 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>['BD', 'AU']</t>
+          <t>['https://openalex.org/W4952878', 'https://openalex.org/W28669376', 'https://openalex.org/W44815768', 'https://openalex.org/W1128809682', 'https://openalex.org/W1484413656', 'https://openalex.org/W1484780623', 'https://openalex.org/W1491541693', 'https://openalex.org/W1498810706', 'https://openalex.org/W1508065755', 'https://openalex.org/W1515231270', 'https://openalex.org/W1543320899', 'https://openalex.org/W1566114229', 'https://openalex.org/W1570448133', 'https://openalex.org/W1594031697', 'https://openalex.org/W1629143244', 'https://openalex.org/W1673310716', 'https://openalex.org/W1806329564', 'https://openalex.org/W1912123407', 'https://openalex.org/W1917795079', 'https://openalex.org/W1927026191', 'https://openalex.org/W1948199107', 'https://openalex.org/W1965702297', 'https://openalex.org/W1967661515', 'https://openalex.org/W1974016210', 'https://openalex.org/W1977496278', 'https://openalex.org/W1981276685', 'https://openalex.org/W1982582425', 'https://openalex.org/W1989344766', 'https://openalex.org/W1990517717', 'https://openalex.org/W2015057666', 'https://openalex.org/W2018936209', 'https://openalex.org/W2026513874', 'https://openalex.org/W2058401212', 'https://openalex.org/W2064853889', 'https://openalex.org/W2069140227', 'https://openalex.org/W2071128523', 'https://openalex.org/W2083620785', 'https://openalex.org/W2088093492', 'https://openalex.org/W2090991262', 'https://openalex.org/W2097117768', 'https://openalex.org/W2099404336', 'https://openalex.org/W2099940443', 'https://openalex.org/W2101234009', 'https://openalex.org/W2106393550', 'https://openalex.org/W2107726111', 'https://openalex.org/W2109255472', 'https://openalex.org/W2112076978', 'https://openalex.org/W2112796928', 'https://openalex.org/W2119567691', 'https://openalex.org/W2120240539', 'https://openalex.org/W2120636621', 'https://openalex.org/W2127218421', 'https://openalex.org/W2132166479', 'https://openalex.org/W2134089414', 'https://openalex.org/W2140190241', 'https://openalex.org/W2142827986', 'https://openalex.org/W2143554828', 'https://openalex.org/W2144219012', 'https://openalex.org/W2147169507', 'https://openalex.org/W2149706766', 'https://openalex.org/W2151040995', 'https://openalex.org/W2154298720', 'https://openalex.org/W2160642098', 'https://openalex.org/W2163605009', 'https://openalex.org/W2164500538', 'https://openalex.org/W2166559705', 'https://openalex.org/W2194775991', 'https://openalex.org/W2215376118', 'https://openalex.org/W2257979135', 'https://openalex.org/W2294798173', 'https://openalex.org/W2296509296', 'https://openalex.org/W2341117600', 'https://openalex.org/W2394309960', 'https://openalex.org/W2395579298', 'https://openalex.org/W2504658994', 'https://openalex.org/W2510496529', 'https://openalex.org/W2518882834', 'https://openalex.org/W2531409750', 'https://openalex.org/W2557283755', 'https://openalex.org/W2580909119', 'https://openalex.org/W2581465409', 'https://openalex.org/W2603678388', 'https://openalex.org/W2609368436', 'https://openalex.org/W2617585083', 'https://openalex.org/W2617697157', 'https://openalex.org/W2622382573', 'https://openalex.org/W2713640100', 'https://openalex.org/W2724111113', 'https://openalex.org/W2752236180', 'https://openalex.org/W2762644836', 'https://openalex.org/W2771053518', 'https://openalex.org/W2802574842', 'https://openalex.org/W2803881474', 'https://openalex.org/W2806407311', 'https://openalex.org/W2889193967', 'https://openalex.org/W2904346290', 'https://openalex.org/W2906027675', 'https://openalex.org/W2909445826', 'https://openalex.org/W2910891387', 'https://openalex.org/W2911964244', 'https://openalex.org/W2912934387', 'https://openalex.org/W2913771179', 'https://openalex.org/W2940523548', 'https://openalex.org/W2950722229', 'https://openalex.org/W2954936648', 'https://openalex.org/W2955285339', 'https://openalex.org/W2960015156', 'https://openalex.org/W2962824709', 'https://openalex.org/W2963748489', 'https://openalex.org/W2971145443', 'https://openalex.org/W2982291760', 'https://openalex.org/W2990933508', 'https://openalex.org/W2991970757', 'https://openalex.org/W2998019206', 'https://openalex.org/W2998574808', 'https://openalex.org/W2999729612', 'https://openalex.org/W3002041203', 'https://openalex.org/W3003734944', 'https://openalex.org/W3007397514', 'https://openalex.org/W3011204221', 'https://openalex.org/W3014867431', 'https://openalex.org/W3016540417', 'https://openalex.org/W3017881119', 'https://openalex.org/W3019166713', 'https://openalex.org/W3023402713', 'https://openalex.org/W3034560014', 'https://openalex.org/W3037163353', 'https://openalex.org/W3038955483', 'https://openalex.org/W3039828206', 'https://openalex.org/W3041463877', 'https://openalex.org/W3044397306', 'https://openalex.org/W3044730720', 'https://openalex.org/W3049757379', 'https://openalex.org/W3083228182', 'https://openalex.org/W3084246142', 'https://openalex.org/W3085162807', 'https://openalex.org/W3086286002', 'https://openalex.org/W3095217282', 'https://openalex.org/W3099185017', 'https://openalex.org/W3100378204', 'https://openalex.org/W3102116369', 'https://openalex.org/W3121263745', 'https://openalex.org/W3122594683', 'https://openalex.org/W3129290453', 'https://openalex.org/W3130145150', 'https://openalex.org/W3139008799', 'https://openalex.org/W3149084432', 'https://openalex.org/W4212883601', 'https://openalex.org/W4230470477', 'https://openalex.org/W4236137412', 'https://openalex.org/W4244238212', 'https://openalex.org/W4245160364', 'https://openalex.org/W4298023569', 'https://openalex.org/W4298882835', 'https://openalex.org/W6601142415', 'https://openalex.org/W6674887505', 'https://openalex.org/W6675354045', 'https://openalex.org/W6675567579', 'https://openalex.org/W6676769703', 'https://openalex.org/W6843735874']</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>['LeCun Y, 1998, PROCEEDINGS OF THE IEEE', 'Szegedy C, 2015, ', 'Witten I, 2011, ELSEVIER EBOOKS', 'Gordon A, 1984, BIOMETRICS', 'Cios K, 1997, NEUROCOMPUTING', 'Ester M, 1996, ', 'He K, 2015, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Agrawal R, 1998, ', 'Hotelling H, 1933, JOURNAL OF EDUCATIONAL PSYCHOLOGY', 'Kaelbling L, 1996, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Hazeghi K, 1995, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Kohonen T, 1990, PROCEEDINGS OF THE IEEE', 'Freund Y, 1996, ', 'Han J, 2000, ACM SIGMOD RECORD', 'Zanella A, 2014, IEEE INTERNET OF THINGS JOURNAL', 'Dey A, 2001, PERSONAL AND UBIQUITOUS COMPUTING', 'Tavallaee M, 2009, ', 'Hinton G, 2012, LECTURE NOTES IN COMPUTER SCIENCE', 'Agrawal R, 1998, ', 'Park H, 2008, EXPERT SYSTEMS WITH APPLICATIONS', 'Xu D, 2015, ANNALS OF DATA SCIENCE', 'Zaki M, 2000, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Cessie S, 1992, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Amit Y, 1997, NEURAL COMPUTATION', 'Wang W, 1997, ', ', 1993, CHOICE REVIEWS ONLINE', 'Sneath P, 1957, MICROBIOLOGY', 'MTW, 1999, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Witten I, 1999, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Bishop C, 2007, ', 'Houtsma M, 2002, ', 'Agrawal R, 1998, KNOWLEDGE DISCOVERY AND DATA MINING', 'Rokach L, 2009, ', 'Zheng Y, 2015, ', 'Scheffer T, 2001, LECTURE NOTES IN COMPUTER SCIENCE', 'Zhu H, 2014, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Zhao Q, 2003, PALLIATIVE &amp; SUPPORTIVE CARE', 'Flach P, 2001, MACHINE LEARNING', 'Cobuloglu H, 2015, EXPERT SYSTEMS WITH APPLICATIONS', 'McCallum A, 2005, QUEUE', 'Das A, 2001, ', 'Phithakkitnukoon S, 2011, ACM TRANSACTIONS ON AUTONOMOUS AND ADAPTIVE SYSTEMS', 'Zhu H, 2012, ', 'Zulkernain S, 2010, E-PUBLICATIONS@MARQUETTE (MARQUETTE UNIVERSITY)', 'Amorim R, 2012, ', 'Sheng S, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Bell A, 2005, QUEUE', 'Zulkernain S, 2010, LECTURE NOTES OF THE INSTITUTE FOR COMPUTER SCIENCES, SOCIAL INFORMATICS AND TELECOMMUNICATIONS ENGINEERING', 'Pedregosa F, 2012, ARXIV (CORNELL UNIVERSITY)', 'John G, 2013, ARXIV (CORNELL UNIVERSITY)', 'He K, 2016, ', 'Breiman L, 2001, MACHINE LEARNING', 'Krizhevsky A, 2017, COMMUNICATIONS OF THE ACM', 'Han J, 2012, CHOICE REVIEWS ONLINE', 'MacQueen J, 1967, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', 'Chollet F, 2017, ', 'Silver D, 2016, NATURE', 'Quinlan J, 1986, MACHINE LEARNING', 'Agrawal R, 1993, ', 'Pearson K, 1901, THE LONDON EDINBURGH AND DUBLIN PHILOSOPHICAL MAGAZINE AND JOURNAL OF SCIENCE', 'Goodfellow I, 2016, MIT PRESS EBOOKS', 'Weiss K, 2016, JOURNAL OF BIG DATA', 'Wu X, 2007, KNOWLEDGE AND INFORMATION SYSTEMS', 'Aha D, 1991, MACHINE LEARNING', 'Ankerst M, 1999, ACM SIGMOD RECORD', 'Moustafa N, 2015, ', 'Fukunaga K, 1975, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Eagle N, 2005, PERSONAL AND UBIQUITOUS COMPUTING', 'Carpenter G, 1987, COMPUTER VISION GRAPHICS AND IMAGE PROCESSING', 'Wagstaff K, 2001, ', 'Keerthi S, 2001, NEURAL COMPUTATION', 'Holte R, 1993, MACHINE LEARNING', 'Kamble S, 2018, PROCESS SAFETY AND ENVIRONMENTAL PROTECTION', 'Ravi K, 2015, KNOWLEDGE-BASED SYSTEMS', 'Xin Y, 2018, IEEE ACCESS', 'Rasmussen C, 1999, ', 'Mahdavinejad M, 2017, DIGITAL COMMUNICATIONS AND NETWORKS', 'Fatima M, 2017, JOURNAL OF INTELLIGENT LEARNING SYSTEMS AND APPLICATIONS', 'Ibáñez J, 2018, SENSORS', 'Liu H, 1998, ', 'Polydoros A, 2017, JOURNAL OF INTELLIGENT &amp; ROBOTIC SYSTEMS', 'Ślusarczyk B, 2018, POLISH JOURNAL OF MANAGEMENT STUDIES', 'Ismail A, 2019, JOURNAL OF BIG DATA', 'López G, 2017, ADVANCES IN INTELLIGENT SYSTEMS AND COMPUTING', 'Lade P, 2017, IEEE INTELLIGENT SYSTEMS', 'Mohammed M, 2016, ', 'Balducci F, 2018, MACHINES', 'Nilashi M, 2017, COMPUTERS &amp; CHEMICAL ENGINEERING', 'Safdar S, 2017, ARTIFICIAL INTELLIGENCE REVIEW', 'Srinivasan V, 2014, ', 'Mehrotra A, 2016, ', 'Sarker I, 2017, THE COMPUTER JOURNAL', 'Perveen S, 2018, IEEE ACCESS', 'Adnan N, 2017, WORLD JOURNAL OF SCIENCE TECHNOLOGY AND SUSTAINABLE DEVELOPMENT', 'Cai J, 2003, ', 'Essien A, 2019, ', 'Wu C, 2016, APPLIED INTELLIGENCE', 'Sarker I, 2016, ', 'Cao L, 2020, ARXIV (CORNELL UNIVERSITY)', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Breiman L, 1996, MACHINE LEARNING', 'Breiman L, 1996, MACHINE LEARNING', 'Quinlan J, 1986, MACHINE LEARNING', ', 1991, CHOICE REVIEWS ONLINE', 'Agrawal R, 1993, ACM SIGMOD RECORD', 'Saeid M, 2017, VIEW', 'Kamble S, 2019, INTERNATIONAL JOURNAL OF PRODUCTION ECONOMICS', 'Lalmuanawma S, 2020, CHAOS SOLITONS &amp; FRACTALS', 'Sharma R, 2020, COMPUTERS &amp; OPERATIONS RESEARCH', 'Sarker I, 2020, JOURNAL OF BIG DATA', 'Agrawal R, 1998, ACM SIGMOD RECORD', 'Harmon S, 2020, NATURE COMMUNICATIONS', 'Jamshidi M, 2020, IEEE ACCESS', 'Sarker I, 2021, SN COMPUTER SCIENCE', 'Fujiyoshi H, 2019, IATSS RESEARCH', 'Kalan A, 2020, NATURE COMMUNICATIONS', 'Zheng T, 2016, INTERNATIONAL JOURNAL OF MEDICAL INFORMATICS', 'Ardabili S, 2020, ALGORITHMS', 'Alakuş T, 2020, CHAOS SOLITONS &amp; FRACTALS', 'Mohamadou Y, 2020, APPLIED INTELLIGENCE', 'Shorten C, 2021, JOURNAL OF BIG DATA', 'Sarker I, 2020, SYMMETRY', 'Boukerche A, 2020, COMPUTER NETWORKS', 'Sarker I, 2019, JOURNAL OF BIG DATA', 'Sarker I, 2021, SN COMPUTER SCIENCE', 'Tao J, 2020, JOURNAL OF BIG DATA', 'Sarker I, 2020, MOBILE NETWORKS AND APPLICATIONS', 'Essien A, 2020, WORLD WIDE WEB', 'Kushwaha S, 2020, JOURNAL OF INDUSTRIAL INTEGRATION AND MANAGEMENT', 'Wei P, 2019, IEEE ACCESS', 'Sarker I, 2019, MOBILE NETWORKS AND APPLICATIONS', 'Sarker I, 2019, INTERNET OF THINGS', 'Sarker I, 2019, JOURNAL OF BIG DATA', 'Tsagkias M, 2020, ACM SIGIR FORUM', 'Marchand A, 2020, JOURNAL OF RETAILING', 'Sarker I, 2020, JOURNAL OF NETWORK AND COMPUTER APPLICATIONS', 'Sarker I, 2020, SYMMETRY', 'Scheffer T, 2005, INTELLIGENT DATA ANALYSIS', 'Sarker I, 2019, INTERNET OF THINGS', 'Sarker I, 2020, JOURNAL OF BIG DATA', 'Khadse V, 2018, ', 'Zi-kang H, 2020, ', 'Sarker I, 2021, PREPRINTS.ORG', 'Sarker I, 2021, PREPRINTS.ORG', 'Sarle W, 1991, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Aha D, 1991, MACHINE LEARNING', 'Baxter L, 1995, TECHNOMETRICS', 'Mohammed M, 2016, ']</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W41" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Iqbal H. Sarker, 2021, SN Computer Science</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>Sarker I, 2021, SN COMPUTER SCIENCE</t>
-        </is>
-      </c>
-      <c r="Z41" t="inlineStr">
-        <is>
-          <t>Sarker I, 2021, SN COMPUTER SCIENCE</t>
+          <t>Iqbal H. Sarker, 2021, SN Computer Science</t>
         </is>
       </c>
     </row>
@@ -4951,33 +4746,28 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://openalex.org/W4919037', 'https://openalex.org/W2112796928', 'https://openalex.org/W2590796488']</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>['LeCun Y, 1998, PROCEEDINGS OF THE IEEE', 'Wan L, 2013, INTERNATIONAL REVIEW OF CYTOLOGY', 'Cohen G, 2017, ARXIV (CORNELL UNIVERSITY)']</t>
-        </is>
-      </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W42" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Xiao Han, 2017, arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>Xiao H, 2017, ARXIV (CORNELL UNIVERSITY)</t>
-        </is>
-      </c>
-      <c r="Z42" t="inlineStr">
-        <is>
-          <t>Xiao H, 2017, ARXIV (CORNELL UNIVERSITY)</t>
+          <t>Xiao Han, 2017, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -5051,23 +4841,18 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">NA, 2008, </t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NA, 2008, </t>
-        </is>
-      </c>
-      <c r="Z43" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2008, </t>
         </is>
@@ -5151,33 +4936,28 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>['GR']</t>
+          <t>['https://openalex.org/W5472403', 'https://openalex.org/W135311109', 'https://openalex.org/W177590838', 'https://openalex.org/W203696055', 'https://openalex.org/W1007293483', 'https://openalex.org/W1497605902', 'https://openalex.org/W1506588750', 'https://openalex.org/W1515851193', 'https://openalex.org/W1520605446', 'https://openalex.org/W1522114398', 'https://openalex.org/W1528113134', 'https://openalex.org/W1537143578', 'https://openalex.org/W1538041071', 'https://openalex.org/W1547833367', 'https://openalex.org/W1554309553', 'https://openalex.org/W1560955742', 'https://openalex.org/W1562368284', 'https://openalex.org/W1563088657', 'https://openalex.org/W1567012231', 'https://openalex.org/W1570329253', 'https://openalex.org/W1570448133', 'https://openalex.org/W1570706771', 'https://openalex.org/W1587647246', 'https://openalex.org/W1588516554', 'https://openalex.org/W1594031697', 'https://openalex.org/W1594781927', 'https://openalex.org/W1602492977', 'https://openalex.org/W1605688901', 'https://openalex.org/W1605844890', 'https://openalex.org/W1637435380', 'https://openalex.org/W1670263352', 'https://openalex.org/W1671614046', 'https://openalex.org/W1746680969', 'https://openalex.org/W1780185704', 'https://openalex.org/W1808644423', 'https://openalex.org/W1813387235', 'https://openalex.org/W1817561967', 'https://openalex.org/W1827261456', 'https://openalex.org/W1904009171', 'https://openalex.org/W1935515061', 'https://openalex.org/W1973991804', 'https://openalex.org/W1974545290', 'https://openalex.org/W1979711143', 'https://openalex.org/W1983479840', 'https://openalex.org/W1983690667', 'https://openalex.org/W1986883011', 'https://openalex.org/W1992419399', 'https://openalex.org/W1993066733', 'https://openalex.org/W2006345381', 'https://openalex.org/W2011101028', 'https://openalex.org/W2016441117', 'https://openalex.org/W2022058268', 'https://openalex.org/W2026718556', 'https://openalex.org/W2037322594', 'https://openalex.org/W2046649434', 'https://openalex.org/W2050829396', 'https://openalex.org/W2063783806', 'https://openalex.org/W2074584355', 'https://openalex.org/W2075932270', 'https://openalex.org/W2093825590', 'https://openalex.org/W2096756482', 'https://openalex.org/W2104333211', 'https://openalex.org/W2110179049', 'https://openalex.org/W2119479037', 'https://openalex.org/W2120199131', 'https://openalex.org/W2122111042', 'https://openalex.org/W2122496402', 'https://openalex.org/W2123623606', 'https://openalex.org/W2125055259', 'https://openalex.org/W2126333738', 'https://openalex.org/W2128912745', 'https://openalex.org/W2133160781', 'https://openalex.org/W2133218851', 'https://openalex.org/W2133632100', 'https://openalex.org/W2136000097', 'https://openalex.org/W2136132422', 'https://openalex.org/W2137130182', 'https://openalex.org/W2139212933', 'https://openalex.org/W2140586694', 'https://openalex.org/W2140785063', 'https://openalex.org/W2142857211', 'https://openalex.org/W2143603257', 'https://openalex.org/W2144731007', 'https://openalex.org/W2145467382', 'https://openalex.org/W2145680191', 'https://openalex.org/W2150796457', 'https://openalex.org/W2151450140', 'https://openalex.org/W2156440942', 'https://openalex.org/W2156571267', 'https://openalex.org/W2156909104', 'https://openalex.org/W2157815868', 'https://openalex.org/W2158724449', 'https://openalex.org/W2159895197', 'https://openalex.org/W2161349318', 'https://openalex.org/W2161782846', 'https://openalex.org/W2161960932', 'https://openalex.org/W2164359548', 'https://openalex.org/W2166985738', 'https://openalex.org/W2167277498', 'https://openalex.org/W2167467747', 'https://openalex.org/W2168754135', 'https://openalex.org/W2171265988', 'https://openalex.org/W2172429451', 'https://openalex.org/W2322002063', 'https://openalex.org/W2488399954', 'https://openalex.org/W2603390332', 'https://openalex.org/W2766736793', 'https://openalex.org/W2911678770', 'https://openalex.org/W2912276539', 'https://openalex.org/W2912934387', 'https://openalex.org/W3015462599']</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>['Witten I, 2011, ELSEVIER EBOOKS', 'Gordon A, 1984, BIOMETRICS', 'Cristianini N, 2000, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Jain A, 1999, ACM COMPUTING SURVEYS', 'Sutton R, 1998, MIT PRESS EBOOKS', 'Friedman N, 1997, MACHINE LEARNING', 'Cohen W, 1995, ELSEVIER EBOOKS', 'Kononenko I, 1994, LECTURE NOTES IN COMPUTER SCIENCE', 'Dietterich T, 2000, MACHINE LEARNING', 'Jordan M, 1998, ', 'Frank E, 1998, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Freund Y, 1998, ', 'Murthy S, 1998, DATA MINING AND KNOWLEDGE DISCOVERY', 'Batista G, 2003, APPLIED ARTIFICIAL INTELLIGENCE', 'Cheng J, 2002, ARTIFICIAL INTELLIGENCE', 'Wettschereck D, 1997, ARTIFICIAL INTELLIGENCE REVIEW', 'Veropoulos K, 1999, ', 'Crammer K, 2002, MACHINE LEARNING', 'Genton M, 2002, ', 'Fürnkranz J, 1999, ARTIFICIAL INTELLIGENCE REVIEW', 'Cestnik B, 1990, EUROPEAN CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Cestnik B, 1987, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Gehrke J, 2000, DATA MINING AND KNOWLEDGE DISCOVERY', 'Breslow L, 1997, THE KNOWLEDGE ENGINEERING REVIEW', 'Kononenko I, 1991, LECTURE NOTES IN COMPUTER SCIENCE', 'Cheng J, 2001, LECTURE NOTES IN COMPUTER SCIENCE', 'Smyth P, 1991, ', 'F�rnkranz J, 2005, MACHINE LEARNING', 'Blum A, 1997, MACHINE LEARNING', 'Setiono R, 2000, APPLIED INTELLIGENCE', 'Elomaa T, 1999, MACHINE LEARNING', 'Rastogi R, 2000, DATA MINING AND KNOWLEDGE DISCOVERY', 'Siddique M, 2002, ', 'Yang Y, 2003, LECTURE NOTES IN COMPUTER SCIENCE', 'Mántaras R, 1998, DATA &amp; KNOWLEDGE ENGINEERING', 'Bonarini A, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Csiszár I, 1996, ', 'An A, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Wall R, 2003, ARTIFICIAL INTELLIGENCE IN MEDICINE', 'Brůha I, 2000, INTELLIGENT DATA ANALYSIS', 'Elomaa T, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Fürnkranz J, 2001, ', 'Zheng Z, 2000, MACHINE LEARNING', 'An A, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Lindgren T, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Kubát M, 2001, INTELLIGENT DATA ANALYSIS', 'Baik S, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Vivarelli F, 2001, NEURAL NETWORKS', 'Cowell R, 2013, ARXIV (CORNELL UNIVERSITY)', 'Vapnik V, 1995, ', 'Quinlan J, 1992, ', 'Burges C, 1998, DATA MINING AND KNOWLEDGE DISCOVERY', 'Cover T, 1967, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Dietterich T, 1998, NEURAL COMPUTATION', ', 2000, APPLIED PHYSICS LETTERS', 'Hodge J, 2004, ARTIFICIAL INTELLIGENCE REVIEW', 'Domingos P, 1997, MACHINE LEARNING', 'Mika S, 2003, ', 'Friedman J, 1989, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Guo G, 2003, LECTURE NOTES IN COMPUTER SCIENCE', 'Littlestone N, 1994, INFORMATION AND COMPUTATION', 'Clark P, 1989, MACHINE LEARNING', 'Yu L, 2004, ', 'Zhang G, 2000, IEEE TRANSACTIONS ON SYSTEMS MAN AND CYBERNETICS PART C (APPLICATIONS AND REVIEWS)', 'Wilson D, 2000, MACHINE LEARNING', 'Lim T, 2000, MACHINE LEARNING', 'Vilalta R, 2002, ARTIFICIAL INTELLIGENCE REVIEW', 'Nadeau C, 2003, MACHINE LEARNING', 'Friedman N, 2003, MACHINE LEARNING', 'Hunt E, 1966, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Weigend A, 1990, ', 'Brighton H, 2002, DATA MINING AND KNOWLEDGE DISCOVERY', 'Zhang S, 2003, APPLIED ARTIFICIAL INTELLIGENCE', ', 2000, APPLIED PHYSICS LETTERS', 'Brazdil P, 2003, MACHINE LEARNING', 'Ruggieri S, 2002, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Utgoff P, 1997, MACHINE LEARNING', 'Keerthi S, 2002, MACHINE LEARNING', 'Kononenko I, 1993, APPLIED ARTIFICIAL INTELLIGENCE', 'Castellano G, 1997, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Heckerman D, 2006, STUDIES IN FUZZINESS AND SOFT COMPUTING', 'Parekh R, 2000, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Bouckaert R, 2003, ', 'Reinartz T, 2002, DATA MINING AND KNOWLEDGE DISCOVERY', 'Fürnkranz J, 1997, MACHINE LEARNING', 'Yam J, 2001, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Dutton D, 1997, THE KNOWLEDGE ENGINEERING REVIEW', 'Kalousis A, 2004, MACHINE LEARNING', 'McSherry D, 1999, KNOWLEDGE-BASED SYSTEMS', 'Zhou Z, 2004, JOURNAL OF COMPUTER SCIENCE AND TECHNOLOGY', 'Camargo L, 2001, NEURAL COMPUTATION', 'Yen G, 2002, ', 'Yıldız O, 2007, PATTERN RECOGNITION LETTERS', 'Roy A, 2000, IEEE TRANSACTIONS ON FUZZY SYSTEMS', 'Basak J, 2004, NEURAL COMPUTATION', 'Kon M, 2000, NEURAL NETWORKS', 'Okamoto S, 2003, THEORETICAL COMPUTER SCIENCE', 'Zheng Z, 1998, KNOWLEDGE-BASED SYSTEMS', 'Sánchez J, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Breiman L, 1996, MACHINE LEARNING', 'Mullin A, 1963, AMERICAN MATHEMATICAL MONTHLY', 'M. P, 1950, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (GENERAL)', 'Bouckaert R, 2004, LECTURE NOTES IN COMPUTER SCIENCE', ', 2001, STUDIES IN FUZZINESS AND SOFT COMPUTING', 'Gama J, 1999, INTELLIGENT DATA ANALYSIS', 'Flach P, 2000, ', 'Kivinen J, 2003, LECTURE NOTES IN COMPUTER SCIENCE', 'Rumelhart D, 1985, ', ', 2019, ', 'Aha D, 1997, ']</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W44" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kotsiantis S, 2007, </t>
-        </is>
-      </c>
-      <c r="Z44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kotsiantis S, 2007, </t>
+          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
         </is>
       </c>
     </row>
@@ -5211,7 +4991,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>2916</v>
+        <v>2920</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -5255,7 +5035,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>['IL', 'CA']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5263,25 +5043,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>Shalev‐Shwartz S, 2014, CAMBRIDGE UNIVERSITY PRESS EBOOKS</t>
-        </is>
-      </c>
-      <c r="Z45" t="inlineStr">
-        <is>
-          <t>Shalev‐Shwartz S, 2014, CAMBRIDGE UNIVERSITY PRESS EBOOKS</t>
+          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
         </is>
       </c>
     </row>
@@ -5315,7 +5090,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>4344</v>
+        <v>4348</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -5383,25 +5158,20 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W46" t="inlineStr"/>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>Samuel A, 1959, IBM JOURNAL OF RESEARCH AND DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="Z46" t="inlineStr">
-        <is>
-          <t>Samuel A, 1959, IBM JOURNAL OF RESEARCH AND DEVELOPMENT</t>
+          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5205,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>4210</v>
+        <v>4214</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
@@ -5479,33 +5249,28 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>['US', 'FR']</t>
+          <t>['https://openalex.org/W1473189865', 'https://openalex.org/W1510952750', 'https://openalex.org/W1528076390', 'https://openalex.org/W1535019556', 'https://openalex.org/W1554944419', 'https://openalex.org/W1760458529', 'https://openalex.org/W1811750039', 'https://openalex.org/W1821462560', 'https://openalex.org/W1826232489', 'https://openalex.org/W1873763122', 'https://openalex.org/W1992926795', 'https://openalex.org/W2009733253', 'https://openalex.org/W2024594469', 'https://openalex.org/W2040228409', 'https://openalex.org/W2051267297', 'https://openalex.org/W2053637704', 'https://openalex.org/W2077905990', 'https://openalex.org/W2095272373', 'https://openalex.org/W2095705004', 'https://openalex.org/W2096633407', 'https://openalex.org/W2106313770', 'https://openalex.org/W2106463421', 'https://openalex.org/W2112380340', 'https://openalex.org/W2114229504', 'https://openalex.org/W2119874464', 'https://openalex.org/W2123147099', 'https://openalex.org/W2130051287', 'https://openalex.org/W2151320232', 'https://openalex.org/W2162379889', 'https://openalex.org/W2186645727', 'https://openalex.org/W2198253679', 'https://openalex.org/W2329660289', 'https://openalex.org/W2461943168', 'https://openalex.org/W2473418344', 'https://openalex.org/W2532520288', 'https://openalex.org/W2950943617', 'https://openalex.org/W2951114885', 'https://openalex.org/W2962835266', 'https://openalex.org/W2963794891', 'https://openalex.org/W2964318098', 'https://openalex.org/W3118608800', 'https://openalex.org/W3215186461', 'https://openalex.org/W4248649186', 'https://openalex.org/W6628547770', 'https://openalex.org/W6631628602', 'https://openalex.org/W6632160336', 'https://openalex.org/W6638214083', 'https://openalex.org/W6639246211', 'https://openalex.org/W6661425395', 'https://openalex.org/W6674330103', 'https://openalex.org/W6676639149', 'https://openalex.org/W6677855611', 'https://openalex.org/W6686761782', 'https://openalex.org/W6731627051']</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>['Srivastava N, 2014, ', 'Hastie T, 2013, ', 'Dwork C, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Abadi M, 2016, ', 'Fredrikson M, 2015, ', 'Shokri R, 2015, ', 'Franklin J, 2005, THE MATHEMATICAL INTELLIGENCER', 'Homer N, 2008, PLOS GENETICS', 'Lindell Y, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Chaudhuri K, 2011, PUBMED', 'Bassily R, 2014, ', 'Fredrikson M, 2014, PUBMED', 'Chaudhuri K, 2008, ', 'Jagannathan G, 2005, ', 'Hardt M, 2016, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Du W, 2004, ', 'Zhang J, 2012, PROCEEDINGS OF THE VLDB ENDOWMENT', 'Dwork C, 2011, ', 'Yang D, 2016, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Calandrino J, 2011, ', 'Bos J, 2014, JOURNAL OF BIOMEDICAL INFORMATICS', 'Rubinstein B, 2012, JOURNAL OF PRIVACY AND CONFIDENTIALITY', 'Sankararaman S, 2009, NATURE GENETICS', 'Vaidya J, 2007, THE VLDB JOURNAL', 'Barni M, 2011, IEEE TRANSACTIONS ON INFORMATION FORENSICS AND SECURITY', 'Duchi J, 2014, JOURNAL OF THE ACM', 'Schneider I, 2005, THE MATHEMATICAL INTELLIGENCER', 'Dwork C, 2015, ', 'Backes M, 2016, ', 'Zhu J, 2001, ', 'Dwork C, 2010, JOURNAL OF PRIVACY AND CONFIDENTIALITY', 'Diakonikolas I, 2015, EDINBURGH RESEARCH EXPLORER (UNIVERSITY OF EDINBURGH)', 'Krizhevsky A, 2024, ', 'Hinton G, 2015, ARXIV (CORNELL UNIVERSITY)', 'Tramèr F, 2016, ARXIV (CORNELL UNIVERSITY)', 'Chaudhuri K, 2009, ARXIV (CORNELL UNIVERSITY)', ', 2016, IRIS RESEARCH PRODUCT CATALOG (SAPIENZA UNIVERSITY OF ROME)', 'Hardt M, 2015, ARXIV (CORNELL UNIVERSITY)', 'Xie P, 2014, ARXIV (CORNELL UNIVERSITY)', 'Duchi J, 2012, ARXIV (CORNELL UNIVERSITY)', 'Jain P, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kusner M, 2015, POLYPUBLIE (ÉCOLE POLYTECHNIQUE DE MONTRÉAL)']</t>
-        </is>
-      </c>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W47" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t xml:space="preserve">Reza Shokri, 2017, </t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shokri R, 2017, </t>
-        </is>
-      </c>
-      <c r="Z47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Shokri R, 2017, </t>
+          <t xml:space="preserve">Reza Shokri, 2017, </t>
         </is>
       </c>
     </row>
@@ -5587,33 +5352,28 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>['GB']</t>
+          <t>['https://openalex.org/W1505641881', 'https://openalex.org/W1541642243', 'https://openalex.org/W1564419782', 'https://openalex.org/W1580529010', 'https://openalex.org/W1639227073', 'https://openalex.org/W1676552347', 'https://openalex.org/W1773272891', 'https://openalex.org/W1926270821', 'https://openalex.org/W1970393892', 'https://openalex.org/W2000701155', 'https://openalex.org/W2003262222', 'https://openalex.org/W2012778485', 'https://openalex.org/W2048677751', 'https://openalex.org/W2059389571', 'https://openalex.org/W2069295011', 'https://openalex.org/W2075746031', 'https://openalex.org/W2099046646', 'https://openalex.org/W2111308925', 'https://openalex.org/W2111589119', 'https://openalex.org/W2114785422', 'https://openalex.org/W2115168188', 'https://openalex.org/W2119747362', 'https://openalex.org/W2130103520', 'https://openalex.org/W2148278638', 'https://openalex.org/W2149706766', 'https://openalex.org/W2151103935', 'https://openalex.org/W2162430761', 'https://openalex.org/W2163205713', 'https://openalex.org/W2166221155', 'https://openalex.org/W2169741726', 'https://openalex.org/W2914011225', 'https://openalex.org/W2999811158', 'https://openalex.org/W6733008967']</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>['Lowe D, 2004, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Quinlan J, 1986, MACHINE LEARNING', 'Harris C, 1988, ', 'Shi J, 1994, ', 'Haralock R, 1991, ADDISON-WESLEY LONGMAN PUBLISHING CO., INC. EBOOKS', 'Smith S, 1997, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Schmid C, 2000, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Mikolajczyk K, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Rosten E, 2005, ', 'Mikolajczyk K, 2002, ', 'Sklar B, 1987, ', 'Moravec H, 2018, RESEARCH SHOWCASE @ CARNEGIE MELLON UNIVERSITY (CARNEGIE MELLON UNIVERSITY)', 'Kitchen L, 1982, PATTERN RECOGNITION LETTERS', 'Brown M, 2002, ', 'Mokhtarian F, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Schaffalitzky F, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Trajković M, 1998, IMAGE AND VISION COMPUTING', 'Schmid C, 2002, ', 'Wang H, 1995, IMAGE AND VISION COMPUTING', 'Zheng Z, 1999, PATTERN RECOGNITION LETTERS', 'Loy G, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Trucco E, 1995, AI COMMUNICATIONS', 'Noble J, 1988, IMAGE AND VISION COMPUTING', 'Rosten E, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Medioni G, 1987, COMPUTER VISION GRAPHICS AND IMAGE PROCESSING', 'Dias P, 2002, ', 'Cooper D, 1993, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Zuliani M, 2005, ', 'Guiducci A, 1988, PATTERN RECOGNITION LETTERS', 'Kenney C, 2003, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Langridge D, 1982, COMPUTER GRAPHICS AND IMAGE PROCESSING', 'Acharya R, 1987, COMPUTER VISION GRAPHICS AND IMAGE PROCESSING']</t>
-        </is>
-      </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W48" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Edward Rosten, 2006, Lecture notes in computer science</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
-          <t>Rosten E, 2006, LECTURE NOTES IN COMPUTER SCIENCE</t>
-        </is>
-      </c>
-      <c r="Z48" t="inlineStr">
-        <is>
-          <t>Rosten E, 2006, LECTURE NOTES IN COMPUTER SCIENCE</t>
+          <t>Edward Rosten, 2006, Lecture notes in computer science</t>
         </is>
       </c>
     </row>
@@ -5647,7 +5407,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3016</v>
+        <v>3027</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -5707,33 +5467,28 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>['GR', 'IT', 'GB']</t>
+          <t>['https://openalex.org/W94523489', 'https://openalex.org/W189596042', 'https://openalex.org/W1179140510', 'https://openalex.org/W1496317909', 'https://openalex.org/W1596717185', 'https://openalex.org/W1689445748', 'https://openalex.org/W1916445479', 'https://openalex.org/W1963579367', 'https://openalex.org/W1963790103', 'https://openalex.org/W1966124853', 'https://openalex.org/W1967320885', 'https://openalex.org/W1968452917', 'https://openalex.org/W1984530193', 'https://openalex.org/W1990517717', 'https://openalex.org/W1995341919', 'https://openalex.org/W1998871699', 'https://openalex.org/W2000972253', 'https://openalex.org/W2001619934', 'https://openalex.org/W2009986810', 'https://openalex.org/W2015263929', 'https://openalex.org/W2018435387', 'https://openalex.org/W2019207321', 'https://openalex.org/W2024081693', 'https://openalex.org/W2025279987', 'https://openalex.org/W2028606616', 'https://openalex.org/W2040104179', 'https://openalex.org/W2040870580', 'https://openalex.org/W2049633694', 'https://openalex.org/W2063304499', 'https://openalex.org/W2065165083', 'https://openalex.org/W2072680624', 'https://openalex.org/W2075320162', 'https://openalex.org/W2076857888', 'https://openalex.org/W2081544115', 'https://openalex.org/W2087877962', 'https://openalex.org/W2095727900', 'https://openalex.org/W2102201073', 'https://openalex.org/W2106855632', 'https://openalex.org/W2108703480', 'https://openalex.org/W2110642273', 'https://openalex.org/W2111072639', 'https://openalex.org/W2119821739', 'https://openalex.org/W2128084896', 'https://openalex.org/W2138178898', 'https://openalex.org/W2143908786', 'https://openalex.org/W2149723649', 'https://openalex.org/W2150593711', 'https://openalex.org/W2153476503', 'https://openalex.org/W2153635508', 'https://openalex.org/W2154350719', 'https://openalex.org/W2161673710', 'https://openalex.org/W2174918471', 'https://openalex.org/W2200121095', 'https://openalex.org/W2209382794', 'https://openalex.org/W2216013554', 'https://openalex.org/W2231576311', 'https://openalex.org/W2270460811', 'https://openalex.org/W2270641383', 'https://openalex.org/W2273322351', 'https://openalex.org/W2286091602', 'https://openalex.org/W2294798173', 'https://openalex.org/W2298521547', 'https://openalex.org/W2337945771', 'https://openalex.org/W2339447311', 'https://openalex.org/W2399675776', 'https://openalex.org/W2417395753', 'https://openalex.org/W2419137750', 'https://openalex.org/W2470803522', 'https://openalex.org/W2497210317', 'https://openalex.org/W2502044482', 'https://openalex.org/W2552660223', 'https://openalex.org/W2560811704', 'https://openalex.org/W2577148968', 'https://openalex.org/W2580808806', 'https://openalex.org/W2586821267', 'https://openalex.org/W2591104514', 'https://openalex.org/W2598645336', 'https://openalex.org/W2603364874', 'https://openalex.org/W2603417106', 'https://openalex.org/W2604196786', 'https://openalex.org/W2606244344', 'https://openalex.org/W2606916050', 'https://openalex.org/W2612828053', 'https://openalex.org/W2619390517', 'https://openalex.org/W2620473470', 'https://openalex.org/W2620542418', 'https://openalex.org/W2621525431', 'https://openalex.org/W2622758479', 'https://openalex.org/W2622999711', 'https://openalex.org/W2738911869', 'https://openalex.org/W2775111183', 'https://openalex.org/W2789255992', 'https://openalex.org/W2790639095', 'https://openalex.org/W2791690647', 'https://openalex.org/W2794415089', 'https://openalex.org/W2796501058', 'https://openalex.org/W2806779833', 'https://openalex.org/W2903950532', 'https://openalex.org/W2911964244', 'https://openalex.org/W2919115771', 'https://openalex.org/W3125807057', 'https://openalex.org/W4210451417', 'https://openalex.org/W4212883601', 'https://openalex.org/W4232670376', 'https://openalex.org/W4239510810', 'https://openalex.org/W4250143236', 'https://openalex.org/W4400360174', 'https://openalex.org/W6607775107', 'https://openalex.org/W6632223008', 'https://openalex.org/W6675321329', 'https://openalex.org/W6675436802', 'https://openalex.org/W6676769703']</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>['Dempster A, 1977, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Chang C, 2011, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Cortes C, 1995, MACHINE LEARNING', 'Hopfield J, 1982, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'McCulloch W, 1943, BULLETIN OF MATHEMATICAL BIOLOGY', 'Jang J, 1993, IEEE TRANSACTIONS ON SYSTEMS MAN AND CYBERNETICS', 'Lloyd S, 1982, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Fisher R, 1936, ANNALS OF EUGENICS', 'Huang G, 2006, NEUROCOMPUTING', 'Rosenblatt F, 1958, PSYCHOLOGICAL REVIEW', 'Cleveland W, 1979, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Suykens J, 1999, NEURAL PROCESSING LETTERS', 'Kohonen T, 1990, PROCEEDINGS OF THE IEEE', 'Friedman J, 1991, THE ANNALS OF STATISTICS', 'Johnson S, 1967, PSYCHOMETRIKA', 'Specht D, 1991, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Riedmiller M, 2002, IEEE INTERNATIONAL CONFERENCE ON NEURAL NETWORKS', 'Suykens J, 2002, WORLD SCIENTIFIC EBOOKS', 'Broomhead D, 1988, COMPLEX SYSTEMS', 'Kong L, 2007, NUCLEIC ACIDS RESEARCH', 'Kass G, 1980, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Fix E, 1989, INTERNATIONAL STATISTICAL REVIEW', 'Salakhutdinov R, 2009, ', 'Atkeson C, 1997, ARTIFICIAL INTELLIGENCE REVIEW', 'Samuel A, 2000, IBM JOURNAL OF RESEARCH AND DEVELOPMENT', 'Pal S, 1992, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Moshou D, 2004, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Linnainmaa S, 1976, BIT NUMERICAL MATHEMATICS', 'Cao J, 2012, NEURAL PROCESSING LETTERS', 'Galvão R, 2008, CHEMOMETRICS AND INTELLIGENT LABORATORY SYSTEMS', 'Mackowiak S, 2015, GENOME BIOLOGY', 'Moshou D, 2005, REAL-TIME IMAGING', 'Asadi H, 2014, PLOS ONE', 'Melssen W, 2006, CHEMOMETRICS AND INTELLIGENT LABORATORY SYSTEMS', 'Dutta R, 2014, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Sengupta S, 2013, BIOSYSTEMS ENGINEERING', 'Amatya S, 2015, BIOSYSTEMS ENGINEERING', 'Mohammadi K, 2015, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Thomas P, 2002, BRITISH JOURNAL OF EDUCATIONAL TECHNOLOGY', 'Coopersmith E, 2014, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Moshou D, 2006, PRECISION AGRICULTURE', 'Craninx M, 2007, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Moshou D, 2013, BIOSYSTEMS ENGINEERING', 'Alonso J, 2013, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Hossain M, 2011, JOURNAL OF HAND SURGERY (EUROPEAN VOLUME)', 'Alonso J, 2014, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Gastaldo P, 2014, ROBOTICS AND AUTONOMOUS SYSTEMS', 'Tryon R, 1957, PSYCHOMETRIKA', 'Neapolitan R, 1987, APPLIED ARTIFICIAL INTELLIGENCE', 'Smith D, 1978, SOCIETY', 'Breiman L, 2001, MACHINE LEARNING', 'LeCun Y, 2015, NATURE', 'Pearson K, 1901, THE LONDON EDINBURGH AND DUBLIN PHILOSOPHICAL MAGAZINE AND JOURNAL OF SCIENCE', 'Ferentinos K, 2018, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Cox D, 1958, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Barboza F, 2017, EXPERT SYSTEMS WITH APPLICATIONS', 'Grinblat G, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2015, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Ebrahimi M, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Morellos A, 2016, BIOSYSTEMS ENGINEERING', 'Zhao Y, 2017, ENERGY ECONOMICS', 'Hansen M, 2018, COMPUTERS IN INDUSTRY', 'Fang K, 2017, GEOPHYSICAL RESEARCH LETTERS', 'Feng Y, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Zhang B, 2017, CANCER LETTERS', 'Rhee J, 2017, AGRICULTURAL AND FOREST METEOROLOGY', 'Mehdizadeh S, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Kang J, 2015, INTERNATIONAL JOURNAL OF RADIATION ONCOLOGY*BIOLOGY*PHYSICS', 'Cramer S, 2017, EXPERT SYSTEMS WITH APPLICATIONS', 'Chung C, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Matthews S, 2017, SCIENTIFIC REPORTS', 'Zhou C, 2018, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2016, BIOSYSTEMS ENGINEERING', 'Ramos P, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Ali I, 2016, IEEE JOURNAL OF SELECTED TOPICS IN APPLIED EARTH OBSERVATIONS AND REMOTE SENSING', 'Bohanec M, 2016, EXPERT SYSTEMS WITH APPLICATIONS', 'Senthilnath J, 2016, BIOSYSTEMS ENGINEERING', 'Patil A, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Belson W, 1959, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Nahvi B, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Maione C, 2015, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Wildenhain J, 2015, CELL SYSTEMS', 'Su Y, 2017, SAUDI JOURNAL OF BIOLOGICAL SCIENCES', 'Aybar-Ruíz A, 2016, SOLAR ENERGY', 'Maione C, 2018, CRITICAL REVIEWS IN FOOD SCIENCE AND NUTRITION', 'Pantazi X, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Binch A, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2017, PRECISION AGRICULTURE', 'Ramírez-Morales I, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Zhang M, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Johann A, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Kung H, 2016, SUSTAINABILITY', 'Pegorini V, 2015, SENSORS', 'Richardson A, 2016, CLINICAL BIOCHEMISTRY', 'López-Cortés X, 2016, AQUACULTURE', 'Takahashi K, 2017, ROBOTICS AND AUTONOMOUS SYSTEMS', 'Fragni R, 2018, FOOD CONTROL', 'Hu H, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Craninx M, 2006, PUBMED', 'Cortes C, 1995, MACHINE LEARNING', 'Breiman L, 1996, MACHINE LEARNING', ', 1988, ELSEVIER EBOOKS', 'Hecht-Nielsen R, 1987, APPLIED OPTICS', ', 1988, NEURAL NETWORKS', 'Strunk K, 2024, ']</t>
-        </is>
-      </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W49" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
         </is>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>Λιάκος Κ, 2018, SENSORS</t>
-        </is>
-      </c>
-      <c r="Z49" t="inlineStr">
-        <is>
-          <t>Λιάκος Κ, 2018, SENSORS</t>
+          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5522,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>4647</v>
+        <v>4649</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -5827,33 +5582,28 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>['NL', 'RS', 'CN', 'DE', 'CA', 'AT', 'US']</t>
+          <t>['https://openalex.org/W30646539', 'https://openalex.org/W92141931', 'https://openalex.org/W191102129', 'https://openalex.org/W429766147', 'https://openalex.org/W595863337', 'https://openalex.org/W1482533224', 'https://openalex.org/W1513618424', 'https://openalex.org/W1573647811', 'https://openalex.org/W1606754933', 'https://openalex.org/W1689749838', 'https://openalex.org/W1727844347', 'https://openalex.org/W1786856418', 'https://openalex.org/W1831050183', 'https://openalex.org/W1895518694', 'https://openalex.org/W1969543759', 'https://openalex.org/W1980225565', 'https://openalex.org/W1983650914', 'https://openalex.org/W1984828485', 'https://openalex.org/W1985839444', 'https://openalex.org/W1990590197', 'https://openalex.org/W1993415357', 'https://openalex.org/W2005164184', 'https://openalex.org/W2006929658', 'https://openalex.org/W2018337952', 'https://openalex.org/W2023312901', 'https://openalex.org/W2023942604', 'https://openalex.org/W2027120296', 'https://openalex.org/W2032518966', 'https://openalex.org/W2033585087', 'https://openalex.org/W2036376676', 'https://openalex.org/W2037789405', 'https://openalex.org/W2050179592', 'https://openalex.org/W2057779644', 'https://openalex.org/W2066626803', 'https://openalex.org/W2078720475', 'https://openalex.org/W2088449361', 'https://openalex.org/W2102467070', 'https://openalex.org/W2112776483', 'https://openalex.org/W2114727579', 'https://openalex.org/W2123845623', 'https://openalex.org/W2126822776', 'https://openalex.org/W2130089270', 'https://openalex.org/W2130560194', 'https://openalex.org/W2131347105', 'https://openalex.org/W2131822674', 'https://openalex.org/W2133505387', 'https://openalex.org/W2135479785', 'https://openalex.org/W2140389576', 'https://openalex.org/W2142800341', 'https://openalex.org/W2145126338', 'https://openalex.org/W2151135366', 'https://openalex.org/W2151666808', 'https://openalex.org/W2155544089', 'https://openalex.org/W2156713494', 'https://openalex.org/W2157395790', 'https://openalex.org/W2158441306', 'https://openalex.org/W2160615957', 'https://openalex.org/W2179669825', 'https://openalex.org/W2191676425', 'https://openalex.org/W2199578048', 'https://openalex.org/W2205945645', 'https://openalex.org/W2287354130', 'https://openalex.org/W2295598076', 'https://openalex.org/W2310573451', 'https://openalex.org/W2346841190', 'https://openalex.org/W2417209869', 'https://openalex.org/W2463898247', 'https://openalex.org/W2479339604', 'https://openalex.org/W2514977123', 'https://openalex.org/W2522985694', 'https://openalex.org/W2554693566', 'https://openalex.org/W2557963070', 'https://openalex.org/W2564901692', 'https://openalex.org/W2580821229', 'https://openalex.org/W2582718246', 'https://openalex.org/W2727623211', 'https://openalex.org/W2730460668', 'https://openalex.org/W2736166619', 'https://openalex.org/W2890624634', 'https://openalex.org/W2890805913', 'https://openalex.org/W2917425395', 'https://openalex.org/W2917661374', 'https://openalex.org/W3022713798', 'https://openalex.org/W3102027041', 'https://openalex.org/W3102476541', 'https://openalex.org/W3163617311', 'https://openalex.org/W4211056572', 'https://openalex.org/W4250720198', 'https://openalex.org/W4252713891', 'https://openalex.org/W4285719527', 'https://openalex.org/W4399271987', 'https://openalex.org/W4399569501', 'https://openalex.org/W6634147026', 'https://openalex.org/W6727196412', 'https://openalex.org/W6870084398', 'https://openalex.org/W6891733106']</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>['Venables W, 2002, STATISCTICS AND COMPUTING/STATISTICS AND COMPUTING', 'Hijmans R, 2005, INTERNATIONAL JOURNAL OF CLIMATOLOGY', 'Kühn M, 2008, JOURNAL OF STATISTICAL SOFTWARE', 'Cohen J, 1968, PSYCHOLOGICAL BULLETIN', 'Kühn M, 2013, ', 'Shannon C, 1998, PROCEEDINGS OF THE IEEE', 'Sing T, 2005, COMPUTER APPLICATIONS IN THE BIOSCIENCES', 'Chen J, 2014, ISPRS JOURNAL OF PHOTOGRAMMETRY AND REMOTE SENSING', 'Rabus B, 2003, ISPRS JOURNAL OF PHOTOGRAMMETRY AND REMOTE SENSING', 'Pendleton R, 1945, GEOGRAPHICAL REVIEW', 'Scharlemann J, 2014, CARBON MANAGEMENT', 'Meinshausen N, 2006, ', 'Goldewijk K, 2010, GLOBAL ECOLOGY AND BIOGEOGRAPHY', 'Fan Y, 2013, SCIENCE', 'Hengl T, 2014, PLOS ONE', 'Hartmann J, 2012, GEOCHEMISTRY GEOPHYSICS GEOSYSTEMS', 'Minasny B, 2006, COMPUTERS &amp; GEOSCIENCES', 'Hall D, 2007, HYDROLOGICAL PROCESSES', 'Pebesma E, 2015, ', 'Statnikov A, 2008, BMC BIOINFORMATICS', 'Shangguan W, 2013, JOURNAL OF ADVANCES IN MODELING EARTH SYSTEMS', 'Sánchez P, 2009, SCIENCE', 'Raup B, 2006, GLOBAL AND PLANETARY CHANGE', 'Brus D, 2011, EUROPEAN JOURNAL OF SOIL SCIENCE', 'Carroll M, 2009, INTERNATIONAL JOURNAL OF DIGITAL EARTH', 'Arrouays D, 2014, ADVANCES IN AGRONOMY', 'Hugelius G, 2013, EARTH SYSTEM SCIENCE DATA', 'Stockmann U, 2015, GLOBAL FOOD SECURITY', 'Grunwald S, 2011, SOIL SCIENCE SOCIETY OF AMERICA JOURNAL', 'Batjes N, 2009, SOIL USE AND MANAGEMENT', 'Savtchenko A, 2004, ADVANCES IN SPACE RESEARCH', 'Wan Z, 2006, INTERNATIONAL JOURNAL OF ENVIRONMENTAL RESEARCH AND PUBLIC HEALTH', 'Kilibarda M, 2014, JOURNAL OF GEOPHYSICAL RESEARCH ATMOSPHERES', 'Fitzpatrick M, 2013, ECOSPHERE', 'Borda M, 2011, ', 'Malone B, 2014, GEODERMA', "Sayre R, 2014, DIGITAL ACCESS TO LIBRARIES (UNIVERSITÉ CATHOLIQUE DE LOUVAIN (UCL), L'UNIVERSITÉ DE NAMUR (UNAMUR) AND THE UNIVERSITÉ SAINT-LOUIS (USL-B))", 'Montanarella L, 2012, CURRENT OPINION IN ENVIRONMENTAL SUSTAINABILITY', 'Gasch C, 2015, SPATIAL STATISTICS', 'Bauer-Marschallinger B, 2014, COMPUTERS &amp; GEOSCIENCES', 'Griffiths R, 2015, APPLIED SOIL ECOLOGY', 'Shani U, 2007, WATER RESOURCES RESEARCH', 'Cooper M, 2005, SOIL SCIENCE SOCIETY OF AMERICA JOURNAL', 'Knaus J, 2009, THE R JOURNAL', 'Láng V, 2012, GEODERMA', 'Pogson M, 2011, ENVIRONMENTAL MODELLING &amp; SOFTWARE', 'Kidd D, 2015, SOIL RESEARCH', 'Mantel S, 2007, DATA ARCHIVING AND NETWORKED SERVICES (DANS)', 'Baade J, 2014, ', 'Danielson J, 2011, ANTARCTICA A KEYSTONE IN A CHANGING WORLD', 'Chen T, 2016, ', 'Shannon C, 1949, PROCEEDINGS OF THE IRE', 'Anonim A, 2010, ', 'Wright M, 2017, JOURNAL OF STATISTICAL SOFTWARE', 'Giri C, 2010, GLOBAL ECOLOGY AND BIOGEOGRAPHY', 'Conrad O, 2015, GEOSCIENTIFIC MODEL DEVELOPMENT', 'Krämer W, 2003, COMPUTATIONAL STATISTICS &amp; DATA ANALYSIS', 'FAO, 2023, ', 'Kühn M, 2008, ', 'Hengl T, 2015, PLOS ONE', 'Nachtergaele F, 2012, SOCIO-ENVIRONMENTAL SYSTEMS MODELING', 'Conrad O, 2015, ', 'Rome, 1977, ', 'Shangguan W, 2016, JOURNAL OF ADVANCES IN MODELING EARTH SYSTEMS', 'Sollich P, 1995, CERN DOCUMENT SERVER (EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Pelletier J, 2015, JOURNAL OF ADVANCES IN MODELING EARTH SYSTEMS', 'Brevik E, 2015, GEODERMA', 'Folberth C, 2016, NATURE COMMUNICATIONS', 'Domisch S, 2015, SCIENTIFIC DATA', 'Mulder V, 2015, GEODERMA', 'Krasilnikov P, 2009, ', 'Tóth G, 2013, JOINT RESEARCH CENTRE (EUROPEAN COMMISSION)', 'Mira M, 2015, REMOTE SENSING OF ENVIRONMENT', 'Wang S, 2007, ', 'Shepherd K, 2014, AGRICULTURAL SYSTEMS', 'Aksoy E, 2016, PLOS ONE', 'Searle R, 2014, ', 'Ribeiro E, 2015, ', 'Leenaars J, 2013, DATA ARCHIVING AND NETWORKED SERVICES (DANS)', 'Faison E, 2016, PLOS ONE', 'Ribeiro E, 2015, ', 'Brevik E, 2015, GEODERMA', 'Jagger J, 2007, ELSEVIER EBOOKS', 'Hijmans R, 2010, ', 'Wright M, 2015, ']</t>
-        </is>
-      </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Tomislav Hengl, 2017, PLoS ONE</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>Hengl T, 2017, PLOS ONE</t>
-        </is>
-      </c>
-      <c r="Z50" t="inlineStr">
-        <is>
-          <t>Hengl T, 2017, PLOS ONE</t>
+          <t>Tomislav Hengl, 2017, PLoS ONE</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5637,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>2469</v>
+        <v>2473</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -5943,33 +5693,28 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>['DE']</t>
+          <t>['https://openalex.org/W822801274', 'https://openalex.org/W1506806321', 'https://openalex.org/W1565746575', 'https://openalex.org/W1901616594', 'https://openalex.org/W1978394996', 'https://openalex.org/W2034059032', 'https://openalex.org/W2059111627', 'https://openalex.org/W2076063813', 'https://openalex.org/W2096352448', 'https://openalex.org/W2099419573', 'https://openalex.org/W2106577732', 'https://openalex.org/W2151103935', 'https://openalex.org/W2161969291', 'https://openalex.org/W2164598857', 'https://openalex.org/W2251410821', 'https://openalex.org/W2269742369', 'https://openalex.org/W2585169518', 'https://openalex.org/W2751039952', 'https://openalex.org/W2798302089', 'https://openalex.org/W2800722845', 'https://openalex.org/W2802955324', 'https://openalex.org/W2884001105', 'https://openalex.org/W2888794009', 'https://openalex.org/W2891503716', 'https://openalex.org/W2892341857', 'https://openalex.org/W2895991254', 'https://openalex.org/W2900453322', 'https://openalex.org/W2902907165', 'https://openalex.org/W2915015079', 'https://openalex.org/W2919115771', 'https://openalex.org/W2921353139', 'https://openalex.org/W2945976633', 'https://openalex.org/W2953189907', 'https://openalex.org/W2963095307', 'https://openalex.org/W2963428668', 'https://openalex.org/W2964716450', 'https://openalex.org/W2981207549', 'https://openalex.org/W2989851933', 'https://openalex.org/W2995871253', 'https://openalex.org/W2999321020', 'https://openalex.org/W3000062802', 'https://openalex.org/W3005351117', 'https://openalex.org/W3025420269', 'https://openalex.org/W3094605956', 'https://openalex.org/W3095865939', 'https://openalex.org/W3118496513', 'https://openalex.org/W3120261410', 'https://openalex.org/W3150796314', 'https://openalex.org/W4212902066', 'https://openalex.org/W4236093597', 'https://openalex.org/W4255466416', 'https://openalex.org/W6730267373', 'https://openalex.org/W6750380350']</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>['LeCun Y, 2015, NATURE', 'Lowe D, 2004, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Dalal N, 2005, ', 'Viola P, 2005, ', 'Schmidhuber J, 2014, NEURAL NETWORKS', 'Demšar J, 2006, ', 'Jordan M, 2015, SCIENCE', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Rudin C, 2019, NATURE MACHINE INTELLIGENCE', 'Bishop C, 2006, SPRINGER EBOOKS', 'Searle J, 1980, BEHAVIORAL AND BRAIN SCIENCES', 'Adadi A, 2018, IEEE ACCESS', 'Silver D, 2018, SCIENCE', 'Gama J, 2014, ACM COMPUTING SURVEYS', 'Young T, 2018, IEEE COMPUTATIONAL INTELLIGENCE MAGAZINE', 'Eykholt K, 2018, ', 'Grigorescu S, 2019, JOURNAL OF FIELD ROBOTICS', 'Kotsiantis S, 2006, ARTIFICIAL INTELLIGENCE REVIEW', 'Pouyanfar S, 2018, ACM COMPUTING SURVEYS', 'Shmueli G, 2011, MIS QUARTERLY', 'Westerlund M, 2019, TECHNOLOGY INNOVATION MANAGEMENT REVIEW', 'Zhang Y, 2018, NPJ COMPUTATIONAL MATERIALS', 'Pan Z, 2019, IEEE ACCESS', 'Madani A, 2018, NPJ DIGITAL MEDICINE', 'Chen S, 2008, MATHEMATICS AND COMPUTERS IN SIMULATION', 'Shrestha Y, 2020, JOURNAL OF BUSINESS RESEARCH', 'Ahani A, 2019, INTERNATIONAL JOURNAL OF HOSPITALITY MANAGEMENT', 'Goyal D, 2015, CIRP JOURNAL OF MANUFACTURING SCIENCE AND TECHNOLOGY', 'Paula E, 2016, ', 'Peters M, 2013, MACHINE LEARNING', 'Howard A, 2017, ', 'Assaf R, 2019, ', 'Pentland B, 2020, MIS QUARTERLY', 'Kühl N, 2019, ELECTRONIC MARKETS', 'Liu Z, 2020, ', 'Balaji A, 2018, PROCEDIA COMPUTER SCIENCE', 'Wang S, 2020, IEEE TRANSACTIONS ON SERVICES COMPUTING', 'Ramaswamy S, 2018, PROCEDIA COMPUTER SCIENCE', 'Heinrich K, 2021, DECISION SUPPORT SYSTEMS', 'Fuchs D, 2018, ', 'Fischer M, 2020, ELECTRONIC MARKETS', 'Selz D, 2020, ELECTRONIC MARKETS', 'Wu M, 2018, ', 'Leijnen S, 2020, PROCEEDINGS', 'Wanner J, 2020, JOURNAL OF THE ASSOCIATION FOR INFORMATION SYSTEMS', 'Duin R, 1994, PATTERN RECOGNITION LETTERS', 'Heinrich K, 2019, JOURNAL OF THE ASSOCIATION FOR INFORMATION SYSTEMS', 'Heinrich K, 2020, JOURNAL OF THE ASSOCIATION FOR INFORMATION SYSTEMS', 'Haselton M, 2015, ', 'Widmer G, 1996, MACHINE LEARNING']</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>OPENALEX</t>
+        </is>
+      </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>OPENALEX</t>
+          <t>Christian Janiesch, 2021, Electronic Markets</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>Janiesch C, 2021, ELECTRONIC MARKETS</t>
-        </is>
-      </c>
-      <c r="Z51" t="inlineStr">
-        <is>
-          <t>Janiesch C, 2021, ELECTRONIC MARKETS</t>
+          <t>Christian Janiesch, 2021, Electronic Markets</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "fix: restore corrected ETL files and standardizer improvements"
This reverts commit 8205ed2006c9dd68e81b11e5d0b296204ce231b6.
</commit_message>
<xml_diff>
--- a/test_openalex.xlsx
+++ b/test_openalex.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y51"/>
+  <dimension ref="A1:Z51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,30 +526,35 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>AU_CO</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>CR</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>PMID</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>SR</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SR_FULL</t>
         </is>
@@ -585,7 +590,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>63729</v>
+        <v>63726</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -629,28 +634,33 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1496508106', 'https://openalex.org/W1571024744', 'https://openalex.org/W2024933578', 'https://openalex.org/W2035776949', 'https://openalex.org/W2040387238', 'https://openalex.org/W2047804403', 'https://openalex.org/W2063978378', 'https://openalex.org/W2097360283', 'https://openalex.org/W2097850441', 'https://openalex.org/W2118585731', 'https://openalex.org/W2146292423', 'https://openalex.org/W2152799677', 'https://openalex.org/W2153635508']</t>
+          <t>['FR', 'JP', 'DE', 'CA', 'US']</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr">
+          <t>['Chang C, 2011, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Friedman J, 2010, PUBMED', 'Walt S, 2011, COMPUTING IN SCIENCE &amp; ENGINEERING', 'Efron B, 2004, THE ANNALS OF STATISTICS', 'Fan R, 2008, ', 'Guyon I, 2004, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Hanke M, 2009, NEUROINFORMATICS', 'Rokhlin V, 2009, SIAM JOURNAL ON MATRIX ANALYSIS AND APPLICATIONS', 'Omohundro S, 2009, ', 'Sören S, 2010, MAX PLANCK INSTITUTE FOR PLASMA PHYSICS', 'Michel V, 2011, PATTERN RECOGNITION', 'Zito T, 2008, FRONTIERS IN NEUROINFORMATICS', 'Dubois P, 2007, COMPUTING IN SCIENCE &amp; ENGINEERING']</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Fabián Pedregosa, 2012, arXiv (Cornell University)</t>
-        </is>
-      </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Fabián Pedregosa, 2012, arXiv (Cornell University)</t>
+          <t>Pedregosa F, 2012, ARXIV (CORNELL UNIVERSITY)</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Pedregosa F, 2012, ARXIV (CORNELL UNIVERSITY)</t>
         </is>
       </c>
     </row>
@@ -750,20 +760,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>NA, 1989, Choice Reviews Online</t>
-        </is>
-      </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>NA, 1989, Choice Reviews Online</t>
+          <t>NA, 1989, CHOICE REVIEWS ONLINE</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>NA, 1989, CHOICE REVIEWS ONLINE</t>
         </is>
       </c>
     </row>
@@ -833,7 +848,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['AU']</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -841,20 +856,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">J. R. Quinlan, 1992, </t>
-        </is>
-      </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t xml:space="preserve">J. R. Quinlan, 1992, </t>
+          <t xml:space="preserve">Quinlan J, 1992, </t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quinlan J, 1992, </t>
         </is>
       </c>
     </row>
@@ -936,20 +956,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr">
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Arthur Asuncion, 2007, Medical Entomology and Zoology</t>
-        </is>
-      </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Arthur Asuncion, 2007, Medical Entomology and Zoology</t>
+          <t>Asuncion A, 2007, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Asuncion A, 2007, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
         </is>
       </c>
     </row>
@@ -1027,28 +1052,33 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W23418094', 'https://openalex.org/W24402856', 'https://openalex.org/W28412257', 'https://openalex.org/W43179442', 'https://openalex.org/W64096637', 'https://openalex.org/W66926763', 'https://openalex.org/W69783631', 'https://openalex.org/W122789262', 'https://openalex.org/W123339444', 'https://openalex.org/W138217685', 'https://openalex.org/W149472151', 'https://openalex.org/W173229765', 'https://openalex.org/W187357405', 'https://openalex.org/W586094522', 'https://openalex.org/W589058777', 'https://openalex.org/W1483135265', 'https://openalex.org/W1483679765', 'https://openalex.org/W1492324553', 'https://openalex.org/W1492698999', 'https://openalex.org/W1495859460', 'https://openalex.org/W1500698297', 'https://openalex.org/W1506285740', 'https://openalex.org/W1513366687', 'https://openalex.org/W1516443426', 'https://openalex.org/W1520687314', 'https://openalex.org/W1523856491', 'https://openalex.org/W1524704912', 'https://openalex.org/W1528113134', 'https://openalex.org/W1530010412', 'https://openalex.org/W1533544838', 'https://openalex.org/W1533946607', 'https://openalex.org/W1536719366', 'https://openalex.org/W1550206324', 'https://openalex.org/W1550821944', 'https://openalex.org/W1551066950', 'https://openalex.org/W1553019137', 'https://openalex.org/W1553313034', 'https://openalex.org/W1554663460', 'https://openalex.org/W1555244713', 'https://openalex.org/W1559060276', 'https://openalex.org/W1560107318', 'https://openalex.org/W1563088657', 'https://openalex.org/W1564947197', 'https://openalex.org/W1571836963', 'https://openalex.org/W1572964175', 'https://openalex.org/W1572978214', 'https://openalex.org/W1573228426', 'https://openalex.org/W1576962511', 'https://openalex.org/W1582036668', 'https://openalex.org/W1583700199', 'https://openalex.org/W1584333058', 'https://openalex.org/W1585221258', 'https://openalex.org/W1585610988', 'https://openalex.org/W1585743408', 'https://openalex.org/W1588100052', 'https://openalex.org/W1588282782', 'https://openalex.org/W1597165973', 'https://openalex.org/W1598333443', 'https://openalex.org/W1598696986', 'https://openalex.org/W1600437712', 'https://openalex.org/W1601529450', 'https://openalex.org/W1604345466', 'https://openalex.org/W1605275907', 'https://openalex.org/W1605688901', 'https://openalex.org/W1605957858', 'https://openalex.org/W1619226191', 'https://openalex.org/W1625504505', 'https://openalex.org/W1630964756', 'https://openalex.org/W1641039719', 'https://openalex.org/W1648885110', 'https://openalex.org/W1670263352', 'https://openalex.org/W1673310716', 'https://openalex.org/W1676820704', 'https://openalex.org/W1678889691', 'https://openalex.org/W1679846099', 'https://openalex.org/W1680392829', 'https://openalex.org/W1763728792', 'https://openalex.org/W1781794689', 'https://openalex.org/W1800049145', 'https://openalex.org/W1806329564', 'https://openalex.org/W1817561967', 'https://openalex.org/W1833977909', 'https://openalex.org/W1861764418', 'https://openalex.org/W1881647329', 'https://openalex.org/W1882120692', 'https://openalex.org/W1906182963', 'https://openalex.org/W1907578970', 'https://openalex.org/W1908888846', 'https://openalex.org/W1912123407', 'https://openalex.org/W1932571505', 'https://openalex.org/W1955600018', 'https://openalex.org/W1969482724', 'https://openalex.org/W1978515644', 'https://openalex.org/W1979711143', 'https://openalex.org/W1982161962', 'https://openalex.org/W1985593448', 'https://openalex.org/W1987947967', 'https://openalex.org/W1990748933', 'https://openalex.org/W1995945562', 'https://openalex.org/W2001619934', 'https://openalex.org/W2008906462', 'https://openalex.org/W2014725748', 'https://openalex.org/W2015401436', 'https://openalex.org/W2017337590', 'https://openalex.org/W2019575783', 'https://openalex.org/W2024046085', 'https://openalex.org/W2024646871', 'https://openalex.org/W2024668293', 'https://openalex.org/W2035890032', 'https://openalex.org/W2037603696', 'https://openalex.org/W2037768235', 'https://openalex.org/W2037965136', 'https://openalex.org/W2042385018', 'https://openalex.org/W2048679005', 'https://openalex.org/W2053154970', 'https://openalex.org/W2057720927', 'https://openalex.org/W2058732827', 'https://openalex.org/W2064853889', 'https://openalex.org/W2065861851', 'https://openalex.org/W2066636486', 'https://openalex.org/W2067098334', 'https://openalex.org/W2068337856', 'https://openalex.org/W2073308541', 'https://openalex.org/W2073583237', 'https://openalex.org/W2074610805', 'https://openalex.org/W2075665712', 'https://openalex.org/W2078579128', 'https://openalex.org/W2095749253', 'https://openalex.org/W2095897464', 'https://openalex.org/W2097089247', 'https://openalex.org/W2097569937', 'https://openalex.org/W2100406636', 'https://openalex.org/W2102009083', 'https://openalex.org/W2105494575', 'https://openalex.org/W2105497548', 'https://openalex.org/W2106393550', 'https://openalex.org/W2108949035', 'https://openalex.org/W2110119381', 'https://openalex.org/W2111746072', 'https://openalex.org/W2112076978', 'https://openalex.org/W2112841646', 'https://openalex.org/W2113242816', 'https://openalex.org/W2117812871', 'https://openalex.org/W2118020653', 'https://openalex.org/W2118383892', 'https://openalex.org/W2119821739', 'https://openalex.org/W2119885577', 'https://openalex.org/W2120216197', 'https://openalex.org/W2122111042', 'https://openalex.org/W2122410182', 'https://openalex.org/W2129113961', 'https://openalex.org/W2129249398', 'https://openalex.org/W2132166479', 'https://openalex.org/W2133632100', 'https://openalex.org/W2134696506', 'https://openalex.org/W2138064700', 'https://openalex.org/W2138621811', 'https://openalex.org/W2139059214', 'https://openalex.org/W2140190241', 'https://openalex.org/W2142767931', 'https://openalex.org/W2142819948', 'https://openalex.org/W2142957916', 'https://openalex.org/W2143349571', 'https://openalex.org/W2143426320', 'https://openalex.org/W2144907232', 'https://openalex.org/W2146257637', 'https://openalex.org/W2147492008', 'https://openalex.org/W2147810216', 'https://openalex.org/W2148949939', 'https://openalex.org/W2149706766', 'https://openalex.org/W2153028052', 'https://openalex.org/W2154318594', 'https://openalex.org/W2154642793', 'https://openalex.org/W2156909104', 'https://openalex.org/W2160642098', 'https://openalex.org/W2161077873', 'https://openalex.org/W2163915185', 'https://openalex.org/W2164818318', 'https://openalex.org/W2166559705', 'https://openalex.org/W2167793421', 'https://openalex.org/W2170112109', 'https://openalex.org/W2170654002', 'https://openalex.org/W2170726034', 'https://openalex.org/W2170913656', 'https://openalex.org/W2172162418', 'https://openalex.org/W2172780573', 'https://openalex.org/W2277957941', 'https://openalex.org/W2331052961', 'https://openalex.org/W2621280964', 'https://openalex.org/W2912934387', 'https://openalex.org/W2913066018', 'https://openalex.org/W2914369697', 'https://openalex.org/W2953014340', 'https://openalex.org/W2988864014', 'https://openalex.org/W3017143921', 'https://openalex.org/W3023540311', 'https://openalex.org/W3083113686', 'https://openalex.org/W3085162807', 'https://openalex.org/W3123294050', 'https://openalex.org/W3163638146', 'https://openalex.org/W3193477162', 'https://openalex.org/W3203633735', 'https://openalex.org/W3208887124']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
+          <t>['1959- B, 1994, CHOICE REVIEWS ONLINE', 'Cristianini N, 2000, CAMBRIDGE UNIVERSITY PRESS EBOOKS', ', 2014, APPLE ACADEMIC PRESS EBOOKS', 'Agrawal R, 1994, VERY LARGE DATA BASES', 'Wolpert D, 1992, NEURAL NETWORKS', 'Devroye L, 1996, STOCHASTIC MODELLING AND APPLIED PROBABILITY', 'McCallum A, 1998, ', 'Kira K, 1992, ELSEVIER EBOOKS', 'Hall M, 2000, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Egan J, 1975, ', 'Cavnar W, 1994, ', 'Pyle D, 1999, ', 'Kohavi R, 1996, ', 'Frank E, 1998, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Kimball R, 1996, ', 'Zaki M, 1997, ', 'Kushmerick N, 1997, ', 'Cypher A, 1993, ', 'Cheeseman P, 1996, ', 'Shafer J, 1996, ', 'Mehta M, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Wang Y, 1996, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Liu H, 1996, ', 'Almuallim H, 1991, NATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Drucker H, 1997, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Kerber R, 1992, NATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Schapire R, 1997, QUT EPRINTS (QUEENSLAND UNIVERSITY OF TECHNOLOGY)', 'Langley P, 1995, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Kong E, 1995, ELSEVIER EBOOKS', 'Kononenko I, 1995, ', 'Zheng Z, 2000, MACHINE LEARNING', 'Brodley C, 1996, ', 'Ting K, 1997, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Ramon J, 2000, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Almuallim H, 1992, ', 'Webb G, 1999, ', 'Kohavi R, 1996, ', 'Moore A, 1994, ELSEVIER EBOOKS', 'Bigus J, 1996, ', 'Kibler D, 1987, ELSEVIER EBOOKS', 'Omohundro S, 1987, COMPLEX SYSTEMS', 'Dhar V, 1996, ', 'Chevaleyre Y, 2001, LECTURE NOTES IN COMPUTER SCIENCE', 'Ramakrishnan R, 2000, ASSOCIATION FOR COMPUTING MACHINERY EBOOKS', 'Cherkauer K, 1996, ', 'Mann T, 1993, ', 'Holmes G, 1995, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Domingos P, 1997, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Maron O, 1998, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)', 'Giraud-Carrier C, 1996, ', 'Efron B, 1994, ', 'Ester M, 1996, ', 'Fisher R, 1936, ANNALS OF EUGENICS', 'Swets J, 1988, SCIENCE', 'Friedman N, 1997, MACHINE LEARNING', 'Cohen W, 1995, ELSEVIER EBOOKS', 'Dietterich T, 2000, MACHINE LEARNING', 'Fayyad U, 1993, INTERNATIONAL JOINT CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Dietterich T, 1995, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Srikant R, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'John G, 1994, ELSEVIER EBOOKS', 'Pelleg D, 2000, ', 'Dougherty J, 1995, ELSEVIER EBOOKS', 'Quinlan J, 1996, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Piateski G, 1991, MIT PRESS EBOOKS', 'Berry M, 1997, UNIVERSITY OF MARIBOR DIGITAL LIBRARY (UNIVERSITY OF MARIBOR)', 'Kubát M, 1998, MACHINE LEARNING', 'Kass R, 1995, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Sahami M, 1998, ', 'Langley P, 1992, ', 'Freund Y, 1998, ', 'Cleary J, 1995, ELSEVIER EBOOKS', 'Freund Y, 1999, ', 'Kohavi R, 1995, LECTURE NOTES IN COMPUTER SCIENCE', 'Langley P, 1994, ELSEVIER EBOOKS', 'Cendrowska J, 1987, INTERNATIONAL JOURNAL OF MAN-MACHINE STUDIES', 'Beck, 1986, PUBMED', 'Frank E, 1999, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'Cabena P, 1997, UNIVERSITY OF MARIBOR DIGITAL LIBRARY (UNIVERSITY OF MARIBOR)', 'Frank E, 1998, MACHINE LEARNING', 'Breiman L, 1999, MACHINE LEARNING', 'Holmes G, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Appelt D, 1999, AI COMMUNICATIONS', 'Demiröz G, 1997, LECTURE NOTES IN COMPUTER SCIENCE', 'Flach P, 2001, MACHINE LEARNING', 'Brownston L, 1985, CERN DOCUMENT SERVER (EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Moore A, 1998, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Ting K, 1997, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'Kohavi R, 1997, ', 'Oates T, 1997, ', 'Witten I, 1999, ', ', 1996, COMPUTERS &amp; MATHEMATICS WITH APPLICATIONS', 'Saitta L, 1998, MACHINE LEARNING', 'Frank E, 1999, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'RICHARDS D, 1998, INTERNATIONAL JOURNAL OF HUMAN-COMPUTER STUDIES', 'Ricci⋆ F, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Kohavi R, 1995, ', 'John G, 2013, ARXIV (CORNELL UNIVERSITY)', 'Moore A, 2021, ', 'Paynter G, 2000, RESEARCH COMMONS (UNIVERSITY OF WAIKATO)', 'Cohen J, 1960, EDUCATIONAL AND PSYCHOLOGICAL MEASUREMENT', 'Cortes C, 1995, MACHINE LEARNING', 'Kumar D, 1995, CHOICE REVIEWS ONLINE', 'Cover T, 1967, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Brin S, 1998, COMPUTER NETWORKS AND ISDN SYSTEMS', 'Kohavi R, 1997, ARTIFICIAL INTELLIGENCE', 'Sebastiani F, 2002, ACM COMPUTING SURVEYS', 'Freund Y, 1996, ', 'Lawson C, 1995, SOCIETY FOR INDUSTRIAL AND APPLIED MATHEMATICS EBOOKS', 'Friedman J, 2000, THE ANNALS OF STATISTICS', 'Ho T, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Ripley B, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Han J, 2000, ACM SIGMOD RECORD', 'Blum A, 1998, ', 'Stevens S, 1946, SCIENCE', 'Zhang T, 1996, ', 'Cooper G, 1992, MACHINE LEARNING', 'Dietterich T, 1997, ARTIFICIAL INTELLIGENCE', 'Friedman J, 1977, ACM TRANSACTIONS ON MATHEMATICAL SOFTWARE', 'Nigam K, 2000, MACHINE LEARNING', 'Hoerl A, 1970, TECHNOMETRICS', 'Koestler A, 1967, ', 'Schölkopf B, 1999, ', 'Brin S, 1997, ', 'Fisher D, 1987, MACHINE LEARNING', 'Vitter J, 1985, ACM TRANSACTIONS ON MATHEMATICAL SOFTWARE', 'Cessie S, 1992, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Agrawal R, 1993, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Niknian M, 1995, TECHNOMETRICS', 'Hastie T, 1998, THE ANNALS OF STATISTICS', 'Domingos P, 1999, ', 'Nigam K, 2000, ', 'Day W, 1984, JOURNAL OF CLASSIFICATION', 'Hochbaum D, 1985, MATHEMATICS OF OPERATIONS RESEARCH', 'Utgoff P, 1989, MACHINE LEARNING', 'Webb G, 2000, MACHINE LEARNING', 'Marill T, 1963, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Wang J, 2000, COGPRINTS (UNIVERSITY OF SOUTHAMPTON)', 'Langley P, 1995, COMMUNICATIONS OF THE ACM', 'Mitchell T, 1994, COMMUNICATIONS OF THE ACM', 'Aha D, 1992, INTERNATIONAL JOURNAL OF MAN-MACHINE STUDIES', 'Fürnkranz J, 1994, ELSEVIER EBOOKS', 'Liu H, 1997, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Vafaie H, 2003, ', 'Gaines B, 1995, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Wettschereck D, 1995, MACHINE LEARNING', 'Littlestone N, 1990, ', 'Bay S, 1999, INTELLIGENT DATA ANALYSIS', 'Rexine J, 1986, THE AMERICAN JOURNAL OF PHILOLOGY', 'Frank E, 2000, ', ', 1989, CHOICE REVIEWS ONLINE', 'Vapnik V, 1995, ', 'Han J, 2012, CHOICE REVIEWS ONLINE', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Breiman L, 1996, MACHINE LEARNING', 'Quinlan J, 1986, MACHINE LEARNING', 'Agrawal R, 1993, ', 'Duda R, 1973, ', 'Guyon I, 2002, MACHINE LEARNING', 'Kleinberg J, 1999, JOURNAL OF THE ACM', 'Piepel G, 1989, TECHNOMETRICS', 'Hartigan J, 1975, ', 'Ankerst M, 1999, ACM SIGMOD RECORD', 'Heckerman D, 1995, MACHINE LEARNING', 'BAYES, 1958, BIOMETRIKA', 'Chen⋆ M, 1996, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Liu B, 1998, ', 'Yan X, 2003, ', 'Holte R, 1993, MACHINE LEARNING', 'Atkinson A, 1995, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (STATISTICS IN SOCIETY)', 'Dumais S, 1998, ', 'Littlestone N, 1988, MACHINE LEARNING', 'Stone P, 2000, AUTONOMOUS ROBOTS', 'Maron O, 1997, ', 'Breiman L, 1996, MACHINE LEARNING', 'Provost F, 1997, ', 'Witten I, 1999, MORGAN KAUFMANN PUBLISHERS INC. EBOOKS', 'Friedman J, 1996, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Califf M, 1997, ', 'Buntine W, 1992, STATISTICS AND COMPUTING', 'Utgoff P, 1997, MACHINE LEARNING', 'Freitag D, 2000, MACHINE LEARNING', 'Cardie C, 1993, ELSEVIER EBOOKS', 'John G, 1995, ', 'Drummond C, 2000, ', 'Salzberg S, 1991, MACHINE LEARNING', 'Gluck M, 1985, ESCHOLARSHIP (CALIFORNIA DIGITAL LIBRARY)', 'Schölkopf B, 1998, ', 'Huffman S, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Moore A, 2000, ', 'John G, 1997, ', 'Martin B, 1995, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Li M, 1992, JOURNAL OF COMPUTER AND SYSTEM SCIENCES', 'Jabbour K, 1988, IEEE TRANSACTIONS ON POWER SYSTEMS', 'Mooney U, 2000, ', 'Komarek P, 2000, ', 'Gennari J, 1988, ', 'Bengio Y, 1999, ÉRUDIT DOCUMENTS AND DATA REPOSITORY (ÉRUDIT CONSORTIUM, UNIVERSITY OF MONTREAL)', 'Bouckaert R, 1995, DATA ARCHIVING AND NETWORKED SERVICES (DANS)', 'C.J.C. B, 1998, ', ', 2015, ', 'Johns M, 1959, ']</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>Ian H. Witten, 2011, Elsevier eBooks</t>
-        </is>
-      </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Ian H. Witten, 2011, Elsevier eBooks</t>
+          <t>Witten I, 2011, ELSEVIER EBOOKS</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Witten I, 2011, ELSEVIER EBOOKS</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1112,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>22083</v>
+        <v>22082</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1142,28 +1172,33 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1480376833', 'https://openalex.org/W1496317909', 'https://openalex.org/W2117812871', 'https://openalex.org/W3215037115', 'https://openalex.org/W4232383088', 'https://openalex.org/W4292691288']</t>
+          <t>['US', 'GB']</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr">
+          <t>['Hastie T, 2001, SPRINGER SERIES IN STATISTICS', 'Ripley B, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Robert C, 2004, SPRINGER TEXTS IN STATISTICS', 'Suykens J, 2002, WORLD SCIENTIFIC EBOOKS', 'Waserman L, 2003, ']</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>Nasser M. Nasrabadi, 2007, Journal of Electronic Imaging</t>
-        </is>
-      </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Nasser M. Nasrabadi, 2007, Journal of Electronic Imaging</t>
+          <t>Nasrabadi N, 2007, JOURNAL OF ELECTRONIC IMAGING</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Nasrabadi N, 2007, JOURNAL OF ELECTRONIC IMAGING</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1234,12 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>['David E. Goldberg', 'David Robson']</t>
+          <t>['David E. Goldberg']</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>['D. Goldberg', 'David Robson']</t>
+          <t>['David E. Goldberg']</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1214,7 +1249,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">D. Goldberg (corresponding author), </t>
+          <t xml:space="preserve">David E. Goldberg (corresponding author), </t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1241,20 +1276,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr">
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">David E. Goldberg, 1988, </t>
-        </is>
-      </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t xml:space="preserve">David E. Goldberg, 1988, </t>
+          <t xml:space="preserve">Goldberg D, 1988, </t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Goldberg D, 1988, </t>
         </is>
       </c>
     </row>
@@ -1332,18 +1372,23 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr">
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2007, </t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2007, </t>
         </is>
@@ -1423,28 +1468,33 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W14377099', 'https://openalex.org/W44447720', 'https://openalex.org/W61071295', 'https://openalex.org/W131514509', 'https://openalex.org/W186419298', 'https://openalex.org/W336602872', 'https://openalex.org/W1213006044', 'https://openalex.org/W1484867920', 'https://openalex.org/W1486089539', 'https://openalex.org/W1486164486', 'https://openalex.org/W1496317909', 'https://openalex.org/W1497675750', 'https://openalex.org/W1505043854', 'https://openalex.org/W1506153731', 'https://openalex.org/W1510355813', 'https://openalex.org/W1512098439', 'https://openalex.org/W1512149552', 'https://openalex.org/W1515272691', 'https://openalex.org/W1543996294', 'https://openalex.org/W1549258098', 'https://openalex.org/W1550570395', 'https://openalex.org/W1551209770', 'https://openalex.org/W1554663460', 'https://openalex.org/W1564947197', 'https://openalex.org/W1567512734', 'https://openalex.org/W1571894236', 'https://openalex.org/W1574225613', 'https://openalex.org/W1598589417', 'https://openalex.org/W1601740268', 'https://openalex.org/W1604293137', 'https://openalex.org/W1607751291', 'https://openalex.org/W1618393386', 'https://openalex.org/W1618449801', 'https://openalex.org/W1628829797', 'https://openalex.org/W1633751774', 'https://openalex.org/W1642427530', 'https://openalex.org/W1648445109', 'https://openalex.org/W1654787807', 'https://openalex.org/W1755117326', 'https://openalex.org/W1859781365', 'https://openalex.org/W1963533512', 'https://openalex.org/W1965999112', 'https://openalex.org/W1967396577', 'https://openalex.org/W1975780894', 'https://openalex.org/W1976382401', 'https://openalex.org/W1976625337', 'https://openalex.org/W1978188282', 'https://openalex.org/W1978394996', 'https://openalex.org/W1981025032', 'https://openalex.org/W1982032418', 'https://openalex.org/W1982276155', 'https://openalex.org/W1986280275', 'https://openalex.org/W1995672551', 'https://openalex.org/W1998167411', 'https://openalex.org/W2000241167', 'https://openalex.org/W2003706076', 'https://openalex.org/W2003870625', 'https://openalex.org/W2006314423', 'https://openalex.org/W2008827410', 'https://openalex.org/W2014831690', 'https://openalex.org/W2015904350', 'https://openalex.org/W2018044188', 'https://openalex.org/W2019363670', 'https://openalex.org/W2020999234', 'https://openalex.org/W2023163512', 'https://openalex.org/W2033839039', 'https://openalex.org/W2041863660', 'https://openalex.org/W2047028564', 'https://openalex.org/W2049387919', 'https://openalex.org/W2056735347', 'https://openalex.org/W2062291655', 'https://openalex.org/W2063852603', 'https://openalex.org/W2065540158', 'https://openalex.org/W2069371995', 'https://openalex.org/W2069527924', 'https://openalex.org/W2072555316', 'https://openalex.org/W2078206416', 'https://openalex.org/W2081873601', 'https://openalex.org/W2085877024', 'https://openalex.org/W2087978636', 'https://openalex.org/W2088538739', 'https://openalex.org/W2090102379', 'https://openalex.org/W2090353374', 'https://openalex.org/W2093268114', 'https://openalex.org/W2094169479', 'https://openalex.org/W2094212611', 'https://openalex.org/W2096335861', 'https://openalex.org/W2098115979', 'https://openalex.org/W2098626000', 'https://openalex.org/W2098949458', 'https://openalex.org/W2100136038', 'https://openalex.org/W2101709642', 'https://openalex.org/W2103972570', 'https://openalex.org/W2104533781', 'https://openalex.org/W2106868411', 'https://openalex.org/W2107152312', 'https://openalex.org/W2107636931', 'https://openalex.org/W2107725114', 'https://openalex.org/W2108966602', 'https://openalex.org/W2111176881', 'https://openalex.org/W2111494971', 'https://openalex.org/W2112545207', 'https://openalex.org/W2114229504', 'https://openalex.org/W2114412769', 'https://openalex.org/W2115606304', 'https://openalex.org/W2116723448', 'https://openalex.org/W2117063635', 'https://openalex.org/W2117812871', 'https://openalex.org/W2118195892', 'https://openalex.org/W2123687908', 'https://openalex.org/W2124101779', 'https://openalex.org/W2124225821', 'https://openalex.org/W2126455177', 'https://openalex.org/W2127713198', 'https://openalex.org/W2129564505', 'https://openalex.org/W2129869373', 'https://openalex.org/W2130475491', 'https://openalex.org/W2130859329', 'https://openalex.org/W2137467792', 'https://openalex.org/W2137557016', 'https://openalex.org/W2137956165', 'https://openalex.org/W2139479120', 'https://openalex.org/W2140170995', 'https://openalex.org/W2140251433', 'https://openalex.org/W2141274633', 'https://openalex.org/W2141436719', 'https://openalex.org/W2142182841', 'https://openalex.org/W2142387771', 'https://openalex.org/W2142575165', 'https://openalex.org/W2143022286', 'https://openalex.org/W2143956139', 'https://openalex.org/W2144286620', 'https://openalex.org/W2145295623', 'https://openalex.org/W2146766088', 'https://openalex.org/W2148603752', 'https://openalex.org/W2149417376', 'https://openalex.org/W2149846618', 'https://openalex.org/W2151238122', 'https://openalex.org/W2152701363', 'https://openalex.org/W2152937653', 'https://openalex.org/W2153347097', 'https://openalex.org/W2153756422', 'https://openalex.org/W2156909104', 'https://openalex.org/W2158451137', 'https://openalex.org/W2158529569', 'https://openalex.org/W2160840682', 'https://openalex.org/W2161767008', 'https://openalex.org/W2162114812', 'https://openalex.org/W2163057507', 'https://openalex.org/W2167061265', 'https://openalex.org/W2167986580', 'https://openalex.org/W2168022998', 'https://openalex.org/W2169779569', 'https://openalex.org/W2170076406', 'https://openalex.org/W2170078560', 'https://openalex.org/W2170120409', 'https://openalex.org/W2170334710', 'https://openalex.org/W2171522835', 'https://openalex.org/W2172039283', 'https://openalex.org/W2296319761', 'https://openalex.org/W2408196097', 'https://openalex.org/W2464224693', 'https://openalex.org/W2548695521', 'https://openalex.org/W2554813760', 'https://openalex.org/W2782810849', 'https://openalex.org/W2797583072', 'https://openalex.org/W2798909945', 'https://openalex.org/W2904816695', 'https://openalex.org/W2916304084', 'https://openalex.org/W2989448192', 'https://openalex.org/W3014600732', 'https://openalex.org/W3017143921', 'https://openalex.org/W3023786531', 'https://openalex.org/W3048078645', 'https://openalex.org/W3119264854', 'https://openalex.org/W3127325877', 'https://openalex.org/W3134067276', 'https://openalex.org/W3140968660', 'https://openalex.org/W3148924112', 'https://openalex.org/W3165771198']</t>
+          <t>['DE']</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr">
+          <t>['1959- B, 1994, CHOICE REVIEWS ONLINE', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Platt J, 1998, THE MIT PRESS EBOOKS', 'Wiener N, 1949, THE MIT PRESS EBOOKS', 'Neal R, 1996, LECTURE NOTES IN STATISTICS', 'Cristianini N, 2000, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Suykens J, 2002, WORLD SCIENTIFIC EBOOKS', 'Devroye L, 1996, STOCHASTIC MODELLING AND APPLIED PROBABILITY', '1950- G, 2004, ELSEVIER EBOOKS', 'Wendland H, 2004, CAMBRIDGE UNIVERSITY PRESS EBOOKS', ', 2000, APPLIED PHYSICS LETTERS', 'Györfi L, 2002, SPRINGER SERIES IN STATISTICS', 'Girosi F, 1995, NEURAL COMPUTATION', 'Bartlett P, 2006, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Geisser S, 1979, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Saunders C, 1998, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Tipping M, 2003, ', 'Smola A, 2000, ', 'Winkler G, 1995, ', 'König H, 1986, OPERATOR THEORY', 'Silverman B, 1984, THE ANNALS OF STATISTICS', 'Seeger M, 2003, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Collobert R, 2000, APPLIED PHYSICS LETTERS', 'Wong E, 1979, ', 'Ritter K, 2000, LECTURE NOTES IN MATHEMATICS', 'Kammler D, 2008, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Teh Y, 2005, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'McAllester D, 2003, MACHINE LEARNING', 'Rasmussen C, 2003, ', 'Gibbs M, 1997, ', 'Seeger M, 2005, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Stitson M, 1998, THE MIT PRESS EBOOKS', 'Grenander U, 1990, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Plaskota L, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Gao F, 2000, THE ANNALS OF STATISTICS', 'Zhu H, 1997, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Silverman B, 1978, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Seeger M, 2004, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Arató M, 1982, LECTURE NOTES IN CONTROL AND INFORMATION SCIENCES', 'Pontil M, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Micchelli C, 1979, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', 'Choi T, 2018, FIGSHARE', 'Cornford D, 2002, JOURNAL OF NONPARAMETRIC STATISTICS', 'Szeliski R, 1987, NATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Grünwald P, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Hawkins D, 1989, COMMUNICATIONS IN STATISTICS - SIMULATION AND COMPUTATION', 'Minka T, 2001, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)', 'Hinton G, 1997, ', 'Neal R, 1997, ARXIV.ORG', 'Mandelbrot B, 1983, AMERICAN JOURNAL OF PHYSICS', 'Geman S, 1984, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Sacks J, 1989, STATISTICAL SCIENCE', 'Hoerl A, 2000, TECHNOMETRICS', 'Aronszajn N, 1950, TRANSACTIONS OF THE AMERICAN MATHEMATICAL SOCIETY', 'Valiant L, 1984, ', 'Arfken G, 1967, AMERICAN JOURNAL OF PHYSICS', 'Green P, 1994, ', ', 1992, CHOICE REVIEWS ONLINE', 'Bishop C, 1998, NEURAL COMPUTATION', 'Kimeldorf G, 1971, JOURNAL OF MATHEMATICAL ANALYSIS AND APPLICATIONS', 'Hand D, 2007, DRUG SAFETY', 'Mazur P, 1959, PHYSICA', 'Zhang T, 2004, THE ANNALS OF STATISTICS', 'Mackay D, 1992, NEURAL COMPUTATION', 'Schoenberg I, 1938, TRANSACTIONS OF THE AMERICAN MATHEMATICAL SOCIETY', 'Diaconis P, 1986, THE ANNALS OF STATISTICS', 'Wahba G, 1985, THE ANNALS OF STATISTICS', 'Schoenberg I, 1964, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Girard A, 2002, ', 'Rasmussen C, 2001, ', 'Solak E, 2002, ', 'O’Sullivan F, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Baxter L, 1996, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES D (THE STATISTICIAN)', 'Mackay D, 2000, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Dawid A, 1976, BIOMETRICS', 'Meir R, 2003, ', 'Cox D, 1984, SIAM JOURNAL ON NUMERICAL ANALYSIS', 'Hansen L, 1997, OPEN SYSTEMS &amp; INFORMATION DYNAMICS', 'Shepp L, 1966, THE ANNALS OF MATHEMATICAL STATISTICS', 'Eskin E, 2002, ', 'Kashyap R, 1981, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Cox D, 1990, THE ANNALS OF STATISTICS', 'Luo Z, 1997, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Williams C, 1998, NEURAL COMPUTATION', 'Freedman D, 1999, THE ANNALS OF STATISTICS', 'Poggio T, 1988, JOURNAL OF COMPLEXITY', 'Tsuda K, 2002, NEURAL COMPUTATION', 'Wahba G, 1995, MONTHLY WEATHER REVIEW', 'Rasmussen C, 2005, ', 'Schwaighofer A, 2002, ', 'Kohn R, 1987, SIAM JOURNAL ON SCIENTIFIC AND STATISTICAL COMPUTING', 'Blight B, 1975, BIOMETRIKA', 'Williams C, 2002, CAMBRIDGE UNIVERSITY ENGINEERING DEPARTMENT PUBLICATIONS DATABASE', 'Wood S, 1998, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Williams C, 2002, NEURAL INFORMATION PROCESSING SYSTEMS', 'Stein M, 1991, ANNALS OF THE INSTITUTE OF STATISTICAL MATHEMATICS', 'Girosi F, 1991, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', 'Thompson P, 1956, TELLUS A DYNAMIC METEOROLOGY AND OCEANOGRAPHY', 'Seeger M, 2003, ERA', 'Vapnik V, 1995, ', 'Wu Y, 1999, TECHNOMETRICS', 'Cressie N, 1992, TERRA NOVA', 'Bell J, 1978, MATHEMATICS OF COMPUTATION', 'Ripley B, 1996, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Müller H, 1991, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Rousseeuw P, 1984, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Dickey D, 1991, TECHNOMETRICS', 'Poggio T, 1990, PROCEEDINGS OF THE IEEE', 'Øksendal B, 2003, UNIVERSITEXT', 'Jones D, 2001, JOURNAL OF GLOBAL OPTIMIZATION', 'Williams C, 2000, ', 'Wahba G, 1975, NUMERISCHE MATHEMATIK', 'Duchon J, 1977, LECTURE NOTES IN MATHEMATICS', 'Williams C, 1995, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Cristianini N, 2006, STUDIES IN FUZZINESS AND SOFT COMPUTING', 'Collins M, 2002, THE MIT PRESS EBOOKS', 'Williams C, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Csató L, 2002, NEURAL COMPUTATION', 'Drineas P, 2005, ', ', 2000, APPLIED PHYSICS LETTERS', 'Fine S, 2002, ', 'Herbrich R, 2002, NEURAL INFORMATION PROCESSING SYSTEMS', 'Chu W, 2005, CAMBRIDGE UNIVERSITY ENGINEERING DEPARTMENT PUBLICATIONS DATABASE', 'Farlie D, 1964, OR', 'Smola A, 2000, ', 'Paciorek C, 2003, ', 'Vishwanathan S, 2004, THE MIT PRESS EBOOKS', 'Faul A, 2002, THE MIT PRESS EBOOKS', 'Mackay D, 1999, NEURAL COMPUTATION', 'Simard P, 1991, NEURAL INFORMATION PROCESSING SYSTEMS', 'Opper M, 2000, NEURAL COMPUTATION', 'Ghahramani Z, 2002, NEURAL INFORMATION PROCESSING SYSTEMS', 'Sundararajan S, 2001, NEURAL COMPUTATION', 'Rasmussen C, 2000, NEURAL INFORMATION PROCESSING SYSTEMS', 'Micchelli C, 2004, UCL DISCOVERY (UNIVERSITY COLLEGE LONDON)', 'Zhu J, 2001, ', 'Vijayakumar S, 2002, AUTONOMOUS ROBOTS', 'Murray‐Smith R, 2001, ENLIGHTEN (JURNAL BIMBINGAN DAN KONSELING ISLAM)', 'Sollich P, 2004, ', 'Seeger M, 1999, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', "Sollich P, 1998, RESEARCH PORTAL (KING'S COLLEGE LONDON)", 'Opper M, 1998, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Vivarelli F, 1998, NEURAL INFORMATION PROCESSING SYSTEMS', 'Ferrari‐Trecate G, 1998, NEURAL INFORMATION PROCESSING SYSTEMS', 'Saunders C, 2002, EPRINTS SOTON (UNIVERSITY OF SOUTHAMPTON)', 'Malzahn D, 2002, THE MIT PRESS EBOOKS', 'Csató L, 2002, THE MIT PRESS EBOOKS', 'Kuß M, 2005, ', 'Boyd S, 2004, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Golub G, 2012, JOHNS HOPKINS UNIVERSITY PRESS EBOOKS', 'Press W, 1994, ', 'Duda R, 1973, ', 'Kölbig K, 1995, MATHEMATICS OF COMPUTATION', 'Brown R, 1991, BIOMETRICS', ', 2004, CHOICE REVIEWS ONLINE', 'Cox D, 1966, PHYSICS TODAY', 'Ripley B, 1981, ', 'Schölkopf B, 2001, MPG.PURE (MAX PLANCK SOCIETY)', 'Platt J, 2000, THE MIT PRESS EBOOKS', 'Iaglom A, 1987, SPRINGER EBOOKS', 'Lawrence N, 2003, ', 'O’Hagan A, 1978, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Tsokos C, 1992, TECHNOMETRICS', ', 1964, ELSEVIER EBOOKS', 'Goldberg P, 1997, ASTON PUBLICATIONS EXPLORER (ASTON UNIVERSITY)', 'Seeger M, 2003, JOURNAL OF MACHINE LEARNING RESEARCH', 'Boyle P, 2004, ', 'Berk R, 1996, TECHNOMETRICS', 'Jaakkola T, 1999, ', 'Dym H, 1989, REGIONAL CONFERENCE SERIES IN MATHEMATICS', 'Kailath T, 1971, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Yang C, 2004, ', 'Blake I, 1973, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Watkins C, 2000, THE MIT PRESS EBOOKS', 'Fowlkes C, 2005, ', 'Hájek J, 1958, CZECHOSLOVAK MATHEMATICAL JOURNAL', 'Quiñonero-Candela J, 2004, MPG.PURE (MAX PLANCK SOCIETY)']</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
-        </is>
-      </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
+          <t>Rasmussen C, 2005, THE MIT PRESS EBOOKS</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Rasmussen C, 2005, THE MIT PRESS EBOOKS</t>
         </is>
       </c>
     </row>
@@ -1522,20 +1572,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
-        </is>
-      </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
+          <t xml:space="preserve">Murphy K, 2012, </t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Murphy K, 2012, </t>
         </is>
       </c>
     </row>
@@ -1569,7 +1624,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9559</v>
+        <v>9550</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1629,28 +1684,33 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W99485931', 'https://openalex.org/W1503398984', 'https://openalex.org/W1512585804', 'https://openalex.org/W1554944419', 'https://openalex.org/W1569098853', 'https://openalex.org/W1873763122', 'https://openalex.org/W1970472910', 'https://openalex.org/W1992570774', 'https://openalex.org/W1999352252', 'https://openalex.org/W2006452405', 'https://openalex.org/W2019363670', 'https://openalex.org/W2042469398', 'https://openalex.org/W2047281923', 'https://openalex.org/W2076063813', 'https://openalex.org/W2097381042', 'https://openalex.org/W2100495367', 'https://openalex.org/W2117726420', 'https://openalex.org/W2127180992', 'https://openalex.org/W2132001804', 'https://openalex.org/W2145339207', 'https://openalex.org/W2146774335', 'https://openalex.org/W2151320232', 'https://openalex.org/W2160815625', 'https://openalex.org/W2163605009', 'https://openalex.org/W2174706414', 'https://openalex.org/W2618530766', 'https://openalex.org/W3102480238', 'https://openalex.org/W4214717370', 'https://openalex.org/W4231109964', 'https://openalex.org/W4238893454', 'https://openalex.org/W4244670803', 'https://openalex.org/W4292363360']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr">
+          <t>['Krizhevsky A, 2017, COMMUNICATIONS OF THE ACM', 'Mnih V, 2015, NATURE', 'Sutton R, 1998, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Hinton G, 2006, SCIENCE', 'Hastie T, 2013, ', 'Schmidhuber J, 2014, NEURAL NETWORKS', 'Boyd S, 2011, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Schultz W, 1997, SCIENCE', 'Murphy K, 2012, ', 'Dwork C, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Bengio Y, 2009, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Blei D, 2012, COMMUNICATIONS OF THE ACM', 'Valiant L, 1984, ', 'Valiant L, 1984, COMMUNICATIONS OF THE ACM', 'Taylor M, 2009, JOURNAL OF MACHINE LEARNING RESEARCH', 'Thrun S, 1998, ', 'Sra S, 2011, THE MIT PRESS EBOOKS', 'Mahoney M, 2012, CHAPMAN &amp; HALL/CRC DATA MINING AND KNOWLEDGE DISCOVERY SERIES', 'Kleiner A, 2014, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Wehbe L, 2014, PLOS ONE', 'Duan R, 2014, JOURNAL OF THE ACM', 'Berthet Q, 2013, THE ANNALS OF STATISTICS', 'Blum A, 2013, JOURNAL OF THE ACM', 'Boyd M, 2011, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Chandrasekaran V, 2013, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Duchi J, 2014, JOURNAL OF THE ACM', 'Balcan M, 2012, ARXIV (CORNELL UNIVERSITY)', 'Decatur S, 2000, SIAM JOURNAL ON COMPUTING', 'Yaylalı E, 2011, WILEY ENCYCLOPEDIA OF OPERATIONS RESEARCH AND MANAGEMENT SCIENCE']</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>Michael I. Jordan, 2015, Science</t>
-        </is>
-      </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Michael I. Jordan, 2015, Science</t>
+          <t>Jordan M, 2015, SCIENCE</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Jordan M, 2015, SCIENCE</t>
         </is>
       </c>
     </row>
@@ -1724,18 +1784,23 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr">
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2006, </t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2006, </t>
         </is>
@@ -1819,20 +1884,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr">
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>Catherine Blake, 1998, Medical Entomology and Zoology</t>
-        </is>
-      </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Catherine Blake, 1998, Medical Entomology and Zoology</t>
+          <t>Blake C, 1998, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Blake C, 1998, MEDICAL ENTOMOLOGY AND ZOOLOGY</t>
         </is>
       </c>
     </row>
@@ -1866,7 +1936,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>8216</v>
+        <v>8215</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1918,20 +1988,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr">
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>PedregosaFabian, 2011, Journal of Machine Learning Research</t>
-        </is>
-      </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>PedregosaFabian, 2011, Journal of Machine Learning Research</t>
+          <t>PedregosaFabian, 2011, JOURNAL OF MACHINE LEARNING RESEARCH</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>PedregosaFabian, 2011, JOURNAL OF MACHINE LEARNING RESEARCH</t>
         </is>
       </c>
     </row>
@@ -2009,28 +2084,33 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W104184427', 'https://openalex.org/W145476170', 'https://openalex.org/W941230081', 'https://openalex.org/W1442374986', 'https://openalex.org/W1484210532', 'https://openalex.org/W1485981043', 'https://openalex.org/W1493893823', 'https://openalex.org/W1498436455', 'https://openalex.org/W1548328233', 'https://openalex.org/W1598866093', 'https://openalex.org/W1658008008', 'https://openalex.org/W1667652561', 'https://openalex.org/W1869752048', 'https://openalex.org/W1978660892', 'https://openalex.org/W1992479210', 'https://openalex.org/W2041517243', 'https://openalex.org/W2055312318', 'https://openalex.org/W2061570747', 'https://openalex.org/W2066443755', 'https://openalex.org/W2072566913', 'https://openalex.org/W2083842231', 'https://openalex.org/W2099471712', 'https://openalex.org/W2100664567', 'https://openalex.org/W2109722477', 'https://openalex.org/W2117539524', 'https://openalex.org/W2120480077', 'https://openalex.org/W2131400476', 'https://openalex.org/W2131975293', 'https://openalex.org/W2132339004', 'https://openalex.org/W2140833774', 'https://openalex.org/W2141992894', 'https://openalex.org/W2145339207', 'https://openalex.org/W2146757372', 'https://openalex.org/W2160815625', 'https://openalex.org/W2163961697', 'https://openalex.org/W2168231600', 'https://openalex.org/W2173213060', 'https://openalex.org/W2186615578', 'https://openalex.org/W2198403777', 'https://openalex.org/W2259472270', 'https://openalex.org/W2308045930', 'https://openalex.org/W2336650964', 'https://openalex.org/W2339765813', 'https://openalex.org/W2384495648', 'https://openalex.org/W2591588155', 'https://openalex.org/W2949117887', 'https://openalex.org/W2949245006', 'https://openalex.org/W2949501655', 'https://openalex.org/W2949605076', 'https://openalex.org/W2949650786', 'https://openalex.org/W2949888546', 'https://openalex.org/W2950094539', 'https://openalex.org/W2950179405', 'https://openalex.org/W2950577311', 'https://openalex.org/W2951714314', 'https://openalex.org/W2951781666']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr">
+          <t>['Russakovsky O, 2015, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Rumelhart D, 1986, NATURE', 'Mnih V, 2015, NATURE', '淳司 柴, 2017, JOURNAL OF JAPAN SOCIETY FOR FUZZY THEORY AND INTELLIGENT INFORMATICS', 'Dean J, 2008, COMMUNICATIONS OF THE ACM', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Zaharia M, 2012, ', 'Sutskever I, 2013, ', 'Dean J, 2012, ', ', 2000, APPLIED PHYSICS LETTERS', 'Sifis L, 2016, ARXIV (CORNELL UNIVERSITY)', 'Le Q, 2013, ', 'Hindman B, 2011, UC BERKELEY', 'Verma A, 2015, ', 'Karpathy A, 2014, ', 'Chu C, 2007, THE MIT PRESS EBOOKS', 'Jordan M, 1997, ADVANCES IN PSYCHOLOGY', 'Larochelle H, 2009, ', 'Li M, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Burrows M, 2006, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Ragan‐Kelley J, 2013, ', 'Jean S, 2015, ', 'Hinton G, 1989, ESCHOLARSHIP (CALIFORNIA DIGITAL LIBRARY)', 'Li M, 2014, ', 'Yu Y, 2008, ', 'Chilimbi T, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Collobert R, 2002, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Smola A, 2010, PROCEEDINGS OF THE VLDB ENDOWMENT', 'Byrd R, 2012, MATHEMATICAL PROGRAMMING', 'Cui H, 2016, ', 'Heigold G, 2013, ', 'Rossbach C, 2013, ', 'Chung E, 2013, ', 'Ovtcharov K, 2015, ', 'Ioffe S, 2024, ARXIV (CORNELL UNIVERSITY)', 'He K, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chen T, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chetlur S, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Józefowicz R, 2016, ARXIV (CORNELL UNIVERSITY)', 'Ba J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Xinghao P, 2017, ARXIV (CORNELL UNIVERSITY)', 'Szegedy C, 2015, ARXIV (CORNELL UNIVERSITY)', 'Nair A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Vinyals O, 2014, ARXIV (CORNELL UNIVERSITY)', 'Dai A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Crankshaw D, 2014, ARXIV (CORNELL UNIVERSITY)', 'Lavin A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Moritz P, 2015, ARXIV (CORNELL UNIVERSITY)', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Jia Y, 2014, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Szegedy C, 2014, ARXIV (CORNELL UNIVERSITY)', 'Niu F, 2011, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>Martı́n Abadi, 2016, arXiv (Cornell University)</t>
-        </is>
-      </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Martı́n Abadi, 2016, arXiv (Cornell University)</t>
+          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2144,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>7891</v>
+        <v>7890</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2124,28 +2204,33 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W12876238', 'https://openalex.org/W22906612', 'https://openalex.org/W35304842', 'https://openalex.org/W59979790', 'https://openalex.org/W74894479', 'https://openalex.org/W81384683', 'https://openalex.org/W81511778', 'https://openalex.org/W104970664', 'https://openalex.org/W107306860', 'https://openalex.org/W112196149', 'https://openalex.org/W116328816', 'https://openalex.org/W148103248', 'https://openalex.org/W166124110', 'https://openalex.org/W1482260847', 'https://openalex.org/W1487445520', 'https://openalex.org/W1490175418', 'https://openalex.org/W1493526108', 'https://openalex.org/W1505794130', 'https://openalex.org/W1507179106', 'https://openalex.org/W1508175965', 'https://openalex.org/W1513874326', 'https://openalex.org/W1514707997', 'https://openalex.org/W1520963883', 'https://openalex.org/W1522930027', 'https://openalex.org/W1523389133', 'https://openalex.org/W1523949738', 'https://openalex.org/W1533946607', 'https://openalex.org/W1544227718', 'https://openalex.org/W1547553618', 'https://openalex.org/W1550961891', 'https://openalex.org/W1553682320', 'https://openalex.org/W1556094091', 'https://openalex.org/W1561056154', 'https://openalex.org/W1574901103', 'https://openalex.org/W1576676390', 'https://openalex.org/W1577216492', 'https://openalex.org/W1578881253', 'https://openalex.org/W1591234214', 'https://openalex.org/W1592212241', 'https://openalex.org/W1594962278', 'https://openalex.org/W1597379537', 'https://openalex.org/W1601145406', 'https://openalex.org/W1619226191', 'https://openalex.org/W1620204465', 'https://openalex.org/W1813610639', 'https://openalex.org/W1857571498', 'https://openalex.org/W1907380269', 'https://openalex.org/W1924689489', 'https://openalex.org/W1966065191', 'https://openalex.org/W1969572066', 'https://openalex.org/W1970858159', 'https://openalex.org/W1970974276', 'https://openalex.org/W1971666241', 'https://openalex.org/W1973911615', 'https://openalex.org/W1975496312', 'https://openalex.org/W1977182536', 'https://openalex.org/W1978394996', 'https://openalex.org/W1979648751', 'https://openalex.org/W1980776671', 'https://openalex.org/W1983078185', 'https://openalex.org/W1986913017', 'https://openalex.org/W1988711048', 'https://openalex.org/W1989568037', 'https://openalex.org/W1989738209', 'https://openalex.org/W1993657037', 'https://openalex.org/W1993934121', 'https://openalex.org/W1995014490', 'https://openalex.org/W2001664274', 'https://openalex.org/W2002675557', 'https://openalex.org/W2002857471', 'https://openalex.org/W2003436527', 'https://openalex.org/W2004180556', 'https://openalex.org/W2004871537', 'https://openalex.org/W2005422315', 'https://openalex.org/W2005758492', 'https://openalex.org/W2006119904', 'https://openalex.org/W2006187024', 'https://openalex.org/W2007395264', 'https://openalex.org/W2007512902', 'https://openalex.org/W2008931716', 'https://openalex.org/W2009190245', 'https://openalex.org/W2010652031', 'https://openalex.org/W2013657661', 'https://openalex.org/W2015267443', 'https://openalex.org/W2015518873', 'https://openalex.org/W2017867386', 'https://openalex.org/W2019778169', 'https://openalex.org/W2020316999', 'https://openalex.org/W2025451713', 'https://openalex.org/W2029609769', 'https://openalex.org/W2033751006', 'https://openalex.org/W2035754578', 'https://openalex.org/W2040424159', 'https://openalex.org/W2041726831', 'https://openalex.org/W2043909051', 'https://openalex.org/W2045812729', 'https://openalex.org/W2047031127', 'https://openalex.org/W2049384587', 'https://openalex.org/W2053463056', 'https://openalex.org/W2058982198', 'https://openalex.org/W2059019405', 'https://openalex.org/W2060216474', 'https://openalex.org/W2060476676', 'https://openalex.org/W2060704583', 'https://openalex.org/W2062847911', 'https://openalex.org/W2062914707', 'https://openalex.org/W2063198646', 'https://openalex.org/W2063862666', 'https://openalex.org/W2064580901', 'https://openalex.org/W2065010255', 'https://openalex.org/W2065747622', 'https://openalex.org/W2066462377', 'https://openalex.org/W2071415686', 'https://openalex.org/W2071664212', 'https://openalex.org/W2076008912', 'https://openalex.org/W2077777431', 'https://openalex.org/W2080251601', 'https://openalex.org/W2084044465', 'https://openalex.org/W2085302848', 'https://openalex.org/W2085989833', 'https://openalex.org/W2087609354', 'https://openalex.org/W2088658068', 'https://openalex.org/W2092134162', 'https://openalex.org/W2092488901', 'https://openalex.org/W2092689128', 'https://openalex.org/W2093098531', 'https://openalex.org/W2094934653', 'https://openalex.org/W2096152098', 'https://openalex.org/W2096411881', 'https://openalex.org/W2097089247', 'https://openalex.org/W2097847889', 'https://openalex.org/W2101154521', 'https://openalex.org/W2104808840', 'https://openalex.org/W2106365165', 'https://openalex.org/W2107008379', 'https://openalex.org/W2107827038', 'https://openalex.org/W2110224739', 'https://openalex.org/W2114535528', 'https://openalex.org/W2125776553', 'https://openalex.org/W2126502509', 'https://openalex.org/W2126631147', 'https://openalex.org/W2126850915', 'https://openalex.org/W2127994451', 'https://openalex.org/W2130337399', 'https://openalex.org/W2132315067', 'https://openalex.org/W2133890944', 'https://openalex.org/W2135276756', 'https://openalex.org/W2139578439', 'https://openalex.org/W2140785063', 'https://openalex.org/W2140956226', 'https://openalex.org/W2142515059', 'https://openalex.org/W2145036943', 'https://openalex.org/W2145296344', 'https://openalex.org/W2146888100', 'https://openalex.org/W2147152072', 'https://openalex.org/W2149684865', 'https://openalex.org/W2151801809', 'https://openalex.org/W2153211312', 'https://openalex.org/W2153962014', 'https://openalex.org/W2158738673', 'https://openalex.org/W2165612380', 'https://openalex.org/W2169384781', 'https://openalex.org/W2170654002', 'https://openalex.org/W2172142456', 'https://openalex.org/W2174678383', 'https://openalex.org/W2435251607', 'https://openalex.org/W2561675875', 'https://openalex.org/W2798573942', 'https://openalex.org/W2915186198', 'https://openalex.org/W2949696181', 'https://openalex.org/W2952299822', 'https://openalex.org/W2953123431', 'https://openalex.org/W3042893949', 'https://openalex.org/W3157411736', 'https://openalex.org/W4205241946', 'https://openalex.org/W4240008182', 'https://openalex.org/W4249379282', 'https://openalex.org/W4285719527', 'https://openalex.org/W6604296810', 'https://openalex.org/W6614676750', 'https://openalex.org/W6629232668', 'https://openalex.org/W6630268012', 'https://openalex.org/W6631307659', 'https://openalex.org/W6632118081', 'https://openalex.org/W6633640926', 'https://openalex.org/W6635379667', 'https://openalex.org/W6635548358', 'https://openalex.org/W6636628491', 'https://openalex.org/W6638423001', 'https://openalex.org/W6641777427', 'https://openalex.org/W6643036076', 'https://openalex.org/W6644484350', 'https://openalex.org/W6666817399', 'https://openalex.org/W6673691841', 'https://openalex.org/W6673781366', 'https://openalex.org/W6679004887', 'https://openalex.org/W6679453733', 'https://openalex.org/W6681835404', 'https://openalex.org/W6682342947', 'https://openalex.org/W6738852829', 'https://openalex.org/W6792154874', 'https://openalex.org/W6794861161', 'https://openalex.org/W7046466245', 'https://openalex.org/W7064660697']</t>
+          <t>['IT']</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr">
+          <t>['John G, 1994, ELSEVIER EBOOKS', 'Lewis D, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Lang K, 1995, ELSEVIER EBOOKS', 'Cavnar W, 1994, ', 'Lewis D, 1994, ELSEVIER EBOOKS', 'Jones K, 1997, MORGAN KAUFMANN PUBLISHERS INC. EBOOKS', 'Koller D, 1997, ', 'McCallum A, 1998, ', 'Klinkenberg R, 2000, ', 'Cohen W, 1996, ', 'Lewis D, 1991, SCHOLARWORKS@UMASSAMHERST (UNIVERSITY OF MASSACHUSETTS AMHERST)', 'Cohen W, 1999, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Yang Y, 2002, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Scott S, 1999, ', 'Galavotti L, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Liere R, 1997, ', 'Caropreso M, 2001, ', 'Mladenić D, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Weigend A, 1999, INFORMATION RETRIEVAL', 'Wermter S, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Taira H, 1999, ', 'Willett P, 1988, ', 'Roussinov D, 1998, UA CAMPUS REPOSITORY (THE UNIVERSITY OF ARIZONA)', 'Fuhr N, 1991, ', 'Diao Y, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Escudero G, 2000, EUROPEAN CONFERENCE ON MACHINE LEARNING', 'Frasconi P, 2002, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Myers K, 2000, ', 'Joachims T, 2002, JOURNAL OF INTELLIGENT INFORMATION SYSTEMS', 'Forsyth R, 1999, ', 'Cohen W, 1995, ELSEVIER EBOOKS', ', 2002, PROGRAM ELECTRONIC LIBRARY AND INFORMATION SYSTEMS', 'Lam W, 1997, INTERNATIONAL JOINT CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Fuhr N, 1985, ', 'Fuhr N, 1984, INTERNATIONAL ACM SIGIR CONFERENCE ON RESEARCH AND DEVELOPMENT IN INFORMATION RETRIEVAL', 'Attardi G, 1998, ZENODO (CERN EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Hull D, 1997, ', 'Sable C, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Lim J, 1999, ', 'Manning C, 1999, ', 'McCallum A, 2022, ', 'Roth D, 1998, ARXIV.ORG', 'Dagan I, 1997, ARXIV.ORG', 'Rodríguez M, 1997, ARXIV.ORG', 'Lewis D, 1994, ACM TRANSACTIONS ON OFFICE INFORMATION SYSTEMS', 'Knorz G, 1982, INTERNATIONAL ACM SIGIR CONFERENCE ON RESEARCH AND DEVELOPMENT IN INFORMATION RETRIEVAL', 'Fangmeyer H, 1968, IFIP CONGRESS', 'Díaz A, 1998, ', 'Lewis D, 1999, INTERNATIONAL ACM SIGIR CONFERENCE ON RESEARCH AND DEVELOPMENT IN INFORMATION RETRIEVAL', 'Tong R, 1992, TEXT RETRIEVAL CONFERENCE', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Yang Y, 1999, ', 'Schapire R, 2000, MACHINE LEARNING', 'Robertson S, 1976, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Chakrabarti S, 1998, COMPUTER NETWORKS AND ISDN SYSTEMS', 'Weikum G, 2002, ACM SIGMOD RECORD', 'Tumer K, 1996, CONNECTION SCIENCE', 'Maron M, 1961, JOURNAL OF THE ACM', 'Gale W, 1992, COMPUTERS AND THE HUMANITIES', 'Schütze H, 1995, ', 'Ng H, 1997, ', 'Larkey L, 1996, ', 'Yang Y, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Crestani F, 1998, ACM COMPUTING SURVEYS', 'Schapire R, 1998, ', 'Masand B, 1992, ', 'Weiss S, 1999, IEEE INTELLIGENT SYSTEMS AND THEIR APPLICATIONS', 'Fuhr N, 1991, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Singhal A, 1996, INFORMATION PROCESSING &amp; MANAGEMENT', 'Yang Y, 1995, ', 'Lam W, 1998, ', 'Wong S, 1995, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Hull D, 1994, ', 'Dörre J, 1999, ', 'Tzeras K, 1993, ', 'Fürnkranz J, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Iwayama M, 1995, ', 'Merkl D, 1998, NEUROCOMPUTING', 'Cooper W, 1995, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Fuhr N, 1989, INFORMATION PROCESSING &amp; MANAGEMENT', 'Singhal A, 1997, ', 'Kim Y, 2000, ', 'Frasconi P, 2001, ', 'Biebricher P, 1988, ', 'Iyer R, 2000, ', 'Knight K, 1999, COMMUNICATIONS OF THE ACM', 'Li P, 1996, CONNECTION SCIENCE', 'Papka R, 1998, ', 'Yu K, 1998, ', 'Cooper W, 1991, ', 'Klingbiel P, 1973, INFORMATION STORAGE AND RETRIEVAL', 'Field B, 1975, JOURNAL OF DOCUMENTATION', 'Guthrie L, 1994, ', 'Sable C, 2000, INTERNATIONAL JOURNAL ON DIGITAL LIBRARIES', 'Liddy E, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Klingbiel P, 1973, INFORMATION STORAGE AND RETRIEVAL', 'Robertson S, 1984, JOURNAL OF DOCUMENTATION', 'Hoyle W, 1973, INFORMATION STORAGE AND RETRIEVAL', 'Wong J, 1996, ACM SIGIR FORUM', 'Cleverdon C, 1984, INFORMATION SERVICES &amp; USE', 'Domingos P, 1997, MACHINE LEARNING', 'Nigam K, 2000, MACHINE LEARNING', 'Joachims T, 1999, ', 'Yang Y, 1999, INFORMATION RETRIEVAL', 'Lewis D, 1994, ARXIV (CORNELL UNIVERSITY)', 'Belkin N, 1992, COMMUNICATIONS OF THE ACM', 'Schütze H, 1998, ', 'Joachims T, 1997, ', 'Apté C, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Saračević T, 1975, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Dumais S, 2000, ', 'Chakrabarti S, 1998, ', 'Baker L, 1998, ', 'Lewis D, 1992, ', 'Lewis D, 1996, ', 'Rijsbergen C, 1977, JOURNAL OF DOCUMENTATION', 'Androutsopoulos I, 2000, ', 'Lewis D, 1995, ACM SIGIR FORUM', 'Li Y, 1998, THE COMPUTER JOURNAL', 'Nigam K, 1998, ', 'Larkey L, 1998, ', 'Chakrabarti S, 1998, THE VLDB JOURNAL', 'Larkey L, 1999, ', 'Lam S, 2003, ', 'Borko H, 1963, JOURNAL OF THE ACM', 'Creecy R, 1992, COMMUNICATIONS OF THE ACM', 'Oh H, 2000, ', 'Attardi G, 1999, CINECA IRIS INSTITUTIAL RESEARCH INFORMATION SYSTEM (UNIVERSITY OF PISA)', 'Hayes P, 2002, ', 'Amati G, 1999, INFORMATION PROCESSING &amp; MANAGEMENT', 'Heaps H, 1973, INFORMATION AND CONTROL', 'Riloff E, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Cohen W, 1998, ', 'Hull D, 1996, ', 'Ruiz M, 1999, ', 'Gövert N, 1999, ', 'Ragas H, 1998, ', 'Li H, 1999, ', 'Clack C, 1997, ', 'Hamill K, 1980, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Fuhr N, 1994, ACM TRANSACTIONS ON INFORMATION SYSTEMS', 'Moulinier I, 1996, LECTURE NOTES IN COMPUTER SCIENCE', 'Rau L, 1991, ', 'Goodman M, 1990, INNOVATIVE APPLICATIONS OF ARTIFICIAL INTELLIGENCE', 'Junker M, 1998, INTERNATIONAL JOURNAL ON DOCUMENT ANALYSIS AND RECOGNITION (IJDAR)', 'Gray W, 1971, INFORMATION STORAGE AND RETRIEVAL', 'Brückner T, 1997, TEXT RETRIEVAL CONFERENCE', ', 1999, INDUSTRIAL ROBOT THE INTERNATIONAL JOURNAL OF ROBOTICS RESEARCH AND APPLICATION', 'Deerwester S, 1990, JOURNAL OF THE AMERICAN SOCIETY FOR INFORMATION SCIENCE', 'Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Salton G, 1975, COMMUNICATIONS OF THE ACM', 'Yang Y, 1997, ', 'Drucker H, 1999, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Dumais S, 1998, ', 'Subashini D, 1993, JOURNAL OF COMPUTATIONAL AND APPLIED MATHEMATICS', 'Willett P, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Kessler B, 1997, ', 'Lewis D, 1995, ', 'Lam W, 1999, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Escudero G, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Raghavan V, 2004, CHAPMAN &amp; HALL/CRC COMPUTER AND INFORMATION SCIENCE SERIES', 'Robertson S, 1988, TAYLOR GRAHAM PUBLISHING EBOOKS', 'Riloff E, 1995, ', 'Ruiz M, 1999, ACM SIGIR FORUM', 'Moulinier I, 1996, ', 'Sebastiani F, 2000, ', 'Denoyer L, 2001, ', 'Tauritz D, 2000, INFORMATION SCIENCES', 'Ignatow G, 2017, ', 'Kessler B, 1997, ARXIV.ORG', 'Dagan I, 1997, ARXIV (CORNELL UNIVERSITY)', 'Institute N, 2020, DEFINITIONS', 'Escudero G, 2000, ARXIV.ORG']</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>Fabrizio Sebastiani, 2002, ACM Computing Surveys</t>
-        </is>
-      </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Fabrizio Sebastiani, 2002, ACM Computing Surveys</t>
+          <t>Sebastiani F, 2002, ACM COMPUTING SURVEYS</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Sebastiani F, 2002, ACM COMPUTING SURVEYS</t>
         </is>
       </c>
     </row>
@@ -2211,28 +2296,33 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1534707631', 'https://openalex.org/W1573640198', 'https://openalex.org/W1594031697', 'https://openalex.org/W1604329830', 'https://openalex.org/W2149706766', 'https://openalex.org/W3085162807']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr">
+          <t>['Gordon A, 1984, BIOMETRICS', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Quinlan J, 1986, MACHINE LEARNING', 'Mingers J, 1989, MACHINE LEARNING', 'Quinlan J, 1989, ELSEVIER EBOOKS', 'Schaffer C, 1992, ELSEVIER EBOOKS']</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
-        </is>
-      </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
+          <t xml:space="preserve">Salzberg S, 1994, </t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salzberg S, 1994, </t>
         </is>
       </c>
     </row>
@@ -2326,20 +2416,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr">
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>NA, 2007, Kybernetes</t>
-        </is>
-      </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>NA, 2007, Kybernetes</t>
+          <t>NA, 2007, KYBERNETES</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>NA, 2007, KYBERNETES</t>
         </is>
       </c>
     </row>
@@ -2417,28 +2512,33 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1442374986', 'https://openalex.org/W1484210532', 'https://openalex.org/W1487337216', 'https://openalex.org/W1498436455', 'https://openalex.org/W1526734559', 'https://openalex.org/W1548328233', 'https://openalex.org/W1598866093', 'https://openalex.org/W1614298861', 'https://openalex.org/W1658008008', 'https://openalex.org/W1667652561', 'https://openalex.org/W1738019091', 'https://openalex.org/W1827297289', 'https://openalex.org/W1869752048', 'https://openalex.org/W1947291763', 'https://openalex.org/W1978660892', 'https://openalex.org/W1978924650', 'https://openalex.org/W2002257715', 'https://openalex.org/W2016053056', 'https://openalex.org/W2017351599', 'https://openalex.org/W2032036568', 'https://openalex.org/W2035424729', 'https://openalex.org/W2055312318', 'https://openalex.org/W2064675550', 'https://openalex.org/W2082171780', 'https://openalex.org/W2097117768', 'https://openalex.org/W2100830825', 'https://openalex.org/W2123024445', 'https://openalex.org/W2130942839', 'https://openalex.org/W2131975293', 'https://openalex.org/W2138243089', 'https://openalex.org/W2141992894', 'https://openalex.org/W2146757372', 'https://openalex.org/W2155893237', 'https://openalex.org/W2160815625', 'https://openalex.org/W2168231600', 'https://openalex.org/W2171532807', 'https://openalex.org/W2181607856', 'https://openalex.org/W2253807446', 'https://openalex.org/W2507756961', 'https://openalex.org/W2949117887', 'https://openalex.org/W2950789693', 'https://openalex.org/W2951781666']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr">
+          <t>['Hochreiter S, 1997, NEURAL COMPUTATION', 'Szegedy C, 2015, ', 'Rumelhart D, 1986, NATURE', 'Jia Y, 2014, ', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Karpathy A, 2014, ', 'Zaharia M, 2012, ', 'Dean J, 2012, ', 'Isard M, 2007, ', 'Frome A, 2013, ', 'Dongarra J, 1990, ACM TRANSACTIONS ON MATHEMATICAL SOFTWARE', 'Verma A, 2015, ', 'Vinyals O, 2015, NEURAL INFORMATION PROCESSING SYSTEMS', 'Recht B, 2011, NEURAL INFORMATION PROCESSING SYSTEMS', 'Ragan‐Kelley J, 2013, ', 'Ranzato M, 2012, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Murray D, 2013, ', 'Chilimbi T, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Collobert R, 2002, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Zeiler M, 2013, ', 'Arvind A, 1990, IEEE TRANSACTIONS ON COMPUTERS', 'Yu D, 2014, ', 'Chambers C, 2010, ', 'Heigold G, 2013, ', 'Murray D, 2011, ', 'Rossbach C, 2013, ', 'Angelova A, 2015, ', 'Click C, 1995, ', 'Gónzalez-Domínguez J, 2014, NEURAL NETWORKS', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Ioffe S, 2024, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Niu F, 2011, ARXIV (CORNELL UNIVERSITY)', 'Chetlur S, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ba J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Goodfellow I, 2013, ARXIV (CORNELL UNIVERSITY)', 'Nair A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Vinyals O, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ramsundar B, 2015, ARXIV (CORNELL UNIVERSITY)', 'Le Q, 2011, ARXIV (CORNELL UNIVERSITY)', 'Maddison C, 2014, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>Martı́n Abadi, 2016, arXiv (Cornell University)-a</t>
-        </is>
-      </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Martı́n Abadi, 2016, arXiv (Cornell University)</t>
+          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)-a</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Abadi M, 2016, ARXIV (CORNELL UNIVERSITY)</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2572,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>6533</v>
+        <v>6503</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2524,28 +2624,33 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W196871588', 'https://openalex.org/W1538131130', 'https://openalex.org/W1543241987', 'https://openalex.org/W1731081199', 'https://openalex.org/W1856502440', 'https://openalex.org/W1899249567', 'https://openalex.org/W1972005403', 'https://openalex.org/W1972576201', 'https://openalex.org/W1976068300', 'https://openalex.org/W1979769287', 'https://openalex.org/W2000359198', 'https://openalex.org/W2002355073', 'https://openalex.org/W2017880874', 'https://openalex.org/W2018159038', 'https://openalex.org/W2019465613', 'https://openalex.org/W2020561998', 'https://openalex.org/W2025444507', 'https://openalex.org/W2060229389', 'https://openalex.org/W2072072671', 'https://openalex.org/W2099471712', 'https://openalex.org/W2101371964', 'https://openalex.org/W2125645174', 'https://openalex.org/W2134164499', 'https://openalex.org/W2142894919', 'https://openalex.org/W2143225719', 'https://openalex.org/W2149498546', 'https://openalex.org/W2158985775', 'https://openalex.org/W2194775991', 'https://openalex.org/W2212370034', 'https://openalex.org/W2234882433', 'https://openalex.org/W2239232218', 'https://openalex.org/W2261689926', 'https://openalex.org/W2277172374', 'https://openalex.org/W2323851192', 'https://openalex.org/W2402144811', 'https://openalex.org/W2474090883', 'https://openalex.org/W2486824498', 'https://openalex.org/W2507348356', 'https://openalex.org/W2534240011', 'https://openalex.org/W2550848904', 'https://openalex.org/W2551156993', 'https://openalex.org/W2558748708', 'https://openalex.org/W2573864470', 'https://openalex.org/W2600297185', 'https://openalex.org/W2605147767', 'https://openalex.org/W2619381903', 'https://openalex.org/W2742127985', 'https://openalex.org/W2749028154', 'https://openalex.org/W2777417212', 'https://openalex.org/W2783378529', 'https://openalex.org/W2786232134', 'https://openalex.org/W2787931125', 'https://openalex.org/W2803629276', 'https://openalex.org/W2809090039', 'https://openalex.org/W2810026216', 'https://openalex.org/W2811199191', 'https://openalex.org/W2856628251', 'https://openalex.org/W2884775584', 'https://openalex.org/W2886802770', 'https://openalex.org/W2887569307', 'https://openalex.org/W2890889625', 'https://openalex.org/W2890968382', 'https://openalex.org/W2893749619', 'https://openalex.org/W2893813411', 'https://openalex.org/W2896549049', 'https://openalex.org/W2897097528', 'https://openalex.org/W2899283552', 'https://openalex.org/W2899971035', 'https://openalex.org/W2900369848', 'https://openalex.org/W2901203181', 'https://openalex.org/W2907047316', 'https://openalex.org/W2908541468', 'https://openalex.org/W2909320927', 'https://openalex.org/W2912389156', 'https://openalex.org/W2912465314', 'https://openalex.org/W2912649832', 'https://openalex.org/W2913323966', 'https://openalex.org/W2914483840', 'https://openalex.org/W2914520121', 'https://openalex.org/W2919958648', 'https://openalex.org/W2936357167', 'https://openalex.org/W2945102878', 'https://openalex.org/W2946794331', 'https://openalex.org/W2946866513', 'https://openalex.org/W2947072793', 'https://openalex.org/W2951392159', 'https://openalex.org/W2952046647', 'https://openalex.org/W2959995783', 'https://openalex.org/W2962793481', 'https://openalex.org/W2963021886', 'https://openalex.org/W2963063862', 'https://openalex.org/W2963095610', 'https://openalex.org/W2963190151', 'https://openalex.org/W2963518130', 'https://openalex.org/W2963634130', 'https://openalex.org/W2963716063', 'https://openalex.org/W2963755523', 'https://openalex.org/W2963901342', 'https://openalex.org/W2964059111', 'https://openalex.org/W2964088238', 'https://openalex.org/W2964121744', 'https://openalex.org/W2964135722', 'https://openalex.org/W2964212578', 'https://openalex.org/W2964268978', 'https://openalex.org/W2966284335', 'https://openalex.org/W2969381807', 'https://openalex.org/W2970100546', 'https://openalex.org/W2970971581', 'https://openalex.org/W2971095480', 'https://openalex.org/W2971343405', 'https://openalex.org/W2972153210', 'https://openalex.org/W2973886134', 'https://openalex.org/W2975003945', 'https://openalex.org/W2977109506', 'https://openalex.org/W2978281981', 'https://openalex.org/W2979712029', 'https://openalex.org/W2979786244', 'https://openalex.org/W2980147119', 'https://openalex.org/W2980592884', 'https://openalex.org/W2980973551', 'https://openalex.org/W2983902802', 'https://openalex.org/W2991298115', 'https://openalex.org/W2991550674', 'https://openalex.org/W2994626356', 'https://openalex.org/W2994747787', 'https://openalex.org/W2997814214', 'https://openalex.org/W2999026783', 'https://openalex.org/W2999467285', 'https://openalex.org/W3003747211', 'https://openalex.org/W3003922491', 'https://openalex.org/W3004450693', 'https://openalex.org/W3005610174', 'https://openalex.org/W3007470329', 'https://openalex.org/W3007740214', 'https://openalex.org/W3008453832', 'https://openalex.org/W3009784374', 'https://openalex.org/W3010849941', 'https://openalex.org/W3011147100', 'https://openalex.org/W3011806874', 'https://openalex.org/W3012417314', 'https://openalex.org/W3012621877', 'https://openalex.org/W3014009018', 'https://openalex.org/W3014468003', 'https://openalex.org/W3015176898', 'https://openalex.org/W3015606043', 'https://openalex.org/W3015865829', 'https://openalex.org/W3016703299', 'https://openalex.org/W3022657828', 'https://openalex.org/W3023982288', 'https://openalex.org/W3025645353', 'https://openalex.org/W3026222427', 'https://openalex.org/W3028316595', 'https://openalex.org/W3028529071', 'https://openalex.org/W3035493266', 'https://openalex.org/W3036843665', 'https://openalex.org/W3037090957', 'https://openalex.org/W3039304986', 'https://openalex.org/W3040277050', 'https://openalex.org/W3041984619', 'https://openalex.org/W3043174105', 'https://openalex.org/W3043516796', 'https://openalex.org/W3045146186', 'https://openalex.org/W3046173836', 'https://openalex.org/W3047001618', 'https://openalex.org/W3048241795', 'https://openalex.org/W3049075514', 'https://openalex.org/W3080393992', 'https://openalex.org/W3081814969', 'https://openalex.org/W3082908155', 'https://openalex.org/W3082977546', 'https://openalex.org/W3084017095', 'https://openalex.org/W3088681382', 'https://openalex.org/W3088691598', 'https://openalex.org/W3088877001', 'https://openalex.org/W3093018961', 'https://openalex.org/W3093190107', 'https://openalex.org/W3093786597', 'https://openalex.org/W3093990252', 'https://openalex.org/W3096173239', 'https://openalex.org/W3096732413', 'https://openalex.org/W3098172061', 'https://openalex.org/W3098195931', 'https://openalex.org/W3098370560', 'https://openalex.org/W3098546160', 'https://openalex.org/W3098951945', 'https://openalex.org/W3099849883', 'https://openalex.org/W3100156752', 'https://openalex.org/W3101260193', 'https://openalex.org/W3101396145', 'https://openalex.org/W3102139197', 'https://openalex.org/W3102569296', 'https://openalex.org/W3102697518', 'https://openalex.org/W3102845444', 'https://openalex.org/W3102921872', 'https://openalex.org/W3103242287', 'https://openalex.org/W3104150464', 'https://openalex.org/W3104873019', 'https://openalex.org/W3105982350', 'https://openalex.org/W3106050203', 'https://openalex.org/W3107691001', 'https://openalex.org/W3107973042', 'https://openalex.org/W3112233611', 'https://openalex.org/W3112264320', 'https://openalex.org/W3116268267', 'https://openalex.org/W3118310857', 'https://openalex.org/W3125167458', 'https://openalex.org/W3128400532', 'https://openalex.org/W3129530645', 'https://openalex.org/W3129610195', 'https://openalex.org/W3132277775', 'https://openalex.org/W3133338006', 'https://openalex.org/W3133608513', 'https://openalex.org/W3137240924', 'https://openalex.org/W3137474564', 'https://openalex.org/W3138463430', 'https://openalex.org/W3145000844', 'https://openalex.org/W3148629269', 'https://openalex.org/W3168386838', 'https://openalex.org/W3181271387', 'https://openalex.org/W3201460085', 'https://openalex.org/W3207890637', 'https://openalex.org/W4230953281', 'https://openalex.org/W4234008654', 'https://openalex.org/W6694756022', 'https://openalex.org/W6713134421', 'https://openalex.org/W6755308174', 'https://openalex.org/W6763197053', 'https://openalex.org/W6787451610']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr">
+          <t>['He K, 2016, ', 'Plimpton S, 1995, JOURNAL OF COMPUTATIONAL PHYSICS', '淳司 柴, 2017, JOURNAL OF JAPAN SOCIETY FOR FUZZY THEORY AND INTELLIGENT INFORMATICS', 'Ganin Y, 2017, ADVANCES IN COMPUTER VISION AND PATTERN RECOGNITION', 'Abadi M, 2016, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Byrd R, 1995, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Behler J, 2007, PHYSICAL REVIEW LETTERS', 'Xiu D, 2002, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Brunton S, 2016, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'LeCun Y, 1998, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Bronstein M, 2017, IEEE SIGNAL PROCESSING MAGAZINE', 'Schmidt M, 2009, SCIENCE', 'Lagaris I, 1998, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Zhang L, 2018, PHYSICAL REVIEW LETTERS', 'Sirignano J, 2018, JOURNAL OF COMPUTATIONAL PHYSICS', 'Alnæs M, 2015, DEPARTMENT OF EARTH SCIENCES EPRINTS REPOSITORY', 'Stuart A, 2010, ACTA NUMERICA', 'Rackauckas C, 2017, JOURNAL OF OPEN RESEARCH SOFTWARE', 'Bruna J, 2013, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Ling J, 2016, JOURNAL OF FLUID MECHANICS', 'Lusch B, 2018, NATURE COMMUNICATIONS', 'Kimeldorf G, 1970, THE ANNALS OF MATHEMATICAL STATISTICS', 'Hart J, 2006, EARTH-SCIENCE REVIEWS', 'Jasak H, 2007, ', 'Hachmann J, 2011, THE JOURNAL OF PHYSICAL CHEMISTRY LETTERS', 'Mallat S, 2016, PHILOSOPHICAL TRANSACTIONS OF THE ROYAL SOCIETY A MATHEMATICAL PHYSICAL AND ENGINEERING SCIENCES', 'Weinan E, 2017, COMMUNICATIONS IN MATHEMATICS AND STATISTICS', 'Raissi M, 2017, JOURNAL OF COMPUTATIONAL PHYSICS', 'Poggio T, 2017, INTERNATIONAL JOURNAL OF AUTOMATION AND COMPUTING', 'Blum A, 1992, NEURAL NETWORKS', 'Marzouk Y, 2006, JOURNAL OF COMPUTATIONAL PHYSICS', 'Lee J, 2016, CONFERENCE ON LEARNING THEORY', 'Micchelli C, 1977, ', 'Raissi M, 2017, JOURNAL OF COMPUTATIONAL PHYSICS', 'Raissi M, 2018, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'González‐García R, 1998, COMPUTERS &amp; CHEMICAL ENGINEERING', 'Diaconis P, 1988, ', 'Owhadi H, 2015, MULTISCALE MODELING AND SIMULATION', 'Stoudenmire E, 2016, NEURAL INFORMATION PROCESSING SYSTEMS', 'Owhadi H, 2006, COMMUNICATIONS ON PURE AND APPLIED MATHEMATICS', 'McFall K, 2009, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Rico-Martı́nez R, 1992, CHEMICAL ENGINEERING COMMUNICATIONS', 'Larkin F, 1972, ROCKY MOUNTAIN JOURNAL OF MATHEMATICS', 'Beidokhti R, 2009, JOURNAL OF THE FRANKLIN INSTITUTE', 'Rovelli C, 2011, FOUNDATIONS OF PHYSICS', 'Rico-Martı́nez R, 2002, ', 'Reisert M, 2007, ', 'Choromanska A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Kondor R, 2018, ARXIV (CORNELL UNIVERSITY)', 'Kadri H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Zhu J, 2017, ', 'Raissi M, 2018, JOURNAL OF COMPUTATIONAL PHYSICS', 'Reichstein M, 2019, NATURE', 'Han J, 2018, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Belkin M, 2019, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Zhu Y, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Bianco S, 2018, IEEE ACCESS', 'Meng X, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Mei S, 2018, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Zhang D, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Xu Z, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Iten R, 2020, PHYSICAL REVIEW LETTERS', 'Tripathy R, 2018, JOURNAL OF COMPUTATIONAL PHYSICS', 'Yang Y, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Geneva N, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Pun G, 2019, NATURE COMMUNICATIONS', 'Kurth T, 2018, ', 'Gardner J, 2018, NEURAL INFORMATION PROCESSING SYSTEMS', 'Poole B, 2016, ARXIV (CORNELL UNIVERSITY)', 'Frostig R, 2018, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Reddy D, 2018, MODELING EARTH SYSTEMS AND ENVIRONMENT', 'Geiger M, 2020, JOURNAL OF STATISTICAL MECHANICS THEORY AND EXPERIMENT', 'Wu J, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Karumuri S, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Grohs P, 2023, MEMOIRS OF THE AMERICAN MATHEMATICAL SOCIETY', 'He J, 2020, JOURNAL OF COMPUTATIONAL MATHEMATICS', 'Geiger M, 2019, PHYSICAL REVIEW. E', 'He J, 2019, SCIENCE CHINA MATHEMATICS', 'Winovich N, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Owhadi H, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Pang G, 2019, JOURNAL OF COMPUTATIONAL PHYSICS', 'Hy T, 2018, THE JOURNAL OF CHEMICAL PHYSICS', 'Spigler S, 2019, JOURNAL OF PHYSICS A MATHEMATICAL AND THEORETICAL', 'Yang Y, 2019, COMPUTATIONAL MECHANICS', 'Yang G, 2017, NEURAL INFORMATION PROCESSING SYSTEMS', 'Kemeth F, 2018, IEEE ACCESS', 'Tai K, 2019, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Winkens J, 2018, ', 'Huang D, 2019, ARXIV (CORNELL UNIVERSITY)', 'Gal Y, 2015, ARXIV (CORNELL UNIVERSITY)', 'Brock A, 2018, ARXIV (CORNELL UNIVERSITY)', 'Jacot A, 2018, ARXIV (CORNELL UNIVERSITY)', 'Cohen T, 2019, ARXIV (CORNELL UNIVERSITY)', 'Rahaman N, 2018, ARXIV (CORNELL UNIVERSITY)', 'Erichson N, 2019, ARXIV (CORNELL UNIVERSITY)', 'Mattheakis M, 2019, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2019, ARXIV (CORNELL UNIVERSITY)', 'Kuan-Lin C, 2021, DROPS (SCHLOSS DAGSTUHL – LEIBNIZ CENTER FOR INFORMATICS)', 'Lu L, 2021, NATURE MACHINE INTELLIGENCE', 'Yu L, 2017, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Raissi M, 2020, SCIENCE', 'He X, 2020, KNOWLEDGE-BASED SYSTEMS', 'Jagtap A, 2020, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Yang L, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Newman D, 1998, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Elsken T, 2019, ARXIV (CORNELL UNIVERSITY)', 'Kharazmi E, 2020, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Kissas G, 2019, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Alber M, 2019, NPJ DIGITAL MEDICINE', 'Tartakovsky A, 2020, WATER RESOURCES RESEARCH', 'Pfau D, 2020, PHYSICAL REVIEW RESEARCH', 'Yang L, 2020, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Haghighat E, 2020, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Lu L, 2020, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Zhang D, 2020, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Hospedales T, 2021, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Jagtap A, 2020, PROCEEDINGS OF THE ROYAL SOCIETY A MATHEMATICAL PHYSICAL AND ENGINEERING SCIENCES', 'Wang W, 2019, NPJ COMPUTATIONAL MATERIALS', 'Xu K, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Sheng H, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Nakata A, 2020, THE JOURNAL OF CHEMICAL PHYSICS', 'Chen F, 2020, THE JOURNAL OF OPEN SOURCE SOFTWARE', 'Owhadi H, 2019, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Fan D, 2019, SCIENCE ROBOTICS', 'Darbon J, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Basri R, 2019, ARXIV (CORNELL UNIVERSITY)', 'Novak R, 2020, INTERNATIONAL CONFERENCE ON LEARNING REPRESENTATIONS', 'Jia J, 2019, ARXIV (CORNELL UNIVERSITY)', 'Jo H, 2020, NETWORKS AND HETEROGENEOUS MEDIA', 'Tsai Y, 2019, ', 'Owhadi H, 2019, NOTICES OF THE AMERICAN MATHEMATICAL SOCIETY', 'Bettencourt J, 2019, ', 'Paszke A, 2019, ARXIV (CORNELL UNIVERSITY)', 'Rackauckas C, 2020, RESEARCH SQUARE', 'Kharazmi E, 2019, ARXIV (CORNELL UNIVERSITY)', 'Wang S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Jia X, 2020, ARXIV (CORNELL UNIVERSITY)', 'Koryagin A, 2019, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2019, ARXIV (CORNELL UNIVERSITY)', 'Kunitski M, 2019, GSI REPOSITORY (GERMAN FEDERAL GOVERNMENT)', 'Lagaris I, 1998, ', 'Jagtap A, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'N. K, 2019, REPEC: RESEARCH PAPERS IN ECONOMICS', 'Kashefi A, 2021, PHYSICS OF FLUIDS', 'Shin Y, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Jin P, 2020, NEURAL NETWORKS', 'Liu Z, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Dong S, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Sirignano J, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Tancik M, 2020, NEURAL INFORMATION PROCESSING SYSTEMS', 'Mu S, 2019, UNIVERSITY OF REGENSBURG PUBLICATION SERVER (UNIVERSITY OF REGENSBURG)', 'Wang S, 2020, JOURNAL OF COMPUTATIONAL PHYSICS', 'Mathews A, 2021, PHYSICAL REVIEW. E', 'Cai W, 2020, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Li D, 2020, WATER RESOURCES RESEARCH', 'Reyes B, 2021, PHYSICAL REVIEW FLUIDS', 'Lagari P, 2020, INTERNATIONAL JOURNAL OF ARTIFICIAL INTELLIGENCE TOOLS', 'Wang B, 2020, COMMUNICATIONS IN COMPUTATIONAL PHYSICS', 'Li Z, 2020, CALTECHAUTHORS (CALIFORNIA INSTITUTE OF TECHNOLOGY)', 'Arbabi H, 2020, JOM', 'Guo M, 2022, JOURNAL OF ENGINEERING MECHANICS', 'Nelsen N, 2021, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Mishra S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Tancik M, 2020, ARXIV (CORNELL UNIVERSITY)', 'Pun G, , REPEC: RESEARCH PAPERS IN ECONOMICS', 'Wujie W, 2019, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)', 'Wang S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Wight C, 2020, ARXIV (CORNELL UNIVERSITY)', 'Mishra S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Mao Z, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Owhadi H, 2020, CALTECHAUTHORS (CALIFORNIA INSTITUTE OF TECHNOLOGY)', 'Pfrommer S, 2020, ARXIV (CORNELL UNIVERSITY)', 'Rotskoff G, 2020, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2020, ARXIV (CORNELL UNIVERSITY)', 'Lee J, 2020, ARXIV (CORNELL UNIVERSITY)', 'Wang S, 2021, COMPUTER METHODS IN APPLIED MECHANICS AND ENGINEERING', 'Cai S, 2021, JOURNAL OF FLUID MECHANICS', 'Sard A, 1963, MATHEMATICAL SURVEYS AND MONOGRAPHS', 'Jia W, 2020, ', 'Li Z, 2021, CALTECHAUTHORS (CALIFORNIA INSTITUTE OF TECHNOLOGY)', 'Cai S, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', ', 2017, AUERBACH PUBLICATIONS EBOOKS', 'Lanthaler S, 2022, TRANSACTIONS OF MATHEMATICS AND ITS APPLICATIONS', 'Hennigh O, 2021, LECTURE NOTES IN COMPUTER SCIENCE', 'Patel R, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Mao Z, 2021, JOURNAL OF COMPUTATIONAL PHYSICS', 'Hamzi B, 2021, PHYSICA D NONLINEAR PHENOMENA', 'Yang Y, 2020, PROCEEDINGS OF THE ROYAL SOCIETY A MATHEMATICAL PHYSICAL AND ENGINEERING SCIENCES', 'Yang L, 2022, SIAM JOURNAL ON SCIENTIFIC COMPUTING', 'Manickam I, 2021, ', 'Zhu W, 2020, AGU FALL MEETING ABSTRACTS', 'Hennigh O, 2020, ARXIV (CORNELL UNIVERSITY)', 'Deng B, 2021, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
-        </is>
-      </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
+          <t>Karniadakis G, 2021, NATURE REVIEWS PHYSICS</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Karniadakis G, 2021, NATURE REVIEWS PHYSICS</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2684,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>7843</v>
+        <v>7839</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2631,28 +2736,33 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W195465510', 'https://openalex.org/W1482451543', 'https://openalex.org/W1553313034', 'https://openalex.org/W1578772208', 'https://openalex.org/W1605688901', 'https://openalex.org/W1676820704', 'https://openalex.org/W1970074386', 'https://openalex.org/W1988790447', 'https://openalex.org/W1991418450', 'https://openalex.org/W2019778169', 'https://openalex.org/W2027197837', 'https://openalex.org/W2032210760', 'https://openalex.org/W2037699108', 'https://openalex.org/W2042614373', 'https://openalex.org/W2098191394', 'https://openalex.org/W2112076978', 'https://openalex.org/W2135293965', 'https://openalex.org/W2148520070', 'https://openalex.org/W2152761983', 'https://openalex.org/W2912934387', 'https://openalex.org/W2914859268', 'https://openalex.org/W4212774754', 'https://openalex.org/W4242746271', 'https://openalex.org/W6676769703', 'https://openalex.org/W6808111085']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr">
+          <t>['Freund Y, 1997, JOURNAL OF COMPUTER AND SYSTEM SCIENCES', 'Breiman L, 1996, MACHINE LEARNING', ', 1996, COMPUTERS &amp; MATHEMATICS WITH APPLICATIONS', 'Freund Y, 1996, ', 'Hansen L, 1990, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Dietterich T, 2000, MACHINE LEARNING', 'Dietterich T, 1995, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Bauer E, 1999, MACHINE LEARNING', 'Schapire R, 1998, ', 'Hornik K, 1990, NEURAL NETWORKS', 'Neal R, 2011, ', 'Hyafil L, 1976, INFORMATION PROCESSING LETTERS', 'Tumer K, 1996, CONNECTION SCIENCE', 'Schapire R, 1997, QUT EPRINTS (QUEENSLAND UNIVERSITY OF TECHNOLOGY)', 'Fisher D, 1997, ', 'Kolen J, 1990, ', 'Schapire R, 1997, ', 'Ali K, 1994, MACHINE LEARNING', 'Raviv Y, 1996, CONNECTION SCIENCE', 'Ali K, 1996, MACHINE LEARNING', 'Kwok S, 1990, MACHINE INTELLIGENCE AND PATTERN RECOGNITION', 'Parmanto B, 1995, ']</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>Thomas G. Dietterich, 2000, Lecture notes in computer science</t>
-        </is>
-      </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Thomas G. Dietterich, 2000, Lecture notes in computer science</t>
+          <t>Dietterich T, 2000, LECTURE NOTES IN COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Dietterich T, 2000, LECTURE NOTES IN COMPUTER SCIENCE</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2796,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>4433</v>
+        <v>4429</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -2742,28 +2852,33 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W51943945', 'https://openalex.org/W118877790', 'https://openalex.org/W199424061', 'https://openalex.org/W882068046', 'https://openalex.org/W999198455', 'https://openalex.org/W1479793620', 'https://openalex.org/W1492999010', 'https://openalex.org/W1503870031', 'https://openalex.org/W1529944915', 'https://openalex.org/W1534582174', 'https://openalex.org/W1559984405', 'https://openalex.org/W1568345435', 'https://openalex.org/W1631356911', 'https://openalex.org/W1684389741', 'https://openalex.org/W1703581136', 'https://openalex.org/W1743210689', 'https://openalex.org/W1872619987', 'https://openalex.org/W1965702053', 'https://openalex.org/W1968390152', 'https://openalex.org/W1968561119', 'https://openalex.org/W1979692035', 'https://openalex.org/W1980314119', 'https://openalex.org/W1981783889', 'https://openalex.org/W1983561139', 'https://openalex.org/W1988369744', 'https://openalex.org/W1994630055', 'https://openalex.org/W2001157051', 'https://openalex.org/W2010505240', 'https://openalex.org/W2015811642', 'https://openalex.org/W2019658260', 'https://openalex.org/W2021276590', 'https://openalex.org/W2022786335', 'https://openalex.org/W2028918948', 'https://openalex.org/W2030545386', 'https://openalex.org/W2035551859', 'https://openalex.org/W2040792108', 'https://openalex.org/W2040870580', 'https://openalex.org/W2041506125', 'https://openalex.org/W2042127289', 'https://openalex.org/W2046481556', 'https://openalex.org/W2051446825', 'https://openalex.org/W2055784634', 'https://openalex.org/W2064517571', 'https://openalex.org/W2069563009', 'https://openalex.org/W2075236172', 'https://openalex.org/W2086236885', 'https://openalex.org/W2097981279', 'https://openalex.org/W2101403221', 'https://openalex.org/W2103956991', 'https://openalex.org/W2104944940', 'https://openalex.org/W2106090814', 'https://openalex.org/W2110322033', 'https://openalex.org/W2120480077', 'https://openalex.org/W2120802379', 'https://openalex.org/W2124269824', 'https://openalex.org/W2153346333', 'https://openalex.org/W2153887174', 'https://openalex.org/W2155728415', 'https://openalex.org/W2156909104', 'https://openalex.org/W2170504083', 'https://openalex.org/W2188879252', 'https://openalex.org/W2195198640', 'https://openalex.org/W2207520826', 'https://openalex.org/W2207698480', 'https://openalex.org/W2221147613', 'https://openalex.org/W2262683142', 'https://openalex.org/W2266138411', 'https://openalex.org/W2272691542', 'https://openalex.org/W2306477081', 'https://openalex.org/W2327049932', 'https://openalex.org/W2334150129', 'https://openalex.org/W2337082154', 'https://openalex.org/W2341702711', 'https://openalex.org/W2397157153', 'https://openalex.org/W2409645286', 'https://openalex.org/W2419175238', 'https://openalex.org/W2468412683', 'https://openalex.org/W2478948476', 'https://openalex.org/W2489886790', 'https://openalex.org/W2490964415', 'https://openalex.org/W2495424399', 'https://openalex.org/W2516533688', 'https://openalex.org/W2517233404', 'https://openalex.org/W2521267242', 'https://openalex.org/W2528744766', 'https://openalex.org/W2557392572', 'https://openalex.org/W2560386163', 'https://openalex.org/W2571629069', 'https://openalex.org/W2579928628', 'https://openalex.org/W2580674237', 'https://openalex.org/W2582909346', 'https://openalex.org/W2595654587', 'https://openalex.org/W2604642811', 'https://openalex.org/W2607911764', 'https://openalex.org/W2612799626', 'https://openalex.org/W2751668559', 'https://openalex.org/W2764347725', 'https://openalex.org/W2766518897', 'https://openalex.org/W2768556639', 'https://openalex.org/W2919115771', 'https://openalex.org/W2949537205', 'https://openalex.org/W2951663210', 'https://openalex.org/W2952050628', 'https://openalex.org/W2962688653', 'https://openalex.org/W2962821153', 'https://openalex.org/W2962954040', 'https://openalex.org/W2963060324', 'https://openalex.org/W2963331258', 'https://openalex.org/W2963614945', 'https://openalex.org/W2963762919', 'https://openalex.org/W2964039664', 'https://openalex.org/W3022610800', 'https://openalex.org/W3023478445', 'https://openalex.org/W3098126014', 'https://openalex.org/W3098768946', 'https://openalex.org/W3098965398', 'https://openalex.org/W3099695580', 'https://openalex.org/W3100863707', 'https://openalex.org/W3101664568', 'https://openalex.org/W3102047485', 'https://openalex.org/W3103372543', 'https://openalex.org/W3104450852', 'https://openalex.org/W3104599990', 'https://openalex.org/W3105377867', 'https://openalex.org/W3106418633', 'https://openalex.org/W3111297213', 'https://openalex.org/W4230674625', 'https://openalex.org/W4297801632', 'https://openalex.org/W4301805094', 'https://openalex.org/W6687462962']</t>
+          <t>['RU', 'ES', 'DE', 'US']</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr">
+          <t>['Nielsen M, 2002, AMERICAN JOURNAL OF PHYSICS', 'Rosenblatt F, 1958, PSYCHOLOGICAL REVIEW', 'Harrow A, 2009, PHYSICAL REVIEW LETTERS', 'Lloyd S, 1996, SCIENCE', 'Rebentrost P, 2014, PHYSICAL REVIEW LETTERS', 'Lloyd S, 2014, NATURE PHYSICS', 'Schuld M, 2014, CONTEMPORARY PHYSICS', 'Giovannetti V, 2008, PHYSICAL REVIEW LETTERS', 'Brunner D, 2013, NATURE COMMUNICATIONS', 'Rønnow T, 2014, SCIENCE', 'Wiebe N, 2012, PHYSICAL REVIEW LETTERS', 'Aaronson S, 2015, NATURE PHYSICS', 'Wittek P, 2014, ', 'Temme K, 2011, NATURE', 'Dolde F, 2014, NATURE COMMUNICATIONS', 'Clader B, 2013, PHYSICAL REVIEW LETTERS', 'Ventura D, 2000, INFORMATION SCIENCES', 'Li Z, 2015, PHYSICAL REVIEW LETTERS', 'Wiebe N, 2014, PHYSICAL REVIEW LETTERS', 'Zeidler D, 2001, PHYSICAL REVIEW A', 'Cai X, 2015, PHYSICAL REVIEW LETTERS', 'Paparo G, 2014, PHYSICAL REVIEW X', 'Hentschel A, 2010, PHYSICAL REVIEW LETTERS', 'Biamonte J, 2008, PHYSICAL REVIEW A', 'Bisio A, 2010, PHYSICAL REVIEW A', 'Zahedinejad E, 2015, PHYSICAL REVIEW LETTERS', 'Low G, 2014, PHYSICAL REVIEW A', 'Anguita D, 2003, NEURAL NETWORKS', 'Lovett N, 2013, PHYSICAL REVIEW LETTERS', 'Sasaki M, 2001, PHYSICAL REVIEW A', 'Sentís G, 2012, SCIENTIFIC REPORTS', 'Whitfield J, 2012, EUROPHYSICS LETTERS (EPL)', 'Neigovzen R, 2009, PHYSICAL REVIEW A', 'Wiebe N, 2015, NEW JOURNAL OF PHYSICS', 'Karimi K, 2011, QUANTUM INFORMATION PROCESSING', 'Dunjko V, 2015, NEW JOURNAL OF PHYSICS', 'Sentís G, 2015, EPJ QUANTUM TECHNOLOGY', 'Tezak N, 2015, EPJ QUANTUM TECHNOLOGY', 'Pons M, 2007, PHYSICAL REVIEW LETTERS', 'Freitas N, 2011, ', 'Lloyd S, 2016, NEW JOURNAL OF PHYSICS', 'Amstrup B, 1995, THE JOURNAL OF PHYSICAL CHEMISTRY', 'Farhi E, 2014, ARXIV (CORNELL UNIVERSITY)', 'Lloyd S, 2013, ARXIV (CORNELL UNIVERSITY)', 'Hermans M, 2015, ARXIV (CORNELL UNIVERSITY)', 'Denchev V, 2012, ARXIV (CORNELL UNIVERSITY)', 'Denchev V, 2015, ARXIV (CORNELL UNIVERSITY)', 'Scherer A, 2015, ARXIV (CORNELL UNIVERSITY)', 'LeCun Y, 2015, NATURE', 'Vapnik V, 1995, ', 'Law J, 2001, ACM SIGSOFT SOFTWARE ENGINEERING NOTES', 'Carleo G, 2017, SCIENCE', 'Le Q, 2013, ', 'Carrasquilla J, 2017, NATURE PHYSICS', 'Dunjko V, 2016, PHYSICAL REVIEW LETTERS', 'Christoph D, 1996, ARXIV.ORG', 'Broecker P, 2017, SCIENTIFIC REPORTS', 'Schuld M, 2016, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Wan K, 2017, NPJ QUANTUM INFORMATION', 'Lloyd S, 2016, NATURE COMMUNICATIONS', 'Schuld M, 2017, EUROPHYSICS LETTERS (EPL)', 'Wossnig L, 2018, PHYSICAL REVIEW LETTERS', 'Benedetti M, 2016, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Granade C, 2012, NEW JOURNAL OF PHYSICS', 'Kieferová M, 2017, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Aı̈meur E, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Yung M, 2012, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Rebentrost P, 2018, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Arunachalam S, 2015, NEW JOURNAL OF PHYSICS', 'Zhao Z, 2019, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'Lau H, 2017, PHYSICAL REVIEW LETTERS', 'Palittapongarnpim P, 2017, NEUROCOMPUTING', 'Lamata L, 2017, SCIENTIFIC REPORTS', 'and A, 2017, QUANTUM INFORMATION AND COMPUTATION', 'Kimmel S, 2017, NPJ QUANTUM INFORMATION', 'Zahedinejad E, 2016, PHYSICAL REVIEW APPLIED', 'August M, 2017, PHYSICAL REVIEW. A/PHYSICAL REVIEW, A', 'O’Gorman B, 2015, THE EUROPEAN PHYSICAL JOURNAL SPECIAL TOPICS', 'Mavadia S, 2017, NATURE COMMUNICATIONS', 'Scherer A, 2017, QUANTUM INFORMATION PROCESSING', 'Banchi L, 2016, NPJ QUANTUM INFORMATION', 'Heras U, 2016, PHYSICAL REVIEW LETTERS', 'Alvarez-Rodriguez U, 2017, SCIENTIFIC REPORTS', 'Sentís G, 2017, ARXIV (CORNELL UNIVERSITY)', 'Monràs A, 2017, PHYSICAL REVIEW LETTERS', 'Dumoulin V, 2014, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Wittek P, 2017, SCIENTIFIC REPORTS', 'Bisio A, 2011, PHYSICS LETTERS A', 'Somma R, 2016, BULLETIN OF THE AMERICAN PHYSICAL SOCIETY', 'Palittapongarnpim P, 2016, KTH PUBLICATION DATABASE DIVA (KTH ROYAL INSTITUTE OF TECHNOLOGY)', 'Alvarez-Rodriguez U, 2016, ARXIV (CORNELL UNIVERSITY)', 'Lu D, 2017, ARXIV (CORNELL UNIVERSITY)', 'Adachi S, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kerenidis I, 2016, ARXIV (CORNELL UNIVERSITY)', 'Adcock J, 2015, ARXIV (CORNELL UNIVERSITY)', 'Marvian I, 2016, ARXIV (CORNELL UNIVERSITY)', 'Dridi R, 2015, ARXIV (CORNELL UNIVERSITY)', 'Schuld M, 2017, ARXIV (CORNELL UNIVERSITY)', 'Vapnik V, 2000, ', 'Shor P, 1997, SIAM JOURNAL ON COMPUTING', 'Schuld M, 2014, ', 'Kerenidis I, 2017, DR-NTU (NANYANG TECHNOLOGICAL UNIVERSITY)', 'Wiebe N, 2015, QUANTUM INFORMATION AND COMPUTATION', 'Wittek P, 2014, ELSEVIER EBOOKS', 'Wiebe N, 2016, NEURAL INFORMATION PROCESSING SYSTEMS', 'Banchi L, 2016, MPG.PURE (MAX PLANCK SOCIETY)', 'Tiersch M, 2015, SCIENTIFIC REPORTS', 'Unai Á, 2018, LA REFERENCIA (RED FEDERADA DE REPOSITORIOS INSTITUCIONALES DE PUBLICACIONES CIENTÍFICAS)', 'M F, 2013, OXFORD UNIVERSITY RESEARCH ARCHIVE (ORA) (UNIVERSITY OF OXFORD)', 'Chatterjee R, 2017, QUANTUM INFORMATION AND COMPUTATION', 'Seth L, 2016, RWTH PUBLICATIONS (RWTH AACHEN)', 'Kulchytskyy B, 2016, BULLETIN OF THE AMERICAN PHYSICAL SOCIETY', 'Adcock J, , BRISTOL RESEARCH (UNIVERSITY OF BRISTOL)', 'Arunachalam S, 2017, ARXIV (CORNELL UNIVERSITY)', 'Low G, 2014, DSPACE@MIT (MASSACHUSETTS INSTITUTE OF TECHNOLOGY)']</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>Jacob Biamonte, 2017, Nature</t>
-        </is>
-      </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Jacob Biamonte, 2017, Nature</t>
+          <t>Biamonte J, 2017, NATURE</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>Biamonte J, 2017, NATURE</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2912,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>5862</v>
+        <v>5851</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2853,28 +2968,33 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W150223756', 'https://openalex.org/W162878246', 'https://openalex.org/W199752024', 'https://openalex.org/W1484769234', 'https://openalex.org/W1485800369', 'https://openalex.org/W1488526968', 'https://openalex.org/W1510952750', 'https://openalex.org/W1559506103', 'https://openalex.org/W1574534563', 'https://openalex.org/W1964366273', 'https://openalex.org/W1968265138', 'https://openalex.org/W1971991172', 'https://openalex.org/W1985511977', 'https://openalex.org/W2016758618', 'https://openalex.org/W2024652123', 'https://openalex.org/W2027471022', 'https://openalex.org/W2041416246', 'https://openalex.org/W2053637704', 'https://openalex.org/W2082624086', 'https://openalex.org/W2092422002', 'https://openalex.org/W2093367651', 'https://openalex.org/W2109426455', 'https://openalex.org/W2112022568', 'https://openalex.org/W2112340198', 'https://openalex.org/W2128906841', 'https://openalex.org/W2132737349', 'https://openalex.org/W2137351756', 'https://openalex.org/W2139336600', 'https://openalex.org/W2159024459', 'https://openalex.org/W2165698076', 'https://openalex.org/W2257979135', 'https://openalex.org/W2283463896', 'https://openalex.org/W2295292576', 'https://openalex.org/W2317339301', 'https://openalex.org/W2435473771', 'https://openalex.org/W2473418344', 'https://openalex.org/W2530417694', 'https://openalex.org/W2536058570', 'https://openalex.org/W2577421826', 'https://openalex.org/W2585580772', 'https://openalex.org/W2591882872', 'https://openalex.org/W2606882085', 'https://openalex.org/W2618494520', 'https://openalex.org/W2679684481', 'https://openalex.org/W2701059868', 'https://openalex.org/W2757853533', 'https://openalex.org/W2765200655', 'https://openalex.org/W2766255512', 'https://openalex.org/W2767079719', 'https://openalex.org/W2768347741', 'https://openalex.org/W2773194476', 'https://openalex.org/W2774000609', 'https://openalex.org/W2777914285', 'https://openalex.org/W2781091734', 'https://openalex.org/W2788629937', 'https://openalex.org/W2793216106', 'https://openalex.org/W2793925626', 'https://openalex.org/W2794888826', 'https://openalex.org/W2798551148', 'https://openalex.org/W2799803467', 'https://openalex.org/W2801958627', 'https://openalex.org/W2807006176', 'https://openalex.org/W2810065831', 'https://openalex.org/W2886722183', 'https://openalex.org/W2895865029', 'https://openalex.org/W2914304175', 'https://openalex.org/W2949140995', 'https://openalex.org/W2950460048', 'https://openalex.org/W2951152347', 'https://openalex.org/W2951368041', 'https://openalex.org/W2951798842', 'https://openalex.org/W2962877476', 'https://openalex.org/W2963106566', 'https://openalex.org/W2990138404', 'https://openalex.org/W3029558105', 'https://openalex.org/W3209546151', 'https://openalex.org/W4248358572', 'https://openalex.org/W4249529812', 'https://openalex.org/W4300427714', 'https://openalex.org/W4301418013', 'https://openalex.org/W4301483968', 'https://openalex.org/W6606067566', 'https://openalex.org/W6732586565', 'https://openalex.org/W6738383168', 'https://openalex.org/W6807767519']</t>
+          <t>['HK', 'CN']</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr">
+          <t>['Pan S, 2009, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Silver D, 2016, NATURE', 'Sweeney L, 2002, INTERNATIONAL JOURNAL OF UNCERTAINTY FUZZINESS AND KNOWLEDGE-BASED SYSTEMS', 'Abadi M, 2016, ', 'Goldreich O, 1987, ', 'Bonawitz K, 2017, ', 'Dwork C, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Agrawal R, 2000, ACM SIGMOD RECORD', 'Yao A, 1982, FOUNDATIONS OF COMPUTER SCIENCE', 'Shokri R, 2015, ', 'Mohassel P, 2017, ', 'Rivest R, 1978, ', 'Dowlin N, 2016, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Hitaj B, 2017, ', 'Acar A, 2018, ACM COMPUTING SURVEYS', 'Vaidya J, 2002, ', 'Clifton C, 2010, ', 'Liu J, 2017, ', 'Bogdanov D, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Vaidya J, 2003, ', 'Ho Q, 2013, PUBMED', 'Song S, 2013, ', 'Nikolaenko V, 2013, ', 'Araki T, 2016, ', 'Du W, 2004, ', 'Du W, 2002, SYRACUSE UNIVERSITY LIBRARIES (SYRACUSE UNIVERSITY)', 'Du W, 2005, ', 'Zhang Q, 2015, IEEE TRANSACTIONS ON COMPUTERS', 'Vaidya J, 2004, ', 'Yuan J, 2013, IEEE TRANSACTIONS ON PARALLEL AND DISTRIBUTED SYSTEMS', 'Yu H, 2006, ', 'Yu H, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Scannapieco M, 2007, ', 'Aono Y, 2016, ', 'Sanil A, 2004, ', 'Karr A, 2009, ', 'Hall R, 2011, ', 'Mohassel P, 2015, ', 'Bahmani R, 2017, LECTURE NOTES IN COMPUTER SCIENCE', 'McMahan H, 2017, ', 'Vaidya J, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Wan L, 2007, ', 'Liang G, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Faltings B, 2017, SYNTHESIS LECTURES ON ARTIFICIAL INTELLIGENCE AND MACHINE LEARNING', 'Konečný J, 2016, ARXIV (CORNELL UNIVERSITY)', 'McMahan H, 2016, ARXIV (CORNELL UNIVERSITY)', 'Hesamifard E, 2017, ARXIV (CORNELL UNIVERSITY)', 'Chabanne H, 2017, IACR CRYPTOLOGY EPRINT ARCHIVE', 'Smith V, 2017, ARXIV (CORNELL UNIVERSITY)', ', 2007, THE MIT PRESS EBOOKS', 'Leen T, 2000, ', 'Agrawal R, 2000, ', 'Phong L, 2017, IEEE TRANSACTIONS ON INFORMATION FORENSICS AND SECURITY', 'Mohassel P, 2018, ', 'Riazi M, 2018, ', 'Bourse F, 2018, LECTURE NOTES IN COMPUTER SCIENCE', 'Kim M, 2018, JMIR MEDICAL INFORMATICS', 'Wang S, 2018, ', 'Rouhani B, 2018, 2018 55TH ACM/ESDA/IEEE DESIGN AUTOMATION CONFERENCE (DAC)', 'Kim H, 2018, ', 'Melis L, 2018, ARXIV (CORNELL UNIVERSITY)', 'Chen F, 2018, ', 'Cheng Y, 2019, ', 'Bourse F, 2018, IACR CRYPTOLOGY EPRINT ARCHIVE', 'Faltings B, 2017, SYNTHESIS LECTURES ON ARTIFICIAL INTELLIGENCE AND MACHINE LEARNING', 'Zhao Y, 2018, ARXIV (CORNELL UNIVERSITY)', 'Dariusz W, 2019, SGEM INTERNATIONAL MULTIDISCIPLINARY SCIENTIFIC CONFERENCES ON SOCIAL SCIENCES AND ARTS', 'Bagdasaryan E, 2018, ARXIV (CORNELL UNIVERSITY)', 'Lin Y, 2017, ARXIV (CORNELL UNIVERSITY)', 'Geyer R, 2017, ARXIV (CORNELL UNIVERSITY)', 'Hardy S, 2017, ARXIV (CORNELL UNIVERSITY)', 'Hitaj B, 2017, ARXIV (CORNELL UNIVERSITY)', 'Gascón A, 2016, IACR CRYPTOLOGY EPRINT ARCHIVE', ', 1999, ', 'Nock R, 2018, ARXIV (CORNELL UNIVERSITY)', 'Kilbertus N, 2025, WARWICK RESEARCH ARCHIVE PORTAL (UNIVERSITY OF WARWICK)', 'Su L, 2018, ARXIV (CORNELL UNIVERSITY)', 'Giacomelli I, 2017, IACR CRYPTOLOGY EPRINT ARCHIVE']</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>Qiang Yang, 2019, ACM Transactions on Intelligent Systems and Technology</t>
-        </is>
-      </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Qiang Yang, 2019, ACM Transactions on Intelligent Systems and Technology</t>
+          <t>Yang Q, 2019, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>Yang Q, 2019, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY</t>
         </is>
       </c>
     </row>
@@ -2960,28 +3080,33 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W104184427', 'https://openalex.org/W145476170', 'https://openalex.org/W1425731158', 'https://openalex.org/W1442374986', 'https://openalex.org/W1485981043', 'https://openalex.org/W1493893823', 'https://openalex.org/W1498436455', 'https://openalex.org/W1526734559', 'https://openalex.org/W1539309091', 'https://openalex.org/W1548328233', 'https://openalex.org/W1598866093', 'https://openalex.org/W1658008008', 'https://openalex.org/W1667652561', 'https://openalex.org/W1815076433', 'https://openalex.org/W1947291763', 'https://openalex.org/W1978660892', 'https://openalex.org/W2016053056', 'https://openalex.org/W2032036568', 'https://openalex.org/W2035424729', 'https://openalex.org/W2041517243', 'https://openalex.org/W2061570747', 'https://openalex.org/W2064675550', 'https://openalex.org/W2066443755', 'https://openalex.org/W2083842231', 'https://openalex.org/W2097117768', 'https://openalex.org/W2100664567', 'https://openalex.org/W2100830825', 'https://openalex.org/W2117539524', 'https://openalex.org/W2122465391', 'https://openalex.org/W2131975293', 'https://openalex.org/W2132339004', 'https://openalex.org/W2140833774', 'https://openalex.org/W2141992894', 'https://openalex.org/W2145339207', 'https://openalex.org/W2146502635', 'https://openalex.org/W2146757372', 'https://openalex.org/W2147527908', 'https://openalex.org/W2160815625', 'https://openalex.org/W2168231600', 'https://openalex.org/W2172654076', 'https://openalex.org/W2186615578', 'https://openalex.org/W2194775991', 'https://openalex.org/W2253807446', 'https://openalex.org/W2259472270', 'https://openalex.org/W2336650964', 'https://openalex.org/W2339765813', 'https://openalex.org/W2384495648', 'https://openalex.org/W2521218765', 'https://openalex.org/W2525778437', 'https://openalex.org/W2618530766', 'https://openalex.org/W2949117887', 'https://openalex.org/W2949888546', 'https://openalex.org/W2950577311', 'https://openalex.org/W2951781666', 'https://openalex.org/W2962844195']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr">
+          <t>['He K, 2016, ', 'Hochreiter S, 1997, NEURAL COMPUTATION', 'Szegedy C, 2015, ', 'Russakovsky O, 2015, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Rumelhart D, 1986, NATURE', 'Mnih V, 2015, NATURE', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Duchi J, 2010, ', 'Karpathy A, 2014, ', 'Zaharia M, 2012, ', 'Sutskever I, 2013, ', 'Dayalan M, 2018, INTERNATIONAL JOURNAL OF RESEARCH AND ENGINEERING', 'Dean J, 2012, ', 'Isard M, 2007, ', ', 2000, APPLIED PHYSICS LETTERS', 'Sifis L, 2016, ARXIV (CORNELL UNIVERSITY)', 'Verma A, 2015, ', 'Jordan M, 1997, ADVANCES IN PSYCHOLOGY', 'Larochelle H, 2009, ', 'Li M, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Lavin A, 2016, ', 'Jean S, 2015, ', 'Hinton G, 1989, ESCHOLARSHIP (CALIFORNIA DIGITAL LIBRARY)', 'Yu Y, 2008, ', 'Ranzato M, 2012, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Chilimbi T, 2014, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION', 'Collobert R, 2002, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Smola A, 2010, PROCEEDINGS OF THE VLDB ENDOWMENT', 'Zeiler M, 2013, ', 'Byrd R, 2012, MATHEMATICAL PROGRAMMING', 'Cui H, 2016, ', 'Heigold G, 2013, ', 'McSherry F, 2015, ', 'Rossbach C, 2013, ', 'Chung E, 2013, ', 'Chelba C, 2014, ', 'Angelova A, 2015, ', 'Gónzalez-Domínguez J, 2014, NEURAL NETWORKS', 'Murray D, 2016, COMMUNICATIONS OF THE ACM', 'Wu Y, 2016, ARXIV (CORNELL UNIVERSITY)', 'Pascanu R, 2012, ARXIV (CORNELL UNIVERSITY)', 'Chen T, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chetlur S, 2014, ARXIV (CORNELL UNIVERSITY)', 'Mnih V, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Józefowicz R, 2016, ARXIV (CORNELL UNIVERSITY)', 'Xinghao P, 2017, ARXIV (CORNELL UNIVERSITY)', 'Nair A, 2015, ARXIV (CORNELL UNIVERSITY)', 'Maddison C, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ioffe S, 2024, ARXIV (CORNELL UNIVERSITY)', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Niu F, 2011, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>Martı́n Abadi, 2016, Operating Systems Design and Implementation</t>
-        </is>
-      </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Martı́n Abadi, 2016, Operating Systems Design and Implementation</t>
+          <t>Abadi M, 2016, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Abadi M, 2016, OPERATING SYSTEMS DESIGN AND IMPLEMENTATION</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3140,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>7225</v>
+        <v>7219</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -3071,28 +3196,33 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W102612133', 'https://openalex.org/W1479940792', 'https://openalex.org/W1488460165', 'https://openalex.org/W1489095897', 'https://openalex.org/W1515026043', 'https://openalex.org/W1533986854', 'https://openalex.org/W1541145887', 'https://openalex.org/W1587362683', 'https://openalex.org/W1588861010', 'https://openalex.org/W1594031697', 'https://openalex.org/W1623080549', 'https://openalex.org/W1704669313', 'https://openalex.org/W1770825568', 'https://openalex.org/W1784695092', 'https://openalex.org/W1967760155', 'https://openalex.org/W1969341260', 'https://openalex.org/W1969557815', 'https://openalex.org/W1983523174', 'https://openalex.org/W1989164753', 'https://openalex.org/W1995023359', 'https://openalex.org/W2002096058', 'https://openalex.org/W2026980413', 'https://openalex.org/W2049172236', 'https://openalex.org/W2050206309', 'https://openalex.org/W2060136512', 'https://openalex.org/W2102150307', 'https://openalex.org/W2110323455', 'https://openalex.org/W2116939452', 'https://openalex.org/W2117897510', 'https://openalex.org/W2125055259', 'https://openalex.org/W2135346934', 'https://openalex.org/W2145224695', 'https://openalex.org/W2157825442', 'https://openalex.org/W2322002063', 'https://openalex.org/W2766736793', 'https://openalex.org/W2921629193', 'https://openalex.org/W2988864014', 'https://openalex.org/W3015981925', 'https://openalex.org/W3085162807', 'https://openalex.org/W3137161744', 'https://openalex.org/W4233107852', 'https://openalex.org/W4254952533', 'https://openalex.org/W4300993416', 'https://openalex.org/W4400445037', 'https://openalex.org/W6629338572', 'https://openalex.org/W6632481002', 'https://openalex.org/W6635398855', 'https://openalex.org/W6642591540', 'https://openalex.org/W6650814897', 'https://openalex.org/W6676534550', 'https://openalex.org/W6682610290', 'https://openalex.org/W7020983598']</t>
+          <t>['AU']</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr">
+          <t>['Gordon A, 1984, BIOMETRICS', 'Quinlan J, 1992, ', 'Hanley J, 1982, RADIOLOGY', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Efron B, 1979, THE ANNALS OF STATISTICS', 'Fukunaga K, 1990, ELSEVIER EBOOKS', 'Green D, 1966, ', 'Ingleby J, 1967, JOURNAL OF SOUND AND VIBRATION', 'Hanley J, 1983, RADIOLOGY', 'Fukunaga K, 1990, ACADEMIC PRESS PROFESSIONAL, INC. EBOOKS', ', 2009, ', 'Devijver P, 1982, PRENTICE-HALL INTERNATIONAL EBOOKS', 'Beckman R, 1973, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Mullin A, 1963, AMERICAN MATHEMATICAL MONTHLY', 'Nguyen D, 1990, ', 'Swets J, 1982, ', 'Ziegel E, 2000, TECHNOMETRICS', 'Kavzoğlu T, 2024, ', 'Wolberg W, 1990, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Loader C, 1999, STATISCTICS AND COMPUTING/STATISTICS AND COMPUTING', 'Weiss S, 1991, ', 'Dorfman D, 1969, JOURNAL OF MATHEMATICAL PSYCHOLOGY', 'Smith J, 1988, PUBMED CENTRAL', 'Moore B, 1982, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (GENERAL)', 'Swets J, 1979, INVESTIGATIVE RADIOLOGY', 'Detrano R, 1989, THE AMERICAN JOURNAL OF CARDIOLOGY', 'Gennari J, 1989, ARTIFICIAL INTELLIGENCE', 'Robinson J, 1990, TECHNOMETRICS', 'Schaffer C, 1993, MACHINE LEARNING', 'Picinbono B, 1995, IEEE TRANSACTIONS ON AEROSPACE AND ELECTRONIC SYSTEMS', 'Ivakhnenko A, 1976, CYBERNETICS AND SYSTEMS ANALYSIS', ', 1989, CHOICE REVIEWS ONLINE', 'Schaffer C, 1993, MACHINE LEARNING', 'Friedman J, 1994, ', 'Cherkassky V, 1996, CERN DOCUMENT SERVER (EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Nelson L, 1994, JOURNAL OF QUALITY TECHNOLOGY', 'Walker R, 2002, ', 'Ray M, 1994, THE ANNALS OF THORACIC SURGERY', 'Lovell B, 1996, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Raubertas R, 1994, MEDICAL DECISION MAKING', 'Bradley A, 2002, ', 'Rumelhart D, 1985, ', 'Gennari J, 1988, ', 'Twomey J, 2002, IEEE INTERNATIONAL CONFERENCE ON NEURAL NETWORKS']</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
-        </is>
-      </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
+          <t>Bradley A, 1997, PATTERN RECOGNITION</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Bradley A, 1997, PATTERN RECOGNITION</t>
         </is>
       </c>
     </row>
@@ -3174,20 +3304,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr">
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>Chris Bishop, 2006, Springer eBooks</t>
-        </is>
-      </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Chris Bishop, 2006, Springer eBooks</t>
+          <t>Bishop C, 2006, SPRINGER EBOOKS</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>Bishop C, 2006, SPRINGER EBOOKS</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3416,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['CA']</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3289,20 +3424,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr">
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>Radford M. Neal, 2007, Technometrics</t>
-        </is>
-      </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Radford M. Neal, 2007, Technometrics</t>
+          <t>Neal R, 2007, TECHNOMETRICS</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>Neal R, 2007, TECHNOMETRICS</t>
         </is>
       </c>
     </row>
@@ -3380,28 +3520,33 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W60686164', 'https://openalex.org/W78356000', 'https://openalex.org/W84569508', 'https://openalex.org/W1497675750', 'https://openalex.org/W1746819321', 'https://openalex.org/W1973333099', 'https://openalex.org/W2061144551', 'https://openalex.org/W2097998348', 'https://openalex.org/W2099201756', 'https://openalex.org/W2106411961', 'https://openalex.org/W2106869737', 'https://openalex.org/W2119595900', 'https://openalex.org/W2129458072', 'https://openalex.org/W2132984949', 'https://openalex.org/W2141125852', 'https://openalex.org/W2147196093', 'https://openalex.org/W2151238122', 'https://openalex.org/W2165599843', 'https://openalex.org/W2189424119', 'https://openalex.org/W2197776371', 'https://openalex.org/W2951665052', 'https://openalex.org/W2964172739', 'https://openalex.org/W3118608800']</t>
+          <t>['CA', 'US']</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr">
+          <t>['Rasmussen C, 2005, THE MIT PRESS EBOOKS', 'Bergstra J, 2012, ', 'Kennedy M, 2001, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Cireşan D, 2012, ', 'Bergstra J, 2011, ', 'Hutter F, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Jones D, 2001, JOURNAL OF GLOBAL OPTIMIZATION', 'Hoffman M, 2010, ', 'Kushner H, 1964, JOURNAL OF BASIC ENGINEERING', 'Kumar M, 2010, NEURAL INFORMATION PROCESSING SYSTEMS', 'Bonilla E, 2007, EDINBURGH RESEARCH EXPLORER', 'Yu C, 2009, ', 'Saxe A, 2011, ', 'Bull A, 2011, JOURNAL OF MACHINE LEARNING RESEARCH', 'Teh Y, 2005, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Mahendran N, 2012, ', 'Miller K, 2012, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Krizhevsky A, 2024, ', 'Brochu E, 2010, ARXIV (CORNELL UNIVERSITY)', 'Srinivas N, 2009, INFOSCIENCE (ECOLE POLYTECHNIQUE FÉDÉRALE DE LAUSANNE)', 'Coates A, 2024, ', 'Murray I, 2010, ARXIV (CORNELL UNIVERSITY)', 'Ginsbourger D, 2011, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)']</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
-        </is>
-      </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
+          <t>Snoek J, 2012, ARXIV (CORNELL UNIVERSITY)</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Snoek J, 2012, ARXIV (CORNELL UNIVERSITY)</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3580,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>4515</v>
+        <v>4501</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -3491,28 +3636,33 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W617139115', 'https://openalex.org/W639205477', 'https://openalex.org/W1491105865', 'https://openalex.org/W1492999010', 'https://openalex.org/W1510073064', 'https://openalex.org/W1565640256', 'https://openalex.org/W1625305535', 'https://openalex.org/W1710476689', 'https://openalex.org/W1757990252', 'https://openalex.org/W1865667476', 'https://openalex.org/W1968761064', 'https://openalex.org/W1976492731', 'https://openalex.org/W1979769287', 'https://openalex.org/W1982589276', 'https://openalex.org/W1982598895', 'https://openalex.org/W1992985800', 'https://openalex.org/W1997974358', 'https://openalex.org/W2007400012', 'https://openalex.org/W2020786104', 'https://openalex.org/W2025679679', 'https://openalex.org/W2030843415', 'https://openalex.org/W2030976617', 'https://openalex.org/W2032026767', 'https://openalex.org/W2034097448', 'https://openalex.org/W2036524141', 'https://openalex.org/W2052226480', 'https://openalex.org/W2052891002', 'https://openalex.org/W2057069496', 'https://openalex.org/W2058452634', 'https://openalex.org/W2063007245', 'https://openalex.org/W2067250248', 'https://openalex.org/W2074616700', 'https://openalex.org/W2076063813', 'https://openalex.org/W2081413236', 'https://openalex.org/W2083415705', 'https://openalex.org/W2104489082', 'https://openalex.org/W2123306226', 'https://openalex.org/W2124234891', 'https://openalex.org/W2127168465', 'https://openalex.org/W2128245586', 'https://openalex.org/W2134164499', 'https://openalex.org/W2138178257', 'https://openalex.org/W2157886206', 'https://openalex.org/W2164524421', 'https://openalex.org/W2173027866', 'https://openalex.org/W2194321275', 'https://openalex.org/W2217912240', 'https://openalex.org/W2230728100', 'https://openalex.org/W2279490987', 'https://openalex.org/W2310703973', 'https://openalex.org/W2324964582', 'https://openalex.org/W2325264655', 'https://openalex.org/W2328928309', 'https://openalex.org/W2337082154', 'https://openalex.org/W2338402873', 'https://openalex.org/W2346180883', 'https://openalex.org/W2346400664', 'https://openalex.org/W2347129741', 'https://openalex.org/W2349487082', 'https://openalex.org/W2418973097', 'https://openalex.org/W2468638527', 'https://openalex.org/W2477622860', 'https://openalex.org/W2478294658', 'https://openalex.org/W2503662290', 'https://openalex.org/W2509907061', 'https://openalex.org/W2520022941', 'https://openalex.org/W2520500207', 'https://openalex.org/W2521267242', 'https://openalex.org/W2525748878', 'https://openalex.org/W2531602199', 'https://openalex.org/W2537064446', 'https://openalex.org/W2540627216', 'https://openalex.org/W2541404351', 'https://openalex.org/W2559394418', 'https://openalex.org/W2565684601', 'https://openalex.org/W2571050567', 'https://openalex.org/W2580919858', 'https://openalex.org/W2591366729', 'https://openalex.org/W2599053724', 'https://openalex.org/W2606044016', 'https://openalex.org/W2611413954', 'https://openalex.org/W2618625858', 'https://openalex.org/W2619580215', 'https://openalex.org/W2620846205', 'https://openalex.org/W2621738901', 'https://openalex.org/W2621742623', 'https://openalex.org/W2734520197', 'https://openalex.org/W2740407088', 'https://openalex.org/W2746244909', 'https://openalex.org/W2747592475', 'https://openalex.org/W2752180799', 'https://openalex.org/W2753962198', 'https://openalex.org/W2766362701', 'https://openalex.org/W2789615344', 'https://openalex.org/W2951016506', 'https://openalex.org/W2963094133', 'https://openalex.org/W2964113829', 'https://openalex.org/W2964116922', 'https://openalex.org/W2964217201', 'https://openalex.org/W3037315640', 'https://openalex.org/W3099950071', 'https://openalex.org/W4240502307', 'https://openalex.org/W4252359241', 'https://openalex.org/W6637568146', 'https://openalex.org/W6730103093', 'https://openalex.org/W6735944222', 'https://openalex.org/W6910696677']</t>
+          <t>['GB', 'US', 'KR']</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr">
+          <t>['Kohn W, 1965, PHYSICAL REVIEW', 'Schmidhuber J, 2014, NEURAL NETWORKS', 'Jain A, 2013, APL MATERIALS', 'Shawe‐Taylor J, 2004, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Sterling T, 2015, JOURNAL OF CHEMICAL INFORMATION AND MODELING', 'Harrow A, 2009, PHYSICAL REVIEW LETTERS', 'Bartók A, 2010, PHYSICAL REVIEW LETTERS', 'Lake B, 2015, SCIENCE', 'Schmidt M, 2009, SCIENCE', 'Drori I, 2022, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Saal J, 2013, JOM', 'Rupp M, 2012, PHYSICAL REVIEW LETTERS', 'Hansch C, 1964, JOURNAL OF THE AMERICAN CHEMICAL SOCIETY', 'Curtarolo S, 2013, NATURE MATERIALS', 'Tropsha A, 2010, MOLECULAR INFORMATICS', 'Dirac P, 1929, PROCEEDINGS OF THE ROYAL SOCIETY OF LONDON SERIES A CONTAINING PAPERS OF A MATHEMATICAL AND PHYSICAL CHARACTER', 'Lejaeghere K, 2016, SCIENCE', 'Aspuru‐Guzik A, 2005, SCIENCE', 'Ghiringhelli L, 2015, PHYSICAL REVIEW LETTERS', 'Hand D, 2001, INTERNATIONAL STATISTICAL REVIEW', 'Pilania G, 2013, SCIENTIFIC REPORTS', 'Fourches D, 2010, JOURNAL OF CHEMICAL INFORMATION AND MODELING', 'Billinge S, 2007, SCIENCE', 'Corey E, 1969, SCIENCE', 'Hachmann J, 2011, THE JOURNAL OF PHYSICAL CHEMISTRY LETTERS', 'Snyder J, 2012, PHYSICAL REVIEW LETTERS', 'Havu V, 2009, JOURNAL OF COMPUTATIONAL PHYSICS', 'Hautier G, 2010, CHEMISTRY OF MATERIALS', 'Schütt K, 2014, PHYSICAL REVIEW B', 'Calderón C, 2015, COMPUTATIONAL MATERIALS SCIENCE', 'Faber F, 2016, PHYSICAL REVIEW LETTERS', 'Shakhnarovich G, 2005, ', 'Kalinin S, 2015, NATURE MATERIALS', 'Handley C, 2010, THE JOURNAL OF PHYSICAL CHEMISTRY A', 'Franceschetti A, 1999, NATURE', 'Christensen R, 2015, CATALYSIS SCIENCE &amp; TECHNOLOGY', 'Fleuren W, 2015, METHODS', 'Kireeva N, 2012, MOLECULAR INFORMATICS', 'Pople J, 1999, ANGEWANDTE CHEMIE INTERNATIONAL EDITION', 'Bonchev D, 1994, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Albuquerque V, 2008, NONDESTRUCTIVE TESTING AND EVALUATION', 'Wicker J, 2014, CRYSTENGCOMM', 'Kühn C, 1996, THE JOURNAL OF PHYSICAL CHEMISTRY', 'Walsh A, 2015, NATURE CHEMISTRY', ', 2013, ', 'Oprea T, 2006, DRUG DISCOVERY TODAY TECHNOLOGIES', 'Kiselyova N, 1998, JOURNAL OF ALLOYS AND COMPOUNDS', 'Duvenaud D, 2015, ARXIV (CORNELL UNIVERSITY)', 'Jastrzȩbski S, 2016, ARXIV (CORNELL UNIVERSITY)', 'Biamonte J, 2017, NATURE', 'Smith J, 2017, CHEMICAL SCIENCE', 'Segler M, 2018, NATURE', 'Raccuglia P, 2016, NATURE', ', 2021, ENCYCLOPEDIA OF THE UN SUSTAINABLE DEVELOPMENT GOALS', 'Rudy S, 2017, SCIENCE ADVANCES', 'Wellendorff J, 2012, PHYSICAL REVIEW B', 'Carrasquilla J, 2017, NATURE PHYSICS', 'Steane A, 1998, REPORTS ON PROGRESS IN PHYSICS', 'Agrawal A, 2016, APL MATERIALS', 'Mardirossian N, 2016, THE JOURNAL OF CHEMICAL PHYSICS', 'Gómez‐Bombarelli R, 2016, NATURE MATERIALS', 'Altae-Tran H, 2017, ACS CENTRAL SCIENCE', 'Reiher M, 2017, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Behler J, 2017, ANGEWANDTE CHEMIE INTERNATIONAL EDITION', 'Faber F, 2017, JOURNAL OF CHEMICAL THEORY AND COMPUTATION', 'Isayev O, 2017, NATURE COMMUNICATIONS', 'Szymkuć S, 2016, ANGEWANDTE CHEMIE INTERNATIONAL EDITION', 'Segler M, 2017, CHEMISTRY - A EUROPEAN JOURNAL', 'Brockherde F, 2017, NATURE COMMUNICATIONS', 'Liu B, 2017, ACS CENTRAL SCIENCE', 'Pulido A, 2017, NATURE', 'Kim E, 2017, CHEMISTRY OF MATERIALS', 'Dunjko V, 2016, PHYSICAL REVIEW LETTERS', 'Ward L, 2017, PHYSICAL REVIEW. B./PHYSICAL REVIEW. B', 'Oliynyk A, 2016, CHEMISTRY OF MATERIALS', 'Klucznik T, 2018, CHEM', 'Duan Y, 2017, NEURAL INFORMATION PROCESSING SYSTEMS', 'Hill J, 2016, MRS BULLETIN', 'Davies D, 2016, CHEM', 'Pensak D, 1977, ACS SYMPOSIUM SERIES', 'Legrain F, 2017, THE JOURNAL OF PHYSICAL CHEMISTRY B', 'Ziatdinov M, 2017, NPJ COMPUTATIONAL MATERIALS', 'Dragone V, 2017, NATURE COMMUNICATIONS', 'Wilkinson K, 2014, JOURNAL OF CHEMICAL THEORY AND COMPUTATION', 'Norbert J, 2011, STUDIES IN COMPUTATIONAL INTELLIGENCE', 'Seko A, 2018, ', 'Arita M, 2014, JOURNAL OF CHEMICAL THEORY AND COMPUTATION', 'Coudert F, 2017, CHEMISTRY OF MATERIALS', 'Tetko I, 2016, MOLECULAR INFORMATICS', 'Cole J, 2016, ACTA CRYSTALLOGRAPHICA SECTION B STRUCTURAL SCIENCE CRYSTAL ENGINEERING AND MATERIALS', 'Boyd D, 2013, ACS SYMPOSIUM SERIES', 'Moot T, 2016, MATERIALS DISCOVERY', 'Pillong M, 2017, CRYSTENGCOMM', 'Trabesinger A, 2017, NATURE', 'Hui Y, 2019, ADVANCES IN INTELLIGENT SYSTEMS AND COMPUTING', 'Guimaraes G, 2017, ARXIV (CORNELL UNIVERSITY)', 'Nam J, 2016, ARXIV (CORNELL UNIVERSITY)', 'Calderón C, 2015, ARXIV (CORNELL UNIVERSITY)', 'F. B, 2017, MPG.PURE (MAX PLANCK SOCIETY)', 'R.B. M, 1993, JOURNAL OF MOLECULAR STRUCTURE THEOCHEM', 'Rokach L, 2009, ']</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>Keith T. Butler, 2018, Nature</t>
-        </is>
-      </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Keith T. Butler, 2018, Nature</t>
+          <t>Butler K, 2018, NATURE</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>Butler K, 2018, NATURE</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3731,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['US', 'CA']</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3589,20 +3739,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr">
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">William W. Cohen, 2008, </t>
-        </is>
-      </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t xml:space="preserve">William W. Cohen, 2008, </t>
+          <t xml:space="preserve">Cohen W, 2008, </t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cohen W, 2008, </t>
         </is>
       </c>
     </row>
@@ -3636,7 +3791,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>3948</v>
+        <v>3936</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -3692,28 +3847,33 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1524493166', 'https://openalex.org/W1529983430', 'https://openalex.org/W2005440935', 'https://openalex.org/W2009184733', 'https://openalex.org/W2009954208', 'https://openalex.org/W2027540165', 'https://openalex.org/W2033163059', 'https://openalex.org/W2033609349', 'https://openalex.org/W2043092953', 'https://openalex.org/W2054076956', 'https://openalex.org/W2083721602', 'https://openalex.org/W2096849439', 'https://openalex.org/W2103018059', 'https://openalex.org/W2103889389', 'https://openalex.org/W2119472226', 'https://openalex.org/W2137767404', 'https://openalex.org/W2147246123', 'https://openalex.org/W2166187912', 'https://openalex.org/W2167414941', 'https://openalex.org/W2174931596', 'https://openalex.org/W2267932926', 'https://openalex.org/W2276530525', 'https://openalex.org/W2337116044', 'https://openalex.org/W2415841860', 'https://openalex.org/W2468431774', 'https://openalex.org/W2512902140', 'https://openalex.org/W2515682654', 'https://openalex.org/W2528491735', 'https://openalex.org/W2530247697', 'https://openalex.org/W2548723212', 'https://openalex.org/W2557738935', 'https://openalex.org/W2581082771', 'https://openalex.org/W2598272139', 'https://openalex.org/W2732701910', 'https://openalex.org/W2734356183', 'https://openalex.org/W2738975713', 'https://openalex.org/W2740060821', 'https://openalex.org/W2752747624', 'https://openalex.org/W2753059860', 'https://openalex.org/W2754518417', 'https://openalex.org/W2758348074', 'https://openalex.org/W2762741128', 'https://openalex.org/W2772246530', 'https://openalex.org/W2772723798', 'https://openalex.org/W2782945064', 'https://openalex.org/W2784499877', 'https://openalex.org/W2785268987', 'https://openalex.org/W2785526886', 'https://openalex.org/W2788633781', 'https://openalex.org/W2789894922', 'https://openalex.org/W2790444357', 'https://openalex.org/W2791819448', 'https://openalex.org/W2792902933', 'https://openalex.org/W2793267369', 'https://openalex.org/W2794457162', 'https://openalex.org/W2799837895', 'https://openalex.org/W2804685074', 'https://openalex.org/W2809453031', 'https://openalex.org/W2886281300', 'https://openalex.org/W2887623535', 'https://openalex.org/W2887719255', 'https://openalex.org/W2888109941', 'https://openalex.org/W2889242407', 'https://openalex.org/W2889494558', 'https://openalex.org/W2894917609', 'https://openalex.org/W2896385413', 'https://openalex.org/W2896817483', 'https://openalex.org/W2897434820', 'https://openalex.org/W2899560923', 'https://openalex.org/W2902802452', 'https://openalex.org/W2908201961', 'https://openalex.org/W2914579361', 'https://openalex.org/W2916105049', 'https://openalex.org/W2919115771', 'https://openalex.org/W3098949126', 'https://openalex.org/W4205374244', 'https://openalex.org/W4212774754', 'https://openalex.org/W4296220420']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr">
+          <t>['Esteva A, 2017, NATURE', 'Gulshan V, 2016, JAMA', 'Haynes A, 2009, NEW ENGLAND JOURNAL OF MEDICINE', 'Kermany D, 2018, CELL', 'Bejnordi B, 2017, JAMA', 'Rajkomar A, 2018, NPJ DIGITAL MEDICINE', 'Ting D, 2017, JAMA', 'Beam A, 2018, JAMA', 'Poplin R, 2018, NATURE BIOMEDICAL ENGINEERING', 'Halevy A, 2009, IEEE INTELLIGENT SYSTEMS', 'Castelvecchi D, 2016, NATURE', 'Sinsky C, 2016, ANNALS OF INTERNAL MEDICINE', 'Bates D, 2014, HEALTH AFFAIRS', 'Cabitza F, 2017, JAMA', 'Arndt B, 2017, THE ANNALS OF FAMILY MEDICINE', 'Mandel J, 2016, JOURNAL OF THE AMERICAN MEDICAL INFORMATICS ASSOCIATION', 'Frieden T, 2017, NEW ENGLAND JOURNAL OF MEDICINE', 'Muntner P, 2014, JAMA', 'Krumholz H, 2014, HEALTH AFFAIRS', 'Hersh W, 2013, MEDICAL CARE', 'Krause J, 2018, OPHTHALMOLOGY', 'Elmore J, 2017, BMJ', 'Jong M, 2017, THE LANCET', 'Lyell D, 2016, JOURNAL OF THE AMERICAN MEDICAL INFORMATICS ASSOCIATION', 'Schneeweiß S, 2014, NEW ENGLAND JOURNAL OF MEDICINE', 'Mandl K, 2001, BMJ', 'Cohen I, 2014, HEALTH AFFAIRS', 'Lindenauer P, 2012, JAMA', 'Kesselheim A, 2011, HEALTH AFFAIRS', 'Obermeyer Z, 2017, NEW ENGLAND JOURNAL OF MEDICINE', 'Erickson S, 2017, ANNALS OF INTERNAL MEDICINE', 'Schwartz W, 1970, NEW ENGLAND JOURNAL OF MEDICINE', 'Hill R, 2013, THE AMERICAN JOURNAL OF EMERGENCY MEDICINE', 'Amarasingham R, 2014, HEALTH AFFAIRS', 'Mamykina L, 2016, ACADEMIC MEDICINE', 'Shuren J, 2016, JAMA', 'Fiore L, 2016, NEW ENGLAND JOURNAL OF MEDICINE', 'Bakris G, 2018, NEW ENGLAND JOURNAL OF MEDICINE', 'Escobar G, 2016, JOURNAL OF HOSPITAL MEDICINE', 'McGlynn E, 2015, JAMA', 'Mandl K, 2016, NEW ENGLAND JOURNAL OF MEDICINE', 'Sniderman A, 2015, JAMA', 'Steinhubl S, 2018, THE LANCET', 'Schuster M, 2017, JAMA', 'Slack W, 1966, NEW ENGLAND JOURNAL OF MEDICINE', 'Oxentenko A, 2010, ARCHIVES OF INTERNAL MEDICINE', 'Reis B, 2009, BMJ', 'Gabriels K, 2018, JOURNAL OF MEDICAL INTERNET RESEARCH', 'Sittig D, 2015, JOURNAL OF THE AMERICAN MEDICAL INFORMATICS ASSOCIATION', 'Rajkomar A, 2016, JMIR MEDICAL INFORMATICS', 'LeCun Y, 2015, NATURE', ', 1996, COMPUTERS &amp; MATHEMATICS WITH APPLICATIONS', 'Topol E, 2018, NATURE MEDICINE', 'Fauw J, 2018, NATURE MEDICINE', 'Alvin R, 2018, ', 'Ford I, 2016, NEW ENGLAND JOURNAL OF MEDICINE', 'Gianfrancesco M, 2018, JAMA INTERNAL MEDICINE', 'Rajkomar A, 2018, ANNALS OF INTERNAL MEDICINE', 'Chilamkurthy S, 2018, THE LANCET', 'Wang P, 2019, GUT', 'Hinton G, 2018, JAMA', 'Grinfeld J, 2018, NEW ENGLAND JOURNAL OF MEDICINE', 'Denis F, 2019, JAMA', 'Tison G, 2018, JAMA CARDIOLOGY', 'Mori Y, 2018, ANNALS OF INTERNAL MEDICINE', 'Steiner D, 2018, THE AMERICAN JOURNAL OF SURGICAL PATHOLOGY', 'Liu Y, 2018, ARCHIVES OF PATHOLOGY &amp; LABORATORY MEDICINE', 'Morawski K, 2018, JAMA INTERNAL MEDICINE', 'Howe J, 2018, JAMA', 'Fraser H, 2018, THE LANCET', 'Kale M, 2018, BMJ', 'Das J, 2018, BMJ', 'Schwartz W, 1987, NEW ENGLAND JOURNAL OF MEDICINE', 'Galloway C, 2018, JOURNAL OF THE AMERICAN COLLEGE OF CARDIOLOGY', 'Berwick D, 2018, JAMA', 'Auerbach A, 2018, ANNALS OF INTERNAL MEDICINE', 'Kannan A, 2018, ', 'Lee V, 2018, JAMA']</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
-        </is>
-      </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
+          <t>Rajkomar A, 2019, NEW ENGLAND JOURNAL OF MEDICINE</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>Rajkomar A, 2019, NEW ENGLAND JOURNAL OF MEDICINE</t>
         </is>
       </c>
     </row>
@@ -3799,28 +3959,33 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W740415', 'https://openalex.org/W1504694836', 'https://openalex.org/W1978394996', 'https://openalex.org/W2023677852', 'https://openalex.org/W2087614174', 'https://openalex.org/W2096152098', 'https://openalex.org/W2114535528', 'https://openalex.org/W2119821739', 'https://openalex.org/W2125055259', 'https://openalex.org/W2149684865', 'https://openalex.org/W2156909104', 'https://openalex.org/W2164547069', 'https://openalex.org/W2435251607', 'https://openalex.org/W6821113053']</t>
+          <t>['DE']</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr">
+          <t>['Vapnik V, 1995, ', 'Cortes C, 1995, MACHINE LEARNING', 'Quinlan J, 1992, ', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE', 'Salzberg S, 1994, ', 'Yang Y, 1997, ', 'Rocchio J, 1971, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Vapnik V, 1995, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Yang Y, 1999, INFORMATION RETRIEVAL', 'Joachims T, 1997, ', 'Kivinen J, 1997, ARTIFICIAL INTELLIGENCE', 'Kivinen J, 1995, ']</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>Thorsten Joachims, 1998, Lecture notes in computer science</t>
-        </is>
-      </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Thorsten Joachims, 1998, Lecture notes in computer science</t>
+          <t>Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Joachims T, 1998, LECTURE NOTES IN COMPUTER SCIENCE</t>
         </is>
       </c>
     </row>
@@ -3854,7 +4019,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>6648</v>
+        <v>6646</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -3898,28 +4063,33 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W588441650', 'https://openalex.org/W962117656', 'https://openalex.org/W1514535095', 'https://openalex.org/W1568514080', 'https://openalex.org/W1606347560', 'https://openalex.org/W1810943226', 'https://openalex.org/W1815076433', 'https://openalex.org/W1867429401', 'https://openalex.org/W1903029394', 'https://openalex.org/W1905882502', 'https://openalex.org/W1947481528', 'https://openalex.org/W1982479097', 'https://openalex.org/W2024414272', 'https://openalex.org/W2030459037', 'https://openalex.org/W2064675550', 'https://openalex.org/W2079565659', 'https://openalex.org/W2116435618', 'https://openalex.org/W2130942839', 'https://openalex.org/W2157331557', 'https://openalex.org/W2557283755', 'https://openalex.org/W2787727108', 'https://openalex.org/W2950635152', 'https://openalex.org/W2951183276', 'https://openalex.org/W2952453038', 'https://openalex.org/W4233546237', 'https://openalex.org/W4294306266', 'https://openalex.org/W4308909683']</t>
+          <t>['HK', 'CN']</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr">
+          <t>['Hochreiter S, 1997, NEURAL COMPUTATION', 'Long J, 2015, ', 'Cho K, 2014, ', 'Goodfellow I, 2016, MIT PRESS EBOOKS', 'Donahue J, 2015, ', 'Karpathy A, 2015, ', 'Davide B, 2013, DROPS (SCHLOSS DAGSTUHL – LEIBNIZ CENTER FOR INFORMATICS)', 'Brox T, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Sun J, 2013, BULLETIN OF THE AMERICAN METEOROLOGICAL SOCIETY', 'Germann U, 2002, MONTHLY WEATHER REVIEW', 'Bridson R, 2011, ', 'Bridson R, 2015, ', 'Klein B, 2015, ', 'Sakaino H, 2012, IEEE TRANSACTIONS ON GEOSCIENCE AND REMOTE SENSING', 'Woo W, 2014, 27TH CONFERENCE ON SEVERE LOCAL STORMS', 'Douglas R, 1990, AMERICAN METEOROLOGICAL SOCIETY EBOOKS', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2015, ARXIV (CORNELL UNIVERSITY)', 'Pascanu R, 2012, ARXIV (CORNELL UNIVERSITY)', 'Cho K, 2014, ARXIV (CORNELL UNIVERSITY)', 'Long J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Srivastava N, 2015, ARXIV (CORNELL UNIVERSITY)', 'Donahue J, 2014, ', 'Bastien F, 2012, ARXIV (CORNELL UNIVERSITY)', 'Ranzato M, 2014, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>Xingjian Shi, 2015, arXiv (Cornell University)</t>
-        </is>
-      </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Xingjian Shi, 2015, arXiv (Cornell University)</t>
+          <t>Shi X, 2015, ARXIV (CORNELL UNIVERSITY)</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Shi X, 2015, ARXIV (CORNELL UNIVERSITY)</t>
         </is>
       </c>
     </row>
@@ -4005,28 +4175,33 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1657213141', 'https://openalex.org/W1746680969', 'https://openalex.org/W2117063635', 'https://openalex.org/W2129564505']</t>
+          <t>['DE']</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr">
+          <t>['Jordan M, 1998, ', 'Williams C, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Csató L, 2002, NEURAL COMPUTATION', 'Williams C, 1998, ']</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>Carl Edward Rasmussen, 2004, Lecture notes in computer science</t>
-        </is>
-      </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Carl Edward Rasmussen, 2004, Lecture notes in computer science</t>
+          <t>Rasmussen C, 2004, LECTURE NOTES IN COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>Rasmussen C, 2004, LECTURE NOTES IN COMPUTER SCIENCE</t>
         </is>
       </c>
     </row>
@@ -4108,28 +4283,33 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1505356468', 'https://openalex.org/W1535810436', 'https://openalex.org/W1629097610', 'https://openalex.org/W2029538739', 'https://openalex.org/W2030811966', 'https://openalex.org/W2035720976', 'https://openalex.org/W2043919728', 'https://openalex.org/W2068484625', 'https://openalex.org/W2086161653', 'https://openalex.org/W2098921539', 'https://openalex.org/W2101159990', 'https://openalex.org/W2113651538', 'https://openalex.org/W2119821739', 'https://openalex.org/W2127218421', 'https://openalex.org/W2129191766', 'https://openalex.org/W2135046866', 'https://openalex.org/W2137515395', 'https://openalex.org/W2147880316', 'https://openalex.org/W2150102617', 'https://openalex.org/W2154451187', 'https://openalex.org/W2322150470', 'https://openalex.org/W2416173357', 'https://openalex.org/W2766736793', 'https://openalex.org/W2990138404', 'https://openalex.org/W3207342693', 'https://openalex.org/W4238284510']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr">
+          <t>['Tibshirani R, 1996, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Cortes C, 1995, MACHINE LEARNING', 'MacQueen J, 1967, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', ', 2007, THE MIT PRESS EBOOKS', 'Lafferty J, 2001, SCHOLARLY COMMONS (UNIVERSITY OF PENNSYLVANIA)', 'Dennis J, 1996, SOCIETY FOR INDUSTRIAL AND APPLIED MATHEMATICS EBOOKS', 'Vapnik V, 2015, ', 'Lewis D, 2004, GOLDSMITHS (UNIVERSITY OF LONDON)', 'Vapnik V, 1971, THEORY OF PROBABILITY AND ITS APPLICATIONS', 'Joachims T, 2006, ', 'Polyak B, 1992, SIAM JOURNAL ON CONTROL AND OPTIMIZATION', 'Bottou L, 2011, THE MIT PRESS EBOOKS', 'Tsybakov A, 2004, THE ANNALS OF STATISTICS', 'Bordes A, 2009, HAL (LE CENTRE POUR LA COMMUNICATION SCIENTIFIQUE DIRECTE)', 'Lin C, 2007, ', 'Shalev‐Shwartz S, 2008, ', 'Massart P, 2000, ANNALES DE LA FACULTÉ DES SCIENCES DE TOULOUSE MATHÉMATIQUES', 'Bottou L, 2005, APPLIED STOCHASTIC MODELS IN BUSINESS AND INDUSTRY', 'Lee W, 1998, IEEE TRANSACTIONS ON INFORMATION THEORY', "Bousquet O, 2002, OPENGREY (INSTITUT DE L'INFORMATION SCIENTIFIQUE ET TECHNIQUE)", 'Murata N, 1999, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Rumelhart D, 1985, ', 'Widrow B, 1960, ', 'Xu W, 2011, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Léon Bottou, 2010, </t>
-        </is>
-      </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Léon Bottou, 2010, </t>
+          <t xml:space="preserve">Bottou L, 2010, </t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottou L, 2010, </t>
         </is>
       </c>
     </row>
@@ -4174,7 +4354,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>['Sammut, Claude 1956-']</t>
+          <t>['Nijssen, Siegfried']</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -4184,7 +4364,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Sammut, Claude 1956- (corresponding author), University Of New south Wales</t>
+          <t>Nijssen, Siegfried (corresponding author), University Of New south Wales</t>
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -4199,7 +4379,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['AU']</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4207,20 +4387,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr">
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claude Sammut, 2010, </t>
-        </is>
-      </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claude Sammut, 2010, </t>
+          <t xml:space="preserve">Sammut C, 2010, </t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sammut C, 2010, </t>
         </is>
       </c>
     </row>
@@ -4254,7 +4439,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>8918</v>
+        <v>8893</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -4310,28 +4495,33 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1492170170', 'https://openalex.org/W1537462412', 'https://openalex.org/W1731081199', 'https://openalex.org/W1746506709', 'https://openalex.org/W1905782493', 'https://openalex.org/W1973682096', 'https://openalex.org/W1984314602', 'https://openalex.org/W1994407253', 'https://openalex.org/W2013587512', 'https://openalex.org/W2026905436', 'https://openalex.org/W2046945713', 'https://openalex.org/W2072136246', 'https://openalex.org/W2082262280', 'https://openalex.org/W2132166479', 'https://openalex.org/W2134598164', 'https://openalex.org/W2141097525', 'https://openalex.org/W2149033360', 'https://openalex.org/W2163598528', 'https://openalex.org/W2239135493', 'https://openalex.org/W2248060815', 'https://openalex.org/W2467510144', 'https://openalex.org/W2493343568', 'https://openalex.org/W2579555219', 'https://openalex.org/W2604231045', 'https://openalex.org/W2613140028', 'https://openalex.org/W2621305858', 'https://openalex.org/W2743731382', 'https://openalex.org/W2752988282', 'https://openalex.org/W2765813195', 'https://openalex.org/W2767442356', 'https://openalex.org/W2778670458', 'https://openalex.org/W2798857668', 'https://openalex.org/W2811104224', 'https://openalex.org/W2811374795', 'https://openalex.org/W2894881080', 'https://openalex.org/W2895051075', 'https://openalex.org/W2896176822', 'https://openalex.org/W2898694742', 'https://openalex.org/W2899360465', 'https://openalex.org/W2901939789', 'https://openalex.org/W2902991393', 'https://openalex.org/W2910705748', 'https://openalex.org/W2962689739', 'https://openalex.org/W2963125461', 'https://openalex.org/W2963533879', 'https://openalex.org/W2963816926', 'https://openalex.org/W2964134873', 'https://openalex.org/W2964180856', 'https://openalex.org/W3085162807', 'https://openalex.org/W3098636317', 'https://openalex.org/W3102221121', 'https://openalex.org/W3102834905', 'https://openalex.org/W3122175177', 'https://openalex.org/W4234008654', 'https://openalex.org/W6743543778']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr">
+          <t>['Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Miller G, 1956, PSYCHOLOGICAL REVIEW', 'Miller G, 1994, PSYCHOLOGICAL REVIEW', 'Ganin Y, 2017, ADVANCES IN COMPUTER VISION AND PATTERN RECOGNITION', 'Fayyad U, 1996, ', 'Goodman B, 2017, AI MAGAZINE', 'Murdoch W, 2019, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'Holte R, 1993, MACHINE LEARNING', 'Zech J, 2018, PLOS MEDICINE', 'Cowan N, 2010, CURRENT DIRECTIONS IN PSYCHOLOGICAL SCIENCE', 'Mittelstadt B, 2019, ', 'Hand D, 2006, STATISTICAL SCIENCE', 'Freitas A, 2014, ACM SIGKDD EXPLORATIONS NEWSLETTER', 'Lou Y, 2013, ', 'Lou Y, 2012, ', 'Huysmans J, 2010, DECISION SUPPORT SYSTEMS', 'Li O, 2018, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Ustun B, 2017, JAMA PSYCHIATRY', 'Brennan T, 2008, CRIMINAL JUSTICE AND BEHAVIOR', 'Flores A, 2016, FEDERAL PROBATION', 'Razavian N, 2015, BIG DATA', 'Zeng J, 2016, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (STATISTICS IN SOCIETY)', 'Wang F, 2015, INTERNATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE AND STATISTICS', 'Rudin C, 2018, ARXIV (CORNELL UNIVERSITY)', 'Goodman B, 2016, ARXIV (CORNELL UNIVERSITY)', 'Tollenaar N, 2012, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (STATISTICS IN SOCIETY)', 'Rudin C, 2018, INFORMS JOURNAL ON APPLIED ANALYTICS', 'Gupta M, 2016, JOURNAL OF MACHINE LEARNING RESEARCH', 'Rudin C, 2020, HARVARD DATA SCIENCE REVIEW', 'Rüping S, 2006, ', 'Rudin C, 2010, MACHINE LEARNING', 'Ustun B, 2017, ', 'Auer P, 1995, ELSEVIER EBOOKS', 'Carrizosa E, 2009, INFORMS JOURNAL ON COMPUTING', 'Wang J, 2018, ', 'Gallagher N, 2017, NEURAL INFORMATION PROCESSING SYSTEMS', 'Chang A, 2012, MACHINE LEARNING', 'Goel A, 2017, AI MAGAZINE', 'Wang F, 2018, BIOSTATISTICS', 'Mannshardt E, 2018, SIGNIFICANCE', 'Neri P, 2018, INFORMS JOURNAL ON APPLIED ANALYTICS', ', , VIEW', 'Chen C, 2018, ARXIV (CORNELL UNIVERSITY)', 'Li O, 2017, ARXIV (CORNELL UNIVERSITY)', 'Chen C, 2018, ARXIV (CORNELL UNIVERSITY)', 'Carrière M, 2017, ARXIV (CORNELL UNIVERSITY)', "Sokolovska N, 2018, BASE INSTITUTIONNELLE DE RECHERCHE DE L'UNIVERSITÉ PARIS-DAUPHINE (BIRD) (UNIVERSITY PARIS-DAUPHINE)", ', 2017, AUERBACH PUBLICATIONS EBOOKS']</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
-        </is>
-      </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
+          <t>Rudin C, 2019, NATURE MACHINE INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Rudin C, 2019, NATURE MACHINE INTELLIGENCE</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4555,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>3409</v>
+        <v>3407</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -4425,28 +4615,33 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W40442397', 'https://openalex.org/W1480376833', 'https://openalex.org/W1678356000', 'https://openalex.org/W1808991731', 'https://openalex.org/W1902027874', 'https://openalex.org/W1976196376', 'https://openalex.org/W2011999110', 'https://openalex.org/W2021701428', 'https://openalex.org/W2029243817', 'https://openalex.org/W2052825782', 'https://openalex.org/W2072128103', 'https://openalex.org/W2073751243', 'https://openalex.org/W2105464873', 'https://openalex.org/W2106665921', 'https://openalex.org/W2110243528', 'https://openalex.org/W2112289645', 'https://openalex.org/W2112592817', 'https://openalex.org/W2113606819', 'https://openalex.org/W2116802246', 'https://openalex.org/W2119361626', 'https://openalex.org/W2120480077', 'https://openalex.org/W2121495423', 'https://openalex.org/W2122111042', 'https://openalex.org/W2127482775', 'https://openalex.org/W2135046866', 'https://openalex.org/W2139212933', 'https://openalex.org/W2147461734', 'https://openalex.org/W2149298154', 'https://openalex.org/W2152072062', 'https://openalex.org/W2158927033', 'https://openalex.org/W2162586165', 'https://openalex.org/W2163697531', 'https://openalex.org/W2164434252', 'https://openalex.org/W2345255551', 'https://openalex.org/W2787894218', 'https://openalex.org/W2911964244', 'https://openalex.org/W2912934387', 'https://openalex.org/W2963481018', 'https://openalex.org/W2998216295', 'https://openalex.org/W3099478002', 'https://openalex.org/W4212883601', 'https://openalex.org/W4231109964', 'https://openalex.org/W4243607236', 'https://openalex.org/W4285719527', 'https://openalex.org/W6601599523', 'https://openalex.org/W6676903177', 'https://openalex.org/W7066667914']</t>
+          <t>['US']</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr">
+          <t>['Breiman L, 2001, MACHINE LEARNING', 'Tibshirani R, 1996, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Friedman J, 2001, THE ANNALS OF STATISTICS', 'Hastie T, 2001, SPRINGER SERIES IN STATISTICS', 'Hastie T, 2009, SPRINGER SERIES IN STATISTICS', 'Breiman L, 1996, MACHINE LEARNING', 'Burges C, 1998, DATA MINING AND KNOWLEDGE DISCOVERY', 'Breiman L, 1996, MACHINE LEARNING', 'Cover T, 1967, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Lee D, 1999, NATURE', 'GuyonIsabelle, 2003, JOURNAL OF MACHINE LEARNING RESEARCH', 'Bengio Y, 2009, FOUNDATIONS AND TRENDS® IN MACHINE LEARNING', 'Lip G, 2009, CHEST JOURNAL', 'Vapnik V, 1999, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Bengio Y, 2009, NOW PUBLISHERS, INC. EBOOKS', 'Olshausen B, 1997, VISION RESEARCH', 'Pitt B, 2014, NEW ENGLAND JOURNAL OF MEDICINE', 'Ishwaran H, 2008, THE ANNALS OF APPLIED STATISTICS', 'Lee H, 2007, THE MIT PRESS EBOOKS', 'D’Agostino R, 2001, JAMA', 'Woodruff P, 2009, AMERICAN JOURNAL OF RESPIRATORY AND CRITICAL CARE MEDICINE', 'Le Q, 2013, ', 'Corren J, 2011, NEW ENGLAND JOURNAL OF MEDICINE', 'Ishwaran H, 2008, ', 'O’Mahony C, 2013, EUROPEAN HEART JOURNAL', 'James M, 2012, PHYSIOLOGICAL REVIEWS', 'Shah S, 2014, CIRCULATION', 'Beck A, 2011, SCIENCE TRANSLATIONAL MEDICINE', 'Koren Y, 2009, ', 'Peña‐Castillo L, 2008, GENOME BIOLOGY', 'Abu‐Mostafa Y, 2012, ', 'Hsich E, 2010, CIRCULATION CARDIOVASCULAR QUALITY AND OUTCOMES', 'Cheng W, 2013, SCIENCE TRANSLATIONAL MEDICINE', 'Margolin A, 2013, SCIENCE TRANSLATIONAL MEDICINE', 'Udelson J, 2011, CIRCULATION', 'Kannel W, 1975, CIRCULATION', 'Cheng W, 2013, PLOS COMPUTATIONAL BIOLOGY', 'Gorodeski E, 2011, CIRCULATION CARDIOVASCULAR QUALITY AND OUTCOMES', 'Deo R, 2014, GENOME BIOLOGY', 'Yogatama D, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ausiello D, 2014, EUROPE PMC (PUBMED CENTRAL)']</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>Rahul C. Deo, 2015, Circulation</t>
-        </is>
-      </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>Rahul C. Deo, 2015, Circulation</t>
+          <t>Deo R, 2015, CIRCULATION</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Deo R, 2015, CIRCULATION</t>
         </is>
       </c>
     </row>
@@ -4480,7 +4675,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>4207</v>
+        <v>4194</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -4536,28 +4731,33 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W8316075', 'https://openalex.org/W21006490', 'https://openalex.org/W22229905', 'https://openalex.org/W59175527', 'https://openalex.org/W68733909', 'https://openalex.org/W129606432', 'https://openalex.org/W155596317', 'https://openalex.org/W189596042', 'https://openalex.org/W199018803', 'https://openalex.org/W262578090', 'https://openalex.org/W854541894', 'https://openalex.org/W877909479', 'https://openalex.org/W956551720', 'https://openalex.org/W1123427201', 'https://openalex.org/W1480583224', 'https://openalex.org/W1481820510', 'https://openalex.org/W1488163396', 'https://openalex.org/W1503933356', 'https://openalex.org/W1514535095', 'https://openalex.org/W1522301498', 'https://openalex.org/W1523385540', 'https://openalex.org/W1527575280', 'https://openalex.org/W1528056001', 'https://openalex.org/W1533861849', 'https://openalex.org/W1540429825', 'https://openalex.org/W1555767263', 'https://openalex.org/W1566289585', 'https://openalex.org/W1572567476', 'https://openalex.org/W1573040851', 'https://openalex.org/W1586939924', 'https://openalex.org/W1601567445', 'https://openalex.org/W1628307106', 'https://openalex.org/W1651753422', 'https://openalex.org/W1664311846', 'https://openalex.org/W1686810756', 'https://openalex.org/W1687846465', 'https://openalex.org/W1753482797', 'https://openalex.org/W1762503104', 'https://openalex.org/W1766290689', 'https://openalex.org/W1773149199', 'https://openalex.org/W1811254738', 'https://openalex.org/W1822526425', 'https://openalex.org/W1828348983', 'https://openalex.org/W1836465849', 'https://openalex.org/W1858383477', 'https://openalex.org/W1870428314', 'https://openalex.org/W1872883209', 'https://openalex.org/W1883346539', 'https://openalex.org/W1889038981', 'https://openalex.org/W1889081078', 'https://openalex.org/W1893116441', 'https://openalex.org/W1895577753', 'https://openalex.org/W1897761818', 'https://openalex.org/W1905882502', 'https://openalex.org/W1906515132', 'https://openalex.org/W1922557984', 'https://openalex.org/W1931795219', 'https://openalex.org/W1933065844', 'https://openalex.org/W1933349210', 'https://openalex.org/W1956340063', 'https://openalex.org/W1963540633', 'https://openalex.org/W1964073652', 'https://openalex.org/W1966811077', 'https://openalex.org/W1969616664', 'https://openalex.org/W1970055505', 'https://openalex.org/W1971791733', 'https://openalex.org/W1976066595', 'https://openalex.org/W1977547683', 'https://openalex.org/W1985867508', 'https://openalex.org/W1986451414', 'https://openalex.org/W1987835821', 'https://openalex.org/W1996418862', 'https://openalex.org/W1996478295', 'https://openalex.org/W2000911139', 'https://openalex.org/W2003333103', 'https://openalex.org/W2006969979', 'https://openalex.org/W2009059481', 'https://openalex.org/W2012237712', 'https://openalex.org/W2015394094', 'https://openalex.org/W2015412875', 'https://openalex.org/W2019024625', 'https://openalex.org/W2022799064', 'https://openalex.org/W2025341678', 'https://openalex.org/W2025638820', 'https://openalex.org/W2026012689', 'https://openalex.org/W2026243162', 'https://openalex.org/W2038698865', 'https://openalex.org/W2041288440', 'https://openalex.org/W2042608483', 'https://openalex.org/W2048343491', 'https://openalex.org/W2048679005', 'https://openalex.org/W2051721233', 'https://openalex.org/W2053101950', 'https://openalex.org/W2057568625', 'https://openalex.org/W2058616948', 'https://openalex.org/W2061781940', 'https://openalex.org/W2062632672', 'https://openalex.org/W2062955551', 'https://openalex.org/W2063036810', 'https://openalex.org/W2063330527', 'https://openalex.org/W2064675550', 'https://openalex.org/W2066667210', 'https://openalex.org/W2068676460', 'https://openalex.org/W2069682406', 'https://openalex.org/W2077395415', 'https://openalex.org/W2080576537', 'https://openalex.org/W2083885588', 'https://openalex.org/W2090048052', 'https://openalex.org/W2095705004', 'https://openalex.org/W2096391593', 'https://openalex.org/W2098411764', 'https://openalex.org/W2098562545', 'https://openalex.org/W2099471712', 'https://openalex.org/W2100235303', 'https://openalex.org/W2100561338', 'https://openalex.org/W2101105183', 'https://openalex.org/W2101534792', 'https://openalex.org/W2102765684', 'https://openalex.org/W2105103432', 'https://openalex.org/W2106277773', 'https://openalex.org/W2108710284', 'https://openalex.org/W2109586012', 'https://openalex.org/W2109743529', 'https://openalex.org/W2111078031', 'https://openalex.org/W2111645492', 'https://openalex.org/W2112019442', 'https://openalex.org/W2112184938', 'https://openalex.org/W2112912048', 'https://openalex.org/W2113507809', 'https://openalex.org/W2118714046', 'https://openalex.org/W2119288237', 'https://openalex.org/W2120776756', 'https://openalex.org/W2123024445', 'https://openalex.org/W2124033848', 'https://openalex.org/W2124372976', 'https://openalex.org/W2125336414', 'https://openalex.org/W2125366733', 'https://openalex.org/W2126598020', 'https://openalex.org/W2128856065', 'https://openalex.org/W2129142580', 'https://openalex.org/W2129360799', 'https://openalex.org/W2129382193', 'https://openalex.org/W2130055251', 'https://openalex.org/W2130162821', 'https://openalex.org/W2130942839', 'https://openalex.org/W2131179926', 'https://openalex.org/W2133459682', 'https://openalex.org/W2133564696', 'https://openalex.org/W2135776491', 'https://openalex.org/W2136922672', 'https://openalex.org/W2136985729', 'https://openalex.org/W2137735870', 'https://openalex.org/W2137806537', 'https://openalex.org/W2141477623', 'https://openalex.org/W2142192571', 'https://openalex.org/W2142900973', 'https://openalex.org/W2143449221', 'https://openalex.org/W2143492886', 'https://openalex.org/W2143612262', 'https://openalex.org/W2143926884', 'https://openalex.org/W2145056192', 'https://openalex.org/W2147880316', 'https://openalex.org/W2147885303', 'https://openalex.org/W2148298736', 'https://openalex.org/W2149172860', 'https://openalex.org/W2149557440', 'https://openalex.org/W2149940198', 'https://openalex.org/W2150295085', 'https://openalex.org/W2150658333', 'https://openalex.org/W2150696241', 'https://openalex.org/W2150824314', 'https://openalex.org/W2151096985', 'https://openalex.org/W2151103935', 'https://openalex.org/W2152239535', 'https://openalex.org/W2153579005', 'https://openalex.org/W2153927146', 'https://openalex.org/W2156303437', 'https://openalex.org/W2156503193', 'https://openalex.org/W2159973364', 'https://openalex.org/W2160815625', 'https://openalex.org/W2163108352', 'https://openalex.org/W2163605009', 'https://openalex.org/W2163922914', 'https://openalex.org/W2164186291', 'https://openalex.org/W2164450870', 'https://openalex.org/W2164587673', 'https://openalex.org/W2164699598', 'https://openalex.org/W2167103782', 'https://openalex.org/W2173180041', 'https://openalex.org/W2180844455', 'https://openalex.org/W2181691731', 'https://openalex.org/W2184045248', 'https://openalex.org/W2184188583', 'https://openalex.org/W2185175083', 'https://openalex.org/W2201007611', 'https://openalex.org/W2203543769', 'https://openalex.org/W2220981600', 'https://openalex.org/W2250742840', 'https://openalex.org/W2250842428', 'https://openalex.org/W2251353663', 'https://openalex.org/W2251394420', 'https://openalex.org/W2251885125', 'https://openalex.org/W2251970440', 'https://openalex.org/W2252122141', 'https://openalex.org/W2252238675', 'https://openalex.org/W2266728343', 'https://openalex.org/W2267126114', 'https://openalex.org/W2282219577', 'https://openalex.org/W2291822808', 'https://openalex.org/W2293453011', 'https://openalex.org/W2294797155', 'https://openalex.org/W2296613712', 'https://openalex.org/W2316138215', 'https://openalex.org/W2327501763', 'https://openalex.org/W2342662179', 'https://openalex.org/W2388114291', 'https://openalex.org/W2397159106', 'https://openalex.org/W2399507222', 'https://openalex.org/W2399733683', 'https://openalex.org/W2402955625', 'https://openalex.org/W2405756170', 'https://openalex.org/W2411037331', 'https://openalex.org/W2418349398', 'https://openalex.org/W2434537049', 'https://openalex.org/W2462496837', 'https://openalex.org/W2470413457', 'https://openalex.org/W2489434015', 'https://openalex.org/W2494980014', 'https://openalex.org/W2519091744', 'https://openalex.org/W2519656895', 'https://openalex.org/W2520160253', 'https://openalex.org/W2546919788', 'https://openalex.org/W2557865186', 'https://openalex.org/W2579317665', 'https://openalex.org/W2914699769', 'https://openalex.org/W2949465329', 'https://openalex.org/W2953318193', 'https://openalex.org/W2962706528', 'https://openalex.org/W2962756039', 'https://openalex.org/W2962835968', 'https://openalex.org/W2963082528', 'https://openalex.org/W2963109634', 'https://openalex.org/W2963143316', 'https://openalex.org/W2963192057', 'https://openalex.org/W2963260436', 'https://openalex.org/W2963324994', 'https://openalex.org/W2963383024', 'https://openalex.org/W2963389687', 'https://openalex.org/W2963410018', 'https://openalex.org/W2963576560', 'https://openalex.org/W2963579811', 'https://openalex.org/W2963605190', 'https://openalex.org/W2963656855', 'https://openalex.org/W2963735856', 'https://openalex.org/W2963811219', 'https://openalex.org/W2963899908', 'https://openalex.org/W2963954913', 'https://openalex.org/W2964040984', 'https://openalex.org/W2964118342', 'https://openalex.org/W2964121744', 'https://openalex.org/W2964217371', 'https://openalex.org/W2964241990', 'https://openalex.org/W2964308564', 'https://openalex.org/W2964345931', 'https://openalex.org/W3000384245', 'https://openalex.org/W3023993913', 'https://openalex.org/W3087871082', 'https://openalex.org/W3125032682', 'https://openalex.org/W4211232216', 'https://openalex.org/W4212844288', 'https://openalex.org/W4240592325', 'https://openalex.org/W4244018879', 'https://openalex.org/W4245655784', 'https://openalex.org/W4252331534', 'https://openalex.org/W4285719527', 'https://openalex.org/W4293665662', 'https://openalex.org/W4294170691', 'https://openalex.org/W4297813007', 'https://openalex.org/W4299801216', 'https://openalex.org/W4302613066', 'https://openalex.org/W4320013936', 'https://openalex.org/W6600334730', 'https://openalex.org/W6600827882', 'https://openalex.org/W6605295763', 'https://openalex.org/W6606244218', 'https://openalex.org/W6606327593', 'https://openalex.org/W6607775107', 'https://openalex.org/W6608183366', 'https://openalex.org/W6623517193', 'https://openalex.org/W6623995992', 'https://openalex.org/W6625044600', 'https://openalex.org/W6628794645', 'https://openalex.org/W6629203210', 'https://openalex.org/W6630875275', 'https://openalex.org/W6631190155', 'https://openalex.org/W6631216910', 'https://openalex.org/W6631516269', 'https://openalex.org/W6631943919', 'https://openalex.org/W6634126550', 'https://openalex.org/W6636447180', 'https://openalex.org/W6636942303', 'https://openalex.org/W6637306801', 'https://openalex.org/W6637373629', 'https://openalex.org/W6637698695', 'https://openalex.org/W6637971603', 'https://openalex.org/W6637989529', 'https://openalex.org/W6638549007', 'https://openalex.org/W6638667902', 'https://openalex.org/W6638742206', 'https://openalex.org/W6639103823', 'https://openalex.org/W6639118148', 'https://openalex.org/W6639283537', 'https://openalex.org/W6639358663', 'https://openalex.org/W6639432524', 'https://openalex.org/W6639434097', 'https://openalex.org/W6640257717', 'https://openalex.org/W6640296258', 'https://openalex.org/W6640764460', 'https://openalex.org/W6650605322', 'https://openalex.org/W6652311901', 'https://openalex.org/W6674330103', 'https://openalex.org/W6675048546', 'https://openalex.org/W6676380891', 'https://openalex.org/W6676497082', 'https://openalex.org/W6676647902', 'https://openalex.org/W6676709516', 'https://openalex.org/W6678360021', 'https://openalex.org/W6678470764', 'https://openalex.org/W6678809451', 'https://openalex.org/W6679434410', 'https://openalex.org/W6679436768', 'https://openalex.org/W6680094886', 'https://openalex.org/W6680336390', 'https://openalex.org/W6681184217', 'https://openalex.org/W6682082992', 'https://openalex.org/W6682086108', 'https://openalex.org/W6682222085', 'https://openalex.org/W6682511423', 'https://openalex.org/W6682691769', 'https://openalex.org/W6682864246', 'https://openalex.org/W6683074461', 'https://openalex.org/W6683167905', 'https://openalex.org/W6683277684', 'https://openalex.org/W6684191040', 'https://openalex.org/W6684209796', 'https://openalex.org/W6685183736', 'https://openalex.org/W6685527872', 'https://openalex.org/W6686207219', 'https://openalex.org/W6687543112', 'https://openalex.org/W6687672932', 'https://openalex.org/W6688143368', 'https://openalex.org/W6691419566', 'https://openalex.org/W6691647468', 'https://openalex.org/W6692004142', 'https://openalex.org/W6696843773', 'https://openalex.org/W6697449767', 'https://openalex.org/W6712426025', 'https://openalex.org/W6712802073', 'https://openalex.org/W6713645886', 'https://openalex.org/W6717487601', 'https://openalex.org/W6726977916', 'https://openalex.org/W6727336983', 'https://openalex.org/W6729831399', 'https://openalex.org/W6730042849', 'https://openalex.org/W6730666313', 'https://openalex.org/W6732843983', 'https://openalex.org/W6845679800', 'https://openalex.org/W6898505805', 'https://openalex.org/W7011438494']</t>
+          <t>['GB', 'US']</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr">
+          <t>['Glorot X, 2010, ', 'Zhu Y, 2015, ', 'Salakhutdinov R, 2009, ', 'Plummer B, 2015, ', 'Kalchbrenner N, 2013, ', 'Hodosh M, 2013, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Andrew G, 2013, ', 'Ghahramani Z, 1997, MACHINE LEARNING', 'Yao L, 2015, ', 'Sutton C, 2007, THE MIT PRESS EBOOKS', 'Weston J, 2011, ', 'Pan Y, 2016, ', 'Wang W, 2015, ', 'Kumar S, 2012, ', 'Mitchell M, 2012, CONFERENCE OF THE EUROPEAN CHAPTER OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Louwerse M, 2010, TOPICS IN COGNITIVE SCIENCE', 'Kahou S, 2015, JOURNAL ON MULTIMODAL USER INTERFACES', 'Gregory K, 2014, IT UNIVERSITY OF COPENHAGEN (IT UNIVERSITY OF COPENHAGEN)', 'Li S, 2011, ', 'Kojima A, 2002, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Yang Y, 2011, ', 'Xu R, 2015, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Castellano G, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Mroueh Y, 2015, ', 'Glodek M, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Cour T, 2008, LECTURE NOTES IN COMPUTER SCIENCE', 'Gupta A, 2021, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Morvant E, 2014, LECTURE NOTES IN COMPUTER SCIENCE', 'Bojanowski P, 2015, ', 'Feng Y, 2010, EDINBURGH RESEARCH EXPLORER (UNIVERSITY OF EDINBURGH)', 'Wei Y, 2016, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Chen Y, 2004, ', 'Sjölander K, 2003, ', 'Wu Z, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Naim I, 2014, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Khapra M, 2010, ', 'Deena S, 2009, LECTURE NOTES IN COMPUTER SCIENCE', 'Kingma D, 2014, UVA-DARE (UNIVERSITY OF AMSTERDAM)', 'Simonyan K, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ioffe S, 2015, ARXIV (CORNELL UNIVERSITY)', 'Xu K, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chorowski J, 2015, ARXIV (CORNELL UNIVERSITY)', 'Chen X, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kiros R, 2014, ARXIV (CORNELL UNIVERSITY)', 'Mao J, 2014, ARXIV (CORNELL UNIVERSITY)', 'Gao H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Torabi A, 2015, ARXIV (CORNELL UNIVERSITY)', 'McFee B, 2010, ARXIV (CORNELL UNIVERSITY)', 'Christoudias C, 2012, ARXIV (CORNELL UNIVERSITY)', 'Lebret R, 2015, ARXIV (CORNELL UNIVERSITY)', 'Vinyals O, 2015, ', 'McGurk H, 1976, NATURE', 'Blum A, 1998, ', 'Hotelling H, 1936, BIOMETRIKA', 'Karpathy A, 2015, ', 'Vedantam R, 2015, ', 'Antol S, 2015, ', 'Brown P, 1993, ', 'Farhadi A, 2010, LECTURE NOTES IN COMPUTER SCIENCE', 'Atrey P, 2010, MULTIMEDIA SYSTEMS', 'Kulkarni G, 2013, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Vogel S, 1996, ', 'Juang B, 1991, TECHNOMETRICS', 'D’Mello S, 2015, ACM COMPUTING SURVEYS', 'Feng F, 2014, ', 'Valstar M, 2013, ', 'Bronstein M, 2010, ', 'Kim Y, 2013, ', 'Lienhart R, 1998, PROCEEDINGS OF SPIE, THE INTERNATIONAL SOCIETY FOR OPTICAL ENGINEERING/PROCEEDINGS OF SPIE', 'Kruskal J, 1983, SIAM REVIEW', 'Yao B, 2010, PROCEEDINGS OF THE IEEE', 'Wöllmer M, 2012, IMAGE AND VISION COMPUTING', 'Ouyang W, 2014, ', 'Evangelopoulos G, 2013, IEEE TRANSACTIONS ON MULTIMEDIA', 'Socher R, 2010, ', 'Li Y, 2014, NEUROCOMPUTING', 'Zitnick C, 2013, ', 'Kong C, 2014, ', 'Huang J, 2013, ', 'Sargin M, 2007, IEEE TRANSACTIONS ON MULTIMEDIA', 'Zhou F, 2012, ', 'Mei H, 2016, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Liu F, 2013, IEEE JOURNAL OF BIOMEDICAL AND HEALTH INFORMATICS', 'Rohrbach A, 2015, LECTURE NOTES IN COMPUTER SCIENCE', 'Chen S, 2015, ', 'Sarah T, 2012, ', 'Baltrušaitis T, 2013, ', 'Chen J, 2014, ', 'Zen H, 2012, IEEE TRANSACTIONS ON AUDIO SPEECH AND LANGUAGE PROCESSING', 'Tapaswi M, 2015, ', 'Arora R, 2013, ', 'Feng F, 2014, NEUROCOMPUTING', 'Bourlard H, 2002, ', 'Yeh Y, 2012, IEEE TRANSACTIONS ON MULTIMEDIA', 'Noulas A, 2011, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Jiang X, 2014, PATTERN RECOGNITION LETTERS', 'Haubold A, 2007, ', 'Tapaswi M, 2014, INTERNATIONAL JOURNAL OF MULTIMEDIA INFORMATION RETRIEVAL', 'Wu D, 2014, ', 'Klein B, 2014, ARXIV (CORNELL UNIVERSITY)', 'Hochreiter S, 1997, NEURAL COMPUTATION', 'Srivastava N, 2014, ', '淳司 柴, 2017, JOURNAL OF JAPAN SOCIETY FOR FUZZY THEORY AND INTELLIGENT INFORMATICS', 'Papineni K, 2001, ', 'Hinton G, 2006, NEURAL COMPUTATION', 'Hardoon D, 2004, NEURAL COMPUTATION', 'Denkowski M, 2014, ', 'Frome A, 2013, ', 'Farhadi A, 2009, 2009 IEEE CONFERENCE ON COMPUTER VISION AND PATTERN RECOGNITION', 'Gönen M, 2011, ', 'Rasiwasia N, 2010, ', 'Zen H, 2009, SPEECH COMMUNICATION', 'Suk H, 2014, NEUROIMAGE', 'Ordóñez V, 2011, ', 'James A, 2014, INFORMATION FUSION', 'Bruni E, 2014, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Carletta J, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Gehler P, 2009, ', 'Pomianos G, 2003, PROCEEDINGS OF THE IEEE', 'Bigham J, 2010, ', 'Lai P, 2000, INTERNATIONAL JOURNAL OF NEURAL SYSTEMS', 'Quattoni A, 2007, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Regneri M, 2013, TRANSACTIONS OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Snoek C, 2004, MULTIMEDIA TOOLS AND APPLICATIONS', 'Anagnostopoulos C, 2012, ARTIFICIAL INTELLIGENCE REVIEW', 'Weston J, 2010, MACHINE LEARNING', 'Coyne B, 2001, ', 'Bucak S, 2014, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'McKeown G, 2010, ', 'Schuller B, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Devlin J, 2015, ', 'Bojanowski P, 2014, LECTURE NOTES IN COMPUTER SCIENCE', 'Wu Z, 2014, ', 'Elliott D, 2014, ', 'Mason R, 2014, ', 'Ramírez G, 2011, LECTURE NOTES IN COMPUTER SCIENCE', 'Anderson R, 2013, ', 'Song Y, 2012, ', 'Slaney M, 2000, NEURAL INFORMATION PROCESSING SYSTEMS', 'Lan Z, 2013, MULTIMEDIA TOOLS AND APPLICATIONS', 'Chang A, 2015, ', 'Gurban M, 2008, ', 'Krogel M, 2004, MACHINE LEARNING', 'Garg A, 2003, PROCEEDINGS OF THE IEEE', 'Christoudias C, 2006, ', 'Cosi P, 2002, ', 'Bahdanau D, 2014, ARXIV (CORNELL UNIVERSITY)', 'Sutskever I, 2014, ARXIV (CORNELL UNIVERSITY)', 'Socher R, 2013, ARXIV (CORNELL UNIVERSITY)', 'Karpathy A, 2014, ARXIV (CORNELL UNIVERSITY)', 'Krizhevsky A, 2017, COMMUNICATIONS OF THE ACM', 'Lowe D, 2004, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Lafferty J, 2001, SCHOLARLY COMMONS (UNIVERSITY OF PENNSYLVANIA)', 'Bengio Y, 2013, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Hinton G, 2012, IEEE SIGNAL PROCESSING MAGAZINE', 'Graves A, 2013, ', 'Zeng Z, 2008, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Young P, 2014, TRANSACTIONS OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Ngiam J, 2011, ', 'Hinton G, 2012, ', 'Lin C, 2003, ', 'Hunt A, 2002, ', 'Brand M, 2002, ', 'Socher R, 2014, TRANSACTIONS OF THE ASSOCIATION FOR COMPUTATIONAL LINGUISTICS', 'Palatucci M, 2018, FIGSHARE', 'Soleymani M, 2011, IEEE TRANSACTIONS ON AFFECTIVE COMPUTING', 'Bregler C, 1997, ', 'Zhang D, 2014, PROCEEDINGS OF THE AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Malinowski M, 2015, ', 'Guadarrama S, 2013, ', 'Nicolaou M, 2011, IEEE TRANSACTIONS ON AFFECTIVE COMPUTING', 'Jia X, 2015, ', 'Harvey D, 2009, ', 'Bruni E, 2012, INSTITUTIONAL RESEARCH INFORMATION SYSTEM (UNIVERSITÀ DEGLI STUDI DI TRENTO)', 'Кузнецова П, 2012, ', 'Hendricks L, 2016, ', 'Elliott D, 2013, ', 'Kiela D, 2014, ', 'Левин, 2003, ', 'Silberer C, 2014, ', 'Nefian A, 2002, IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS SPEECH AND SIGNAL PROCESSING', 'Yuhas B, 1989, IEEE COMMUNICATIONS MAGAZINE', 'Wöllmer M, 2010, ', 'Zhou F, 2009, ', 'Thomason J, 2014, ', 'Sikka K, 2013, ', 'Qin T, 2008, ', 'Yu H, 2013, ', 'Wang D, 2015, INTERNATIONAL CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Sarkar A, 2001, ', 'Song Y, 2012, ', 'Nakov P, 2012, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Yagcioglu S, 2015, ', 'Shariat S, 2011, ', 'Masuko T, 2002, ', 'Reiter S, 2007, ', 'Mikolov T, 2013, ARXIV (CORNELL UNIVERSITY)', 'Simonyan K, 2014, ARXIV (CORNELL UNIVERSITY)', 'Ratnaparkhi A, 2000, ARXIV.ORG', 'Feichtenhofer C, 2016, ', 'Chan W, 2016, ', 'Fukui A, 2016, ', 'Mao J, 2016, ', 'Yu L, 2016, LECTURE NOTES IN COMPUTER SCIENCE', 'Jiang Q, 2017, ', 'Trigeorgis G, 2016, ', 'Wang L, 2016, ', 'Yu H, 2016, ', 'Poria S, 2015, ', 'Müller M, 2008, ', 'Fan Y, 2014, ', 'Bernardi R, 2016, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Rohrbach A, 2017, INTERNATIONAL JOURNAL OF COMPUTER VISION', ', 2009, ENCYCLOPEDIA OF BIOMETRICS', 'Cao Y, 2016, ', 'Nojavanasghari B, 2016, ', 'Shutova E, 2016, ', 'Srivastava N, 2012, ', 'Mahasseni B, 2016, ', 'Rajagopalan S, 2016, LECTURE NOTES IN COMPUTER SCIENCE', 'Gebru I, 2017, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Baroni M, 2015, LANGUAGE AND LINGUISTICS COMPASS', 'Lazaridou A, 2014, ', 'Kiela D, 2015, ', 'Silberer C, 2012, EDINBURGH RESEARCH EXPLORER (UNIVERSITY OF EDINBURGH)', 'Gao H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kiela D, 2015, ', 'Trigeorgis G, 2016, ', 'Jin Q, 2016, ', 'Song Y, 2016, INTERNATIONAL JOINT CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Naim I, 2015, ', 'Anguera X, 2014, ', 'Moon S, 2014, ', 'Oord A, 2016, ARXIV (CORNELL UNIVERSITY)', 'Reed S, 2016, ARXIV (CORNELL UNIVERSITY)', 'Oord A, 2016, ARXIV (CORNELL UNIVERSITY)', 'Xiong C, 2016, ARXIV (CORNELL UNIVERSITY)', 'Oord A, 2016, ARXIV (CORNELL UNIVERSITY)', 'Collobert R, 2016, ARXIV (CORNELL UNIVERSITY)', 'Lu J, 2016, ARXIV (CORNELL UNIVERSITY)', 'Kuan-Lin C, 2021, DROPS (SCHLOSS DAGSTUHL – LEIBNIZ CENTER FOR INFORMATICS)', 'Labaca-Castro R, 2023, ', 'Barsalou L, 2007, ANNUAL REVIEW OF PSYCHOLOGY', 'Yang Z, 2016, ', ', 2007, ', 'Xu H, 2016, LECTURE NOTES IN COMPUTER SCIENCE', 'Juang B, 1991, TECHNOMETRICS', 'Hu R, 2016, ', 'Xiong C, 2016, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Huang T, 2016, ', 'Zeng K, 2017, ', 'Torre F, 2011, ', 'Nefian, 2002, IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS SPEECH AND SIGNAL PROCESSING', 'McFeeBrian, 2011, JOURNAL OF MACHINE LEARNING RESEARCH', 'Bourlard H, 1996, 4TH INTERNATIONAL CONFERENCE ON SPOKEN LANGUAGE PROCESSING (ICSLP 1996)', 'Zhang H, 2016, ', 'Ghahramani Z, 1996, ', 'Mei H, 2015, ARXIV (CORNELL UNIVERSITY)', 'Klein B, 2014, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>Tadas Baltrušaitis, 2018, IEEE Transactions on Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>Tadas Baltrušaitis, 2018, IEEE Transactions on Pattern Analysis and Machine Intelligence</t>
+          <t>Baltrušaitis T, 2018, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Baltrušaitis T, 2018, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4791,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>5107</v>
+        <v>5100</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -4647,28 +4847,33 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W4952878', 'https://openalex.org/W28669376', 'https://openalex.org/W44815768', 'https://openalex.org/W1128809682', 'https://openalex.org/W1484413656', 'https://openalex.org/W1484780623', 'https://openalex.org/W1491541693', 'https://openalex.org/W1498810706', 'https://openalex.org/W1508065755', 'https://openalex.org/W1515231270', 'https://openalex.org/W1543320899', 'https://openalex.org/W1566114229', 'https://openalex.org/W1570448133', 'https://openalex.org/W1594031697', 'https://openalex.org/W1629143244', 'https://openalex.org/W1673310716', 'https://openalex.org/W1806329564', 'https://openalex.org/W1912123407', 'https://openalex.org/W1917795079', 'https://openalex.org/W1927026191', 'https://openalex.org/W1948199107', 'https://openalex.org/W1965702297', 'https://openalex.org/W1967661515', 'https://openalex.org/W1974016210', 'https://openalex.org/W1977496278', 'https://openalex.org/W1981276685', 'https://openalex.org/W1982582425', 'https://openalex.org/W1989344766', 'https://openalex.org/W1990517717', 'https://openalex.org/W2015057666', 'https://openalex.org/W2018936209', 'https://openalex.org/W2026513874', 'https://openalex.org/W2058401212', 'https://openalex.org/W2064853889', 'https://openalex.org/W2069140227', 'https://openalex.org/W2071128523', 'https://openalex.org/W2083620785', 'https://openalex.org/W2088093492', 'https://openalex.org/W2090991262', 'https://openalex.org/W2097117768', 'https://openalex.org/W2099404336', 'https://openalex.org/W2099940443', 'https://openalex.org/W2101234009', 'https://openalex.org/W2106393550', 'https://openalex.org/W2107726111', 'https://openalex.org/W2109255472', 'https://openalex.org/W2112076978', 'https://openalex.org/W2112796928', 'https://openalex.org/W2119567691', 'https://openalex.org/W2120240539', 'https://openalex.org/W2120636621', 'https://openalex.org/W2127218421', 'https://openalex.org/W2132166479', 'https://openalex.org/W2134089414', 'https://openalex.org/W2140190241', 'https://openalex.org/W2142827986', 'https://openalex.org/W2143554828', 'https://openalex.org/W2144219012', 'https://openalex.org/W2147169507', 'https://openalex.org/W2149706766', 'https://openalex.org/W2151040995', 'https://openalex.org/W2154298720', 'https://openalex.org/W2160642098', 'https://openalex.org/W2163605009', 'https://openalex.org/W2164500538', 'https://openalex.org/W2166559705', 'https://openalex.org/W2194775991', 'https://openalex.org/W2215376118', 'https://openalex.org/W2257979135', 'https://openalex.org/W2294798173', 'https://openalex.org/W2296509296', 'https://openalex.org/W2341117600', 'https://openalex.org/W2394309960', 'https://openalex.org/W2395579298', 'https://openalex.org/W2504658994', 'https://openalex.org/W2510496529', 'https://openalex.org/W2518882834', 'https://openalex.org/W2531409750', 'https://openalex.org/W2557283755', 'https://openalex.org/W2580909119', 'https://openalex.org/W2581465409', 'https://openalex.org/W2603678388', 'https://openalex.org/W2609368436', 'https://openalex.org/W2617585083', 'https://openalex.org/W2617697157', 'https://openalex.org/W2622382573', 'https://openalex.org/W2713640100', 'https://openalex.org/W2724111113', 'https://openalex.org/W2752236180', 'https://openalex.org/W2762644836', 'https://openalex.org/W2771053518', 'https://openalex.org/W2802574842', 'https://openalex.org/W2803881474', 'https://openalex.org/W2806407311', 'https://openalex.org/W2889193967', 'https://openalex.org/W2904346290', 'https://openalex.org/W2906027675', 'https://openalex.org/W2909445826', 'https://openalex.org/W2910891387', 'https://openalex.org/W2911964244', 'https://openalex.org/W2912934387', 'https://openalex.org/W2913771179', 'https://openalex.org/W2940523548', 'https://openalex.org/W2950722229', 'https://openalex.org/W2954936648', 'https://openalex.org/W2955285339', 'https://openalex.org/W2960015156', 'https://openalex.org/W2962824709', 'https://openalex.org/W2963748489', 'https://openalex.org/W2971145443', 'https://openalex.org/W2982291760', 'https://openalex.org/W2990933508', 'https://openalex.org/W2991970757', 'https://openalex.org/W2998019206', 'https://openalex.org/W2998574808', 'https://openalex.org/W2999729612', 'https://openalex.org/W3002041203', 'https://openalex.org/W3003734944', 'https://openalex.org/W3007397514', 'https://openalex.org/W3011204221', 'https://openalex.org/W3014867431', 'https://openalex.org/W3016540417', 'https://openalex.org/W3017881119', 'https://openalex.org/W3019166713', 'https://openalex.org/W3023402713', 'https://openalex.org/W3034560014', 'https://openalex.org/W3037163353', 'https://openalex.org/W3038955483', 'https://openalex.org/W3039828206', 'https://openalex.org/W3041463877', 'https://openalex.org/W3044397306', 'https://openalex.org/W3044730720', 'https://openalex.org/W3049757379', 'https://openalex.org/W3083228182', 'https://openalex.org/W3084246142', 'https://openalex.org/W3085162807', 'https://openalex.org/W3086286002', 'https://openalex.org/W3095217282', 'https://openalex.org/W3099185017', 'https://openalex.org/W3100378204', 'https://openalex.org/W3102116369', 'https://openalex.org/W3121263745', 'https://openalex.org/W3122594683', 'https://openalex.org/W3129290453', 'https://openalex.org/W3130145150', 'https://openalex.org/W3139008799', 'https://openalex.org/W3149084432', 'https://openalex.org/W4212883601', 'https://openalex.org/W4230470477', 'https://openalex.org/W4236137412', 'https://openalex.org/W4244238212', 'https://openalex.org/W4245160364', 'https://openalex.org/W4298023569', 'https://openalex.org/W4298882835', 'https://openalex.org/W6601142415', 'https://openalex.org/W6674887505', 'https://openalex.org/W6675354045', 'https://openalex.org/W6675567579', 'https://openalex.org/W6676769703', 'https://openalex.org/W6843735874']</t>
+          <t>['BD', 'AU']</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr">
+          <t>['LeCun Y, 1998, PROCEEDINGS OF THE IEEE', 'Szegedy C, 2015, ', 'Witten I, 2011, ELSEVIER EBOOKS', 'Gordon A, 1984, BIOMETRICS', 'Cios K, 1997, NEUROCOMPUTING', 'Ester M, 1996, ', 'He K, 2015, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Agrawal R, 1998, ', 'Hotelling H, 1933, JOURNAL OF EDUCATIONAL PSYCHOLOGY', 'Kaelbling L, 1996, JOURNAL OF ARTIFICIAL INTELLIGENCE RESEARCH', 'Hazeghi K, 1995, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Kohonen T, 1990, PROCEEDINGS OF THE IEEE', 'Freund Y, 1996, ', 'Han J, 2000, ACM SIGMOD RECORD', 'Zanella A, 2014, IEEE INTERNET OF THINGS JOURNAL', 'Dey A, 2001, PERSONAL AND UBIQUITOUS COMPUTING', 'Tavallaee M, 2009, ', 'Hinton G, 2012, LECTURE NOTES IN COMPUTER SCIENCE', 'Agrawal R, 1998, ', 'Park H, 2008, EXPERT SYSTEMS WITH APPLICATIONS', 'Xu D, 2015, ANNALS OF DATA SCIENCE', 'Zaki M, 2000, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Cessie S, 1992, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Amit Y, 1997, NEURAL COMPUTATION', 'Wang W, 1997, ', ', 1993, CHOICE REVIEWS ONLINE', 'Sneath P, 1957, MICROBIOLOGY', 'MTW, 1999, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Witten I, 1999, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Bishop C, 2007, ', 'Houtsma M, 2002, ', 'Agrawal R, 1998, KNOWLEDGE DISCOVERY AND DATA MINING', 'Rokach L, 2009, ', 'Zheng Y, 2015, ', 'Scheffer T, 2001, LECTURE NOTES IN COMPUTER SCIENCE', 'Zhu H, 2014, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Zhao Q, 2003, PALLIATIVE &amp; SUPPORTIVE CARE', 'Flach P, 2001, MACHINE LEARNING', 'Cobuloglu H, 2015, EXPERT SYSTEMS WITH APPLICATIONS', 'McCallum A, 2005, QUEUE', 'Das A, 2001, ', 'Phithakkitnukoon S, 2011, ACM TRANSACTIONS ON AUTONOMOUS AND ADAPTIVE SYSTEMS', 'Zhu H, 2012, ', 'Zulkernain S, 2010, E-PUBLICATIONS@MARQUETTE (MARQUETTE UNIVERSITY)', 'Amorim R, 2012, ', 'Sheng S, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Bell A, 2005, QUEUE', 'Zulkernain S, 2010, LECTURE NOTES OF THE INSTITUTE FOR COMPUTER SCIENCES, SOCIAL INFORMATICS AND TELECOMMUNICATIONS ENGINEERING', 'Pedregosa F, 2012, ARXIV (CORNELL UNIVERSITY)', 'John G, 2013, ARXIV (CORNELL UNIVERSITY)', 'He K, 2016, ', 'Breiman L, 2001, MACHINE LEARNING', 'Krizhevsky A, 2017, COMMUNICATIONS OF THE ACM', 'Han J, 2012, CHOICE REVIEWS ONLINE', 'MacQueen J, 1967, DEFENSE TECHNICAL INFORMATION CENTER (DTIC)', 'Chollet F, 2017, ', 'Silver D, 2016, NATURE', 'Quinlan J, 1986, MACHINE LEARNING', 'Agrawal R, 1993, ', 'Pearson K, 1901, THE LONDON EDINBURGH AND DUBLIN PHILOSOPHICAL MAGAZINE AND JOURNAL OF SCIENCE', 'Goodfellow I, 2016, MIT PRESS EBOOKS', 'Weiss K, 2016, JOURNAL OF BIG DATA', 'Wu X, 2007, KNOWLEDGE AND INFORMATION SYSTEMS', 'Aha D, 1991, MACHINE LEARNING', 'Ankerst M, 1999, ACM SIGMOD RECORD', 'Moustafa N, 2015, ', 'Fukunaga K, 1975, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Eagle N, 2005, PERSONAL AND UBIQUITOUS COMPUTING', 'Carpenter G, 1987, COMPUTER VISION GRAPHICS AND IMAGE PROCESSING', 'Wagstaff K, 2001, ', 'Keerthi S, 2001, NEURAL COMPUTATION', 'Holte R, 1993, MACHINE LEARNING', 'Kamble S, 2018, PROCESS SAFETY AND ENVIRONMENTAL PROTECTION', 'Ravi K, 2015, KNOWLEDGE-BASED SYSTEMS', 'Xin Y, 2018, IEEE ACCESS', 'Rasmussen C, 1999, ', 'Mahdavinejad M, 2017, DIGITAL COMMUNICATIONS AND NETWORKS', 'Fatima M, 2017, JOURNAL OF INTELLIGENT LEARNING SYSTEMS AND APPLICATIONS', 'Ibáñez J, 2018, SENSORS', 'Liu H, 1998, ', 'Polydoros A, 2017, JOURNAL OF INTELLIGENT &amp; ROBOTIC SYSTEMS', 'Ślusarczyk B, 2018, POLISH JOURNAL OF MANAGEMENT STUDIES', 'Ismail A, 2019, JOURNAL OF BIG DATA', 'López G, 2017, ADVANCES IN INTELLIGENT SYSTEMS AND COMPUTING', 'Lade P, 2017, IEEE INTELLIGENT SYSTEMS', 'Mohammed M, 2016, ', 'Balducci F, 2018, MACHINES', 'Nilashi M, 2017, COMPUTERS &amp; CHEMICAL ENGINEERING', 'Safdar S, 2017, ARTIFICIAL INTELLIGENCE REVIEW', 'Srinivasan V, 2014, ', 'Mehrotra A, 2016, ', 'Sarker I, 2017, THE COMPUTER JOURNAL', 'Perveen S, 2018, IEEE ACCESS', 'Adnan N, 2017, WORLD JOURNAL OF SCIENCE TECHNOLOGY AND SUSTAINABLE DEVELOPMENT', 'Cai J, 2003, ', 'Essien A, 2019, ', 'Wu C, 2016, APPLIED INTELLIGENCE', 'Sarker I, 2016, ', 'Cao L, 2020, ARXIV (CORNELL UNIVERSITY)', 'Ryzin J, 1986, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Breiman L, 1996, MACHINE LEARNING', 'Breiman L, 1996, MACHINE LEARNING', 'Quinlan J, 1986, MACHINE LEARNING', ', 1991, CHOICE REVIEWS ONLINE', 'Agrawal R, 1993, ACM SIGMOD RECORD', 'Saeid M, 2017, VIEW', 'Kamble S, 2019, INTERNATIONAL JOURNAL OF PRODUCTION ECONOMICS', 'Lalmuanawma S, 2020, CHAOS SOLITONS &amp; FRACTALS', 'Sharma R, 2020, COMPUTERS &amp; OPERATIONS RESEARCH', 'Sarker I, 2020, JOURNAL OF BIG DATA', 'Agrawal R, 1998, ACM SIGMOD RECORD', 'Harmon S, 2020, NATURE COMMUNICATIONS', 'Jamshidi M, 2020, IEEE ACCESS', 'Sarker I, 2021, SN COMPUTER SCIENCE', 'Fujiyoshi H, 2019, IATSS RESEARCH', 'Kalan A, 2020, NATURE COMMUNICATIONS', 'Zheng T, 2016, INTERNATIONAL JOURNAL OF MEDICAL INFORMATICS', 'Ardabili S, 2020, ALGORITHMS', 'Alakuş T, 2020, CHAOS SOLITONS &amp; FRACTALS', 'Mohamadou Y, 2020, APPLIED INTELLIGENCE', 'Shorten C, 2021, JOURNAL OF BIG DATA', 'Sarker I, 2020, SYMMETRY', 'Boukerche A, 2020, COMPUTER NETWORKS', 'Sarker I, 2019, JOURNAL OF BIG DATA', 'Sarker I, 2021, SN COMPUTER SCIENCE', 'Tao J, 2020, JOURNAL OF BIG DATA', 'Sarker I, 2020, MOBILE NETWORKS AND APPLICATIONS', 'Essien A, 2020, WORLD WIDE WEB', 'Kushwaha S, 2020, JOURNAL OF INDUSTRIAL INTEGRATION AND MANAGEMENT', 'Wei P, 2019, IEEE ACCESS', 'Sarker I, 2019, MOBILE NETWORKS AND APPLICATIONS', 'Sarker I, 2019, INTERNET OF THINGS', 'Sarker I, 2019, JOURNAL OF BIG DATA', 'Tsagkias M, 2020, ACM SIGIR FORUM', 'Marchand A, 2020, JOURNAL OF RETAILING', 'Sarker I, 2020, JOURNAL OF NETWORK AND COMPUTER APPLICATIONS', 'Sarker I, 2020, SYMMETRY', 'Scheffer T, 2005, INTELLIGENT DATA ANALYSIS', 'Sarker I, 2019, INTERNET OF THINGS', 'Sarker I, 2020, JOURNAL OF BIG DATA', 'Khadse V, 2018, ', 'Zi-kang H, 2020, ', 'Sarker I, 2021, PREPRINTS.ORG', 'Sarker I, 2021, PREPRINTS.ORG', 'Sarle W, 1991, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Aha D, 1991, MACHINE LEARNING', 'Baxter L, 1995, TECHNOMETRICS', 'Mohammed M, 2016, ']</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>Iqbal H. Sarker, 2021, SN Computer Science</t>
-        </is>
-      </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>Iqbal H. Sarker, 2021, SN Computer Science</t>
+          <t>Sarker I, 2021, SN COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Sarker I, 2021, SN COMPUTER SCIENCE</t>
         </is>
       </c>
     </row>
@@ -4746,28 +4951,33 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W4919037', 'https://openalex.org/W2112796928', 'https://openalex.org/W2590796488']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr">
+          <t>['LeCun Y, 1998, PROCEEDINGS OF THE IEEE', 'Wan L, 2013, INTERNATIONAL REVIEW OF CYTOLOGY', 'Cohen G, 2017, ARXIV (CORNELL UNIVERSITY)']</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr"/>
+      <c r="X42" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>Xiao Han, 2017, arXiv (Cornell University)</t>
-        </is>
-      </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>Xiao Han, 2017, arXiv (Cornell University)</t>
+          <t>Xiao H, 2017, ARXIV (CORNELL UNIVERSITY)</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Xiao H, 2017, ARXIV (CORNELL UNIVERSITY)</t>
         </is>
       </c>
     </row>
@@ -4841,18 +5051,23 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr">
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr"/>
+      <c r="X43" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr">
+      <c r="Y43" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2008, </t>
         </is>
       </c>
-      <c r="Y43" t="inlineStr">
+      <c r="Z43" t="inlineStr">
         <is>
           <t xml:space="preserve">NA, 2008, </t>
         </is>
@@ -4936,28 +5151,33 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W5472403', 'https://openalex.org/W135311109', 'https://openalex.org/W177590838', 'https://openalex.org/W203696055', 'https://openalex.org/W1007293483', 'https://openalex.org/W1497605902', 'https://openalex.org/W1506588750', 'https://openalex.org/W1515851193', 'https://openalex.org/W1520605446', 'https://openalex.org/W1522114398', 'https://openalex.org/W1528113134', 'https://openalex.org/W1537143578', 'https://openalex.org/W1538041071', 'https://openalex.org/W1547833367', 'https://openalex.org/W1554309553', 'https://openalex.org/W1560955742', 'https://openalex.org/W1562368284', 'https://openalex.org/W1563088657', 'https://openalex.org/W1567012231', 'https://openalex.org/W1570329253', 'https://openalex.org/W1570448133', 'https://openalex.org/W1570706771', 'https://openalex.org/W1587647246', 'https://openalex.org/W1588516554', 'https://openalex.org/W1594031697', 'https://openalex.org/W1594781927', 'https://openalex.org/W1602492977', 'https://openalex.org/W1605688901', 'https://openalex.org/W1605844890', 'https://openalex.org/W1637435380', 'https://openalex.org/W1670263352', 'https://openalex.org/W1671614046', 'https://openalex.org/W1746680969', 'https://openalex.org/W1780185704', 'https://openalex.org/W1808644423', 'https://openalex.org/W1813387235', 'https://openalex.org/W1817561967', 'https://openalex.org/W1827261456', 'https://openalex.org/W1904009171', 'https://openalex.org/W1935515061', 'https://openalex.org/W1973991804', 'https://openalex.org/W1974545290', 'https://openalex.org/W1979711143', 'https://openalex.org/W1983479840', 'https://openalex.org/W1983690667', 'https://openalex.org/W1986883011', 'https://openalex.org/W1992419399', 'https://openalex.org/W1993066733', 'https://openalex.org/W2006345381', 'https://openalex.org/W2011101028', 'https://openalex.org/W2016441117', 'https://openalex.org/W2022058268', 'https://openalex.org/W2026718556', 'https://openalex.org/W2037322594', 'https://openalex.org/W2046649434', 'https://openalex.org/W2050829396', 'https://openalex.org/W2063783806', 'https://openalex.org/W2074584355', 'https://openalex.org/W2075932270', 'https://openalex.org/W2093825590', 'https://openalex.org/W2096756482', 'https://openalex.org/W2104333211', 'https://openalex.org/W2110179049', 'https://openalex.org/W2119479037', 'https://openalex.org/W2120199131', 'https://openalex.org/W2122111042', 'https://openalex.org/W2122496402', 'https://openalex.org/W2123623606', 'https://openalex.org/W2125055259', 'https://openalex.org/W2126333738', 'https://openalex.org/W2128912745', 'https://openalex.org/W2133160781', 'https://openalex.org/W2133218851', 'https://openalex.org/W2133632100', 'https://openalex.org/W2136000097', 'https://openalex.org/W2136132422', 'https://openalex.org/W2137130182', 'https://openalex.org/W2139212933', 'https://openalex.org/W2140586694', 'https://openalex.org/W2140785063', 'https://openalex.org/W2142857211', 'https://openalex.org/W2143603257', 'https://openalex.org/W2144731007', 'https://openalex.org/W2145467382', 'https://openalex.org/W2145680191', 'https://openalex.org/W2150796457', 'https://openalex.org/W2151450140', 'https://openalex.org/W2156440942', 'https://openalex.org/W2156571267', 'https://openalex.org/W2156909104', 'https://openalex.org/W2157815868', 'https://openalex.org/W2158724449', 'https://openalex.org/W2159895197', 'https://openalex.org/W2161349318', 'https://openalex.org/W2161782846', 'https://openalex.org/W2161960932', 'https://openalex.org/W2164359548', 'https://openalex.org/W2166985738', 'https://openalex.org/W2167277498', 'https://openalex.org/W2167467747', 'https://openalex.org/W2168754135', 'https://openalex.org/W2171265988', 'https://openalex.org/W2172429451', 'https://openalex.org/W2322002063', 'https://openalex.org/W2488399954', 'https://openalex.org/W2603390332', 'https://openalex.org/W2766736793', 'https://openalex.org/W2911678770', 'https://openalex.org/W2912276539', 'https://openalex.org/W2912934387', 'https://openalex.org/W3015462599']</t>
+          <t>['GR']</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr">
+          <t>['Witten I, 2011, ELSEVIER EBOOKS', 'Gordon A, 1984, BIOMETRICS', 'Cristianini N, 2000, CAMBRIDGE UNIVERSITY PRESS EBOOKS', 'Jain A, 1999, ACM COMPUTING SURVEYS', 'Sutton R, 1998, MIT PRESS EBOOKS', 'Friedman N, 1997, MACHINE LEARNING', 'Cohen W, 1995, ELSEVIER EBOOKS', 'Kononenko I, 1994, LECTURE NOTES IN COMPUTER SCIENCE', 'Dietterich T, 2000, MACHINE LEARNING', 'Jordan M, 1998, ', 'Frank E, 1998, RESEARCH COMMONS (THE UNIVERSITY OF WAIKATO)', 'Freund Y, 1998, ', 'Murthy S, 1998, DATA MINING AND KNOWLEDGE DISCOVERY', 'Batista G, 2003, APPLIED ARTIFICIAL INTELLIGENCE', 'Cheng J, 2002, ARTIFICIAL INTELLIGENCE', 'Wettschereck D, 1997, ARTIFICIAL INTELLIGENCE REVIEW', 'Veropoulos K, 1999, ', 'Crammer K, 2002, MACHINE LEARNING', 'Genton M, 2002, ', 'Fürnkranz J, 1999, ARTIFICIAL INTELLIGENCE REVIEW', 'Cestnik B, 1990, EUROPEAN CONFERENCE ON ARTIFICIAL INTELLIGENCE', 'Cestnik B, 1987, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Gehrke J, 2000, DATA MINING AND KNOWLEDGE DISCOVERY', 'Breslow L, 1997, THE KNOWLEDGE ENGINEERING REVIEW', 'Kononenko I, 1991, LECTURE NOTES IN COMPUTER SCIENCE', 'Cheng J, 2001, LECTURE NOTES IN COMPUTER SCIENCE', 'Smyth P, 1991, ', 'F�rnkranz J, 2005, MACHINE LEARNING', 'Blum A, 1997, MACHINE LEARNING', 'Setiono R, 2000, APPLIED INTELLIGENCE', 'Elomaa T, 1999, MACHINE LEARNING', 'Rastogi R, 2000, DATA MINING AND KNOWLEDGE DISCOVERY', 'Siddique M, 2002, ', 'Yang Y, 2003, LECTURE NOTES IN COMPUTER SCIENCE', 'Mántaras R, 1998, DATA &amp; KNOWLEDGE ENGINEERING', 'Bonarini A, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Csiszár I, 1996, ', 'An A, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Wall R, 2003, ARTIFICIAL INTELLIGENCE IN MEDICINE', 'Brůha I, 2000, INTELLIGENT DATA ANALYSIS', 'Elomaa T, 1999, LECTURE NOTES IN COMPUTER SCIENCE', 'Fürnkranz J, 2001, ', 'Zheng Z, 2000, MACHINE LEARNING', 'An A, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Lindgren T, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Kubát M, 2001, INTELLIGENT DATA ANALYSIS', 'Baik S, 2004, LECTURE NOTES IN COMPUTER SCIENCE', 'Vivarelli F, 2001, NEURAL NETWORKS', 'Cowell R, 2013, ARXIV (CORNELL UNIVERSITY)', 'Vapnik V, 1995, ', 'Quinlan J, 1992, ', 'Burges C, 1998, DATA MINING AND KNOWLEDGE DISCOVERY', 'Cover T, 1967, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Dietterich T, 1998, NEURAL COMPUTATION', ', 2000, APPLIED PHYSICS LETTERS', 'Hodge J, 2004, ARTIFICIAL INTELLIGENCE REVIEW', 'Domingos P, 1997, MACHINE LEARNING', 'Mika S, 2003, ', 'Friedman J, 1989, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Guo G, 2003, LECTURE NOTES IN COMPUTER SCIENCE', 'Littlestone N, 1994, INFORMATION AND COMPUTATION', 'Clark P, 1989, MACHINE LEARNING', 'Yu L, 2004, ', 'Zhang G, 2000, IEEE TRANSACTIONS ON SYSTEMS MAN AND CYBERNETICS PART C (APPLICATIONS AND REVIEWS)', 'Wilson D, 2000, MACHINE LEARNING', 'Lim T, 2000, MACHINE LEARNING', 'Vilalta R, 2002, ARTIFICIAL INTELLIGENCE REVIEW', 'Nadeau C, 2003, MACHINE LEARNING', 'Friedman N, 2003, MACHINE LEARNING', 'Hunt E, 1966, MEDICAL ENTOMOLOGY AND ZOOLOGY', 'Weigend A, 1990, ', 'Brighton H, 2002, DATA MINING AND KNOWLEDGE DISCOVERY', 'Zhang S, 2003, APPLIED ARTIFICIAL INTELLIGENCE', ', 2000, APPLIED PHYSICS LETTERS', 'Brazdil P, 2003, MACHINE LEARNING', 'Ruggieri S, 2002, IEEE TRANSACTIONS ON KNOWLEDGE AND DATA ENGINEERING', 'Utgoff P, 1997, MACHINE LEARNING', 'Keerthi S, 2002, MACHINE LEARNING', 'Kononenko I, 1993, APPLIED ARTIFICIAL INTELLIGENCE', 'Castellano G, 1997, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Heckerman D, 2006, STUDIES IN FUZZINESS AND SOFT COMPUTING', 'Parekh R, 2000, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Bouckaert R, 2003, ', 'Reinartz T, 2002, DATA MINING AND KNOWLEDGE DISCOVERY', 'Fürnkranz J, 1997, MACHINE LEARNING', 'Yam J, 2001, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Dutton D, 1997, THE KNOWLEDGE ENGINEERING REVIEW', 'Kalousis A, 2004, MACHINE LEARNING', 'McSherry D, 1999, KNOWLEDGE-BASED SYSTEMS', 'Zhou Z, 2004, JOURNAL OF COMPUTER SCIENCE AND TECHNOLOGY', 'Camargo L, 2001, NEURAL COMPUTATION', 'Yen G, 2002, ', 'Yıldız O, 2007, PATTERN RECOGNITION LETTERS', 'Roy A, 2000, IEEE TRANSACTIONS ON FUZZY SYSTEMS', 'Basak J, 2004, NEURAL COMPUTATION', 'Kon M, 2000, NEURAL NETWORKS', 'Okamoto S, 2003, THEORETICAL COMPUTER SCIENCE', 'Zheng Z, 1998, KNOWLEDGE-BASED SYSTEMS', 'Sánchez J, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Breiman L, 1996, MACHINE LEARNING', 'Mullin A, 1963, AMERICAN MATHEMATICAL MONTHLY', 'M. P, 1950, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES A (GENERAL)', 'Bouckaert R, 2004, LECTURE NOTES IN COMPUTER SCIENCE', ', 2001, STUDIES IN FUZZINESS AND SOFT COMPUTING', 'Gama J, 1999, INTELLIGENT DATA ANALYSIS', 'Flach P, 2000, ', 'Kivinen J, 2003, LECTURE NOTES IN COMPUTER SCIENCE', 'Rumelhart D, 1985, ', ', 2019, ', 'Aha D, 1997, ']</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
-        </is>
-      </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
+          <t xml:space="preserve">Kotsiantis S, 2007, </t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kotsiantis S, 2007, </t>
         </is>
       </c>
     </row>
@@ -4991,7 +5211,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>2920</v>
+        <v>2916</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -5035,7 +5255,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['IL', 'CA']</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5043,20 +5263,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr">
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr"/>
+      <c r="X45" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr">
-        <is>
-          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
-        </is>
-      </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
+          <t>Shalev‐Shwartz S, 2014, CAMBRIDGE UNIVERSITY PRESS EBOOKS</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Shalev‐Shwartz S, 2014, CAMBRIDGE UNIVERSITY PRESS EBOOKS</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5315,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>4348</v>
+        <v>4344</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -5158,20 +5383,25 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr">
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr"/>
+      <c r="X46" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr">
-        <is>
-          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
-        </is>
-      </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
+          <t>Samuel A, 1959, IBM JOURNAL OF RESEARCH AND DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Samuel A, 1959, IBM JOURNAL OF RESEARCH AND DEVELOPMENT</t>
         </is>
       </c>
     </row>
@@ -5205,7 +5435,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>4214</v>
+        <v>4210</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
@@ -5249,28 +5479,33 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1473189865', 'https://openalex.org/W1510952750', 'https://openalex.org/W1528076390', 'https://openalex.org/W1535019556', 'https://openalex.org/W1554944419', 'https://openalex.org/W1760458529', 'https://openalex.org/W1811750039', 'https://openalex.org/W1821462560', 'https://openalex.org/W1826232489', 'https://openalex.org/W1873763122', 'https://openalex.org/W1992926795', 'https://openalex.org/W2009733253', 'https://openalex.org/W2024594469', 'https://openalex.org/W2040228409', 'https://openalex.org/W2051267297', 'https://openalex.org/W2053637704', 'https://openalex.org/W2077905990', 'https://openalex.org/W2095272373', 'https://openalex.org/W2095705004', 'https://openalex.org/W2096633407', 'https://openalex.org/W2106313770', 'https://openalex.org/W2106463421', 'https://openalex.org/W2112380340', 'https://openalex.org/W2114229504', 'https://openalex.org/W2119874464', 'https://openalex.org/W2123147099', 'https://openalex.org/W2130051287', 'https://openalex.org/W2151320232', 'https://openalex.org/W2162379889', 'https://openalex.org/W2186645727', 'https://openalex.org/W2198253679', 'https://openalex.org/W2329660289', 'https://openalex.org/W2461943168', 'https://openalex.org/W2473418344', 'https://openalex.org/W2532520288', 'https://openalex.org/W2950943617', 'https://openalex.org/W2951114885', 'https://openalex.org/W2962835266', 'https://openalex.org/W2963794891', 'https://openalex.org/W2964318098', 'https://openalex.org/W3118608800', 'https://openalex.org/W3215186461', 'https://openalex.org/W4248649186', 'https://openalex.org/W6628547770', 'https://openalex.org/W6631628602', 'https://openalex.org/W6632160336', 'https://openalex.org/W6638214083', 'https://openalex.org/W6639246211', 'https://openalex.org/W6661425395', 'https://openalex.org/W6674330103', 'https://openalex.org/W6676639149', 'https://openalex.org/W6677855611', 'https://openalex.org/W6686761782', 'https://openalex.org/W6731627051']</t>
+          <t>['US', 'FR']</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr">
+          <t>['Srivastava N, 2014, ', 'Hastie T, 2013, ', 'Dwork C, 2006, LECTURE NOTES IN COMPUTER SCIENCE', 'Abadi M, 2016, ', 'Fredrikson M, 2015, ', 'Shokri R, 2015, ', 'Franklin J, 2005, THE MATHEMATICAL INTELLIGENCER', 'Homer N, 2008, PLOS GENETICS', 'Lindell Y, 2000, LECTURE NOTES IN COMPUTER SCIENCE', 'Chaudhuri K, 2011, PUBMED', 'Bassily R, 2014, ', 'Fredrikson M, 2014, PUBMED', 'Chaudhuri K, 2008, ', 'Jagannathan G, 2005, ', 'Hardt M, 2016, INTERNATIONAL CONFERENCE ON MACHINE LEARNING', 'Du W, 2004, ', 'Zhang J, 2012, PROCEEDINGS OF THE VLDB ENDOWMENT', 'Dwork C, 2011, ', 'Yang D, 2016, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Calandrino J, 2011, ', 'Bos J, 2014, JOURNAL OF BIOMEDICAL INFORMATICS', 'Rubinstein B, 2012, JOURNAL OF PRIVACY AND CONFIDENTIALITY', 'Sankararaman S, 2009, NATURE GENETICS', 'Vaidya J, 2007, THE VLDB JOURNAL', 'Barni M, 2011, IEEE TRANSACTIONS ON INFORMATION FORENSICS AND SECURITY', 'Duchi J, 2014, JOURNAL OF THE ACM', 'Schneider I, 2005, THE MATHEMATICAL INTELLIGENCER', 'Dwork C, 2015, ', 'Backes M, 2016, ', 'Zhu J, 2001, ', 'Dwork C, 2010, JOURNAL OF PRIVACY AND CONFIDENTIALITY', 'Diakonikolas I, 2015, EDINBURGH RESEARCH EXPLORER (UNIVERSITY OF EDINBURGH)', 'Krizhevsky A, 2024, ', 'Hinton G, 2015, ARXIV (CORNELL UNIVERSITY)', 'Tramèr F, 2016, ARXIV (CORNELL UNIVERSITY)', 'Chaudhuri K, 2009, ARXIV (CORNELL UNIVERSITY)', ', 2016, IRIS RESEARCH PRODUCT CATALOG (SAPIENZA UNIVERSITY OF ROME)', 'Hardt M, 2015, ARXIV (CORNELL UNIVERSITY)', 'Xie P, 2014, ARXIV (CORNELL UNIVERSITY)', 'Duchi J, 2012, ARXIV (CORNELL UNIVERSITY)', 'Jain P, 2015, ARXIV (CORNELL UNIVERSITY)', 'Kusner M, 2015, POLYPUBLIE (ÉCOLE POLYTECHNIQUE DE MONTRÉAL)']</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reza Shokri, 2017, </t>
-        </is>
-      </c>
       <c r="Y47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reza Shokri, 2017, </t>
+          <t xml:space="preserve">Shokri R, 2017, </t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shokri R, 2017, </t>
         </is>
       </c>
     </row>
@@ -5352,28 +5587,33 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W1505641881', 'https://openalex.org/W1541642243', 'https://openalex.org/W1564419782', 'https://openalex.org/W1580529010', 'https://openalex.org/W1639227073', 'https://openalex.org/W1676552347', 'https://openalex.org/W1773272891', 'https://openalex.org/W1926270821', 'https://openalex.org/W1970393892', 'https://openalex.org/W2000701155', 'https://openalex.org/W2003262222', 'https://openalex.org/W2012778485', 'https://openalex.org/W2048677751', 'https://openalex.org/W2059389571', 'https://openalex.org/W2069295011', 'https://openalex.org/W2075746031', 'https://openalex.org/W2099046646', 'https://openalex.org/W2111308925', 'https://openalex.org/W2111589119', 'https://openalex.org/W2114785422', 'https://openalex.org/W2115168188', 'https://openalex.org/W2119747362', 'https://openalex.org/W2130103520', 'https://openalex.org/W2148278638', 'https://openalex.org/W2149706766', 'https://openalex.org/W2151103935', 'https://openalex.org/W2162430761', 'https://openalex.org/W2163205713', 'https://openalex.org/W2166221155', 'https://openalex.org/W2169741726', 'https://openalex.org/W2914011225', 'https://openalex.org/W2999811158', 'https://openalex.org/W6733008967']</t>
+          <t>['GB']</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr">
+          <t>['Lowe D, 2004, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Quinlan J, 1986, MACHINE LEARNING', 'Harris C, 1988, ', 'Shi J, 1994, ', 'Haralock R, 1991, ADDISON-WESLEY LONGMAN PUBLISHING CO., INC. EBOOKS', 'Smith S, 1997, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Schmid C, 2000, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Mikolajczyk K, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Rosten E, 2005, ', 'Mikolajczyk K, 2002, ', 'Sklar B, 1987, ', 'Moravec H, 2018, RESEARCH SHOWCASE @ CARNEGIE MELLON UNIVERSITY (CARNEGIE MELLON UNIVERSITY)', 'Kitchen L, 1982, PATTERN RECOGNITION LETTERS', 'Brown M, 2002, ', 'Mokhtarian F, 1998, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Schaffalitzky F, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Trajković M, 1998, IMAGE AND VISION COMPUTING', 'Schmid C, 2002, ', 'Wang H, 1995, IMAGE AND VISION COMPUTING', 'Zheng Z, 1999, PATTERN RECOGNITION LETTERS', 'Loy G, 2002, LECTURE NOTES IN COMPUTER SCIENCE', 'Trucco E, 1995, AI COMMUNICATIONS', 'Noble J, 1988, IMAGE AND VISION COMPUTING', 'Rosten E, 2005, LECTURE NOTES IN COMPUTER SCIENCE', 'Medioni G, 1987, COMPUTER VISION GRAPHICS AND IMAGE PROCESSING', 'Dias P, 2002, ', 'Cooper D, 1993, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Zuliani M, 2005, ', 'Guiducci A, 1988, PATTERN RECOGNITION LETTERS', 'Kenney C, 2003, IEEE TRANSACTIONS ON PATTERN ANALYSIS AND MACHINE INTELLIGENCE', 'Langridge D, 1982, COMPUTER GRAPHICS AND IMAGE PROCESSING', 'Acharya R, 1987, COMPUTER VISION GRAPHICS AND IMAGE PROCESSING']</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr">
-        <is>
-          <t>Edward Rosten, 2006, Lecture notes in computer science</t>
-        </is>
-      </c>
       <c r="Y48" t="inlineStr">
         <is>
-          <t>Edward Rosten, 2006, Lecture notes in computer science</t>
+          <t>Rosten E, 2006, LECTURE NOTES IN COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>Rosten E, 2006, LECTURE NOTES IN COMPUTER SCIENCE</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5647,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3027</v>
+        <v>3016</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -5467,28 +5707,33 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W94523489', 'https://openalex.org/W189596042', 'https://openalex.org/W1179140510', 'https://openalex.org/W1496317909', 'https://openalex.org/W1596717185', 'https://openalex.org/W1689445748', 'https://openalex.org/W1916445479', 'https://openalex.org/W1963579367', 'https://openalex.org/W1963790103', 'https://openalex.org/W1966124853', 'https://openalex.org/W1967320885', 'https://openalex.org/W1968452917', 'https://openalex.org/W1984530193', 'https://openalex.org/W1990517717', 'https://openalex.org/W1995341919', 'https://openalex.org/W1998871699', 'https://openalex.org/W2000972253', 'https://openalex.org/W2001619934', 'https://openalex.org/W2009986810', 'https://openalex.org/W2015263929', 'https://openalex.org/W2018435387', 'https://openalex.org/W2019207321', 'https://openalex.org/W2024081693', 'https://openalex.org/W2025279987', 'https://openalex.org/W2028606616', 'https://openalex.org/W2040104179', 'https://openalex.org/W2040870580', 'https://openalex.org/W2049633694', 'https://openalex.org/W2063304499', 'https://openalex.org/W2065165083', 'https://openalex.org/W2072680624', 'https://openalex.org/W2075320162', 'https://openalex.org/W2076857888', 'https://openalex.org/W2081544115', 'https://openalex.org/W2087877962', 'https://openalex.org/W2095727900', 'https://openalex.org/W2102201073', 'https://openalex.org/W2106855632', 'https://openalex.org/W2108703480', 'https://openalex.org/W2110642273', 'https://openalex.org/W2111072639', 'https://openalex.org/W2119821739', 'https://openalex.org/W2128084896', 'https://openalex.org/W2138178898', 'https://openalex.org/W2143908786', 'https://openalex.org/W2149723649', 'https://openalex.org/W2150593711', 'https://openalex.org/W2153476503', 'https://openalex.org/W2153635508', 'https://openalex.org/W2154350719', 'https://openalex.org/W2161673710', 'https://openalex.org/W2174918471', 'https://openalex.org/W2200121095', 'https://openalex.org/W2209382794', 'https://openalex.org/W2216013554', 'https://openalex.org/W2231576311', 'https://openalex.org/W2270460811', 'https://openalex.org/W2270641383', 'https://openalex.org/W2273322351', 'https://openalex.org/W2286091602', 'https://openalex.org/W2294798173', 'https://openalex.org/W2298521547', 'https://openalex.org/W2337945771', 'https://openalex.org/W2339447311', 'https://openalex.org/W2399675776', 'https://openalex.org/W2417395753', 'https://openalex.org/W2419137750', 'https://openalex.org/W2470803522', 'https://openalex.org/W2497210317', 'https://openalex.org/W2502044482', 'https://openalex.org/W2552660223', 'https://openalex.org/W2560811704', 'https://openalex.org/W2577148968', 'https://openalex.org/W2580808806', 'https://openalex.org/W2586821267', 'https://openalex.org/W2591104514', 'https://openalex.org/W2598645336', 'https://openalex.org/W2603364874', 'https://openalex.org/W2603417106', 'https://openalex.org/W2604196786', 'https://openalex.org/W2606244344', 'https://openalex.org/W2606916050', 'https://openalex.org/W2612828053', 'https://openalex.org/W2619390517', 'https://openalex.org/W2620473470', 'https://openalex.org/W2620542418', 'https://openalex.org/W2621525431', 'https://openalex.org/W2622758479', 'https://openalex.org/W2622999711', 'https://openalex.org/W2738911869', 'https://openalex.org/W2775111183', 'https://openalex.org/W2789255992', 'https://openalex.org/W2790639095', 'https://openalex.org/W2791690647', 'https://openalex.org/W2794415089', 'https://openalex.org/W2796501058', 'https://openalex.org/W2806779833', 'https://openalex.org/W2903950532', 'https://openalex.org/W2911964244', 'https://openalex.org/W2919115771', 'https://openalex.org/W3125807057', 'https://openalex.org/W4210451417', 'https://openalex.org/W4212883601', 'https://openalex.org/W4232670376', 'https://openalex.org/W4239510810', 'https://openalex.org/W4250143236', 'https://openalex.org/W4400360174', 'https://openalex.org/W6607775107', 'https://openalex.org/W6632223008', 'https://openalex.org/W6675321329', 'https://openalex.org/W6675436802', 'https://openalex.org/W6676769703']</t>
+          <t>['GR', 'IT', 'GB']</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr">
+          <t>['Dempster A, 1977, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Chang C, 2011, ACM TRANSACTIONS ON INTELLIGENT SYSTEMS AND TECHNOLOGY', 'Cortes C, 1995, MACHINE LEARNING', 'Hopfield J, 1982, PROCEEDINGS OF THE NATIONAL ACADEMY OF SCIENCES', 'McCulloch W, 1943, BULLETIN OF MATHEMATICAL BIOLOGY', 'Jang J, 1993, IEEE TRANSACTIONS ON SYSTEMS MAN AND CYBERNETICS', 'Lloyd S, 1982, IEEE TRANSACTIONS ON INFORMATION THEORY', 'Fisher R, 1936, ANNALS OF EUGENICS', 'Huang G, 2006, NEUROCOMPUTING', 'Rosenblatt F, 1958, PSYCHOLOGICAL REVIEW', 'Cleveland W, 1979, JOURNAL OF THE AMERICAN STATISTICAL ASSOCIATION', 'Suykens J, 1999, NEURAL PROCESSING LETTERS', 'Kohonen T, 1990, PROCEEDINGS OF THE IEEE', 'Friedman J, 1991, THE ANNALS OF STATISTICS', 'Johnson S, 1967, PSYCHOMETRIKA', 'Specht D, 1991, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Riedmiller M, 2002, IEEE INTERNATIONAL CONFERENCE ON NEURAL NETWORKS', 'Suykens J, 2002, WORLD SCIENTIFIC EBOOKS', 'Broomhead D, 1988, COMPLEX SYSTEMS', 'Kong L, 2007, NUCLEIC ACIDS RESEARCH', 'Kass G, 1980, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Fix E, 1989, INTERNATIONAL STATISTICAL REVIEW', 'Salakhutdinov R, 2009, ', 'Atkeson C, 1997, ARTIFICIAL INTELLIGENCE REVIEW', 'Samuel A, 2000, IBM JOURNAL OF RESEARCH AND DEVELOPMENT', 'Pal S, 1992, IEEE TRANSACTIONS ON NEURAL NETWORKS', 'Moshou D, 2004, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Linnainmaa S, 1976, BIT NUMERICAL MATHEMATICS', 'Cao J, 2012, NEURAL PROCESSING LETTERS', 'Galvão R, 2008, CHEMOMETRICS AND INTELLIGENT LABORATORY SYSTEMS', 'Mackowiak S, 2015, GENOME BIOLOGY', 'Moshou D, 2005, REAL-TIME IMAGING', 'Asadi H, 2014, PLOS ONE', 'Melssen W, 2006, CHEMOMETRICS AND INTELLIGENT LABORATORY SYSTEMS', 'Dutta R, 2014, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Sengupta S, 2013, BIOSYSTEMS ENGINEERING', 'Amatya S, 2015, BIOSYSTEMS ENGINEERING', 'Mohammadi K, 2015, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Thomas P, 2002, BRITISH JOURNAL OF EDUCATIONAL TECHNOLOGY', 'Coopersmith E, 2014, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Moshou D, 2006, PRECISION AGRICULTURE', 'Craninx M, 2007, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Moshou D, 2013, BIOSYSTEMS ENGINEERING', 'Alonso J, 2013, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Hossain M, 2011, JOURNAL OF HAND SURGERY (EUROPEAN VOLUME)', 'Alonso J, 2014, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Gastaldo P, 2014, ROBOTICS AND AUTONOMOUS SYSTEMS', 'Tryon R, 1957, PSYCHOMETRIKA', 'Neapolitan R, 1987, APPLIED ARTIFICIAL INTELLIGENCE', 'Smith D, 1978, SOCIETY', 'Breiman L, 2001, MACHINE LEARNING', 'LeCun Y, 2015, NATURE', 'Pearson K, 1901, THE LONDON EDINBURGH AND DUBLIN PHILOSOPHICAL MAGAZINE AND JOURNAL OF SCIENCE', 'Ferentinos K, 2018, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Cox D, 1958, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES B (STATISTICAL METHODOLOGY)', 'Barboza F, 2017, EXPERT SYSTEMS WITH APPLICATIONS', 'Grinblat G, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2015, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Ebrahimi M, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Morellos A, 2016, BIOSYSTEMS ENGINEERING', 'Zhao Y, 2017, ENERGY ECONOMICS', 'Hansen M, 2018, COMPUTERS IN INDUSTRY', 'Fang K, 2017, GEOPHYSICAL RESEARCH LETTERS', 'Feng Y, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Zhang B, 2017, CANCER LETTERS', 'Rhee J, 2017, AGRICULTURAL AND FOREST METEOROLOGY', 'Mehdizadeh S, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Kang J, 2015, INTERNATIONAL JOURNAL OF RADIATION ONCOLOGY*BIOLOGY*PHYSICS', 'Cramer S, 2017, EXPERT SYSTEMS WITH APPLICATIONS', 'Chung C, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Matthews S, 2017, SCIENTIFIC REPORTS', 'Zhou C, 2018, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2016, BIOSYSTEMS ENGINEERING', 'Ramos P, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Ali I, 2016, IEEE JOURNAL OF SELECTED TOPICS IN APPLIED EARTH OBSERVATIONS AND REMOTE SENSING', 'Bohanec M, 2016, EXPERT SYSTEMS WITH APPLICATIONS', 'Senthilnath J, 2016, BIOSYSTEMS ENGINEERING', 'Patil A, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Belson W, 1959, JOURNAL OF THE ROYAL STATISTICAL SOCIETY SERIES C (APPLIED STATISTICS)', 'Nahvi B, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Maione C, 2015, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Wildenhain J, 2015, CELL SYSTEMS', 'Su Y, 2017, SAUDI JOURNAL OF BIOLOGICAL SCIENCES', 'Aybar-Ruíz A, 2016, SOLAR ENERGY', 'Maione C, 2018, CRITICAL REVIEWS IN FOOD SCIENCE AND NUTRITION', 'Pantazi X, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Binch A, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2017, PRECISION AGRICULTURE', 'Ramírez-Morales I, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Zhang M, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Johann A, 2016, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Pantazi X, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Kung H, 2016, SUSTAINABILITY', 'Pegorini V, 2015, SENSORS', 'Richardson A, 2016, CLINICAL BIOCHEMISTRY', 'López-Cortés X, 2016, AQUACULTURE', 'Takahashi K, 2017, ROBOTICS AND AUTONOMOUS SYSTEMS', 'Fragni R, 2018, FOOD CONTROL', 'Hu H, 2017, COMPUTERS AND ELECTRONICS IN AGRICULTURE', 'Craninx M, 2006, PUBMED', 'Cortes C, 1995, MACHINE LEARNING', 'Breiman L, 1996, MACHINE LEARNING', ', 1988, ELSEVIER EBOOKS', 'Hecht-Nielsen R, 1987, APPLIED OPTICS', ', 1988, NEURAL NETWORKS', 'Strunk K, 2024, ']</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
-        <is>
-          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
-        </is>
-      </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
+          <t>Λιάκος Κ, 2018, SENSORS</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Λιάκος Κ, 2018, SENSORS</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5767,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>4649</v>
+        <v>4647</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -5582,28 +5827,33 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W30646539', 'https://openalex.org/W92141931', 'https://openalex.org/W191102129', 'https://openalex.org/W429766147', 'https://openalex.org/W595863337', 'https://openalex.org/W1482533224', 'https://openalex.org/W1513618424', 'https://openalex.org/W1573647811', 'https://openalex.org/W1606754933', 'https://openalex.org/W1689749838', 'https://openalex.org/W1727844347', 'https://openalex.org/W1786856418', 'https://openalex.org/W1831050183', 'https://openalex.org/W1895518694', 'https://openalex.org/W1969543759', 'https://openalex.org/W1980225565', 'https://openalex.org/W1983650914', 'https://openalex.org/W1984828485', 'https://openalex.org/W1985839444', 'https://openalex.org/W1990590197', 'https://openalex.org/W1993415357', 'https://openalex.org/W2005164184', 'https://openalex.org/W2006929658', 'https://openalex.org/W2018337952', 'https://openalex.org/W2023312901', 'https://openalex.org/W2023942604', 'https://openalex.org/W2027120296', 'https://openalex.org/W2032518966', 'https://openalex.org/W2033585087', 'https://openalex.org/W2036376676', 'https://openalex.org/W2037789405', 'https://openalex.org/W2050179592', 'https://openalex.org/W2057779644', 'https://openalex.org/W2066626803', 'https://openalex.org/W2078720475', 'https://openalex.org/W2088449361', 'https://openalex.org/W2102467070', 'https://openalex.org/W2112776483', 'https://openalex.org/W2114727579', 'https://openalex.org/W2123845623', 'https://openalex.org/W2126822776', 'https://openalex.org/W2130089270', 'https://openalex.org/W2130560194', 'https://openalex.org/W2131347105', 'https://openalex.org/W2131822674', 'https://openalex.org/W2133505387', 'https://openalex.org/W2135479785', 'https://openalex.org/W2140389576', 'https://openalex.org/W2142800341', 'https://openalex.org/W2145126338', 'https://openalex.org/W2151135366', 'https://openalex.org/W2151666808', 'https://openalex.org/W2155544089', 'https://openalex.org/W2156713494', 'https://openalex.org/W2157395790', 'https://openalex.org/W2158441306', 'https://openalex.org/W2160615957', 'https://openalex.org/W2179669825', 'https://openalex.org/W2191676425', 'https://openalex.org/W2199578048', 'https://openalex.org/W2205945645', 'https://openalex.org/W2287354130', 'https://openalex.org/W2295598076', 'https://openalex.org/W2310573451', 'https://openalex.org/W2346841190', 'https://openalex.org/W2417209869', 'https://openalex.org/W2463898247', 'https://openalex.org/W2479339604', 'https://openalex.org/W2514977123', 'https://openalex.org/W2522985694', 'https://openalex.org/W2554693566', 'https://openalex.org/W2557963070', 'https://openalex.org/W2564901692', 'https://openalex.org/W2580821229', 'https://openalex.org/W2582718246', 'https://openalex.org/W2727623211', 'https://openalex.org/W2730460668', 'https://openalex.org/W2736166619', 'https://openalex.org/W2890624634', 'https://openalex.org/W2890805913', 'https://openalex.org/W2917425395', 'https://openalex.org/W2917661374', 'https://openalex.org/W3022713798', 'https://openalex.org/W3102027041', 'https://openalex.org/W3102476541', 'https://openalex.org/W3163617311', 'https://openalex.org/W4211056572', 'https://openalex.org/W4250720198', 'https://openalex.org/W4252713891', 'https://openalex.org/W4285719527', 'https://openalex.org/W4399271987', 'https://openalex.org/W4399569501', 'https://openalex.org/W6634147026', 'https://openalex.org/W6727196412', 'https://openalex.org/W6870084398', 'https://openalex.org/W6891733106']</t>
+          <t>['NL', 'RS', 'CN', 'DE', 'CA', 'AT', 'US']</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr">
+          <t>['Venables W, 2002, STATISCTICS AND COMPUTING/STATISTICS AND COMPUTING', 'Hijmans R, 2005, INTERNATIONAL JOURNAL OF CLIMATOLOGY', 'Kühn M, 2008, JOURNAL OF STATISTICAL SOFTWARE', 'Cohen J, 1968, PSYCHOLOGICAL BULLETIN', 'Kühn M, 2013, ', 'Shannon C, 1998, PROCEEDINGS OF THE IEEE', 'Sing T, 2005, COMPUTER APPLICATIONS IN THE BIOSCIENCES', 'Chen J, 2014, ISPRS JOURNAL OF PHOTOGRAMMETRY AND REMOTE SENSING', 'Rabus B, 2003, ISPRS JOURNAL OF PHOTOGRAMMETRY AND REMOTE SENSING', 'Pendleton R, 1945, GEOGRAPHICAL REVIEW', 'Scharlemann J, 2014, CARBON MANAGEMENT', 'Meinshausen N, 2006, ', 'Goldewijk K, 2010, GLOBAL ECOLOGY AND BIOGEOGRAPHY', 'Fan Y, 2013, SCIENCE', 'Hengl T, 2014, PLOS ONE', 'Hartmann J, 2012, GEOCHEMISTRY GEOPHYSICS GEOSYSTEMS', 'Minasny B, 2006, COMPUTERS &amp; GEOSCIENCES', 'Hall D, 2007, HYDROLOGICAL PROCESSES', 'Pebesma E, 2015, ', 'Statnikov A, 2008, BMC BIOINFORMATICS', 'Shangguan W, 2013, JOURNAL OF ADVANCES IN MODELING EARTH SYSTEMS', 'Sánchez P, 2009, SCIENCE', 'Raup B, 2006, GLOBAL AND PLANETARY CHANGE', 'Brus D, 2011, EUROPEAN JOURNAL OF SOIL SCIENCE', 'Carroll M, 2009, INTERNATIONAL JOURNAL OF DIGITAL EARTH', 'Arrouays D, 2014, ADVANCES IN AGRONOMY', 'Hugelius G, 2013, EARTH SYSTEM SCIENCE DATA', 'Stockmann U, 2015, GLOBAL FOOD SECURITY', 'Grunwald S, 2011, SOIL SCIENCE SOCIETY OF AMERICA JOURNAL', 'Batjes N, 2009, SOIL USE AND MANAGEMENT', 'Savtchenko A, 2004, ADVANCES IN SPACE RESEARCH', 'Wan Z, 2006, INTERNATIONAL JOURNAL OF ENVIRONMENTAL RESEARCH AND PUBLIC HEALTH', 'Kilibarda M, 2014, JOURNAL OF GEOPHYSICAL RESEARCH ATMOSPHERES', 'Fitzpatrick M, 2013, ECOSPHERE', 'Borda M, 2011, ', 'Malone B, 2014, GEODERMA', "Sayre R, 2014, DIGITAL ACCESS TO LIBRARIES (UNIVERSITÉ CATHOLIQUE DE LOUVAIN (UCL), L'UNIVERSITÉ DE NAMUR (UNAMUR) AND THE UNIVERSITÉ SAINT-LOUIS (USL-B))", 'Montanarella L, 2012, CURRENT OPINION IN ENVIRONMENTAL SUSTAINABILITY', 'Gasch C, 2015, SPATIAL STATISTICS', 'Bauer-Marschallinger B, 2014, COMPUTERS &amp; GEOSCIENCES', 'Griffiths R, 2015, APPLIED SOIL ECOLOGY', 'Shani U, 2007, WATER RESOURCES RESEARCH', 'Cooper M, 2005, SOIL SCIENCE SOCIETY OF AMERICA JOURNAL', 'Knaus J, 2009, THE R JOURNAL', 'Láng V, 2012, GEODERMA', 'Pogson M, 2011, ENVIRONMENTAL MODELLING &amp; SOFTWARE', 'Kidd D, 2015, SOIL RESEARCH', 'Mantel S, 2007, DATA ARCHIVING AND NETWORKED SERVICES (DANS)', 'Baade J, 2014, ', 'Danielson J, 2011, ANTARCTICA A KEYSTONE IN A CHANGING WORLD', 'Chen T, 2016, ', 'Shannon C, 1949, PROCEEDINGS OF THE IRE', 'Anonim A, 2010, ', 'Wright M, 2017, JOURNAL OF STATISTICAL SOFTWARE', 'Giri C, 2010, GLOBAL ECOLOGY AND BIOGEOGRAPHY', 'Conrad O, 2015, GEOSCIENTIFIC MODEL DEVELOPMENT', 'Krämer W, 2003, COMPUTATIONAL STATISTICS &amp; DATA ANALYSIS', 'FAO, 2023, ', 'Kühn M, 2008, ', 'Hengl T, 2015, PLOS ONE', 'Nachtergaele F, 2012, SOCIO-ENVIRONMENTAL SYSTEMS MODELING', 'Conrad O, 2015, ', 'Rome, 1977, ', 'Shangguan W, 2016, JOURNAL OF ADVANCES IN MODELING EARTH SYSTEMS', 'Sollich P, 1995, CERN DOCUMENT SERVER (EUROPEAN ORGANIZATION FOR NUCLEAR RESEARCH)', 'Pelletier J, 2015, JOURNAL OF ADVANCES IN MODELING EARTH SYSTEMS', 'Brevik E, 2015, GEODERMA', 'Folberth C, 2016, NATURE COMMUNICATIONS', 'Domisch S, 2015, SCIENTIFIC DATA', 'Mulder V, 2015, GEODERMA', 'Krasilnikov P, 2009, ', 'Tóth G, 2013, JOINT RESEARCH CENTRE (EUROPEAN COMMISSION)', 'Mira M, 2015, REMOTE SENSING OF ENVIRONMENT', 'Wang S, 2007, ', 'Shepherd K, 2014, AGRICULTURAL SYSTEMS', 'Aksoy E, 2016, PLOS ONE', 'Searle R, 2014, ', 'Ribeiro E, 2015, ', 'Leenaars J, 2013, DATA ARCHIVING AND NETWORKED SERVICES (DANS)', 'Faison E, 2016, PLOS ONE', 'Ribeiro E, 2015, ', 'Brevik E, 2015, GEODERMA', 'Jagger J, 2007, ELSEVIER EBOOKS', 'Hijmans R, 2010, ', 'Wright M, 2015, ']</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>Tomislav Hengl, 2017, PLoS ONE</t>
-        </is>
-      </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>Tomislav Hengl, 2017, PLoS ONE</t>
+          <t>Hengl T, 2017, PLOS ONE</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Hengl T, 2017, PLOS ONE</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5887,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>2473</v>
+        <v>2469</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -5693,28 +5943,33 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>['https://openalex.org/W822801274', 'https://openalex.org/W1506806321', 'https://openalex.org/W1565746575', 'https://openalex.org/W1901616594', 'https://openalex.org/W1978394996', 'https://openalex.org/W2034059032', 'https://openalex.org/W2059111627', 'https://openalex.org/W2076063813', 'https://openalex.org/W2096352448', 'https://openalex.org/W2099419573', 'https://openalex.org/W2106577732', 'https://openalex.org/W2151103935', 'https://openalex.org/W2161969291', 'https://openalex.org/W2164598857', 'https://openalex.org/W2251410821', 'https://openalex.org/W2269742369', 'https://openalex.org/W2585169518', 'https://openalex.org/W2751039952', 'https://openalex.org/W2798302089', 'https://openalex.org/W2800722845', 'https://openalex.org/W2802955324', 'https://openalex.org/W2884001105', 'https://openalex.org/W2888794009', 'https://openalex.org/W2891503716', 'https://openalex.org/W2892341857', 'https://openalex.org/W2895991254', 'https://openalex.org/W2900453322', 'https://openalex.org/W2902907165', 'https://openalex.org/W2915015079', 'https://openalex.org/W2919115771', 'https://openalex.org/W2921353139', 'https://openalex.org/W2945976633', 'https://openalex.org/W2953189907', 'https://openalex.org/W2963095307', 'https://openalex.org/W2963428668', 'https://openalex.org/W2964716450', 'https://openalex.org/W2981207549', 'https://openalex.org/W2989851933', 'https://openalex.org/W2995871253', 'https://openalex.org/W2999321020', 'https://openalex.org/W3000062802', 'https://openalex.org/W3005351117', 'https://openalex.org/W3025420269', 'https://openalex.org/W3094605956', 'https://openalex.org/W3095865939', 'https://openalex.org/W3118496513', 'https://openalex.org/W3120261410', 'https://openalex.org/W3150796314', 'https://openalex.org/W4212902066', 'https://openalex.org/W4236093597', 'https://openalex.org/W4255466416', 'https://openalex.org/W6730267373', 'https://openalex.org/W6750380350']</t>
+          <t>['DE']</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr">
+          <t>['LeCun Y, 2015, NATURE', 'Lowe D, 2004, INTERNATIONAL JOURNAL OF COMPUTER VISION', 'Dalal N, 2005, ', 'Viola P, 2005, ', 'Schmidhuber J, 2014, NEURAL NETWORKS', 'Demšar J, 2006, ', 'Jordan M, 2015, SCIENCE', 'Salton G, 1988, INFORMATION PROCESSING &amp; MANAGEMENT', 'Rudin C, 2019, NATURE MACHINE INTELLIGENCE', 'Bishop C, 2006, SPRINGER EBOOKS', 'Searle J, 1980, BEHAVIORAL AND BRAIN SCIENCES', 'Adadi A, 2018, IEEE ACCESS', 'Silver D, 2018, SCIENCE', 'Gama J, 2014, ACM COMPUTING SURVEYS', 'Young T, 2018, IEEE COMPUTATIONAL INTELLIGENCE MAGAZINE', 'Eykholt K, 2018, ', 'Grigorescu S, 2019, JOURNAL OF FIELD ROBOTICS', 'Kotsiantis S, 2006, ARTIFICIAL INTELLIGENCE REVIEW', 'Pouyanfar S, 2018, ACM COMPUTING SURVEYS', 'Shmueli G, 2011, MIS QUARTERLY', 'Westerlund M, 2019, TECHNOLOGY INNOVATION MANAGEMENT REVIEW', 'Zhang Y, 2018, NPJ COMPUTATIONAL MATERIALS', 'Pan Z, 2019, IEEE ACCESS', 'Madani A, 2018, NPJ DIGITAL MEDICINE', 'Chen S, 2008, MATHEMATICS AND COMPUTERS IN SIMULATION', 'Shrestha Y, 2020, JOURNAL OF BUSINESS RESEARCH', 'Ahani A, 2019, INTERNATIONAL JOURNAL OF HOSPITALITY MANAGEMENT', 'Goyal D, 2015, CIRP JOURNAL OF MANUFACTURING SCIENCE AND TECHNOLOGY', 'Paula E, 2016, ', 'Peters M, 2013, MACHINE LEARNING', 'Howard A, 2017, ', 'Assaf R, 2019, ', 'Pentland B, 2020, MIS QUARTERLY', 'Kühl N, 2019, ELECTRONIC MARKETS', 'Liu Z, 2020, ', 'Balaji A, 2018, PROCEDIA COMPUTER SCIENCE', 'Wang S, 2020, IEEE TRANSACTIONS ON SERVICES COMPUTING', 'Ramaswamy S, 2018, PROCEDIA COMPUTER SCIENCE', 'Heinrich K, 2021, DECISION SUPPORT SYSTEMS', 'Fuchs D, 2018, ', 'Fischer M, 2020, ELECTRONIC MARKETS', 'Selz D, 2020, ELECTRONIC MARKETS', 'Wu M, 2018, ', 'Leijnen S, 2020, PROCEEDINGS', 'Wanner J, 2020, JOURNAL OF THE ASSOCIATION FOR INFORMATION SYSTEMS', 'Duin R, 1994, PATTERN RECOGNITION LETTERS', 'Heinrich K, 2019, JOURNAL OF THE ASSOCIATION FOR INFORMATION SYSTEMS', 'Heinrich K, 2020, JOURNAL OF THE ASSOCIATION FOR INFORMATION SYSTEMS', 'Haselton M, 2015, ', 'Widmer G, 1996, MACHINE LEARNING']</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr">
         <is>
           <t>OPENALEX</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>Christian Janiesch, 2021, Electronic Markets</t>
-        </is>
-      </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>Christian Janiesch, 2021, Electronic Markets</t>
+          <t>Janiesch C, 2021, ELECTRONIC MARKETS</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>Janiesch C, 2021, ELECTRONIC MARKETS</t>
         </is>
       </c>
     </row>

</xml_diff>